<commit_message>
Updated dataset to latest IndyCar results and trained new models
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79064C1-D40F-499D-8B73-BC87BDB142F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCD4F19-A542-41C9-8920-BC90C4F1598A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy_Model" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="90">
   <si>
     <t>Model</t>
   </si>
@@ -310,11 +310,17 @@
   <si>
     <t>Streets of Long Beach</t>
   </si>
+  <si>
+    <t>Indianapolis Motor Speedway (Road)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -397,7 +403,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -428,6 +434,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1284,28 +1292,28 @@
         <v>87</v>
       </c>
       <c r="B14" s="1">
-        <v>0.2475</v>
+        <v>0.26190000000000002</v>
       </c>
       <c r="C14" s="1">
-        <v>3.8199999999999998E-2</v>
+        <v>-0.11269999999999999</v>
       </c>
       <c r="D14" s="1">
-        <v>0.2576</v>
+        <v>0.25779999999999997</v>
       </c>
       <c r="E14" s="1">
-        <v>2.2200000000000001E-2</v>
+        <v>2.24E-2</v>
       </c>
       <c r="F14" s="1">
-        <v>0.2248</v>
+        <v>0.25309999999999999</v>
       </c>
       <c r="G14" s="1">
-        <v>0.1782</v>
+        <v>4.5400000000000003E-2</v>
       </c>
       <c r="H14" s="1">
-        <v>0.2321</v>
+        <v>0.2545</v>
       </c>
       <c r="I14" s="1">
-        <v>0.1192</v>
+        <v>3.6600000000000001E-2</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1313,28 +1321,28 @@
         <v>10</v>
       </c>
       <c r="B15" s="1">
-        <v>0.24349999999999999</v>
+        <v>0.24390000000000001</v>
       </c>
       <c r="C15" s="1">
-        <v>8.4599999999999995E-2</v>
+        <v>8.5800000000000001E-2</v>
       </c>
       <c r="D15" s="1">
         <v>0.2361</v>
       </c>
       <c r="E15" s="1">
-        <v>0.13930000000000001</v>
+        <v>0.1421</v>
       </c>
       <c r="F15" s="1">
-        <v>0.21659999999999999</v>
+        <v>0.2165</v>
       </c>
       <c r="G15" s="1">
-        <v>0.2492</v>
+        <v>0.25069999999999998</v>
       </c>
       <c r="H15" s="1">
-        <v>0.22140000000000001</v>
+        <v>0.22209999999999999</v>
       </c>
       <c r="I15" s="1">
-        <v>0.20899999999999999</v>
+        <v>0.20180000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1342,28 +1350,28 @@
         <v>4</v>
       </c>
       <c r="B16" s="1">
-        <v>0.24379999999999999</v>
+        <v>0.245</v>
       </c>
       <c r="C16" s="1">
-        <v>6.1800000000000001E-2</v>
+        <v>5.57E-2</v>
       </c>
       <c r="D16" s="1">
-        <v>0.24030000000000001</v>
+        <v>0.2417</v>
       </c>
       <c r="E16" s="1">
-        <v>0.11940000000000001</v>
+        <v>0.115</v>
       </c>
       <c r="F16" s="1">
-        <v>0.21870000000000001</v>
+        <v>0.218</v>
       </c>
       <c r="G16" s="1">
-        <v>0.22989999999999999</v>
+        <v>0.2334</v>
       </c>
       <c r="H16" s="1">
-        <v>0.22739999999999999</v>
+        <v>0.22789999999999999</v>
       </c>
       <c r="I16" s="1">
-        <v>0.18379999999999999</v>
+        <v>0.18210000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1371,28 +1379,28 @@
         <v>8</v>
       </c>
       <c r="B17" s="1">
-        <v>0.24540000000000001</v>
+        <v>0.24790000000000001</v>
       </c>
       <c r="C17" s="1">
-        <v>4.8500000000000001E-2</v>
+        <v>3.0700000000000002E-2</v>
       </c>
       <c r="D17" s="1">
-        <v>0.23619999999999999</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="E17" s="1">
-        <v>0.12959999999999999</v>
+        <v>0.1263</v>
       </c>
       <c r="F17" s="1">
-        <v>0.21279999999999999</v>
+        <v>0.21560000000000001</v>
       </c>
       <c r="G17" s="1">
-        <v>0.25569999999999998</v>
+        <v>0.25009999999999999</v>
       </c>
       <c r="H17" s="1">
-        <v>0.21859999999999999</v>
+        <v>0.21990000000000001</v>
       </c>
       <c r="I17" s="1">
-        <v>0.19789999999999999</v>
+        <v>0.20269999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1400,28 +1408,28 @@
         <v>9</v>
       </c>
       <c r="B18" s="1">
-        <v>0.24879999999999999</v>
+        <v>0.246</v>
       </c>
       <c r="C18" s="1">
-        <v>-1.9E-3</v>
+        <v>2.5399999999999999E-2</v>
       </c>
       <c r="D18" s="1">
-        <v>0.23580000000000001</v>
+        <v>0.23569999999999999</v>
       </c>
       <c r="E18" s="1">
-        <v>0.1399</v>
+        <v>0.13930000000000001</v>
       </c>
       <c r="F18" s="1">
-        <v>0.2142</v>
+        <v>0.21390000000000001</v>
       </c>
       <c r="G18" s="1">
-        <v>0.25230000000000002</v>
+        <v>0.25159999999999999</v>
       </c>
       <c r="H18" s="1">
-        <v>0.22040000000000001</v>
+        <v>0.219</v>
       </c>
       <c r="I18" s="1">
-        <v>0.1983</v>
+        <v>0.1976</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1432,25 +1440,25 @@
         <v>0.2356</v>
       </c>
       <c r="C19" s="1">
-        <v>0.1429</v>
+        <v>0.14410000000000001</v>
       </c>
       <c r="D19" s="1">
-        <v>0.2356</v>
+        <v>0.23569999999999999</v>
       </c>
       <c r="E19" s="1">
-        <v>0.14280000000000001</v>
+        <v>0.14419999999999999</v>
       </c>
       <c r="F19" s="1">
-        <v>0.2152</v>
+        <v>0.21490000000000001</v>
       </c>
       <c r="G19" s="1">
-        <v>0.25259999999999999</v>
+        <v>0.25330000000000003</v>
       </c>
       <c r="H19" s="1">
-        <v>0.22090000000000001</v>
+        <v>0.22070000000000001</v>
       </c>
       <c r="I19" s="1">
-        <v>0.20549999999999999</v>
+        <v>0.20180000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1458,28 +1466,28 @@
         <v>15</v>
       </c>
       <c r="B20" s="1">
-        <v>0.2354</v>
+        <v>0.23569999999999999</v>
       </c>
       <c r="C20" s="1">
-        <v>0.14199999999999999</v>
+        <v>0.14149999999999999</v>
       </c>
       <c r="D20" s="1">
-        <v>0.23549999999999999</v>
+        <v>0.23569999999999999</v>
       </c>
       <c r="E20" s="1">
-        <v>0.14299999999999999</v>
+        <v>0.14369999999999999</v>
       </c>
       <c r="F20" s="1">
-        <v>0.21429999999999999</v>
+        <v>0.2147</v>
       </c>
       <c r="G20" s="1">
-        <v>0.25559999999999999</v>
+        <v>0.25490000000000002</v>
       </c>
       <c r="H20" s="1">
-        <v>0.2205</v>
+        <v>0.2198</v>
       </c>
       <c r="I20" s="1">
-        <v>0.20569999999999999</v>
+        <v>0.20380000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1487,28 +1495,28 @@
         <v>12</v>
       </c>
       <c r="B21" s="1">
-        <v>0.23680000000000001</v>
+        <v>0.23730000000000001</v>
       </c>
       <c r="C21" s="1">
-        <v>0.1386</v>
+        <v>0.13850000000000001</v>
       </c>
       <c r="D21" s="1">
-        <v>0.23630000000000001</v>
+        <v>0.2366</v>
       </c>
       <c r="E21" s="1">
-        <v>0.14069999999999999</v>
+        <v>0.14119999999999999</v>
       </c>
       <c r="F21" s="1">
-        <v>0.21679999999999999</v>
+        <v>0.2165</v>
       </c>
       <c r="G21" s="1">
-        <v>0.24829999999999999</v>
+        <v>0.24959999999999999</v>
       </c>
       <c r="H21" s="1">
-        <v>0.222</v>
+        <v>0.22170000000000001</v>
       </c>
       <c r="I21" s="1">
-        <v>0.20369999999999999</v>
+        <v>0.20050000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1516,28 +1524,28 @@
         <v>13</v>
       </c>
       <c r="B22" s="1">
-        <v>0.23630000000000001</v>
+        <v>0.2369</v>
       </c>
       <c r="C22" s="1">
-        <v>0.13969999999999999</v>
+        <v>0.13850000000000001</v>
       </c>
       <c r="D22" s="1">
-        <v>0.23569999999999999</v>
+        <v>0.2361</v>
       </c>
       <c r="E22" s="1">
-        <v>0.1416</v>
+        <v>0.1406</v>
       </c>
       <c r="F22" s="1">
-        <v>0.21490000000000001</v>
+        <v>0.21679999999999999</v>
       </c>
       <c r="G22" s="1">
-        <v>0.254</v>
+        <v>0.2495</v>
       </c>
       <c r="H22" s="1">
-        <v>0.2205</v>
+        <v>0.22009999999999999</v>
       </c>
       <c r="I22" s="1">
-        <v>0.2039</v>
+        <v>0.20280000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1545,28 +1553,28 @@
         <v>14</v>
       </c>
       <c r="B23" s="1">
-        <v>0.23569999999999999</v>
+        <v>0.2361</v>
       </c>
       <c r="C23" s="1">
-        <v>0.1389</v>
+        <v>0.13850000000000001</v>
       </c>
       <c r="D23" s="1">
-        <v>0.2359</v>
+        <v>0.23599999999999999</v>
       </c>
       <c r="E23" s="1">
-        <v>0.14030000000000001</v>
+        <v>0.1416</v>
       </c>
       <c r="F23" s="1">
-        <v>0.2145</v>
+        <v>0.21560000000000001</v>
       </c>
       <c r="G23" s="1">
-        <v>0.25490000000000002</v>
+        <v>0.2535</v>
       </c>
       <c r="H23" s="1">
-        <v>0.21970000000000001</v>
+        <v>0.2203</v>
       </c>
       <c r="I23" s="1">
-        <v>0.20610000000000001</v>
+        <v>0.20499999999999999</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1574,28 +1582,28 @@
         <v>58</v>
       </c>
       <c r="B24" s="1">
-        <v>0.23549999999999999</v>
+        <v>0.23580000000000001</v>
       </c>
       <c r="C24" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.1376</v>
       </c>
       <c r="D24" s="1">
-        <v>0.23549999999999999</v>
+        <v>0.23569999999999999</v>
       </c>
       <c r="E24" s="1">
-        <v>0.14119999999999999</v>
+        <v>0.13980000000000001</v>
       </c>
       <c r="F24" s="1">
-        <v>0.21329999999999999</v>
+        <v>0.2142</v>
       </c>
       <c r="G24" s="1">
-        <v>0.25690000000000002</v>
+        <v>0.25490000000000002</v>
       </c>
       <c r="H24" s="1">
         <v>0.21909999999999999</v>
       </c>
       <c r="I24" s="1">
-        <v>0.2019</v>
+        <v>0.2026</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1676,12 +1684,23 @@
         <v>0.20610000000000001</v>
       </c>
       <c r="G30" s="5">
-        <f>D30*25</f>
-        <v>5.4924999999999997</v>
+        <f>D31*25</f>
+        <v>5.4775</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="E31" s="5"/>
+      <c r="A31" s="4">
+        <v>46151</v>
+      </c>
+      <c r="B31" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31">
+        <v>0.21909999999999999</v>
+      </c>
+      <c r="E31" s="14">
+        <v>0.2026</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1749,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80150BC0-64DC-411B-A1B1-FAD28F14CD71}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10.20703125" bestFit="1" customWidth="1"/>
@@ -1812,25 +1831,25 @@
         <v>0.2349</v>
       </c>
       <c r="C3" s="1">
-        <v>0.13819999999999999</v>
+        <v>0.1376</v>
       </c>
       <c r="D3" s="1">
-        <v>0.23119999999999999</v>
+        <v>0.2344</v>
       </c>
       <c r="E3" s="1">
-        <v>0.16539999999999999</v>
+        <v>0.16039999999999999</v>
       </c>
       <c r="F3" s="1">
-        <v>0.2152</v>
+        <v>0.2155</v>
       </c>
       <c r="G3" s="1">
-        <v>0.25700000000000001</v>
+        <v>0.254</v>
       </c>
       <c r="H3" s="1">
-        <v>0.21540000000000001</v>
+        <v>0.21690000000000001</v>
       </c>
       <c r="I3" s="1">
-        <v>0.2346</v>
+        <v>0.2303</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1838,28 +1857,28 @@
         <v>17</v>
       </c>
       <c r="B4" s="1">
-        <v>0.2364</v>
+        <v>0.2374</v>
       </c>
       <c r="C4" s="1">
-        <v>0.12909999999999999</v>
+        <v>0.1278</v>
       </c>
       <c r="D4" s="1">
-        <v>0.2319</v>
+        <v>0.23269999999999999</v>
       </c>
       <c r="E4" s="1">
-        <v>0.16619999999999999</v>
+        <v>0.1638</v>
       </c>
       <c r="F4" s="1">
-        <v>0.21249999999999999</v>
+        <v>0.2127</v>
       </c>
       <c r="G4" s="1">
-        <v>0.27650000000000002</v>
+        <v>0.27310000000000001</v>
       </c>
       <c r="H4" s="1">
-        <v>0.21279999999999999</v>
+        <v>0.21540000000000001</v>
       </c>
       <c r="I4" s="1">
-        <v>0.26069999999999999</v>
+        <v>0.2452</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1867,28 +1886,28 @@
         <v>18</v>
       </c>
       <c r="B5" s="1">
+        <v>0.23669999999999999</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.1069</v>
+      </c>
+      <c r="D5" s="1">
         <v>0.23749999999999999</v>
       </c>
-      <c r="C5" s="1">
-        <v>9.7600000000000006E-2</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0.2364</v>
-      </c>
       <c r="E5" s="1">
-        <v>0.14749999999999999</v>
+        <v>0.1434</v>
       </c>
       <c r="F5" s="1">
-        <v>0.2117</v>
+        <v>0.21060000000000001</v>
       </c>
       <c r="G5" s="1">
-        <v>0.26329999999999998</v>
+        <v>0.26910000000000001</v>
       </c>
       <c r="H5" s="1">
-        <v>0.2107</v>
+        <v>0.21879999999999999</v>
       </c>
       <c r="I5" s="1">
-        <v>0.26879999999999998</v>
+        <v>0.2392</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1896,28 +1915,28 @@
         <v>19</v>
       </c>
       <c r="B6" s="1">
-        <v>0.23980000000000001</v>
+        <v>0.23949999999999999</v>
       </c>
       <c r="C6" s="1">
-        <v>7.8600000000000003E-2</v>
+        <v>8.3099999999999993E-2</v>
       </c>
       <c r="D6" s="1">
-        <v>0.2301</v>
+        <v>0.23100000000000001</v>
       </c>
       <c r="E6" s="1">
-        <v>0.18809999999999999</v>
+        <v>0.1593</v>
       </c>
       <c r="F6" s="1">
-        <v>0.2069</v>
+        <v>0.2054</v>
       </c>
       <c r="G6" s="1">
-        <v>0.27739999999999998</v>
+        <v>0.29480000000000001</v>
       </c>
       <c r="H6" s="1">
-        <v>0.2074</v>
+        <v>0.2077</v>
       </c>
       <c r="I6" s="1">
-        <v>0.25650000000000001</v>
+        <v>0.26979999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1925,28 +1944,28 @@
         <v>20</v>
       </c>
       <c r="B7" s="1">
-        <v>0.24179999999999999</v>
+        <v>0.2424</v>
       </c>
       <c r="C7" s="1">
-        <v>5.0799999999999998E-2</v>
+        <v>5.2400000000000002E-2</v>
       </c>
       <c r="D7" s="1">
-        <v>0.23019999999999999</v>
+        <v>0.23</v>
       </c>
       <c r="E7" s="1">
-        <v>0.16880000000000001</v>
+        <v>0.17080000000000001</v>
       </c>
       <c r="F7" s="1">
-        <v>0.2069</v>
+        <v>0.20619999999999999</v>
       </c>
       <c r="G7" s="1">
-        <v>0.29609999999999997</v>
+        <v>0.29239999999999999</v>
       </c>
       <c r="H7" s="1">
-        <v>0.20660000000000001</v>
+        <v>0.20630000000000001</v>
       </c>
       <c r="I7" s="1">
-        <v>0.28029999999999999</v>
+        <v>0.26950000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1954,28 +1973,28 @@
         <v>24</v>
       </c>
       <c r="B8" s="1">
-        <v>0.22589999999999999</v>
+        <v>0.22639999999999999</v>
       </c>
       <c r="C8" s="1">
-        <v>0.17180000000000001</v>
+        <v>0.17030000000000001</v>
       </c>
       <c r="D8" s="1">
-        <v>0.22550000000000001</v>
+        <v>0.22650000000000001</v>
       </c>
       <c r="E8" s="1">
-        <v>0.17180000000000001</v>
+        <v>0.17030000000000001</v>
       </c>
       <c r="F8" s="1">
-        <v>0.2026</v>
+        <v>0.20230000000000001</v>
       </c>
       <c r="G8" s="1">
-        <v>0.28439999999999999</v>
+        <v>0.28520000000000001</v>
       </c>
       <c r="H8" s="1">
-        <v>0.20530000000000001</v>
+        <v>0.20469999999999999</v>
       </c>
       <c r="I8" s="1">
-        <v>0.25819999999999999</v>
+        <v>0.25359999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1983,28 +2002,28 @@
         <v>21</v>
       </c>
       <c r="B9" s="1">
-        <v>0.2306</v>
+        <v>0.23100000000000001</v>
       </c>
       <c r="C9" s="1">
-        <v>0.17130000000000001</v>
+        <v>0.17119999999999999</v>
       </c>
       <c r="D9" s="1">
-        <v>0.23050000000000001</v>
+        <v>0.2303</v>
       </c>
       <c r="E9" s="1">
-        <v>0.1714</v>
+        <v>0.1719</v>
       </c>
       <c r="F9" s="1">
-        <v>0.20899999999999999</v>
+        <v>0.20710000000000001</v>
       </c>
       <c r="G9" s="1">
-        <v>0.29120000000000001</v>
+        <v>0.2913</v>
       </c>
       <c r="H9" s="1">
-        <v>0.20880000000000001</v>
+        <v>0.2077</v>
       </c>
       <c r="I9" s="1">
-        <v>0.27500000000000002</v>
+        <v>0.26750000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2012,28 +2031,28 @@
         <v>22</v>
       </c>
       <c r="B10" s="1">
-        <v>0.23</v>
+        <v>0.23050000000000001</v>
       </c>
       <c r="C10" s="1">
-        <v>0.17280000000000001</v>
+        <v>0.1714</v>
       </c>
       <c r="D10" s="1">
-        <v>0.2301</v>
+        <v>0.23019999999999999</v>
       </c>
       <c r="E10" s="1">
-        <v>0.17280000000000001</v>
+        <v>0.17249999999999999</v>
       </c>
       <c r="F10" s="1">
-        <v>0.2082</v>
+        <v>0.20680000000000001</v>
       </c>
       <c r="G10" s="1">
-        <v>0.2893</v>
+        <v>0.29339999999999999</v>
       </c>
       <c r="H10" s="1">
-        <v>0.20799999999999999</v>
+        <v>0.2077</v>
       </c>
       <c r="I10" s="1">
-        <v>0.27229999999999999</v>
+        <v>0.26939999999999997</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2041,28 +2060,28 @@
         <v>52</v>
       </c>
       <c r="B11" s="1">
-        <v>0.2296</v>
+        <v>0.23039999999999999</v>
       </c>
       <c r="C11" s="1">
-        <v>0.1749</v>
+        <v>0.17519999999999999</v>
       </c>
       <c r="D11" s="1">
-        <v>0.2291</v>
+        <v>0.2298</v>
       </c>
       <c r="E11" s="1">
-        <v>0.1779</v>
+        <v>0.1774</v>
       </c>
       <c r="F11" s="1">
-        <v>0.2074</v>
+        <v>0.20799999999999999</v>
       </c>
       <c r="G11" s="1">
-        <v>0.29459999999999997</v>
+        <v>0.29249999999999998</v>
       </c>
       <c r="H11" s="1">
-        <v>0.2077</v>
+        <v>0.20899999999999999</v>
       </c>
       <c r="I11" s="1">
-        <v>0.2787</v>
+        <v>0.2681</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2070,13 +2089,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="1">
-        <v>0.2276</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="C12" s="1">
-        <v>0.17829999999999999</v>
+        <v>0.17749999999999999</v>
       </c>
       <c r="D12" s="1">
-        <v>0.22670000000000001</v>
+        <v>0.2273</v>
       </c>
       <c r="E12" s="1">
         <v>0.17929999999999999</v>
@@ -2085,13 +2104,13 @@
         <v>0.20369999999999999</v>
       </c>
       <c r="G12" s="1">
-        <v>0.29289999999999999</v>
+        <v>0.2979</v>
       </c>
       <c r="H12" s="1">
-        <v>0.2056</v>
+        <v>0.20519999999999999</v>
       </c>
       <c r="I12" s="1">
-        <v>0.2727</v>
+        <v>0.27210000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2099,28 +2118,28 @@
         <v>23</v>
       </c>
       <c r="B13" s="1">
-        <v>0.22919999999999999</v>
+        <v>0.2296</v>
       </c>
       <c r="C13" s="1">
-        <v>0.17849999999999999</v>
+        <v>0.17710000000000001</v>
       </c>
       <c r="D13" s="1">
-        <v>0.2278</v>
+        <v>0.2281</v>
       </c>
       <c r="E13" s="1">
-        <v>0.18099999999999999</v>
+        <v>0.1797</v>
       </c>
       <c r="F13" s="1">
         <v>0.20619999999999999</v>
       </c>
       <c r="G13" s="1">
-        <v>0.29459999999999997</v>
+        <v>0.29249999999999998</v>
       </c>
       <c r="H13" s="1">
-        <v>0.20730000000000001</v>
+        <v>0.2079</v>
       </c>
       <c r="I13" s="1">
-        <v>0.27200000000000002</v>
+        <v>0.2661</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2128,28 +2147,28 @@
         <v>56</v>
       </c>
       <c r="B14" s="1">
-        <v>0.23139999999999999</v>
+        <v>0.23280000000000001</v>
       </c>
       <c r="C14" s="1">
-        <v>0.1638</v>
+        <v>0.1661</v>
       </c>
       <c r="D14" s="1">
-        <v>0.23089999999999999</v>
+        <v>0.23200000000000001</v>
       </c>
       <c r="E14" s="1">
-        <v>0.16880000000000001</v>
+        <v>0.1686</v>
       </c>
       <c r="F14" s="1">
-        <v>0.20930000000000001</v>
+        <v>0.2109</v>
       </c>
       <c r="G14" s="1">
-        <v>0.29020000000000001</v>
+        <v>0.28249999999999997</v>
       </c>
       <c r="H14" s="1">
-        <v>0.20910000000000001</v>
+        <v>0.2117</v>
       </c>
       <c r="I14" s="1">
-        <v>0.28120000000000001</v>
+        <v>0.26019999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2157,28 +2176,28 @@
         <v>60</v>
       </c>
       <c r="B15" s="1">
-        <v>0.23069999999999999</v>
+        <v>0.2319</v>
       </c>
       <c r="C15" s="1">
-        <v>0.16719999999999999</v>
+        <v>0.16830000000000001</v>
       </c>
       <c r="D15" s="1">
-        <v>0.23</v>
+        <v>0.23080000000000001</v>
       </c>
       <c r="E15" s="1">
-        <v>0.17199999999999999</v>
+        <v>0.17130000000000001</v>
       </c>
       <c r="F15" s="1">
-        <v>0.2077</v>
+        <v>0.2079</v>
       </c>
       <c r="G15" s="1">
-        <v>0.29189999999999999</v>
+        <v>0.2918</v>
       </c>
       <c r="H15" s="1">
-        <v>0.20730000000000001</v>
+        <v>0.2087</v>
       </c>
       <c r="I15" s="1">
-        <v>0.27800000000000002</v>
+        <v>0.26889999999999997</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2186,28 +2205,28 @@
         <v>54</v>
       </c>
       <c r="B16" s="1">
-        <v>0.2303</v>
+        <v>0.23119999999999999</v>
       </c>
       <c r="C16" s="1">
-        <v>0.1704</v>
+        <v>0.16769999999999999</v>
       </c>
       <c r="D16" s="1">
-        <v>0.23050000000000001</v>
+        <v>0.23130000000000001</v>
       </c>
       <c r="E16" s="1">
-        <v>0.17050000000000001</v>
+        <v>0.16789999999999999</v>
       </c>
       <c r="F16" s="1">
-        <v>0.2092</v>
+        <v>0.20849999999999999</v>
       </c>
       <c r="G16" s="1">
-        <v>0.2828</v>
+        <v>0.28920000000000001</v>
       </c>
       <c r="H16" s="1">
-        <v>0.2092</v>
+        <v>0.21049999999999999</v>
       </c>
       <c r="I16" s="1">
-        <v>0.2651</v>
+        <v>0.26319999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2215,28 +2234,28 @@
         <v>57</v>
       </c>
       <c r="B17" s="1">
-        <v>0.2296</v>
+        <v>0.22989999999999999</v>
       </c>
       <c r="C17" s="1">
-        <v>0.1714</v>
+        <v>0.17030000000000001</v>
       </c>
       <c r="D17" s="1">
-        <v>0.2296</v>
+        <v>0.22989999999999999</v>
       </c>
       <c r="E17" s="1">
         <v>0.1719</v>
       </c>
       <c r="F17" s="1">
-        <v>0.20649999999999999</v>
+        <v>0.2054</v>
       </c>
       <c r="G17" s="1">
-        <v>0.29339999999999999</v>
+        <v>0.29659999999999997</v>
       </c>
       <c r="H17" s="1">
-        <v>0.20610000000000001</v>
+        <v>0.2064</v>
       </c>
       <c r="I17" s="1">
-        <v>0.27639999999999998</v>
+        <v>0.27300000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2244,28 +2263,28 @@
         <v>55</v>
       </c>
       <c r="B18" s="1">
-        <v>0.2291</v>
+        <v>0.23019999999999999</v>
       </c>
       <c r="C18" s="1">
-        <v>0.17430000000000001</v>
+        <v>0.17480000000000001</v>
       </c>
       <c r="D18" s="1">
-        <v>0.2276</v>
+        <v>0.22839999999999999</v>
       </c>
       <c r="E18" s="1">
-        <v>0.17860000000000001</v>
+        <v>0.1777</v>
       </c>
       <c r="F18" s="1">
-        <v>0.2049</v>
+        <v>0.20480000000000001</v>
       </c>
       <c r="G18" s="1">
-        <v>0.29260000000000003</v>
+        <v>0.29680000000000001</v>
       </c>
       <c r="H18" s="1">
-        <v>0.20599999999999999</v>
+        <v>0.20630000000000001</v>
       </c>
       <c r="I18" s="1">
-        <v>0.2737</v>
+        <v>0.27079999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2273,28 +2292,28 @@
         <v>59</v>
       </c>
       <c r="B19" s="1">
-        <v>0.23169999999999999</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="C19" s="1">
-        <v>0.15609999999999999</v>
+        <v>0.1651</v>
       </c>
       <c r="D19" s="1">
-        <v>0.23039999999999999</v>
+        <v>0.23119999999999999</v>
       </c>
       <c r="E19" s="1">
-        <v>0.16880000000000001</v>
+        <v>0.17030000000000001</v>
       </c>
       <c r="F19" s="1">
-        <v>0.2074</v>
+        <v>0.20860000000000001</v>
       </c>
       <c r="G19" s="1">
-        <v>0.29480000000000001</v>
+        <v>0.28899999999999998</v>
       </c>
       <c r="H19" s="1">
-        <v>0.20699999999999999</v>
+        <v>0.20849999999999999</v>
       </c>
       <c r="I19" s="1">
-        <v>0.28510000000000002</v>
+        <v>0.26869999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2302,92 +2321,129 @@
         <v>61</v>
       </c>
       <c r="B20" s="1">
-        <v>0.23230000000000001</v>
+        <v>0.2334</v>
       </c>
       <c r="C20" s="1">
-        <v>0.14779999999999999</v>
+        <v>0.16070000000000001</v>
       </c>
       <c r="D20" s="1">
-        <v>0.2301</v>
+        <v>0.23169999999999999</v>
       </c>
       <c r="E20" s="1">
-        <v>0.16239999999999999</v>
+        <v>0.16200000000000001</v>
       </c>
       <c r="F20" s="1">
-        <v>0.2069</v>
+        <v>0.2077</v>
       </c>
       <c r="G20" s="1">
-        <v>0.2777</v>
+        <v>0.29160000000000003</v>
       </c>
       <c r="H20" s="1">
-        <v>0.20810000000000001</v>
+        <v>0.2092</v>
       </c>
       <c r="I20" s="1">
-        <v>0.27689999999999998</v>
+        <v>0.26889999999999997</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="C21" t="s">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="C22" t="s">
         <v>1</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D22" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="4">
-        <v>46085</v>
-      </c>
-      <c r="B22" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22">
-        <v>0.2147</v>
-      </c>
-      <c r="D22">
-        <v>0.2006</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="4">
-        <v>46090</v>
+        <v>46085</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C23">
-        <v>0.2142</v>
+        <v>0.2147</v>
       </c>
       <c r="D23">
-        <v>0.2334</v>
+        <v>0.2006</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="4">
-        <v>46098</v>
+        <v>46090</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C24">
-        <v>0.20810000000000001</v>
+        <v>0.2142</v>
       </c>
       <c r="D24">
-        <v>0.24890000000000001</v>
+        <v>0.2334</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="4">
-        <v>46112</v>
+        <v>46098</v>
       </c>
       <c r="B25" t="s">
         <v>53</v>
       </c>
       <c r="C25">
+        <v>0.20810000000000001</v>
+      </c>
+      <c r="D25">
+        <v>0.24890000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="4">
+        <v>46112</v>
+      </c>
+      <c r="B26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26">
         <v>0.2056</v>
       </c>
-      <c r="D25">
+      <c r="D26">
         <v>0.2727</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" s="4">
+        <v>46151</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27">
+        <v>0.20519999999999999</v>
+      </c>
+      <c r="D27">
+        <v>0.27210000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2397,31 +2453,31 @@
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:I1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B3:B20">
+  <conditionalFormatting sqref="B3:B21">
     <cfRule type="top10" dxfId="8" priority="46" bottom="1" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C20">
+  <conditionalFormatting sqref="C3:C21">
     <cfRule type="top10" dxfId="7" priority="117" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D20 D23:D25">
+  <conditionalFormatting sqref="D3:D21 D24:D27">
     <cfRule type="top10" dxfId="6" priority="6" bottom="1" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E20">
+  <conditionalFormatting sqref="E3:E21">
     <cfRule type="top10" dxfId="5" priority="3" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E22">
+  <conditionalFormatting sqref="E23">
     <cfRule type="top10" dxfId="4" priority="14" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F20">
+  <conditionalFormatting sqref="F3:F21">
     <cfRule type="top10" dxfId="3" priority="5" bottom="1" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G20">
+  <conditionalFormatting sqref="G3:G21">
     <cfRule type="top10" dxfId="2" priority="2" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H20">
+  <conditionalFormatting sqref="H3:H21">
     <cfRule type="top10" dxfId="1" priority="4" bottom="1" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I20">
+  <conditionalFormatting sqref="I3:I21">
     <cfRule type="top10" dxfId="0" priority="1" rank="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7638,105 +7694,480 @@
       <c r="O126" s="5"/>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F127">
+        <v>1</v>
+      </c>
       <c r="H127" s="8"/>
+      <c r="I127" t="s">
+        <v>89</v>
+      </c>
+      <c r="J127" t="s">
+        <v>76</v>
+      </c>
+      <c r="K127" t="s">
+        <v>77</v>
+      </c>
+      <c r="L127">
+        <v>5.48</v>
+      </c>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F128">
+        <v>2</v>
+      </c>
       <c r="H128" s="8"/>
-    </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I128" t="s">
+        <v>89</v>
+      </c>
+      <c r="J128" t="s">
+        <v>76</v>
+      </c>
+      <c r="K128" t="s">
+        <v>77</v>
+      </c>
+      <c r="L128">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="129" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F129">
+        <v>3</v>
+      </c>
       <c r="H129" s="8"/>
-    </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I129" t="s">
+        <v>89</v>
+      </c>
+      <c r="J129" t="s">
+        <v>76</v>
+      </c>
+      <c r="K129" t="s">
+        <v>77</v>
+      </c>
+      <c r="L129">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="130" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F130">
+        <v>4</v>
+      </c>
       <c r="H130" s="8"/>
-    </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I130" t="s">
+        <v>89</v>
+      </c>
+      <c r="J130" t="s">
+        <v>76</v>
+      </c>
+      <c r="K130" t="s">
+        <v>77</v>
+      </c>
+      <c r="L130">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="131" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F131">
+        <v>5</v>
+      </c>
       <c r="H131" s="8"/>
-    </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I131" t="s">
+        <v>89</v>
+      </c>
+      <c r="J131" t="s">
+        <v>76</v>
+      </c>
+      <c r="K131" t="s">
+        <v>77</v>
+      </c>
+      <c r="L131">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="132" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F132">
+        <v>6</v>
+      </c>
       <c r="H132" s="8"/>
-    </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I132" t="s">
+        <v>89</v>
+      </c>
+      <c r="J132" t="s">
+        <v>76</v>
+      </c>
+      <c r="K132" t="s">
+        <v>77</v>
+      </c>
+      <c r="L132">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="133" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F133">
+        <v>7</v>
+      </c>
       <c r="H133" s="8"/>
-    </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I133" t="s">
+        <v>89</v>
+      </c>
+      <c r="J133" t="s">
+        <v>76</v>
+      </c>
+      <c r="K133" t="s">
+        <v>77</v>
+      </c>
+      <c r="L133">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="134" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F134">
+        <v>8</v>
+      </c>
       <c r="H134" s="8"/>
-    </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I134" t="s">
+        <v>89</v>
+      </c>
+      <c r="J134" t="s">
+        <v>76</v>
+      </c>
+      <c r="K134" t="s">
+        <v>77</v>
+      </c>
+      <c r="L134">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="135" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F135">
+        <v>9</v>
+      </c>
       <c r="H135" s="8"/>
-    </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I135" t="s">
+        <v>89</v>
+      </c>
+      <c r="J135" t="s">
+        <v>76</v>
+      </c>
+      <c r="K135" t="s">
+        <v>77</v>
+      </c>
+      <c r="L135">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="136" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F136">
+        <v>10</v>
+      </c>
       <c r="H136" s="8"/>
-    </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I136" t="s">
+        <v>89</v>
+      </c>
+      <c r="J136" t="s">
+        <v>76</v>
+      </c>
+      <c r="K136" t="s">
+        <v>77</v>
+      </c>
+      <c r="L136">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="137" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F137">
+        <v>11</v>
+      </c>
       <c r="H137" s="8"/>
-    </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I137" t="s">
+        <v>89</v>
+      </c>
+      <c r="J137" t="s">
+        <v>76</v>
+      </c>
+      <c r="K137" t="s">
+        <v>77</v>
+      </c>
+      <c r="L137">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="138" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F138">
+        <v>12</v>
+      </c>
       <c r="H138" s="8"/>
-    </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I138" t="s">
+        <v>89</v>
+      </c>
+      <c r="J138" t="s">
+        <v>76</v>
+      </c>
+      <c r="K138" t="s">
+        <v>77</v>
+      </c>
+      <c r="L138">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="139" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F139">
+        <v>13</v>
+      </c>
       <c r="H139" s="8"/>
-    </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I139" t="s">
+        <v>89</v>
+      </c>
+      <c r="J139" t="s">
+        <v>76</v>
+      </c>
+      <c r="K139" t="s">
+        <v>77</v>
+      </c>
+      <c r="L139">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="140" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F140">
+        <v>14</v>
+      </c>
       <c r="H140" s="8"/>
-    </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I140" t="s">
+        <v>89</v>
+      </c>
+      <c r="J140" t="s">
+        <v>76</v>
+      </c>
+      <c r="K140" t="s">
+        <v>77</v>
+      </c>
+      <c r="L140">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="141" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F141">
+        <v>15</v>
+      </c>
       <c r="H141" s="8"/>
-    </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I141" t="s">
+        <v>89</v>
+      </c>
+      <c r="J141" t="s">
+        <v>76</v>
+      </c>
+      <c r="K141" t="s">
+        <v>77</v>
+      </c>
+      <c r="L141">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="142" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F142">
+        <v>16</v>
+      </c>
       <c r="H142" s="8"/>
-    </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I142" t="s">
+        <v>89</v>
+      </c>
+      <c r="J142" t="s">
+        <v>76</v>
+      </c>
+      <c r="K142" t="s">
+        <v>77</v>
+      </c>
+      <c r="L142">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="143" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F143">
+        <v>17</v>
+      </c>
       <c r="H143" s="8"/>
-    </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I143" t="s">
+        <v>89</v>
+      </c>
+      <c r="J143" t="s">
+        <v>76</v>
+      </c>
+      <c r="K143" t="s">
+        <v>77</v>
+      </c>
+      <c r="L143">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="144" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F144">
+        <v>18</v>
+      </c>
       <c r="H144" s="8"/>
-    </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I144" t="s">
+        <v>89</v>
+      </c>
+      <c r="J144" t="s">
+        <v>76</v>
+      </c>
+      <c r="K144" t="s">
+        <v>77</v>
+      </c>
+      <c r="L144">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="145" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F145">
+        <v>19</v>
+      </c>
       <c r="H145" s="8"/>
-    </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I145" t="s">
+        <v>89</v>
+      </c>
+      <c r="J145" t="s">
+        <v>76</v>
+      </c>
+      <c r="K145" t="s">
+        <v>77</v>
+      </c>
+      <c r="L145">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="146" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F146">
+        <v>20</v>
+      </c>
       <c r="H146" s="8"/>
-    </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I146" t="s">
+        <v>89</v>
+      </c>
+      <c r="J146" t="s">
+        <v>76</v>
+      </c>
+      <c r="K146" t="s">
+        <v>77</v>
+      </c>
+      <c r="L146">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="147" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F147">
+        <v>21</v>
+      </c>
       <c r="H147" s="8"/>
-    </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I147" t="s">
+        <v>89</v>
+      </c>
+      <c r="J147" t="s">
+        <v>76</v>
+      </c>
+      <c r="K147" t="s">
+        <v>77</v>
+      </c>
+      <c r="L147">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="148" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F148">
+        <v>22</v>
+      </c>
       <c r="H148" s="8"/>
-    </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I148" t="s">
+        <v>89</v>
+      </c>
+      <c r="J148" t="s">
+        <v>76</v>
+      </c>
+      <c r="K148" t="s">
+        <v>77</v>
+      </c>
+      <c r="L148">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="149" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F149">
+        <v>23</v>
+      </c>
       <c r="H149" s="8"/>
-    </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I149" t="s">
+        <v>89</v>
+      </c>
+      <c r="J149" t="s">
+        <v>76</v>
+      </c>
+      <c r="K149" t="s">
+        <v>77</v>
+      </c>
+      <c r="L149">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="150" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F150">
+        <v>24</v>
+      </c>
       <c r="H150" s="8"/>
-    </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I150" t="s">
+        <v>89</v>
+      </c>
+      <c r="J150" t="s">
+        <v>76</v>
+      </c>
+      <c r="K150" t="s">
+        <v>77</v>
+      </c>
+      <c r="L150">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="151" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F151">
+        <v>25</v>
+      </c>
       <c r="H151" s="8"/>
-    </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I151" t="s">
+        <v>89</v>
+      </c>
+      <c r="J151" t="s">
+        <v>76</v>
+      </c>
+      <c r="K151" t="s">
+        <v>77</v>
+      </c>
+      <c r="L151">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="152" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H152" s="8"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="153" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H153" s="8"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="154" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H154" s="8"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="155" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H155" s="8"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="156" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H156" s="8"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="157" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H157" s="8"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="158" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H158" s="8"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="159" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H159" s="8"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="160" spans="6:12" x14ac:dyDescent="0.55000000000000004">
       <c r="H160" s="8"/>
     </row>
     <row r="161" spans="8:8" x14ac:dyDescent="0.55000000000000004">
@@ -8345,7 +8776,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:O151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="17.20703125" bestFit="1" customWidth="1"/>
@@ -13575,6 +14006,431 @@
       <c r="N126" s="6"/>
       <c r="O126" s="5"/>
     </row>
+    <row r="127" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F127">
+        <v>1</v>
+      </c>
+      <c r="I127" t="s">
+        <v>89</v>
+      </c>
+      <c r="J127" t="s">
+        <v>76</v>
+      </c>
+      <c r="K127" t="s">
+        <v>86</v>
+      </c>
+      <c r="L127" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="128" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F128">
+        <v>2</v>
+      </c>
+      <c r="I128" t="s">
+        <v>89</v>
+      </c>
+      <c r="J128" t="s">
+        <v>76</v>
+      </c>
+      <c r="K128" t="s">
+        <v>86</v>
+      </c>
+      <c r="L128" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="129" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F129">
+        <v>3</v>
+      </c>
+      <c r="I129" t="s">
+        <v>89</v>
+      </c>
+      <c r="J129" t="s">
+        <v>76</v>
+      </c>
+      <c r="K129" t="s">
+        <v>86</v>
+      </c>
+      <c r="L129" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="130" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F130">
+        <v>4</v>
+      </c>
+      <c r="I130" t="s">
+        <v>89</v>
+      </c>
+      <c r="J130" t="s">
+        <v>76</v>
+      </c>
+      <c r="K130" t="s">
+        <v>86</v>
+      </c>
+      <c r="L130" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="131" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F131">
+        <v>5</v>
+      </c>
+      <c r="I131" t="s">
+        <v>89</v>
+      </c>
+      <c r="J131" t="s">
+        <v>76</v>
+      </c>
+      <c r="K131" t="s">
+        <v>86</v>
+      </c>
+      <c r="L131" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="132" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F132">
+        <v>6</v>
+      </c>
+      <c r="I132" t="s">
+        <v>89</v>
+      </c>
+      <c r="J132" t="s">
+        <v>76</v>
+      </c>
+      <c r="K132" t="s">
+        <v>86</v>
+      </c>
+      <c r="L132" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="133" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F133">
+        <v>7</v>
+      </c>
+      <c r="I133" t="s">
+        <v>89</v>
+      </c>
+      <c r="J133" t="s">
+        <v>76</v>
+      </c>
+      <c r="K133" t="s">
+        <v>86</v>
+      </c>
+      <c r="L133" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="134" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F134">
+        <v>8</v>
+      </c>
+      <c r="I134" t="s">
+        <v>89</v>
+      </c>
+      <c r="J134" t="s">
+        <v>76</v>
+      </c>
+      <c r="K134" t="s">
+        <v>86</v>
+      </c>
+      <c r="L134" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="135" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F135">
+        <v>9</v>
+      </c>
+      <c r="I135" t="s">
+        <v>89</v>
+      </c>
+      <c r="J135" t="s">
+        <v>76</v>
+      </c>
+      <c r="K135" t="s">
+        <v>86</v>
+      </c>
+      <c r="L135" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="136" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F136">
+        <v>10</v>
+      </c>
+      <c r="I136" t="s">
+        <v>89</v>
+      </c>
+      <c r="J136" t="s">
+        <v>76</v>
+      </c>
+      <c r="K136" t="s">
+        <v>86</v>
+      </c>
+      <c r="L136" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="137" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F137">
+        <v>11</v>
+      </c>
+      <c r="I137" t="s">
+        <v>89</v>
+      </c>
+      <c r="J137" t="s">
+        <v>76</v>
+      </c>
+      <c r="K137" t="s">
+        <v>86</v>
+      </c>
+      <c r="L137" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="138" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F138">
+        <v>12</v>
+      </c>
+      <c r="I138" t="s">
+        <v>89</v>
+      </c>
+      <c r="J138" t="s">
+        <v>76</v>
+      </c>
+      <c r="K138" t="s">
+        <v>86</v>
+      </c>
+      <c r="L138" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="139" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F139">
+        <v>13</v>
+      </c>
+      <c r="I139" t="s">
+        <v>89</v>
+      </c>
+      <c r="J139" t="s">
+        <v>76</v>
+      </c>
+      <c r="K139" t="s">
+        <v>86</v>
+      </c>
+      <c r="L139" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="140" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F140">
+        <v>14</v>
+      </c>
+      <c r="I140" t="s">
+        <v>89</v>
+      </c>
+      <c r="J140" t="s">
+        <v>76</v>
+      </c>
+      <c r="K140" t="s">
+        <v>86</v>
+      </c>
+      <c r="L140" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="141" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F141">
+        <v>15</v>
+      </c>
+      <c r="I141" t="s">
+        <v>89</v>
+      </c>
+      <c r="J141" t="s">
+        <v>76</v>
+      </c>
+      <c r="K141" t="s">
+        <v>86</v>
+      </c>
+      <c r="L141" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="142" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F142">
+        <v>16</v>
+      </c>
+      <c r="I142" t="s">
+        <v>89</v>
+      </c>
+      <c r="J142" t="s">
+        <v>76</v>
+      </c>
+      <c r="K142" t="s">
+        <v>86</v>
+      </c>
+      <c r="L142" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="143" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F143">
+        <v>17</v>
+      </c>
+      <c r="I143" t="s">
+        <v>89</v>
+      </c>
+      <c r="J143" t="s">
+        <v>76</v>
+      </c>
+      <c r="K143" t="s">
+        <v>86</v>
+      </c>
+      <c r="L143" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="144" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F144">
+        <v>18</v>
+      </c>
+      <c r="I144" t="s">
+        <v>89</v>
+      </c>
+      <c r="J144" t="s">
+        <v>76</v>
+      </c>
+      <c r="K144" t="s">
+        <v>86</v>
+      </c>
+      <c r="L144" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="145" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F145">
+        <v>19</v>
+      </c>
+      <c r="I145" t="s">
+        <v>89</v>
+      </c>
+      <c r="J145" t="s">
+        <v>76</v>
+      </c>
+      <c r="K145" t="s">
+        <v>86</v>
+      </c>
+      <c r="L145" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="146" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F146">
+        <v>20</v>
+      </c>
+      <c r="I146" t="s">
+        <v>89</v>
+      </c>
+      <c r="J146" t="s">
+        <v>76</v>
+      </c>
+      <c r="K146" t="s">
+        <v>86</v>
+      </c>
+      <c r="L146" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="147" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F147">
+        <v>21</v>
+      </c>
+      <c r="I147" t="s">
+        <v>89</v>
+      </c>
+      <c r="J147" t="s">
+        <v>76</v>
+      </c>
+      <c r="K147" t="s">
+        <v>86</v>
+      </c>
+      <c r="L147" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="148" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F148">
+        <v>22</v>
+      </c>
+      <c r="I148" t="s">
+        <v>89</v>
+      </c>
+      <c r="J148" t="s">
+        <v>76</v>
+      </c>
+      <c r="K148" t="s">
+        <v>86</v>
+      </c>
+      <c r="L148" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="149" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F149">
+        <v>23</v>
+      </c>
+      <c r="I149" t="s">
+        <v>89</v>
+      </c>
+      <c r="J149" t="s">
+        <v>76</v>
+      </c>
+      <c r="K149" t="s">
+        <v>86</v>
+      </c>
+      <c r="L149" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="150" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F150">
+        <v>24</v>
+      </c>
+      <c r="I150" t="s">
+        <v>89</v>
+      </c>
+      <c r="J150" t="s">
+        <v>76</v>
+      </c>
+      <c r="K150" t="s">
+        <v>86</v>
+      </c>
+      <c r="L150" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="151" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F151">
+        <v>25</v>
+      </c>
+      <c r="I151" t="s">
+        <v>89</v>
+      </c>
+      <c r="J151" t="s">
+        <v>76</v>
+      </c>
+      <c r="K151" t="s">
+        <v>86</v>
+      </c>
+      <c r="L151" s="5">
+        <v>5.13</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N102:O126">
     <sortCondition ref="O102:O126"/>

</xml_diff>

<commit_message>
Updated results page for IndyCar
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCD4F19-A542-41C9-8920-BC90C4F1598A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C3FD66-FD97-4ECD-8E55-300680A0E774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="57480" yWindow="-11595" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy_Model" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1326" uniqueCount="90">
   <si>
     <t>Model</t>
   </si>
@@ -319,7 +319,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -403,7 +403,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -422,6 +422,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -434,8 +435,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -957,22 +956,22 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="10" t="s">
+      <c r="C1" s="14"/>
+      <c r="D1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="10"/>
-      <c r="F1" s="11" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11" t="s">
+      <c r="G1" s="12"/>
+      <c r="H1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="11"/>
+      <c r="I1" s="12"/>
       <c r="J1" t="s">
         <v>51</v>
       </c>
@@ -1240,22 +1239,22 @@
       <c r="A12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="10" t="s">
+      <c r="C12" s="14"/>
+      <c r="D12" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="11" t="s">
+      <c r="E12" s="11"/>
+      <c r="F12" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11" t="s">
+      <c r="G12" s="12"/>
+      <c r="H12" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I12" s="11"/>
+      <c r="I12" s="12"/>
       <c r="J12" t="s">
         <v>50</v>
       </c>
@@ -1698,7 +1697,7 @@
       <c r="D31">
         <v>0.21909999999999999</v>
       </c>
-      <c r="E31" s="14">
+      <c r="E31" s="10">
         <v>0.2026</v>
       </c>
     </row>
@@ -1779,22 +1778,22 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="10" t="s">
+      <c r="C1" s="14"/>
+      <c r="D1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="10"/>
-      <c r="F1" s="11" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11" t="s">
+      <c r="G1" s="12"/>
+      <c r="H1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="11"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1"/>
@@ -2346,27 +2345,24 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15" t="s">
+      <c r="B21" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="15" t="s">
+      <c r="F21" t="s">
         <v>65</v>
       </c>
-      <c r="G21" s="15" t="s">
+      <c r="G21" t="s">
         <v>24</v>
       </c>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="C22" t="s">
@@ -7694,7 +7690,27 @@
       <c r="O126" s="5"/>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A127" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B127" s="6">
+        <v>7.58</v>
+      </c>
+      <c r="C127" s="5">
+        <f>B127-L127</f>
+        <v>2.0999999999999996</v>
+      </c>
+      <c r="D127" s="5">
+        <f>B127+L127</f>
+        <v>13.06</v>
+      </c>
+      <c r="E127" s="5">
+        <v>2.1</v>
+      </c>
       <c r="F127">
+        <v>1</v>
+      </c>
+      <c r="G127" s="8">
         <v>1</v>
       </c>
       <c r="H127" s="8"/>
@@ -7712,8 +7728,28 @@
       </c>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A128" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B128" s="6">
+        <v>7.95</v>
+      </c>
+      <c r="C128" s="5">
+        <f t="shared" ref="C128:C151" si="10">B128-L128</f>
+        <v>2.4699999999999998</v>
+      </c>
+      <c r="D128" s="5">
+        <f t="shared" ref="D128:D151" si="11">B128+L128</f>
+        <v>13.43</v>
+      </c>
+      <c r="E128" s="5">
+        <v>7.95</v>
+      </c>
       <c r="F128">
         <v>2</v>
+      </c>
+      <c r="G128" s="8">
+        <v>8</v>
       </c>
       <c r="H128" s="8"/>
       <c r="I128" t="s">
@@ -7728,10 +7764,32 @@
       <c r="L128">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="129" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N128" s="6"/>
+      <c r="O128" s="5"/>
+    </row>
+    <row r="129" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A129" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B129" s="6">
+        <v>8.17</v>
+      </c>
+      <c r="C129" s="5">
+        <f t="shared" si="10"/>
+        <v>2.6899999999999995</v>
+      </c>
+      <c r="D129" s="5">
+        <f t="shared" si="11"/>
+        <v>13.65</v>
+      </c>
+      <c r="E129" s="5">
+        <v>8.17</v>
+      </c>
       <c r="F129">
         <v>3</v>
+      </c>
+      <c r="G129" s="8">
+        <v>9</v>
       </c>
       <c r="H129" s="8"/>
       <c r="I129" t="s">
@@ -7746,10 +7804,32 @@
       <c r="L129">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="130" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N129" s="6"/>
+      <c r="O129" s="5"/>
+    </row>
+    <row r="130" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A130" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B130" s="6">
+        <v>8.92</v>
+      </c>
+      <c r="C130" s="5">
+        <f t="shared" si="10"/>
+        <v>3.4399999999999995</v>
+      </c>
+      <c r="D130" s="5">
+        <f t="shared" si="11"/>
+        <v>14.4</v>
+      </c>
+      <c r="E130" s="5">
+        <v>3.44</v>
+      </c>
       <c r="F130">
         <v>4</v>
+      </c>
+      <c r="G130" s="8">
+        <v>2</v>
       </c>
       <c r="H130" s="8"/>
       <c r="I130" t="s">
@@ -7764,10 +7844,32 @@
       <c r="L130">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="131" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N130" s="6"/>
+      <c r="O130" s="5"/>
+    </row>
+    <row r="131" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A131" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B131" s="6">
+        <v>8.93</v>
+      </c>
+      <c r="C131" s="5">
+        <f t="shared" si="10"/>
+        <v>3.4499999999999993</v>
+      </c>
+      <c r="D131" s="5">
+        <f t="shared" si="11"/>
+        <v>14.41</v>
+      </c>
+      <c r="E131" s="5">
+        <v>3.45</v>
+      </c>
       <c r="F131">
         <v>5</v>
+      </c>
+      <c r="G131" s="8">
+        <v>3</v>
       </c>
       <c r="H131" s="8"/>
       <c r="I131" t="s">
@@ -7782,10 +7884,32 @@
       <c r="L131">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="132" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N131" s="6"/>
+      <c r="O131" s="5"/>
+    </row>
+    <row r="132" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A132" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B132" s="6">
+        <v>8.9700000000000006</v>
+      </c>
+      <c r="C132" s="5">
+        <f t="shared" si="10"/>
+        <v>3.49</v>
+      </c>
+      <c r="D132" s="5">
+        <f t="shared" si="11"/>
+        <v>14.450000000000001</v>
+      </c>
+      <c r="E132" s="5">
+        <v>8.9700000000000006</v>
+      </c>
       <c r="F132">
         <v>6</v>
+      </c>
+      <c r="G132" s="8">
+        <v>11</v>
       </c>
       <c r="H132" s="8"/>
       <c r="I132" t="s">
@@ -7800,10 +7924,32 @@
       <c r="L132">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="133" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N132" s="6"/>
+      <c r="O132" s="5"/>
+    </row>
+    <row r="133" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A133" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B133" s="6">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="C133" s="5">
+        <f t="shared" si="10"/>
+        <v>4.32</v>
+      </c>
+      <c r="D133" s="5">
+        <f t="shared" si="11"/>
+        <v>15.280000000000001</v>
+      </c>
+      <c r="E133" s="5">
+        <v>4.32</v>
+      </c>
       <c r="F133">
         <v>7</v>
+      </c>
+      <c r="G133" s="8">
+        <v>4</v>
       </c>
       <c r="H133" s="8"/>
       <c r="I133" t="s">
@@ -7818,10 +7964,32 @@
       <c r="L133">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="134" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N133" s="6"/>
+      <c r="O133" s="5"/>
+    </row>
+    <row r="134" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A134" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B134" s="6">
+        <v>10.1</v>
+      </c>
+      <c r="C134" s="5">
+        <f t="shared" si="10"/>
+        <v>4.6199999999999992</v>
+      </c>
+      <c r="D134" s="5">
+        <f t="shared" si="11"/>
+        <v>15.58</v>
+      </c>
+      <c r="E134" s="5">
+        <v>10.1</v>
+      </c>
       <c r="F134">
         <v>8</v>
+      </c>
+      <c r="G134" s="8">
+        <v>12</v>
       </c>
       <c r="H134" s="8"/>
       <c r="I134" t="s">
@@ -7836,10 +8004,32 @@
       <c r="L134">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="135" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N134" s="6"/>
+      <c r="O134" s="5"/>
+    </row>
+    <row r="135" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A135" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B135" s="6">
+        <v>10.33</v>
+      </c>
+      <c r="C135" s="5">
+        <f t="shared" si="10"/>
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="D135" s="5">
+        <f t="shared" si="11"/>
+        <v>15.81</v>
+      </c>
+      <c r="E135" s="5">
+        <v>4.8499999999999996</v>
+      </c>
       <c r="F135">
         <v>9</v>
+      </c>
+      <c r="G135" s="8">
+        <v>5</v>
       </c>
       <c r="H135" s="8"/>
       <c r="I135" t="s">
@@ -7854,10 +8044,32 @@
       <c r="L135">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="136" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N135" s="6"/>
+      <c r="O135" s="5"/>
+    </row>
+    <row r="136" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A136" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B136" s="6">
+        <v>10.34</v>
+      </c>
+      <c r="C136" s="5">
+        <f t="shared" si="10"/>
+        <v>4.8599999999999994</v>
+      </c>
+      <c r="D136" s="5">
+        <f t="shared" si="11"/>
+        <v>15.82</v>
+      </c>
+      <c r="E136" s="5">
+        <v>10.34</v>
+      </c>
       <c r="F136">
         <v>10</v>
+      </c>
+      <c r="G136" s="8">
+        <v>13</v>
       </c>
       <c r="H136" s="8"/>
       <c r="I136" t="s">
@@ -7872,10 +8084,32 @@
       <c r="L136">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="137" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N136" s="6"/>
+      <c r="O136" s="5"/>
+    </row>
+    <row r="137" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A137" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B137" s="6">
+        <v>10.58</v>
+      </c>
+      <c r="C137" s="5">
+        <f t="shared" si="10"/>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D137" s="5">
+        <f t="shared" si="11"/>
+        <v>16.060000000000002</v>
+      </c>
+      <c r="E137" s="5">
+        <v>10.58</v>
+      </c>
       <c r="F137">
         <v>11</v>
+      </c>
+      <c r="G137" s="8">
+        <v>14</v>
       </c>
       <c r="H137" s="8"/>
       <c r="I137" t="s">
@@ -7890,10 +8124,32 @@
       <c r="L137">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="138" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N137" s="6"/>
+      <c r="O137" s="5"/>
+    </row>
+    <row r="138" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A138" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B138" s="6">
+        <v>11.18</v>
+      </c>
+      <c r="C138" s="5">
+        <f t="shared" si="10"/>
+        <v>5.6999999999999993</v>
+      </c>
+      <c r="D138" s="5">
+        <f t="shared" si="11"/>
+        <v>16.66</v>
+      </c>
+      <c r="E138" s="5">
+        <v>11.18</v>
+      </c>
       <c r="F138">
         <v>12</v>
+      </c>
+      <c r="G138" s="8">
+        <v>15</v>
       </c>
       <c r="H138" s="8"/>
       <c r="I138" t="s">
@@ -7908,10 +8164,32 @@
       <c r="L138">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="139" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N138" s="6"/>
+      <c r="O138" s="5"/>
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A139" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B139" s="6">
+        <v>11.79</v>
+      </c>
+      <c r="C139" s="5">
+        <f t="shared" si="10"/>
+        <v>6.3099999999999987</v>
+      </c>
+      <c r="D139" s="5">
+        <f t="shared" si="11"/>
+        <v>17.27</v>
+      </c>
+      <c r="E139" s="5">
+        <v>6.31</v>
+      </c>
       <c r="F139">
         <v>13</v>
+      </c>
+      <c r="G139" s="8">
+        <v>6</v>
       </c>
       <c r="H139" s="8"/>
       <c r="I139" t="s">
@@ -7926,10 +8204,32 @@
       <c r="L139">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="140" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N139" s="6"/>
+      <c r="O139" s="5"/>
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A140" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B140" s="6">
+        <v>12.06</v>
+      </c>
+      <c r="C140" s="5">
+        <f t="shared" si="10"/>
+        <v>6.58</v>
+      </c>
+      <c r="D140" s="5">
+        <f t="shared" si="11"/>
+        <v>17.54</v>
+      </c>
+      <c r="E140" s="5">
+        <v>6.58</v>
+      </c>
       <c r="F140">
         <v>14</v>
+      </c>
+      <c r="G140" s="8">
+        <v>7</v>
       </c>
       <c r="H140" s="8"/>
       <c r="I140" t="s">
@@ -7944,10 +8244,32 @@
       <c r="L140">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="141" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N140" s="6"/>
+      <c r="O140" s="5"/>
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A141" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B141" s="6">
+        <v>12.35</v>
+      </c>
+      <c r="C141" s="5">
+        <f t="shared" si="10"/>
+        <v>6.8699999999999992</v>
+      </c>
+      <c r="D141" s="5">
+        <f t="shared" si="11"/>
+        <v>17.829999999999998</v>
+      </c>
+      <c r="E141" s="5">
+        <v>12.35</v>
+      </c>
       <c r="F141">
         <v>15</v>
+      </c>
+      <c r="G141" s="8">
+        <v>16</v>
       </c>
       <c r="H141" s="8"/>
       <c r="I141" t="s">
@@ -7962,10 +8284,32 @@
       <c r="L141">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="142" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N141" s="6"/>
+      <c r="O141" s="5"/>
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A142" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B142" s="6">
+        <v>13.76</v>
+      </c>
+      <c r="C142" s="5">
+        <f t="shared" si="10"/>
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="D142" s="5">
+        <f t="shared" si="11"/>
+        <v>19.240000000000002</v>
+      </c>
+      <c r="E142" s="5">
+        <v>13.76</v>
+      </c>
       <c r="F142">
         <v>16</v>
+      </c>
+      <c r="G142" s="8">
+        <v>17</v>
       </c>
       <c r="H142" s="8"/>
       <c r="I142" t="s">
@@ -7980,10 +8324,32 @@
       <c r="L142">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="143" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N142" s="6"/>
+      <c r="O142" s="5"/>
+    </row>
+    <row r="143" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A143" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B143" s="6">
+        <v>13.83</v>
+      </c>
+      <c r="C143" s="5">
+        <f t="shared" si="10"/>
+        <v>8.35</v>
+      </c>
+      <c r="D143" s="5">
+        <f t="shared" si="11"/>
+        <v>19.310000000000002</v>
+      </c>
+      <c r="E143" s="5">
+        <v>19.309999999999999</v>
+      </c>
       <c r="F143">
         <v>17</v>
+      </c>
+      <c r="G143" s="8">
+        <v>24</v>
       </c>
       <c r="H143" s="8"/>
       <c r="I143" t="s">
@@ -7998,9 +8364,31 @@
       <c r="L143">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="144" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N143" s="6"/>
+      <c r="O143" s="5"/>
+    </row>
+    <row r="144" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A144" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B144" s="6">
+        <v>13.95</v>
+      </c>
+      <c r="C144" s="5">
+        <f t="shared" si="10"/>
+        <v>8.4699999999999989</v>
+      </c>
+      <c r="D144" s="5">
+        <f t="shared" si="11"/>
+        <v>19.43</v>
+      </c>
+      <c r="E144" s="5">
+        <v>13.95</v>
+      </c>
       <c r="F144">
+        <v>18</v>
+      </c>
+      <c r="G144" s="8">
         <v>18</v>
       </c>
       <c r="H144" s="8"/>
@@ -8016,9 +8404,31 @@
       <c r="L144">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="145" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N144" s="6"/>
+      <c r="O144" s="5"/>
+    </row>
+    <row r="145" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A145" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B145" s="6">
+        <v>14.34</v>
+      </c>
+      <c r="C145" s="5">
+        <f t="shared" si="10"/>
+        <v>8.86</v>
+      </c>
+      <c r="D145" s="5">
+        <f t="shared" si="11"/>
+        <v>19.82</v>
+      </c>
+      <c r="E145" s="5">
+        <v>14.34</v>
+      </c>
       <c r="F145">
+        <v>19</v>
+      </c>
+      <c r="G145" s="8">
         <v>19</v>
       </c>
       <c r="H145" s="8"/>
@@ -8034,10 +8444,32 @@
       <c r="L145">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="146" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N145" s="6"/>
+      <c r="O145" s="5"/>
+    </row>
+    <row r="146" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A146" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B146" s="6">
+        <v>14.42</v>
+      </c>
+      <c r="C146" s="5">
+        <f t="shared" si="10"/>
+        <v>8.94</v>
+      </c>
+      <c r="D146" s="5">
+        <f t="shared" si="11"/>
+        <v>19.899999999999999</v>
+      </c>
+      <c r="E146" s="5">
+        <v>8.94</v>
+      </c>
       <c r="F146">
         <v>20</v>
+      </c>
+      <c r="G146" s="8">
+        <v>10</v>
       </c>
       <c r="H146" s="8"/>
       <c r="I146" t="s">
@@ -8052,10 +8484,32 @@
       <c r="L146">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="147" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N146" s="6"/>
+      <c r="O146" s="5"/>
+    </row>
+    <row r="147" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A147" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B147" s="6">
+        <v>14.81</v>
+      </c>
+      <c r="C147" s="5">
+        <f t="shared" si="10"/>
+        <v>9.33</v>
+      </c>
+      <c r="D147" s="5">
+        <f t="shared" si="11"/>
+        <v>20.29</v>
+      </c>
+      <c r="E147" s="5">
+        <v>14.81</v>
+      </c>
       <c r="F147">
         <v>21</v>
+      </c>
+      <c r="G147" s="8">
+        <v>20</v>
       </c>
       <c r="H147" s="8"/>
       <c r="I147" t="s">
@@ -8070,10 +8524,32 @@
       <c r="L147">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="148" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N147" s="6"/>
+      <c r="O147" s="5"/>
+    </row>
+    <row r="148" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A148" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B148" s="6">
+        <v>15.89</v>
+      </c>
+      <c r="C148" s="5">
+        <f t="shared" si="10"/>
+        <v>10.41</v>
+      </c>
+      <c r="D148" s="5">
+        <f t="shared" si="11"/>
+        <v>21.37</v>
+      </c>
+      <c r="E148" s="5">
+        <v>15.89</v>
+      </c>
       <c r="F148">
         <v>22</v>
+      </c>
+      <c r="G148" s="8">
+        <v>21</v>
       </c>
       <c r="H148" s="8"/>
       <c r="I148" t="s">
@@ -8088,10 +8564,32 @@
       <c r="L148">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="149" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N148" s="6"/>
+      <c r="O148" s="5"/>
+    </row>
+    <row r="149" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A149" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B149" s="6">
+        <v>16.03</v>
+      </c>
+      <c r="C149" s="5">
+        <f t="shared" si="10"/>
+        <v>10.55</v>
+      </c>
+      <c r="D149" s="5">
+        <f t="shared" si="11"/>
+        <v>21.51</v>
+      </c>
+      <c r="E149" s="5">
+        <v>16.03</v>
+      </c>
       <c r="F149">
         <v>23</v>
+      </c>
+      <c r="G149" s="8">
+        <v>22</v>
       </c>
       <c r="H149" s="8"/>
       <c r="I149" t="s">
@@ -8106,10 +8604,32 @@
       <c r="L149">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="150" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N149" s="6"/>
+      <c r="O149" s="5"/>
+    </row>
+    <row r="150" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A150" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B150" s="6">
+        <v>16.23</v>
+      </c>
+      <c r="C150" s="5">
+        <f t="shared" si="10"/>
+        <v>10.75</v>
+      </c>
+      <c r="D150" s="5">
+        <f t="shared" si="11"/>
+        <v>21.71</v>
+      </c>
+      <c r="E150" s="5">
+        <v>16.23</v>
+      </c>
       <c r="F150">
         <v>24</v>
+      </c>
+      <c r="G150" s="8">
+        <v>23</v>
       </c>
       <c r="H150" s="8"/>
       <c r="I150" t="s">
@@ -8124,9 +8644,31 @@
       <c r="L150">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="151" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N150" s="6"/>
+      <c r="O150" s="5"/>
+    </row>
+    <row r="151" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A151" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B151" s="6">
+        <v>17.36</v>
+      </c>
+      <c r="C151" s="5">
+        <f t="shared" si="10"/>
+        <v>11.879999999999999</v>
+      </c>
+      <c r="D151" s="5">
+        <f t="shared" si="11"/>
+        <v>22.84</v>
+      </c>
+      <c r="E151" s="5">
+        <v>22.84</v>
+      </c>
       <c r="F151">
+        <v>25</v>
+      </c>
+      <c r="G151" s="8">
         <v>25</v>
       </c>
       <c r="H151" s="8"/>
@@ -8142,32 +8684,36 @@
       <c r="L151">
         <v>5.48</v>
       </c>
-    </row>
-    <row r="152" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N151" s="6"/>
+      <c r="O151" s="5"/>
+    </row>
+    <row r="152" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H152" s="8"/>
-    </row>
-    <row r="153" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N152" s="6"/>
+      <c r="O152" s="5"/>
+    </row>
+    <row r="153" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H153" s="8"/>
     </row>
-    <row r="154" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H154" s="8"/>
     </row>
-    <row r="155" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H155" s="8"/>
     </row>
-    <row r="156" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H156" s="8"/>
     </row>
-    <row r="157" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H157" s="8"/>
     </row>
-    <row r="158" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H158" s="8"/>
     </row>
-    <row r="159" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H159" s="8"/>
     </row>
-    <row r="160" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="H160" s="8"/>
     </row>
     <row r="161" spans="8:8" x14ac:dyDescent="0.55000000000000004">
@@ -8762,8 +9308,8 @@
       <c r="H357" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N102:O126">
-    <sortCondition ref="O102:O126"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N128:O152">
+    <sortCondition ref="O128:O152"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8779,7 +9325,7 @@
   <dimension ref="A1:O151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="17.20703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.3671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.47265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.05078125" customWidth="1"/>
     <col min="5" max="5" width="10.68359375" bestFit="1" customWidth="1"/>
@@ -14007,9 +14553,29 @@
       <c r="O126" s="5"/>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A127" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B127" s="6">
+        <v>5.52</v>
+      </c>
+      <c r="C127" s="5">
+        <f>B127-L127</f>
+        <v>0.38999999999999968</v>
+      </c>
+      <c r="D127" s="5">
+        <f>B127+L127</f>
+        <v>10.649999999999999</v>
+      </c>
+      <c r="E127" s="5">
+        <v>0.39</v>
+      </c>
       <c r="F127">
         <v>1</v>
       </c>
+      <c r="G127" s="8">
+        <v>1</v>
+      </c>
       <c r="I127" t="s">
         <v>89</v>
       </c>
@@ -14022,11 +14588,33 @@
       <c r="L127" s="5">
         <v>5.13</v>
       </c>
+      <c r="N127" s="6"/>
+      <c r="O127" s="5"/>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A128" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B128" s="6">
+        <v>7.15</v>
+      </c>
+      <c r="C128" s="5">
+        <f t="shared" ref="C128:C151" si="9">B128-L128</f>
+        <v>2.0200000000000005</v>
+      </c>
+      <c r="D128" s="5">
+        <f t="shared" ref="D128:D151" si="10">B128+L128</f>
+        <v>12.280000000000001</v>
+      </c>
+      <c r="E128" s="5">
+        <v>2.02</v>
+      </c>
       <c r="F128">
         <v>2</v>
       </c>
+      <c r="G128" s="8">
+        <v>2</v>
+      </c>
       <c r="I128" t="s">
         <v>89</v>
       </c>
@@ -14039,11 +14627,33 @@
       <c r="L128" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="129" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N128" s="6"/>
+      <c r="O128" s="5"/>
+    </row>
+    <row r="129" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A129" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B129" s="6">
+        <v>7.39</v>
+      </c>
+      <c r="C129" s="5">
+        <f t="shared" si="9"/>
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="D129" s="5">
+        <f t="shared" si="10"/>
+        <v>12.52</v>
+      </c>
+      <c r="E129" s="5">
+        <v>7.39</v>
+      </c>
       <c r="F129">
         <v>3</v>
       </c>
+      <c r="G129" s="8">
+        <v>7</v>
+      </c>
       <c r="I129" t="s">
         <v>89</v>
       </c>
@@ -14056,11 +14666,33 @@
       <c r="L129" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="130" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N129" s="6"/>
+      <c r="O129" s="5"/>
+    </row>
+    <row r="130" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A130" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B130" s="6">
+        <v>7.51</v>
+      </c>
+      <c r="C130" s="5">
+        <f t="shared" si="9"/>
+        <v>2.38</v>
+      </c>
+      <c r="D130" s="5">
+        <f t="shared" si="10"/>
+        <v>12.64</v>
+      </c>
+      <c r="E130" s="5">
+        <v>2.38</v>
+      </c>
       <c r="F130">
         <v>4</v>
       </c>
+      <c r="G130" s="8">
+        <v>3</v>
+      </c>
       <c r="I130" t="s">
         <v>89</v>
       </c>
@@ -14073,11 +14705,33 @@
       <c r="L130" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="131" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N130" s="6"/>
+      <c r="O130" s="5"/>
+    </row>
+    <row r="131" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A131" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B131" s="6">
+        <v>8.9</v>
+      </c>
+      <c r="C131" s="5">
+        <f t="shared" si="9"/>
+        <v>3.7700000000000005</v>
+      </c>
+      <c r="D131" s="5">
+        <f t="shared" si="10"/>
+        <v>14.030000000000001</v>
+      </c>
+      <c r="E131" s="5">
+        <v>3.77</v>
+      </c>
       <c r="F131">
         <v>5</v>
       </c>
+      <c r="G131" s="8">
+        <v>4</v>
+      </c>
       <c r="I131" t="s">
         <v>89</v>
       </c>
@@ -14090,11 +14744,33 @@
       <c r="L131" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="132" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N131" s="6"/>
+      <c r="O131" s="5"/>
+    </row>
+    <row r="132" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A132" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B132" s="6">
+        <v>9.32</v>
+      </c>
+      <c r="C132" s="5">
+        <f t="shared" si="9"/>
+        <v>4.1900000000000004</v>
+      </c>
+      <c r="D132" s="5">
+        <f t="shared" si="10"/>
+        <v>14.45</v>
+      </c>
+      <c r="E132" s="5">
+        <v>4.1900000000000004</v>
+      </c>
       <c r="F132">
         <v>6</v>
       </c>
+      <c r="G132" s="8">
+        <v>5</v>
+      </c>
       <c r="I132" t="s">
         <v>89</v>
       </c>
@@ -14107,11 +14783,33 @@
       <c r="L132" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="133" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N132" s="6"/>
+      <c r="O132" s="5"/>
+    </row>
+    <row r="133" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A133" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B133" s="6">
+        <v>9.4</v>
+      </c>
+      <c r="C133" s="5">
+        <f t="shared" si="9"/>
+        <v>4.2700000000000005</v>
+      </c>
+      <c r="D133" s="5">
+        <f t="shared" si="10"/>
+        <v>14.530000000000001</v>
+      </c>
+      <c r="E133" s="5">
+        <v>9.4</v>
+      </c>
       <c r="F133">
         <v>7</v>
       </c>
+      <c r="G133" s="8">
+        <v>8</v>
+      </c>
       <c r="I133" t="s">
         <v>89</v>
       </c>
@@ -14124,11 +14822,33 @@
       <c r="L133" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="134" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N133" s="6"/>
+      <c r="O133" s="5"/>
+    </row>
+    <row r="134" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A134" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B134" s="6">
+        <v>9.68</v>
+      </c>
+      <c r="C134" s="5">
+        <f t="shared" si="9"/>
+        <v>4.55</v>
+      </c>
+      <c r="D134" s="5">
+        <f t="shared" si="10"/>
+        <v>14.809999999999999</v>
+      </c>
+      <c r="E134" s="5">
+        <v>9.68</v>
+      </c>
       <c r="F134">
         <v>8</v>
       </c>
+      <c r="G134" s="8">
+        <v>9</v>
+      </c>
       <c r="I134" t="s">
         <v>89</v>
       </c>
@@ -14141,11 +14861,33 @@
       <c r="L134" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="135" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N134" s="6"/>
+      <c r="O134" s="5"/>
+    </row>
+    <row r="135" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A135" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B135" s="6">
+        <v>9.9700000000000006</v>
+      </c>
+      <c r="C135" s="5">
+        <f t="shared" si="9"/>
+        <v>4.8400000000000007</v>
+      </c>
+      <c r="D135" s="5">
+        <f t="shared" si="10"/>
+        <v>15.100000000000001</v>
+      </c>
+      <c r="E135" s="5">
+        <v>4.84</v>
+      </c>
       <c r="F135">
         <v>9</v>
       </c>
+      <c r="G135" s="8">
+        <v>6</v>
+      </c>
       <c r="I135" t="s">
         <v>89</v>
       </c>
@@ -14158,11 +14900,33 @@
       <c r="L135" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="136" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N135" s="6"/>
+      <c r="O135" s="5"/>
+    </row>
+    <row r="136" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A136" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B136" s="6">
+        <v>11.1</v>
+      </c>
+      <c r="C136" s="5">
+        <f t="shared" si="9"/>
+        <v>5.97</v>
+      </c>
+      <c r="D136" s="5">
+        <f t="shared" si="10"/>
+        <v>16.23</v>
+      </c>
+      <c r="E136" s="5">
+        <v>11.1</v>
+      </c>
       <c r="F136">
         <v>10</v>
       </c>
+      <c r="G136" s="8">
+        <v>11</v>
+      </c>
       <c r="I136" t="s">
         <v>89</v>
       </c>
@@ -14175,11 +14939,33 @@
       <c r="L136" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="137" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N136" s="6"/>
+      <c r="O136" s="5"/>
+    </row>
+    <row r="137" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A137" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B137" s="6">
+        <v>11.61</v>
+      </c>
+      <c r="C137" s="5">
+        <f t="shared" si="9"/>
+        <v>6.4799999999999995</v>
+      </c>
+      <c r="D137" s="5">
+        <f t="shared" si="10"/>
+        <v>16.739999999999998</v>
+      </c>
+      <c r="E137" s="5">
+        <v>11.61</v>
+      </c>
       <c r="F137">
         <v>11</v>
       </c>
+      <c r="G137" s="8">
+        <v>12</v>
+      </c>
       <c r="I137" t="s">
         <v>89</v>
       </c>
@@ -14192,11 +14978,33 @@
       <c r="L137" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="138" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N137" s="6"/>
+      <c r="O137" s="5"/>
+    </row>
+    <row r="138" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A138" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B138" s="6">
+        <v>11.63</v>
+      </c>
+      <c r="C138" s="5">
+        <f t="shared" si="9"/>
+        <v>6.5000000000000009</v>
+      </c>
+      <c r="D138" s="5">
+        <f t="shared" si="10"/>
+        <v>16.760000000000002</v>
+      </c>
+      <c r="E138" s="5">
+        <v>16.760000000000002</v>
+      </c>
       <c r="F138">
         <v>12</v>
       </c>
+      <c r="G138" s="8">
+        <v>21</v>
+      </c>
       <c r="I138" t="s">
         <v>89</v>
       </c>
@@ -14209,11 +15017,33 @@
       <c r="L138" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="139" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N138" s="6"/>
+      <c r="O138" s="5"/>
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A139" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B139" s="6">
+        <v>12.35</v>
+      </c>
+      <c r="C139" s="5">
+        <f t="shared" si="9"/>
+        <v>7.22</v>
+      </c>
+      <c r="D139" s="5">
+        <f t="shared" si="10"/>
+        <v>17.48</v>
+      </c>
+      <c r="E139" s="5">
+        <v>12.35</v>
+      </c>
       <c r="F139">
         <v>13</v>
       </c>
+      <c r="G139" s="8">
+        <v>13</v>
+      </c>
       <c r="I139" t="s">
         <v>89</v>
       </c>
@@ -14226,11 +15056,33 @@
       <c r="L139" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="140" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N139" s="6"/>
+      <c r="O139" s="5"/>
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A140" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B140" s="6">
+        <v>12.71</v>
+      </c>
+      <c r="C140" s="5">
+        <f t="shared" si="9"/>
+        <v>7.580000000000001</v>
+      </c>
+      <c r="D140" s="5">
+        <f t="shared" si="10"/>
+        <v>17.84</v>
+      </c>
+      <c r="E140" s="5">
+        <v>12.71</v>
+      </c>
       <c r="F140">
         <v>14</v>
       </c>
+      <c r="G140" s="8">
+        <v>14</v>
+      </c>
       <c r="I140" t="s">
         <v>89</v>
       </c>
@@ -14243,11 +15095,33 @@
       <c r="L140" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="141" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N140" s="6"/>
+      <c r="O140" s="5"/>
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A141" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B141" s="6">
+        <v>12.85</v>
+      </c>
+      <c r="C141" s="5">
+        <f t="shared" si="9"/>
+        <v>7.72</v>
+      </c>
+      <c r="D141" s="5">
+        <f t="shared" si="10"/>
+        <v>17.98</v>
+      </c>
+      <c r="E141" s="5">
+        <v>12.85</v>
+      </c>
       <c r="F141">
         <v>15</v>
       </c>
+      <c r="G141" s="8">
+        <v>15</v>
+      </c>
       <c r="I141" t="s">
         <v>89</v>
       </c>
@@ -14260,11 +15134,33 @@
       <c r="L141" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="142" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N141" s="6"/>
+      <c r="O141" s="5"/>
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A142" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B142" s="6">
+        <v>12.86</v>
+      </c>
+      <c r="C142" s="5">
+        <f t="shared" si="9"/>
+        <v>7.7299999999999995</v>
+      </c>
+      <c r="D142" s="5">
+        <f t="shared" si="10"/>
+        <v>17.989999999999998</v>
+      </c>
+      <c r="E142" s="5">
+        <v>17.989999999999998</v>
+      </c>
       <c r="F142">
         <v>16</v>
       </c>
+      <c r="G142" s="8">
+        <v>22</v>
+      </c>
       <c r="I142" t="s">
         <v>89</v>
       </c>
@@ -14277,11 +15173,33 @@
       <c r="L142" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="143" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N142" s="6"/>
+      <c r="O142" s="5"/>
+    </row>
+    <row r="143" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A143" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B143" s="6">
+        <v>13.93</v>
+      </c>
+      <c r="C143" s="5">
+        <f t="shared" si="9"/>
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="D143" s="5">
+        <f t="shared" si="10"/>
+        <v>19.059999999999999</v>
+      </c>
+      <c r="E143" s="5">
+        <v>13.93</v>
+      </c>
       <c r="F143">
         <v>17</v>
       </c>
+      <c r="G143" s="8">
+        <v>16</v>
+      </c>
       <c r="I143" t="s">
         <v>89</v>
       </c>
@@ -14294,11 +15212,33 @@
       <c r="L143" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="144" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N143" s="6"/>
+      <c r="O143" s="5"/>
+    </row>
+    <row r="144" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A144" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B144" s="6">
+        <v>14.31</v>
+      </c>
+      <c r="C144" s="5">
+        <f t="shared" si="9"/>
+        <v>9.18</v>
+      </c>
+      <c r="D144" s="5">
+        <f t="shared" si="10"/>
+        <v>19.440000000000001</v>
+      </c>
+      <c r="E144" s="5">
+        <v>14.31</v>
+      </c>
       <c r="F144">
         <v>18</v>
       </c>
+      <c r="G144" s="8">
+        <v>17</v>
+      </c>
       <c r="I144" t="s">
         <v>89</v>
       </c>
@@ -14311,11 +15251,33 @@
       <c r="L144" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="145" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N144" s="6"/>
+      <c r="O144" s="5"/>
+    </row>
+    <row r="145" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A145" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B145" s="6">
+        <v>14.88</v>
+      </c>
+      <c r="C145" s="5">
+        <f t="shared" si="9"/>
+        <v>9.75</v>
+      </c>
+      <c r="D145" s="5">
+        <f t="shared" si="10"/>
+        <v>20.010000000000002</v>
+      </c>
+      <c r="E145" s="5">
+        <v>20.010000000000002</v>
+      </c>
       <c r="F145">
         <v>19</v>
       </c>
+      <c r="G145" s="8">
+        <v>23</v>
+      </c>
       <c r="I145" t="s">
         <v>89</v>
       </c>
@@ -14328,11 +15290,33 @@
       <c r="L145" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="146" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N145" s="6"/>
+      <c r="O145" s="5"/>
+    </row>
+    <row r="146" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A146" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B146" s="6">
+        <v>15.06</v>
+      </c>
+      <c r="C146" s="5">
+        <f t="shared" si="9"/>
+        <v>9.93</v>
+      </c>
+      <c r="D146" s="5">
+        <f t="shared" si="10"/>
+        <v>20.190000000000001</v>
+      </c>
+      <c r="E146" s="5">
+        <v>15.06</v>
+      </c>
       <c r="F146">
         <v>20</v>
       </c>
+      <c r="G146" s="8">
+        <v>18</v>
+      </c>
       <c r="I146" t="s">
         <v>89</v>
       </c>
@@ -14345,11 +15329,33 @@
       <c r="L146" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="147" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N146" s="6"/>
+      <c r="O146" s="5"/>
+    </row>
+    <row r="147" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A147" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B147" s="6">
+        <v>15.23</v>
+      </c>
+      <c r="C147" s="5">
+        <f t="shared" si="9"/>
+        <v>10.100000000000001</v>
+      </c>
+      <c r="D147" s="5">
+        <f t="shared" si="10"/>
+        <v>20.36</v>
+      </c>
+      <c r="E147" s="5">
+        <v>20.6</v>
+      </c>
       <c r="F147">
         <v>21</v>
       </c>
+      <c r="G147" s="8">
+        <v>24</v>
+      </c>
       <c r="I147" t="s">
         <v>89</v>
       </c>
@@ -14362,11 +15368,33 @@
       <c r="L147" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="148" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N147" s="6"/>
+      <c r="O147" s="5"/>
+    </row>
+    <row r="148" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A148" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B148" s="6">
+        <v>15.71</v>
+      </c>
+      <c r="C148" s="5">
+        <f t="shared" si="9"/>
+        <v>10.580000000000002</v>
+      </c>
+      <c r="D148" s="5">
+        <f t="shared" si="10"/>
+        <v>20.84</v>
+      </c>
+      <c r="E148" s="5">
+        <v>15.71</v>
+      </c>
       <c r="F148">
         <v>22</v>
       </c>
+      <c r="G148" s="8">
+        <v>19</v>
+      </c>
       <c r="I148" t="s">
         <v>89</v>
       </c>
@@ -14379,11 +15407,33 @@
       <c r="L148" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="149" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N148" s="6"/>
+      <c r="O148" s="5"/>
+    </row>
+    <row r="149" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A149" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B149" s="6">
+        <v>15.81</v>
+      </c>
+      <c r="C149" s="5">
+        <f t="shared" si="9"/>
+        <v>10.68</v>
+      </c>
+      <c r="D149" s="5">
+        <f t="shared" si="10"/>
+        <v>20.94</v>
+      </c>
+      <c r="E149" s="5">
+        <v>10.68</v>
+      </c>
       <c r="F149">
         <v>23</v>
       </c>
+      <c r="G149" s="8">
+        <v>10</v>
+      </c>
       <c r="I149" t="s">
         <v>89</v>
       </c>
@@ -14396,11 +15446,33 @@
       <c r="L149" s="5">
         <v>5.13</v>
       </c>
-    </row>
-    <row r="150" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N149" s="6"/>
+      <c r="O149" s="5"/>
+    </row>
+    <row r="150" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A150" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B150" s="6">
+        <v>16.32</v>
+      </c>
+      <c r="C150" s="5">
+        <f t="shared" si="9"/>
+        <v>11.190000000000001</v>
+      </c>
+      <c r="D150" s="5">
+        <f t="shared" si="10"/>
+        <v>21.45</v>
+      </c>
+      <c r="E150" s="5">
+        <v>16.32</v>
+      </c>
       <c r="F150">
         <v>24</v>
       </c>
+      <c r="G150" s="8">
+        <v>20</v>
+      </c>
       <c r="I150" t="s">
         <v>89</v>
       </c>
@@ -14414,10 +15486,30 @@
         <v>5.13</v>
       </c>
     </row>
-    <row r="151" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A151" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B151" s="6">
+        <v>17.98</v>
+      </c>
+      <c r="C151" s="5">
+        <f t="shared" si="9"/>
+        <v>12.850000000000001</v>
+      </c>
+      <c r="D151" s="5">
+        <f t="shared" si="10"/>
+        <v>23.11</v>
+      </c>
+      <c r="E151" s="5">
+        <v>23.11</v>
+      </c>
       <c r="F151">
         <v>25</v>
       </c>
+      <c r="G151" s="8">
+        <v>25</v>
+      </c>
       <c r="I151" t="s">
         <v>89</v>
       </c>
@@ -14432,8 +15524,8 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N102:O126">
-    <sortCondition ref="O102:O126"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N125:O149">
+    <sortCondition ref="O125:O149"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Added latest results to retrain models and updated paths
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C3FD66-FD97-4ECD-8E55-300680A0E774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5C4B24-9DAA-46F5-B36D-455A61C9BBF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-11595" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy_Model" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1326" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="91">
   <si>
     <t>Model</t>
   </si>
@@ -313,6 +313,9 @@
   <si>
     <t>Indianapolis Motor Speedway (Road)</t>
   </si>
+  <si>
+    <t>Indianapolis Motor Speedway (Oval)</t>
+  </si>
 </sst>
 </file>
 
@@ -403,7 +406,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -435,6 +438,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -945,7 +949,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF436913-6699-4642-91DA-EC5EA358EA79}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="12.3671875" bestFit="1" customWidth="1"/>
@@ -1320,28 +1324,28 @@
         <v>10</v>
       </c>
       <c r="B15" s="1">
-        <v>0.24390000000000001</v>
+        <v>0.2422</v>
       </c>
       <c r="C15" s="1">
-        <v>8.5800000000000001E-2</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="D15" s="1">
-        <v>0.2361</v>
+        <v>0.2359</v>
       </c>
       <c r="E15" s="1">
-        <v>0.1421</v>
+        <v>0.14430000000000001</v>
       </c>
       <c r="F15" s="1">
-        <v>0.2165</v>
+        <v>0.2162</v>
       </c>
       <c r="G15" s="1">
-        <v>0.25069999999999998</v>
+        <v>0.24759999999999999</v>
       </c>
       <c r="H15" s="1">
-        <v>0.22209999999999999</v>
+        <v>0.21940000000000001</v>
       </c>
       <c r="I15" s="1">
-        <v>0.20180000000000001</v>
+        <v>0.2069</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1349,28 +1353,28 @@
         <v>4</v>
       </c>
       <c r="B16" s="1">
-        <v>0.245</v>
+        <v>0.24560000000000001</v>
       </c>
       <c r="C16" s="1">
-        <v>5.57E-2</v>
+        <v>4.7500000000000001E-2</v>
       </c>
       <c r="D16" s="1">
-        <v>0.2417</v>
+        <v>0.24060000000000001</v>
       </c>
       <c r="E16" s="1">
-        <v>0.115</v>
+        <v>0.1235</v>
       </c>
       <c r="F16" s="1">
-        <v>0.218</v>
+        <v>0.21729999999999999</v>
       </c>
       <c r="G16" s="1">
-        <v>0.2334</v>
+        <v>0.22689999999999999</v>
       </c>
       <c r="H16" s="1">
-        <v>0.22789999999999999</v>
+        <v>0.22420000000000001</v>
       </c>
       <c r="I16" s="1">
-        <v>0.18210000000000001</v>
+        <v>0.19259999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1378,28 +1382,28 @@
         <v>8</v>
       </c>
       <c r="B17" s="1">
-        <v>0.24790000000000001</v>
+        <v>0.24629999999999999</v>
       </c>
       <c r="C17" s="1">
-        <v>3.0700000000000002E-2</v>
+        <v>4.2599999999999999E-2</v>
       </c>
       <c r="D17" s="1">
-        <v>0.23680000000000001</v>
+        <v>0.23669999999999999</v>
       </c>
       <c r="E17" s="1">
-        <v>0.1263</v>
+        <v>0.12920000000000001</v>
       </c>
       <c r="F17" s="1">
-        <v>0.21560000000000001</v>
+        <v>0.2155</v>
       </c>
       <c r="G17" s="1">
-        <v>0.25009999999999999</v>
+        <v>0.24579999999999999</v>
       </c>
       <c r="H17" s="1">
-        <v>0.21990000000000001</v>
+        <v>0.21940000000000001</v>
       </c>
       <c r="I17" s="1">
-        <v>0.20269999999999999</v>
+        <v>0.20699999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1407,28 +1411,28 @@
         <v>9</v>
       </c>
       <c r="B18" s="1">
-        <v>0.246</v>
+        <v>0.24809999999999999</v>
       </c>
       <c r="C18" s="1">
-        <v>2.5399999999999999E-2</v>
+        <v>1.9800000000000002E-2</v>
       </c>
       <c r="D18" s="1">
-        <v>0.23569999999999999</v>
+        <v>0.23519999999999999</v>
       </c>
       <c r="E18" s="1">
-        <v>0.13930000000000001</v>
+        <v>0.14610000000000001</v>
       </c>
       <c r="F18" s="1">
-        <v>0.21390000000000001</v>
+        <v>0.21529999999999999</v>
       </c>
       <c r="G18" s="1">
-        <v>0.25159999999999999</v>
+        <v>0.24479999999999999</v>
       </c>
       <c r="H18" s="1">
-        <v>0.219</v>
+        <v>0.21829999999999999</v>
       </c>
       <c r="I18" s="1">
-        <v>0.1976</v>
+        <v>0.20580000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1436,28 +1440,28 @@
         <v>21</v>
       </c>
       <c r="B19" s="1">
-        <v>0.2356</v>
+        <v>0.23530000000000001</v>
       </c>
       <c r="C19" s="1">
-        <v>0.14410000000000001</v>
+        <v>0.14810000000000001</v>
       </c>
       <c r="D19" s="1">
-        <v>0.23569999999999999</v>
+        <v>0.23519999999999999</v>
       </c>
       <c r="E19" s="1">
-        <v>0.14419999999999999</v>
+        <v>0.1482</v>
       </c>
       <c r="F19" s="1">
-        <v>0.21490000000000001</v>
+        <v>0.21560000000000001</v>
       </c>
       <c r="G19" s="1">
-        <v>0.25330000000000003</v>
+        <v>0.24779999999999999</v>
       </c>
       <c r="H19" s="1">
-        <v>0.22070000000000001</v>
+        <v>0.21870000000000001</v>
       </c>
       <c r="I19" s="1">
-        <v>0.20180000000000001</v>
+        <v>0.2079</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1465,28 +1469,28 @@
         <v>15</v>
       </c>
       <c r="B20" s="1">
-        <v>0.23569999999999999</v>
+        <v>0.2354</v>
       </c>
       <c r="C20" s="1">
-        <v>0.14149999999999999</v>
+        <v>0.14530000000000001</v>
       </c>
       <c r="D20" s="1">
-        <v>0.23569999999999999</v>
+        <v>0.23530000000000001</v>
       </c>
       <c r="E20" s="1">
-        <v>0.14369999999999999</v>
+        <v>0.14749999999999999</v>
       </c>
       <c r="F20" s="1">
-        <v>0.2147</v>
+        <v>0.21529999999999999</v>
       </c>
       <c r="G20" s="1">
-        <v>0.25490000000000002</v>
+        <v>0.25030000000000002</v>
       </c>
       <c r="H20" s="1">
-        <v>0.2198</v>
+        <v>0.21820000000000001</v>
       </c>
       <c r="I20" s="1">
-        <v>0.20380000000000001</v>
+        <v>0.2109</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1494,28 +1498,28 @@
         <v>12</v>
       </c>
       <c r="B21" s="1">
-        <v>0.23730000000000001</v>
+        <v>0.23669999999999999</v>
       </c>
       <c r="C21" s="1">
-        <v>0.13850000000000001</v>
+        <v>0.14369999999999999</v>
       </c>
       <c r="D21" s="1">
-        <v>0.2366</v>
+        <v>0.2361</v>
       </c>
       <c r="E21" s="1">
-        <v>0.14119999999999999</v>
+        <v>0.1459</v>
       </c>
       <c r="F21" s="1">
-        <v>0.2165</v>
+        <v>0.21709999999999999</v>
       </c>
       <c r="G21" s="1">
-        <v>0.24959999999999999</v>
+        <v>0.24479999999999999</v>
       </c>
       <c r="H21" s="1">
-        <v>0.22170000000000001</v>
+        <v>0.21959999999999999</v>
       </c>
       <c r="I21" s="1">
-        <v>0.20050000000000001</v>
+        <v>0.20749999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1523,86 +1527,86 @@
         <v>13</v>
       </c>
       <c r="B22" s="1">
-        <v>0.2369</v>
+        <v>0.2364</v>
       </c>
       <c r="C22" s="1">
-        <v>0.13850000000000001</v>
+        <v>0.14319999999999999</v>
       </c>
       <c r="D22" s="1">
-        <v>0.2361</v>
+        <v>0.23569999999999999</v>
       </c>
       <c r="E22" s="1">
-        <v>0.1406</v>
+        <v>0.1454</v>
       </c>
       <c r="F22" s="1">
-        <v>0.21679999999999999</v>
+        <v>0.21590000000000001</v>
       </c>
       <c r="G22" s="1">
-        <v>0.2495</v>
+        <v>0.2485</v>
       </c>
       <c r="H22" s="1">
-        <v>0.22009999999999999</v>
+        <v>0.2185</v>
       </c>
       <c r="I22" s="1">
-        <v>0.20280000000000001</v>
+        <v>0.21060000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="15" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="1">
-        <v>0.2361</v>
+        <v>0.2359</v>
       </c>
       <c r="C23" s="1">
-        <v>0.13850000000000001</v>
+        <v>0.1409</v>
       </c>
       <c r="D23" s="1">
-        <v>0.23599999999999999</v>
+        <v>0.23580000000000001</v>
       </c>
       <c r="E23" s="1">
-        <v>0.1416</v>
+        <v>0.14380000000000001</v>
       </c>
       <c r="F23" s="1">
-        <v>0.21560000000000001</v>
+        <v>0.21540000000000001</v>
       </c>
       <c r="G23" s="1">
-        <v>0.2535</v>
+        <v>0.25059999999999999</v>
       </c>
       <c r="H23" s="1">
-        <v>0.2203</v>
+        <v>0.21859999999999999</v>
       </c>
       <c r="I23" s="1">
-        <v>0.20499999999999999</v>
+        <v>0.21110000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="3" t="s">
         <v>58</v>
       </c>
       <c r="B24" s="1">
-        <v>0.23580000000000001</v>
+        <v>0.23549999999999999</v>
       </c>
       <c r="C24" s="1">
-        <v>0.1376</v>
+        <v>0.14280000000000001</v>
       </c>
       <c r="D24" s="1">
-        <v>0.23569999999999999</v>
+        <v>0.23519999999999999</v>
       </c>
       <c r="E24" s="1">
-        <v>0.13980000000000001</v>
+        <v>0.1459</v>
       </c>
       <c r="F24" s="1">
-        <v>0.2142</v>
+        <v>0.215</v>
       </c>
       <c r="G24" s="1">
-        <v>0.25490000000000002</v>
+        <v>0.24940000000000001</v>
       </c>
       <c r="H24" s="1">
-        <v>0.21909999999999999</v>
+        <v>0.21790000000000001</v>
       </c>
       <c r="I24" s="1">
-        <v>0.2026</v>
+        <v>0.21060000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1683,8 +1687,8 @@
         <v>0.20610000000000001</v>
       </c>
       <c r="G30" s="5">
-        <f>D31*25</f>
-        <v>5.4775</v>
+        <f>D32*25</f>
+        <v>5.4475000000000007</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1699,6 +1703,20 @@
       </c>
       <c r="E31" s="10">
         <v>0.2026</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" s="4">
+        <v>46154</v>
+      </c>
+      <c r="B32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D32">
+        <v>0.21790000000000001</v>
+      </c>
+      <c r="E32">
+        <v>0.21060000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1767,7 +1785,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80150BC0-64DC-411B-A1B1-FAD28F14CD71}">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10.20703125" bestFit="1" customWidth="1"/>
@@ -1827,28 +1845,28 @@
         <v>16</v>
       </c>
       <c r="B3" s="1">
-        <v>0.2349</v>
+        <v>0.23419999999999999</v>
       </c>
       <c r="C3" s="1">
-        <v>0.1376</v>
+        <v>0.1421</v>
       </c>
       <c r="D3" s="1">
-        <v>0.2344</v>
+        <v>0.2341</v>
       </c>
       <c r="E3" s="1">
-        <v>0.16039999999999999</v>
+        <v>0.16270000000000001</v>
       </c>
       <c r="F3" s="1">
-        <v>0.2155</v>
+        <v>0.21579999999999999</v>
       </c>
       <c r="G3" s="1">
-        <v>0.254</v>
+        <v>0.24510000000000001</v>
       </c>
       <c r="H3" s="1">
-        <v>0.21690000000000001</v>
+        <v>0.21310000000000001</v>
       </c>
       <c r="I3" s="1">
-        <v>0.2303</v>
+        <v>0.24740000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1856,28 +1874,28 @@
         <v>17</v>
       </c>
       <c r="B4" s="1">
-        <v>0.2374</v>
+        <v>0.23699999999999999</v>
       </c>
       <c r="C4" s="1">
-        <v>0.1278</v>
+        <v>0.13109999999999999</v>
       </c>
       <c r="D4" s="1">
-        <v>0.23269999999999999</v>
+        <v>0.23230000000000001</v>
       </c>
       <c r="E4" s="1">
-        <v>0.1638</v>
+        <v>0.1668</v>
       </c>
       <c r="F4" s="1">
-        <v>0.2127</v>
+        <v>0.21279999999999999</v>
       </c>
       <c r="G4" s="1">
-        <v>0.27310000000000001</v>
+        <v>0.27039999999999997</v>
       </c>
       <c r="H4" s="1">
-        <v>0.21540000000000001</v>
+        <v>0.21160000000000001</v>
       </c>
       <c r="I4" s="1">
-        <v>0.2452</v>
+        <v>0.25369999999999998</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1885,28 +1903,28 @@
         <v>18</v>
       </c>
       <c r="B5" s="1">
-        <v>0.23669999999999999</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="C5" s="1">
-        <v>0.1069</v>
+        <v>0.1101</v>
       </c>
       <c r="D5" s="1">
-        <v>0.23749999999999999</v>
+        <v>0.23649999999999999</v>
       </c>
       <c r="E5" s="1">
-        <v>0.1434</v>
+        <v>0.15</v>
       </c>
       <c r="F5" s="1">
-        <v>0.21060000000000001</v>
+        <v>0.2112</v>
       </c>
       <c r="G5" s="1">
-        <v>0.26910000000000001</v>
+        <v>0.25790000000000002</v>
       </c>
       <c r="H5" s="1">
-        <v>0.21879999999999999</v>
+        <v>0.21249999999999999</v>
       </c>
       <c r="I5" s="1">
-        <v>0.2392</v>
+        <v>0.2467</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1914,28 +1932,28 @@
         <v>19</v>
       </c>
       <c r="B6" s="1">
-        <v>0.23949999999999999</v>
+        <v>0.2379</v>
       </c>
       <c r="C6" s="1">
-        <v>8.3099999999999993E-2</v>
+        <v>9.0300000000000005E-2</v>
       </c>
       <c r="D6" s="1">
-        <v>0.23100000000000001</v>
+        <v>0.23039999999999999</v>
       </c>
       <c r="E6" s="1">
-        <v>0.1593</v>
+        <v>0.1618</v>
       </c>
       <c r="F6" s="1">
-        <v>0.2054</v>
+        <v>0.20680000000000001</v>
       </c>
       <c r="G6" s="1">
-        <v>0.29480000000000001</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="H6" s="1">
-        <v>0.2077</v>
+        <v>0.20449999999999999</v>
       </c>
       <c r="I6" s="1">
-        <v>0.26979999999999998</v>
+        <v>0.27810000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1943,28 +1961,28 @@
         <v>20</v>
       </c>
       <c r="B7" s="1">
-        <v>0.2424</v>
+        <v>0.24149999999999999</v>
       </c>
       <c r="C7" s="1">
-        <v>5.2400000000000002E-2</v>
+        <v>5.2900000000000003E-2</v>
       </c>
       <c r="D7" s="1">
-        <v>0.23</v>
+        <v>0.22900000000000001</v>
       </c>
       <c r="E7" s="1">
-        <v>0.17080000000000001</v>
+        <v>0.1749</v>
       </c>
       <c r="F7" s="1">
-        <v>0.20619999999999999</v>
+        <v>0.20660000000000001</v>
       </c>
       <c r="G7" s="1">
-        <v>0.29239999999999999</v>
+        <v>0.28689999999999999</v>
       </c>
       <c r="H7" s="1">
-        <v>0.20630000000000001</v>
+        <v>0.2046</v>
       </c>
       <c r="I7" s="1">
-        <v>0.26950000000000002</v>
+        <v>0.27410000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -1972,28 +1990,28 @@
         <v>24</v>
       </c>
       <c r="B8" s="1">
-        <v>0.22639999999999999</v>
+        <v>0.22589999999999999</v>
       </c>
       <c r="C8" s="1">
-        <v>0.17030000000000001</v>
+        <v>0.1739</v>
       </c>
       <c r="D8" s="1">
-        <v>0.22650000000000001</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="E8" s="1">
-        <v>0.17030000000000001</v>
+        <v>0.17399999999999999</v>
       </c>
       <c r="F8" s="1">
-        <v>0.20230000000000001</v>
+        <v>0.20319999999999999</v>
       </c>
       <c r="G8" s="1">
-        <v>0.28520000000000001</v>
+        <v>0.27539999999999998</v>
       </c>
       <c r="H8" s="1">
-        <v>0.20469999999999999</v>
+        <v>0.20169999999999999</v>
       </c>
       <c r="I8" s="1">
-        <v>0.25359999999999999</v>
+        <v>0.2626</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2001,28 +2019,28 @@
         <v>21</v>
       </c>
       <c r="B9" s="1">
-        <v>0.23100000000000001</v>
+        <v>0.23019999999999999</v>
       </c>
       <c r="C9" s="1">
-        <v>0.17119999999999999</v>
+        <v>0.17499999999999999</v>
       </c>
       <c r="D9" s="1">
-        <v>0.2303</v>
+        <v>0.22939999999999999</v>
       </c>
       <c r="E9" s="1">
-        <v>0.1719</v>
+        <v>0.1759</v>
       </c>
       <c r="F9" s="1">
-        <v>0.20710000000000001</v>
+        <v>0.20749999999999999</v>
       </c>
       <c r="G9" s="1">
-        <v>0.2913</v>
+        <v>0.28599999999999998</v>
       </c>
       <c r="H9" s="1">
-        <v>0.2077</v>
+        <v>0.2056</v>
       </c>
       <c r="I9" s="1">
-        <v>0.26750000000000002</v>
+        <v>0.27239999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2030,28 +2048,28 @@
         <v>22</v>
       </c>
       <c r="B10" s="1">
-        <v>0.23050000000000001</v>
+        <v>0.22989999999999999</v>
       </c>
       <c r="C10" s="1">
-        <v>0.1714</v>
+        <v>0.17449999999999999</v>
       </c>
       <c r="D10" s="1">
-        <v>0.23019999999999999</v>
+        <v>0.22939999999999999</v>
       </c>
       <c r="E10" s="1">
-        <v>0.17249999999999999</v>
+        <v>0.17599999999999999</v>
       </c>
       <c r="F10" s="1">
-        <v>0.20680000000000001</v>
+        <v>0.2074</v>
       </c>
       <c r="G10" s="1">
-        <v>0.29339999999999999</v>
+        <v>0.28720000000000001</v>
       </c>
       <c r="H10" s="1">
-        <v>0.2077</v>
+        <v>0.20530000000000001</v>
       </c>
       <c r="I10" s="1">
-        <v>0.26939999999999997</v>
+        <v>0.2747</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2059,28 +2077,28 @@
         <v>52</v>
       </c>
       <c r="B11" s="1">
-        <v>0.23039999999999999</v>
+        <v>0.2293</v>
       </c>
       <c r="C11" s="1">
-        <v>0.17519999999999999</v>
+        <v>0.17860000000000001</v>
       </c>
       <c r="D11" s="1">
-        <v>0.2298</v>
+        <v>0.2288</v>
       </c>
       <c r="E11" s="1">
-        <v>0.1774</v>
+        <v>0.18140000000000001</v>
       </c>
       <c r="F11" s="1">
-        <v>0.20799999999999999</v>
+        <v>0.20749999999999999</v>
       </c>
       <c r="G11" s="1">
-        <v>0.29249999999999998</v>
+        <v>0.28710000000000002</v>
       </c>
       <c r="H11" s="1">
-        <v>0.20899999999999999</v>
+        <v>0.20569999999999999</v>
       </c>
       <c r="I11" s="1">
-        <v>0.2681</v>
+        <v>0.2777</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2088,28 +2106,28 @@
         <v>53</v>
       </c>
       <c r="B12" s="1">
-        <v>0.22800000000000001</v>
+        <v>0.2273</v>
       </c>
       <c r="C12" s="1">
-        <v>0.17749999999999999</v>
+        <v>0.18079999999999999</v>
       </c>
       <c r="D12" s="1">
-        <v>0.2273</v>
+        <v>0.22670000000000001</v>
       </c>
       <c r="E12" s="1">
-        <v>0.17929999999999999</v>
+        <v>0.18279999999999999</v>
       </c>
       <c r="F12" s="1">
-        <v>0.20369999999999999</v>
+        <v>0.20469999999999999</v>
       </c>
       <c r="G12" s="1">
-        <v>0.2979</v>
+        <v>0.28960000000000002</v>
       </c>
       <c r="H12" s="1">
-        <v>0.20519999999999999</v>
+        <v>0.20250000000000001</v>
       </c>
       <c r="I12" s="1">
-        <v>0.27210000000000001</v>
+        <v>0.27860000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2117,28 +2135,28 @@
         <v>23</v>
       </c>
       <c r="B13" s="1">
-        <v>0.2296</v>
+        <v>0.2291</v>
       </c>
       <c r="C13" s="1">
-        <v>0.17710000000000001</v>
+        <v>0.18090000000000001</v>
       </c>
       <c r="D13" s="1">
-        <v>0.2281</v>
+        <v>0.2276</v>
       </c>
       <c r="E13" s="1">
-        <v>0.1797</v>
+        <v>0.1837</v>
       </c>
       <c r="F13" s="1">
-        <v>0.20619999999999999</v>
+        <v>0.20680000000000001</v>
       </c>
       <c r="G13" s="1">
-        <v>0.29249999999999998</v>
+        <v>0.28439999999999999</v>
       </c>
       <c r="H13" s="1">
-        <v>0.2079</v>
+        <v>0.20469999999999999</v>
       </c>
       <c r="I13" s="1">
-        <v>0.2661</v>
+        <v>0.27589999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2146,28 +2164,28 @@
         <v>56</v>
       </c>
       <c r="B14" s="1">
-        <v>0.23280000000000001</v>
+        <v>0.23089999999999999</v>
       </c>
       <c r="C14" s="1">
-        <v>0.1661</v>
+        <v>0.1696</v>
       </c>
       <c r="D14" s="1">
-        <v>0.23200000000000001</v>
+        <v>0.23039999999999999</v>
       </c>
       <c r="E14" s="1">
-        <v>0.1686</v>
+        <v>0.1736</v>
       </c>
       <c r="F14" s="1">
-        <v>0.2109</v>
+        <v>0.2092</v>
       </c>
       <c r="G14" s="1">
-        <v>0.28249999999999997</v>
+        <v>0.2828</v>
       </c>
       <c r="H14" s="1">
-        <v>0.2117</v>
+        <v>0.2079</v>
       </c>
       <c r="I14" s="1">
-        <v>0.26019999999999999</v>
+        <v>0.2702</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2175,28 +2193,28 @@
         <v>60</v>
       </c>
       <c r="B15" s="1">
-        <v>0.2319</v>
+        <v>0.23039999999999999</v>
       </c>
       <c r="C15" s="1">
-        <v>0.16830000000000001</v>
+        <v>0.17119999999999999</v>
       </c>
       <c r="D15" s="1">
-        <v>0.23080000000000001</v>
+        <v>0.2296</v>
       </c>
       <c r="E15" s="1">
-        <v>0.17130000000000001</v>
+        <v>0.17530000000000001</v>
       </c>
       <c r="F15" s="1">
-        <v>0.2079</v>
+        <v>0.20760000000000001</v>
       </c>
       <c r="G15" s="1">
-        <v>0.2918</v>
+        <v>0.28699999999999998</v>
       </c>
       <c r="H15" s="1">
-        <v>0.2087</v>
+        <v>0.20569999999999999</v>
       </c>
       <c r="I15" s="1">
-        <v>0.26889999999999997</v>
+        <v>0.27629999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -2204,147 +2222,147 @@
         <v>54</v>
       </c>
       <c r="B16" s="1">
-        <v>0.23119999999999999</v>
+        <v>0.23069999999999999</v>
       </c>
       <c r="C16" s="1">
-        <v>0.16769999999999999</v>
+        <v>0.17019999999999999</v>
       </c>
       <c r="D16" s="1">
-        <v>0.23130000000000001</v>
+        <v>0.23089999999999999</v>
       </c>
       <c r="E16" s="1">
-        <v>0.16789999999999999</v>
+        <v>0.17050000000000001</v>
       </c>
       <c r="F16" s="1">
-        <v>0.20849999999999999</v>
+        <v>0.2092</v>
       </c>
       <c r="G16" s="1">
-        <v>0.28920000000000001</v>
+        <v>0.2828</v>
       </c>
       <c r="H16" s="1">
-        <v>0.21049999999999999</v>
+        <v>0.20730000000000001</v>
       </c>
       <c r="I16" s="1">
-        <v>0.26319999999999999</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0.27100000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B17" s="1">
-        <v>0.22989999999999999</v>
+        <v>0.22919999999999999</v>
       </c>
       <c r="C17" s="1">
-        <v>0.17030000000000001</v>
+        <v>0.1734</v>
       </c>
       <c r="D17" s="1">
-        <v>0.22989999999999999</v>
+        <v>0.22900000000000001</v>
       </c>
       <c r="E17" s="1">
-        <v>0.1719</v>
+        <v>0.1754</v>
       </c>
       <c r="F17" s="1">
-        <v>0.2054</v>
+        <v>0.2064</v>
       </c>
       <c r="G17" s="1">
-        <v>0.29659999999999997</v>
+        <v>0.28860000000000002</v>
       </c>
       <c r="H17" s="1">
-        <v>0.2064</v>
+        <v>0.2041</v>
       </c>
       <c r="I17" s="1">
-        <v>0.27300000000000002</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0.2787</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B18" s="1">
-        <v>0.23019999999999999</v>
+        <v>0.2288</v>
       </c>
       <c r="C18" s="1">
-        <v>0.17480000000000001</v>
+        <v>0.1782</v>
       </c>
       <c r="D18" s="1">
-        <v>0.22839999999999999</v>
+        <v>0.22750000000000001</v>
       </c>
       <c r="E18" s="1">
-        <v>0.1777</v>
+        <v>0.1812</v>
       </c>
       <c r="F18" s="1">
-        <v>0.20480000000000001</v>
+        <v>0.2051</v>
       </c>
       <c r="G18" s="1">
-        <v>0.29680000000000001</v>
+        <v>0.28910000000000002</v>
       </c>
       <c r="H18" s="1">
-        <v>0.20630000000000001</v>
+        <v>0.20330000000000001</v>
       </c>
       <c r="I18" s="1">
-        <v>0.27079999999999999</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0.27850000000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B19" s="1">
-        <v>0.23300000000000001</v>
+        <v>0.23089999999999999</v>
       </c>
       <c r="C19" s="1">
-        <v>0.1651</v>
+        <v>0.1641</v>
       </c>
       <c r="D19" s="1">
-        <v>0.23119999999999999</v>
+        <v>0.22919999999999999</v>
       </c>
       <c r="E19" s="1">
-        <v>0.17030000000000001</v>
+        <v>0.1754</v>
       </c>
       <c r="F19" s="1">
-        <v>0.20860000000000001</v>
+        <v>0.20710000000000001</v>
       </c>
       <c r="G19" s="1">
-        <v>0.28899999999999998</v>
+        <v>0.28589999999999999</v>
       </c>
       <c r="H19" s="1">
-        <v>0.20849999999999999</v>
+        <v>0.20580000000000001</v>
       </c>
       <c r="I19" s="1">
-        <v>0.26869999999999999</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0.2757</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B20" s="1">
-        <v>0.2334</v>
+        <v>0.2321</v>
       </c>
       <c r="C20" s="1">
-        <v>0.16070000000000001</v>
+        <v>0.15340000000000001</v>
       </c>
       <c r="D20" s="1">
-        <v>0.23169999999999999</v>
+        <v>0.2306</v>
       </c>
       <c r="E20" s="1">
-        <v>0.16200000000000001</v>
+        <v>0.1628</v>
       </c>
       <c r="F20" s="1">
-        <v>0.2077</v>
+        <v>0.2072</v>
       </c>
       <c r="G20" s="1">
-        <v>0.29160000000000003</v>
+        <v>0.28460000000000002</v>
       </c>
       <c r="H20" s="1">
-        <v>0.2092</v>
+        <v>0.2056</v>
       </c>
       <c r="I20" s="1">
-        <v>0.26889999999999997</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0.27889999999999998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" t="s">
         <v>16</v>
       </c>
@@ -2352,7 +2370,7 @@
         <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E21" t="s">
         <v>64</v>
@@ -2364,7 +2382,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="C22" t="s">
         <v>1</v>
       </c>
@@ -2372,7 +2390,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="4">
         <v>46085</v>
       </c>
@@ -2386,7 +2404,7 @@
         <v>0.2006</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="4">
         <v>46090</v>
       </c>
@@ -2400,7 +2418,7 @@
         <v>0.2334</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="4">
         <v>46098</v>
       </c>
@@ -2414,7 +2432,7 @@
         <v>0.24890000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="4">
         <v>46112</v>
       </c>
@@ -2428,7 +2446,7 @@
         <v>0.2727</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="4">
         <v>46151</v>
       </c>
@@ -2440,6 +2458,21 @@
       </c>
       <c r="D27">
         <v>0.27210000000000001</v>
+      </c>
+      <c r="J27" s="5"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="4">
+        <v>46154</v>
+      </c>
+      <c r="B28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28">
+        <v>0.20250000000000001</v>
+      </c>
+      <c r="D28">
+        <v>0.27860000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2455,7 +2488,7 @@
   <conditionalFormatting sqref="C3:C21">
     <cfRule type="top10" dxfId="7" priority="117" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D21 D24:D27">
+  <conditionalFormatting sqref="D3:D21 D24:D28">
     <cfRule type="top10" dxfId="6" priority="6" bottom="1" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E21">
@@ -7713,7 +7746,9 @@
       <c r="G127" s="8">
         <v>1</v>
       </c>
-      <c r="H127" s="8"/>
+      <c r="H127" s="8">
+        <v>5</v>
+      </c>
       <c r="I127" t="s">
         <v>89</v>
       </c>
@@ -7751,7 +7786,9 @@
       <c r="G128" s="8">
         <v>8</v>
       </c>
-      <c r="H128" s="8"/>
+      <c r="H128" s="8">
+        <v>6</v>
+      </c>
       <c r="I128" t="s">
         <v>89</v>
       </c>
@@ -7791,7 +7828,9 @@
       <c r="G129" s="8">
         <v>9</v>
       </c>
-      <c r="H129" s="8"/>
+      <c r="H129" s="8">
+        <v>16</v>
+      </c>
       <c r="I129" t="s">
         <v>89</v>
       </c>
@@ -7831,7 +7870,9 @@
       <c r="G130" s="8">
         <v>2</v>
       </c>
-      <c r="H130" s="8"/>
+      <c r="H130" s="8">
+        <v>1</v>
+      </c>
       <c r="I130" t="s">
         <v>89</v>
       </c>
@@ -7871,7 +7912,9 @@
       <c r="G131" s="8">
         <v>3</v>
       </c>
-      <c r="H131" s="8"/>
+      <c r="H131" s="8">
+        <v>18</v>
+      </c>
       <c r="I131" t="s">
         <v>89</v>
       </c>
@@ -7911,7 +7954,9 @@
       <c r="G132" s="8">
         <v>11</v>
       </c>
-      <c r="H132" s="8"/>
+      <c r="H132" s="8">
+        <v>4</v>
+      </c>
       <c r="I132" t="s">
         <v>89</v>
       </c>
@@ -7951,7 +7996,9 @@
       <c r="G133" s="8">
         <v>4</v>
       </c>
-      <c r="H133" s="8"/>
+      <c r="H133" s="8">
+        <v>9</v>
+      </c>
       <c r="I133" t="s">
         <v>89</v>
       </c>
@@ -7991,7 +8038,9 @@
       <c r="G134" s="8">
         <v>12</v>
       </c>
-      <c r="H134" s="8"/>
+      <c r="H134" s="8">
+        <v>11</v>
+      </c>
       <c r="I134" t="s">
         <v>89</v>
       </c>
@@ -8031,7 +8080,9 @@
       <c r="G135" s="8">
         <v>5</v>
       </c>
-      <c r="H135" s="8"/>
+      <c r="H135" s="8">
+        <v>2</v>
+      </c>
       <c r="I135" t="s">
         <v>89</v>
       </c>
@@ -8071,7 +8122,9 @@
       <c r="G136" s="8">
         <v>13</v>
       </c>
-      <c r="H136" s="8"/>
+      <c r="H136" s="8">
+        <v>13</v>
+      </c>
       <c r="I136" t="s">
         <v>89</v>
       </c>
@@ -8111,7 +8164,9 @@
       <c r="G137" s="8">
         <v>14</v>
       </c>
-      <c r="H137" s="8"/>
+      <c r="H137" s="8">
+        <v>22</v>
+      </c>
       <c r="I137" t="s">
         <v>89</v>
       </c>
@@ -8151,7 +8206,9 @@
       <c r="G138" s="8">
         <v>15</v>
       </c>
-      <c r="H138" s="8"/>
+      <c r="H138" s="8">
+        <v>25</v>
+      </c>
       <c r="I138" t="s">
         <v>89</v>
       </c>
@@ -8191,7 +8248,9 @@
       <c r="G139" s="8">
         <v>6</v>
       </c>
-      <c r="H139" s="8"/>
+      <c r="H139" s="8">
+        <v>3</v>
+      </c>
       <c r="I139" t="s">
         <v>89</v>
       </c>
@@ -8231,7 +8290,9 @@
       <c r="G140" s="8">
         <v>7</v>
       </c>
-      <c r="H140" s="8"/>
+      <c r="H140" s="8">
+        <v>23</v>
+      </c>
       <c r="I140" t="s">
         <v>89</v>
       </c>
@@ -8271,7 +8332,9 @@
       <c r="G141" s="8">
         <v>16</v>
       </c>
-      <c r="H141" s="8"/>
+      <c r="H141" s="8">
+        <v>12</v>
+      </c>
       <c r="I141" t="s">
         <v>89</v>
       </c>
@@ -8311,7 +8374,9 @@
       <c r="G142" s="8">
         <v>17</v>
       </c>
-      <c r="H142" s="8"/>
+      <c r="H142" s="8">
+        <v>21</v>
+      </c>
       <c r="I142" t="s">
         <v>89</v>
       </c>
@@ -8351,7 +8416,9 @@
       <c r="G143" s="8">
         <v>24</v>
       </c>
-      <c r="H143" s="8"/>
+      <c r="H143" s="8">
+        <v>24</v>
+      </c>
       <c r="I143" t="s">
         <v>89</v>
       </c>
@@ -8391,7 +8458,9 @@
       <c r="G144" s="8">
         <v>18</v>
       </c>
-      <c r="H144" s="8"/>
+      <c r="H144" s="8">
+        <v>15</v>
+      </c>
       <c r="I144" t="s">
         <v>89</v>
       </c>
@@ -8431,7 +8500,9 @@
       <c r="G145" s="8">
         <v>19</v>
       </c>
-      <c r="H145" s="8"/>
+      <c r="H145" s="8">
+        <v>14</v>
+      </c>
       <c r="I145" t="s">
         <v>89</v>
       </c>
@@ -8471,7 +8542,9 @@
       <c r="G146" s="8">
         <v>10</v>
       </c>
-      <c r="H146" s="8"/>
+      <c r="H146" s="8">
+        <v>7</v>
+      </c>
       <c r="I146" t="s">
         <v>89</v>
       </c>
@@ -8511,7 +8584,9 @@
       <c r="G147" s="8">
         <v>20</v>
       </c>
-      <c r="H147" s="8"/>
+      <c r="H147" s="8">
+        <v>10</v>
+      </c>
       <c r="I147" t="s">
         <v>89</v>
       </c>
@@ -8551,7 +8626,9 @@
       <c r="G148" s="8">
         <v>21</v>
       </c>
-      <c r="H148" s="8"/>
+      <c r="H148" s="8">
+        <v>19</v>
+      </c>
       <c r="I148" t="s">
         <v>89</v>
       </c>
@@ -8591,7 +8668,9 @@
       <c r="G149" s="8">
         <v>22</v>
       </c>
-      <c r="H149" s="8"/>
+      <c r="H149" s="8">
+        <v>8</v>
+      </c>
       <c r="I149" t="s">
         <v>89</v>
       </c>
@@ -8631,7 +8710,9 @@
       <c r="G150" s="8">
         <v>23</v>
       </c>
-      <c r="H150" s="8"/>
+      <c r="H150" s="8">
+        <v>20</v>
+      </c>
       <c r="I150" t="s">
         <v>89</v>
       </c>
@@ -8671,7 +8752,9 @@
       <c r="G151" s="8">
         <v>25</v>
       </c>
-      <c r="H151" s="8"/>
+      <c r="H151" s="8">
+        <v>17</v>
+      </c>
       <c r="I151" t="s">
         <v>89</v>
       </c>
@@ -8688,81 +8771,456 @@
       <c r="O151" s="5"/>
     </row>
     <row r="152" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F152">
+        <v>1</v>
+      </c>
       <c r="H152" s="8"/>
+      <c r="I152" t="s">
+        <v>90</v>
+      </c>
+      <c r="J152" t="s">
+        <v>85</v>
+      </c>
+      <c r="K152" t="s">
+        <v>77</v>
+      </c>
+      <c r="L152">
+        <v>5.45</v>
+      </c>
       <c r="N152" s="6"/>
       <c r="O152" s="5"/>
     </row>
     <row r="153" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F153">
+        <v>2</v>
+      </c>
       <c r="H153" s="8"/>
+      <c r="I153" t="s">
+        <v>90</v>
+      </c>
+      <c r="J153" t="s">
+        <v>85</v>
+      </c>
+      <c r="K153" t="s">
+        <v>77</v>
+      </c>
+      <c r="L153">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="154" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F154">
+        <v>3</v>
+      </c>
       <c r="H154" s="8"/>
+      <c r="I154" t="s">
+        <v>90</v>
+      </c>
+      <c r="J154" t="s">
+        <v>85</v>
+      </c>
+      <c r="K154" t="s">
+        <v>77</v>
+      </c>
+      <c r="L154">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="155" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F155">
+        <v>4</v>
+      </c>
       <c r="H155" s="8"/>
+      <c r="I155" t="s">
+        <v>90</v>
+      </c>
+      <c r="J155" t="s">
+        <v>85</v>
+      </c>
+      <c r="K155" t="s">
+        <v>77</v>
+      </c>
+      <c r="L155">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="156" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F156">
+        <v>5</v>
+      </c>
       <c r="H156" s="8"/>
+      <c r="I156" t="s">
+        <v>90</v>
+      </c>
+      <c r="J156" t="s">
+        <v>85</v>
+      </c>
+      <c r="K156" t="s">
+        <v>77</v>
+      </c>
+      <c r="L156">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="157" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F157">
+        <v>6</v>
+      </c>
       <c r="H157" s="8"/>
+      <c r="I157" t="s">
+        <v>90</v>
+      </c>
+      <c r="J157" t="s">
+        <v>85</v>
+      </c>
+      <c r="K157" t="s">
+        <v>77</v>
+      </c>
+      <c r="L157">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="158" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F158">
+        <v>7</v>
+      </c>
       <c r="H158" s="8"/>
+      <c r="I158" t="s">
+        <v>90</v>
+      </c>
+      <c r="J158" t="s">
+        <v>85</v>
+      </c>
+      <c r="K158" t="s">
+        <v>77</v>
+      </c>
+      <c r="L158">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="159" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F159">
+        <v>8</v>
+      </c>
       <c r="H159" s="8"/>
+      <c r="I159" t="s">
+        <v>90</v>
+      </c>
+      <c r="J159" t="s">
+        <v>85</v>
+      </c>
+      <c r="K159" t="s">
+        <v>77</v>
+      </c>
+      <c r="L159">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="160" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F160">
+        <v>9</v>
+      </c>
       <c r="H160" s="8"/>
-    </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I160" t="s">
+        <v>90</v>
+      </c>
+      <c r="J160" t="s">
+        <v>85</v>
+      </c>
+      <c r="K160" t="s">
+        <v>77</v>
+      </c>
+      <c r="L160">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="161" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F161">
+        <v>10</v>
+      </c>
       <c r="H161" s="8"/>
-    </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I161" t="s">
+        <v>90</v>
+      </c>
+      <c r="J161" t="s">
+        <v>85</v>
+      </c>
+      <c r="K161" t="s">
+        <v>77</v>
+      </c>
+      <c r="L161">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="162" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F162">
+        <v>11</v>
+      </c>
       <c r="H162" s="8"/>
-    </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I162" t="s">
+        <v>90</v>
+      </c>
+      <c r="J162" t="s">
+        <v>85</v>
+      </c>
+      <c r="K162" t="s">
+        <v>77</v>
+      </c>
+      <c r="L162">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="163" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F163">
+        <v>12</v>
+      </c>
       <c r="H163" s="8"/>
-    </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I163" t="s">
+        <v>90</v>
+      </c>
+      <c r="J163" t="s">
+        <v>85</v>
+      </c>
+      <c r="K163" t="s">
+        <v>77</v>
+      </c>
+      <c r="L163">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="164" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F164">
+        <v>13</v>
+      </c>
       <c r="H164" s="8"/>
-    </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I164" t="s">
+        <v>90</v>
+      </c>
+      <c r="J164" t="s">
+        <v>85</v>
+      </c>
+      <c r="K164" t="s">
+        <v>77</v>
+      </c>
+      <c r="L164">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="165" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F165">
+        <v>14</v>
+      </c>
       <c r="H165" s="8"/>
-    </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I165" t="s">
+        <v>90</v>
+      </c>
+      <c r="J165" t="s">
+        <v>85</v>
+      </c>
+      <c r="K165" t="s">
+        <v>77</v>
+      </c>
+      <c r="L165">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="166" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F166">
+        <v>15</v>
+      </c>
       <c r="H166" s="8"/>
-    </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I166" t="s">
+        <v>90</v>
+      </c>
+      <c r="J166" t="s">
+        <v>85</v>
+      </c>
+      <c r="K166" t="s">
+        <v>77</v>
+      </c>
+      <c r="L166">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="167" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F167">
+        <v>16</v>
+      </c>
       <c r="H167" s="8"/>
-    </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I167" t="s">
+        <v>90</v>
+      </c>
+      <c r="J167" t="s">
+        <v>85</v>
+      </c>
+      <c r="K167" t="s">
+        <v>77</v>
+      </c>
+      <c r="L167">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="168" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F168">
+        <v>17</v>
+      </c>
       <c r="H168" s="8"/>
-    </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I168" t="s">
+        <v>90</v>
+      </c>
+      <c r="J168" t="s">
+        <v>85</v>
+      </c>
+      <c r="K168" t="s">
+        <v>77</v>
+      </c>
+      <c r="L168">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="169" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F169">
+        <v>18</v>
+      </c>
       <c r="H169" s="8"/>
-    </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I169" t="s">
+        <v>90</v>
+      </c>
+      <c r="J169" t="s">
+        <v>85</v>
+      </c>
+      <c r="K169" t="s">
+        <v>77</v>
+      </c>
+      <c r="L169">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="170" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F170">
+        <v>19</v>
+      </c>
       <c r="H170" s="8"/>
-    </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I170" t="s">
+        <v>90</v>
+      </c>
+      <c r="J170" t="s">
+        <v>85</v>
+      </c>
+      <c r="K170" t="s">
+        <v>77</v>
+      </c>
+      <c r="L170">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="171" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F171">
+        <v>20</v>
+      </c>
       <c r="H171" s="8"/>
-    </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I171" t="s">
+        <v>90</v>
+      </c>
+      <c r="J171" t="s">
+        <v>85</v>
+      </c>
+      <c r="K171" t="s">
+        <v>77</v>
+      </c>
+      <c r="L171">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="172" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F172">
+        <v>21</v>
+      </c>
       <c r="H172" s="8"/>
-    </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I172" t="s">
+        <v>90</v>
+      </c>
+      <c r="J172" t="s">
+        <v>85</v>
+      </c>
+      <c r="K172" t="s">
+        <v>77</v>
+      </c>
+      <c r="L172">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="173" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F173">
+        <v>22</v>
+      </c>
       <c r="H173" s="8"/>
-    </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I173" t="s">
+        <v>90</v>
+      </c>
+      <c r="J173" t="s">
+        <v>85</v>
+      </c>
+      <c r="K173" t="s">
+        <v>77</v>
+      </c>
+      <c r="L173">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="174" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F174">
+        <v>23</v>
+      </c>
       <c r="H174" s="8"/>
-    </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I174" t="s">
+        <v>90</v>
+      </c>
+      <c r="J174" t="s">
+        <v>85</v>
+      </c>
+      <c r="K174" t="s">
+        <v>77</v>
+      </c>
+      <c r="L174">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="175" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F175">
+        <v>24</v>
+      </c>
       <c r="H175" s="8"/>
-    </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I175" t="s">
+        <v>90</v>
+      </c>
+      <c r="J175" t="s">
+        <v>85</v>
+      </c>
+      <c r="K175" t="s">
+        <v>77</v>
+      </c>
+      <c r="L175">
+        <v>5.45</v>
+      </c>
+    </row>
+    <row r="176" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F176">
+        <v>25</v>
+      </c>
       <c r="H176" s="8"/>
+      <c r="I176" t="s">
+        <v>90</v>
+      </c>
+      <c r="J176" t="s">
+        <v>85</v>
+      </c>
+      <c r="K176" t="s">
+        <v>77</v>
+      </c>
+      <c r="L176">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="177" spans="8:8" x14ac:dyDescent="0.55000000000000004">
       <c r="H177" s="8"/>
@@ -9322,7 +9780,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O151"/>
+  <dimension ref="A1:O176"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="18.3671875" bestFit="1" customWidth="1"/>
@@ -14576,6 +15034,9 @@
       <c r="G127" s="8">
         <v>1</v>
       </c>
+      <c r="H127" s="8">
+        <v>5</v>
+      </c>
       <c r="I127" t="s">
         <v>89</v>
       </c>
@@ -14615,6 +15076,9 @@
       <c r="G128" s="8">
         <v>2</v>
       </c>
+      <c r="H128" s="8">
+        <v>18</v>
+      </c>
       <c r="I128" t="s">
         <v>89</v>
       </c>
@@ -14654,6 +15118,9 @@
       <c r="G129" s="8">
         <v>7</v>
       </c>
+      <c r="H129" s="8">
+        <v>6</v>
+      </c>
       <c r="I129" t="s">
         <v>89</v>
       </c>
@@ -14693,6 +15160,9 @@
       <c r="G130" s="8">
         <v>3</v>
       </c>
+      <c r="H130" s="8">
+        <v>1</v>
+      </c>
       <c r="I130" t="s">
         <v>89</v>
       </c>
@@ -14732,6 +15202,9 @@
       <c r="G131" s="8">
         <v>4</v>
       </c>
+      <c r="H131" s="8">
+        <v>2</v>
+      </c>
       <c r="I131" t="s">
         <v>89</v>
       </c>
@@ -14771,6 +15244,9 @@
       <c r="G132" s="8">
         <v>5</v>
       </c>
+      <c r="H132" s="8">
+        <v>9</v>
+      </c>
       <c r="I132" t="s">
         <v>89</v>
       </c>
@@ -14810,6 +15286,9 @@
       <c r="G133" s="8">
         <v>8</v>
       </c>
+      <c r="H133" s="8">
+        <v>4</v>
+      </c>
       <c r="I133" t="s">
         <v>89</v>
       </c>
@@ -14849,6 +15328,9 @@
       <c r="G134" s="8">
         <v>9</v>
       </c>
+      <c r="H134" s="8">
+        <v>23</v>
+      </c>
       <c r="I134" t="s">
         <v>89</v>
       </c>
@@ -14888,6 +15370,9 @@
       <c r="G135" s="8">
         <v>6</v>
       </c>
+      <c r="H135" s="8">
+        <v>3</v>
+      </c>
       <c r="I135" t="s">
         <v>89</v>
       </c>
@@ -14927,6 +15412,9 @@
       <c r="G136" s="8">
         <v>11</v>
       </c>
+      <c r="H136" s="8">
+        <v>16</v>
+      </c>
       <c r="I136" t="s">
         <v>89</v>
       </c>
@@ -14966,6 +15454,9 @@
       <c r="G137" s="8">
         <v>12</v>
       </c>
+      <c r="H137" s="8">
+        <v>11</v>
+      </c>
       <c r="I137" t="s">
         <v>89</v>
       </c>
@@ -15005,6 +15496,9 @@
       <c r="G138" s="8">
         <v>21</v>
       </c>
+      <c r="H138" s="8">
+        <v>22</v>
+      </c>
       <c r="I138" t="s">
         <v>89</v>
       </c>
@@ -15044,6 +15538,9 @@
       <c r="G139" s="8">
         <v>13</v>
       </c>
+      <c r="H139" s="8">
+        <v>13</v>
+      </c>
       <c r="I139" t="s">
         <v>89</v>
       </c>
@@ -15083,6 +15580,9 @@
       <c r="G140" s="8">
         <v>14</v>
       </c>
+      <c r="H140" s="8">
+        <v>7</v>
+      </c>
       <c r="I140" t="s">
         <v>89</v>
       </c>
@@ -15122,6 +15622,9 @@
       <c r="G141" s="8">
         <v>15</v>
       </c>
+      <c r="H141" s="8">
+        <v>25</v>
+      </c>
       <c r="I141" t="s">
         <v>89</v>
       </c>
@@ -15161,6 +15664,9 @@
       <c r="G142" s="8">
         <v>22</v>
       </c>
+      <c r="H142" s="8">
+        <v>12</v>
+      </c>
       <c r="I142" t="s">
         <v>89</v>
       </c>
@@ -15200,6 +15706,9 @@
       <c r="G143" s="8">
         <v>16</v>
       </c>
+      <c r="H143" s="8">
+        <v>21</v>
+      </c>
       <c r="I143" t="s">
         <v>89</v>
       </c>
@@ -15239,6 +15748,9 @@
       <c r="G144" s="8">
         <v>17</v>
       </c>
+      <c r="H144" s="8">
+        <v>10</v>
+      </c>
       <c r="I144" t="s">
         <v>89</v>
       </c>
@@ -15278,6 +15790,9 @@
       <c r="G145" s="8">
         <v>23</v>
       </c>
+      <c r="H145" s="8">
+        <v>14</v>
+      </c>
       <c r="I145" t="s">
         <v>89</v>
       </c>
@@ -15317,6 +15832,9 @@
       <c r="G146" s="8">
         <v>18</v>
       </c>
+      <c r="H146" s="8">
+        <v>15</v>
+      </c>
       <c r="I146" t="s">
         <v>89</v>
       </c>
@@ -15356,6 +15874,9 @@
       <c r="G147" s="8">
         <v>24</v>
       </c>
+      <c r="H147" s="8">
+        <v>24</v>
+      </c>
       <c r="I147" t="s">
         <v>89</v>
       </c>
@@ -15395,6 +15916,9 @@
       <c r="G148" s="8">
         <v>19</v>
       </c>
+      <c r="H148" s="8">
+        <v>20</v>
+      </c>
       <c r="I148" t="s">
         <v>89</v>
       </c>
@@ -15434,6 +15958,9 @@
       <c r="G149" s="8">
         <v>10</v>
       </c>
+      <c r="H149" s="8">
+        <v>19</v>
+      </c>
       <c r="I149" t="s">
         <v>89</v>
       </c>
@@ -15473,6 +16000,9 @@
       <c r="G150" s="8">
         <v>20</v>
       </c>
+      <c r="H150" s="8">
+        <v>8</v>
+      </c>
       <c r="I150" t="s">
         <v>89</v>
       </c>
@@ -15510,6 +16040,9 @@
       <c r="G151" s="8">
         <v>25</v>
       </c>
+      <c r="H151" s="8">
+        <v>17</v>
+      </c>
       <c r="I151" t="s">
         <v>89</v>
       </c>
@@ -15521,6 +16054,431 @@
       </c>
       <c r="L151" s="5">
         <v>5.13</v>
+      </c>
+    </row>
+    <row r="152" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F152">
+        <v>1</v>
+      </c>
+      <c r="I152" t="s">
+        <v>90</v>
+      </c>
+      <c r="J152" t="s">
+        <v>85</v>
+      </c>
+      <c r="K152" t="s">
+        <v>86</v>
+      </c>
+      <c r="L152" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="153" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F153">
+        <v>2</v>
+      </c>
+      <c r="I153" t="s">
+        <v>90</v>
+      </c>
+      <c r="J153" t="s">
+        <v>85</v>
+      </c>
+      <c r="K153" t="s">
+        <v>86</v>
+      </c>
+      <c r="L153" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="154" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F154">
+        <v>3</v>
+      </c>
+      <c r="I154" t="s">
+        <v>90</v>
+      </c>
+      <c r="J154" t="s">
+        <v>85</v>
+      </c>
+      <c r="K154" t="s">
+        <v>86</v>
+      </c>
+      <c r="L154" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="155" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F155">
+        <v>4</v>
+      </c>
+      <c r="I155" t="s">
+        <v>90</v>
+      </c>
+      <c r="J155" t="s">
+        <v>85</v>
+      </c>
+      <c r="K155" t="s">
+        <v>86</v>
+      </c>
+      <c r="L155" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="156" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F156">
+        <v>5</v>
+      </c>
+      <c r="I156" t="s">
+        <v>90</v>
+      </c>
+      <c r="J156" t="s">
+        <v>85</v>
+      </c>
+      <c r="K156" t="s">
+        <v>86</v>
+      </c>
+      <c r="L156" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="157" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F157">
+        <v>6</v>
+      </c>
+      <c r="I157" t="s">
+        <v>90</v>
+      </c>
+      <c r="J157" t="s">
+        <v>85</v>
+      </c>
+      <c r="K157" t="s">
+        <v>86</v>
+      </c>
+      <c r="L157" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="158" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F158">
+        <v>7</v>
+      </c>
+      <c r="I158" t="s">
+        <v>90</v>
+      </c>
+      <c r="J158" t="s">
+        <v>85</v>
+      </c>
+      <c r="K158" t="s">
+        <v>86</v>
+      </c>
+      <c r="L158" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="159" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F159">
+        <v>8</v>
+      </c>
+      <c r="I159" t="s">
+        <v>90</v>
+      </c>
+      <c r="J159" t="s">
+        <v>85</v>
+      </c>
+      <c r="K159" t="s">
+        <v>86</v>
+      </c>
+      <c r="L159" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="160" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="F160">
+        <v>9</v>
+      </c>
+      <c r="I160" t="s">
+        <v>90</v>
+      </c>
+      <c r="J160" t="s">
+        <v>85</v>
+      </c>
+      <c r="K160" t="s">
+        <v>86</v>
+      </c>
+      <c r="L160" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="161" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F161">
+        <v>10</v>
+      </c>
+      <c r="I161" t="s">
+        <v>90</v>
+      </c>
+      <c r="J161" t="s">
+        <v>85</v>
+      </c>
+      <c r="K161" t="s">
+        <v>86</v>
+      </c>
+      <c r="L161" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="162" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F162">
+        <v>11</v>
+      </c>
+      <c r="I162" t="s">
+        <v>90</v>
+      </c>
+      <c r="J162" t="s">
+        <v>85</v>
+      </c>
+      <c r="K162" t="s">
+        <v>86</v>
+      </c>
+      <c r="L162" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="163" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F163">
+        <v>12</v>
+      </c>
+      <c r="I163" t="s">
+        <v>90</v>
+      </c>
+      <c r="J163" t="s">
+        <v>85</v>
+      </c>
+      <c r="K163" t="s">
+        <v>86</v>
+      </c>
+      <c r="L163" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="164" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F164">
+        <v>13</v>
+      </c>
+      <c r="I164" t="s">
+        <v>90</v>
+      </c>
+      <c r="J164" t="s">
+        <v>85</v>
+      </c>
+      <c r="K164" t="s">
+        <v>86</v>
+      </c>
+      <c r="L164" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="165" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F165">
+        <v>14</v>
+      </c>
+      <c r="I165" t="s">
+        <v>90</v>
+      </c>
+      <c r="J165" t="s">
+        <v>85</v>
+      </c>
+      <c r="K165" t="s">
+        <v>86</v>
+      </c>
+      <c r="L165" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="166" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F166">
+        <v>15</v>
+      </c>
+      <c r="I166" t="s">
+        <v>90</v>
+      </c>
+      <c r="J166" t="s">
+        <v>85</v>
+      </c>
+      <c r="K166" t="s">
+        <v>86</v>
+      </c>
+      <c r="L166" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="167" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F167">
+        <v>16</v>
+      </c>
+      <c r="I167" t="s">
+        <v>90</v>
+      </c>
+      <c r="J167" t="s">
+        <v>85</v>
+      </c>
+      <c r="K167" t="s">
+        <v>86</v>
+      </c>
+      <c r="L167" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="168" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F168">
+        <v>17</v>
+      </c>
+      <c r="I168" t="s">
+        <v>90</v>
+      </c>
+      <c r="J168" t="s">
+        <v>85</v>
+      </c>
+      <c r="K168" t="s">
+        <v>86</v>
+      </c>
+      <c r="L168" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="169" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F169">
+        <v>18</v>
+      </c>
+      <c r="I169" t="s">
+        <v>90</v>
+      </c>
+      <c r="J169" t="s">
+        <v>85</v>
+      </c>
+      <c r="K169" t="s">
+        <v>86</v>
+      </c>
+      <c r="L169" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="170" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F170">
+        <v>19</v>
+      </c>
+      <c r="I170" t="s">
+        <v>90</v>
+      </c>
+      <c r="J170" t="s">
+        <v>85</v>
+      </c>
+      <c r="K170" t="s">
+        <v>86</v>
+      </c>
+      <c r="L170" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="171" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F171">
+        <v>20</v>
+      </c>
+      <c r="I171" t="s">
+        <v>90</v>
+      </c>
+      <c r="J171" t="s">
+        <v>85</v>
+      </c>
+      <c r="K171" t="s">
+        <v>86</v>
+      </c>
+      <c r="L171" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="172" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F172">
+        <v>21</v>
+      </c>
+      <c r="I172" t="s">
+        <v>90</v>
+      </c>
+      <c r="J172" t="s">
+        <v>85</v>
+      </c>
+      <c r="K172" t="s">
+        <v>86</v>
+      </c>
+      <c r="L172" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="173" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F173">
+        <v>22</v>
+      </c>
+      <c r="I173" t="s">
+        <v>90</v>
+      </c>
+      <c r="J173" t="s">
+        <v>85</v>
+      </c>
+      <c r="K173" t="s">
+        <v>86</v>
+      </c>
+      <c r="L173" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="174" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F174">
+        <v>23</v>
+      </c>
+      <c r="I174" t="s">
+        <v>90</v>
+      </c>
+      <c r="J174" t="s">
+        <v>85</v>
+      </c>
+      <c r="K174" t="s">
+        <v>86</v>
+      </c>
+      <c r="L174" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="175" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F175">
+        <v>24</v>
+      </c>
+      <c r="I175" t="s">
+        <v>90</v>
+      </c>
+      <c r="J175" t="s">
+        <v>85</v>
+      </c>
+      <c r="K175" t="s">
+        <v>86</v>
+      </c>
+      <c r="L175" s="5">
+        <v>5.0599999999999996</v>
+      </c>
+    </row>
+    <row r="176" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="F176">
+        <v>25</v>
+      </c>
+      <c r="I176" t="s">
+        <v>90</v>
+      </c>
+      <c r="J176" t="s">
+        <v>85</v>
+      </c>
+      <c r="K176" t="s">
+        <v>86</v>
+      </c>
+      <c r="L176" s="5">
+        <v>5.0599999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Pages for the IndyCar May Edition
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5C4B24-9DAA-46F5-B36D-455A61C9BBF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6B6850-4FD4-4812-9933-2CE7F20C7CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy_Model" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="99">
   <si>
     <t>Model</t>
   </si>
@@ -316,6 +316,30 @@
   <si>
     <t>Indianapolis Motor Speedway (Oval)</t>
   </si>
+  <si>
+    <t>Conor Daly</t>
+  </si>
+  <si>
+    <t>Helio Castroneves</t>
+  </si>
+  <si>
+    <t>Ryan Hunter-Reay</t>
+  </si>
+  <si>
+    <t>Takuma Sato</t>
+  </si>
+  <si>
+    <t>Jacob Abel</t>
+  </si>
+  <si>
+    <t>Ed Carpenter</t>
+  </si>
+  <si>
+    <t>Jack Harvey</t>
+  </si>
+  <si>
+    <t>Katherine Legge</t>
+  </si>
 </sst>
 </file>
 
@@ -406,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -438,7 +462,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1552,7 +1575,7 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="1">
@@ -2528,6 +2551,7 @@
     <col min="11" max="11" width="8.3671875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.20703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17.3125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.20703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="17.26171875" customWidth="1"/>
     <col min="18" max="18" width="10.68359375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9.47265625" bestFit="1" customWidth="1"/>
@@ -8476,7 +8500,7 @@
       <c r="N144" s="6"/>
       <c r="O144" s="5"/>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A145" s="6" t="s">
         <v>29</v>
       </c>
@@ -8518,7 +8542,7 @@
       <c r="N145" s="6"/>
       <c r="O145" s="5"/>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A146" s="6" t="s">
         <v>30</v>
       </c>
@@ -8560,7 +8584,7 @@
       <c r="N146" s="6"/>
       <c r="O146" s="5"/>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A147" s="6" t="s">
         <v>47</v>
       </c>
@@ -8602,7 +8626,7 @@
       <c r="N147" s="6"/>
       <c r="O147" s="5"/>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A148" s="6" t="s">
         <v>26</v>
       </c>
@@ -8644,7 +8668,7 @@
       <c r="N148" s="6"/>
       <c r="O148" s="5"/>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A149" s="6" t="s">
         <v>32</v>
       </c>
@@ -8686,7 +8710,7 @@
       <c r="N149" s="6"/>
       <c r="O149" s="5"/>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A150" s="6" t="s">
         <v>46</v>
       </c>
@@ -8728,7 +8752,7 @@
       <c r="N150" s="6"/>
       <c r="O150" s="5"/>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A151" s="6" t="s">
         <v>43</v>
       </c>
@@ -8770,9 +8794,29 @@
       <c r="N151" s="6"/>
       <c r="O151" s="5"/>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A152" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B152" s="6">
+        <v>10.19</v>
+      </c>
+      <c r="C152" s="5">
+        <f>B152-L152</f>
+        <v>4.7399999999999993</v>
+      </c>
+      <c r="D152" s="5">
+        <f>B152+L152</f>
+        <v>15.64</v>
+      </c>
+      <c r="E152" s="5">
+        <v>10.19</v>
+      </c>
       <c r="F152">
         <v>1</v>
+      </c>
+      <c r="G152" s="8">
+        <v>4</v>
       </c>
       <c r="H152" s="8"/>
       <c r="I152" t="s">
@@ -8788,11 +8832,32 @@
         <v>5.45</v>
       </c>
       <c r="N152" s="6"/>
-      <c r="O152" s="5"/>
-    </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="O152" s="7"/>
+      <c r="P152" s="5"/>
+    </row>
+    <row r="153" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A153" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B153" s="6">
+        <v>10.6</v>
+      </c>
+      <c r="C153" s="5">
+        <f t="shared" ref="C153:C184" si="12">B153-L153</f>
+        <v>5.1499999999999995</v>
+      </c>
+      <c r="D153" s="5">
+        <f t="shared" ref="D153:D184" si="13">B153+L153</f>
+        <v>16.05</v>
+      </c>
+      <c r="E153" s="5">
+        <v>10.6</v>
+      </c>
       <c r="F153">
         <v>2</v>
+      </c>
+      <c r="G153" s="8">
+        <v>7</v>
       </c>
       <c r="H153" s="8"/>
       <c r="I153" t="s">
@@ -8807,10 +8872,32 @@
       <c r="L153">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="O153" s="7"/>
+      <c r="P153" s="5"/>
+    </row>
+    <row r="154" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A154" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B154" s="6">
+        <v>10.78</v>
+      </c>
+      <c r="C154" s="5">
+        <f t="shared" si="12"/>
+        <v>5.3299999999999992</v>
+      </c>
+      <c r="D154" s="5">
+        <f t="shared" si="13"/>
+        <v>16.23</v>
+      </c>
+      <c r="E154" s="5">
+        <v>10.78</v>
+      </c>
       <c r="F154">
         <v>3</v>
+      </c>
+      <c r="G154" s="8">
+        <v>8</v>
       </c>
       <c r="H154" s="8"/>
       <c r="I154" t="s">
@@ -8825,10 +8912,32 @@
       <c r="L154">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="O154" s="7"/>
+      <c r="P154" s="5"/>
+    </row>
+    <row r="155" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A155" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B155" s="6">
+        <v>11.13</v>
+      </c>
+      <c r="C155" s="5">
+        <f t="shared" si="12"/>
+        <v>5.6800000000000006</v>
+      </c>
+      <c r="D155" s="5">
+        <f t="shared" si="13"/>
+        <v>16.580000000000002</v>
+      </c>
+      <c r="E155" s="5">
+        <v>5.68</v>
+      </c>
       <c r="F155">
         <v>4</v>
+      </c>
+      <c r="G155" s="8">
+        <v>1</v>
       </c>
       <c r="H155" s="8"/>
       <c r="I155" t="s">
@@ -8843,10 +8952,33 @@
       <c r="L155">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="N155" s="6"/>
+      <c r="O155" s="7"/>
+      <c r="P155" s="5"/>
+    </row>
+    <row r="156" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A156" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B156" s="6">
+        <v>11.79</v>
+      </c>
+      <c r="C156" s="5">
+        <f t="shared" si="12"/>
+        <v>6.339999999999999</v>
+      </c>
+      <c r="D156" s="5">
+        <f t="shared" si="13"/>
+        <v>17.239999999999998</v>
+      </c>
+      <c r="E156" s="5">
+        <v>6.34</v>
+      </c>
       <c r="F156">
         <v>5</v>
+      </c>
+      <c r="G156" s="8">
+        <v>2</v>
       </c>
       <c r="H156" s="8"/>
       <c r="I156" t="s">
@@ -8861,10 +8993,32 @@
       <c r="L156">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="O156" s="7"/>
+      <c r="P156" s="5"/>
+    </row>
+    <row r="157" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A157" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B157" s="6">
+        <v>12.54</v>
+      </c>
+      <c r="C157" s="5">
+        <f t="shared" si="12"/>
+        <v>7.089999999999999</v>
+      </c>
+      <c r="D157" s="5">
+        <f t="shared" si="13"/>
+        <v>17.989999999999998</v>
+      </c>
+      <c r="E157" s="5">
+        <v>7.09</v>
+      </c>
       <c r="F157">
         <v>6</v>
+      </c>
+      <c r="G157" s="8">
+        <v>3</v>
       </c>
       <c r="H157" s="8"/>
       <c r="I157" t="s">
@@ -8879,10 +9033,32 @@
       <c r="L157">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="O157" s="7"/>
+      <c r="P157" s="5"/>
+    </row>
+    <row r="158" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A158" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B158" s="6">
+        <v>12.83</v>
+      </c>
+      <c r="C158" s="5">
+        <f t="shared" si="12"/>
+        <v>7.38</v>
+      </c>
+      <c r="D158" s="5">
+        <f t="shared" si="13"/>
+        <v>18.28</v>
+      </c>
+      <c r="E158" s="5">
+        <v>12.83</v>
+      </c>
       <c r="F158">
         <v>7</v>
+      </c>
+      <c r="G158" s="8">
+        <v>12</v>
       </c>
       <c r="H158" s="8"/>
       <c r="I158" t="s">
@@ -8897,10 +9073,33 @@
       <c r="L158">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="N158" s="6"/>
+      <c r="O158" s="7"/>
+      <c r="P158" s="5"/>
+    </row>
+    <row r="159" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A159" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B159" s="6">
+        <v>13.74</v>
+      </c>
+      <c r="C159" s="5">
+        <f t="shared" si="12"/>
+        <v>8.2899999999999991</v>
+      </c>
+      <c r="D159" s="5">
+        <f t="shared" si="13"/>
+        <v>19.190000000000001</v>
+      </c>
+      <c r="E159" s="5">
+        <v>13.74</v>
+      </c>
       <c r="F159">
         <v>8</v>
+      </c>
+      <c r="G159" s="8">
+        <v>13</v>
       </c>
       <c r="H159" s="8"/>
       <c r="I159" t="s">
@@ -8915,10 +9114,32 @@
       <c r="L159">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="O159" s="7"/>
+      <c r="P159" s="5"/>
+    </row>
+    <row r="160" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A160" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B160" s="6">
+        <v>14.48</v>
+      </c>
+      <c r="C160" s="5">
+        <f t="shared" si="12"/>
+        <v>9.0300000000000011</v>
+      </c>
+      <c r="D160" s="5">
+        <f t="shared" si="13"/>
+        <v>19.93</v>
+      </c>
+      <c r="E160" s="5">
+        <v>19.93</v>
+      </c>
       <c r="F160">
         <v>9</v>
+      </c>
+      <c r="G160" s="8">
+        <v>23</v>
       </c>
       <c r="H160" s="8"/>
       <c r="I160" t="s">
@@ -8933,10 +9154,32 @@
       <c r="L160">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="161" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O160" s="7"/>
+      <c r="P160" s="5"/>
+    </row>
+    <row r="161" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A161" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B161" s="6">
+        <v>15.16</v>
+      </c>
+      <c r="C161" s="5">
+        <f t="shared" si="12"/>
+        <v>9.7100000000000009</v>
+      </c>
+      <c r="D161" s="5">
+        <f t="shared" si="13"/>
+        <v>20.61</v>
+      </c>
+      <c r="E161" s="5">
+        <v>15.16</v>
+      </c>
       <c r="F161">
         <v>10</v>
+      </c>
+      <c r="G161" s="8">
+        <v>14</v>
       </c>
       <c r="H161" s="8"/>
       <c r="I161" t="s">
@@ -8951,10 +9194,33 @@
       <c r="L161">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="162" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N161" s="6"/>
+      <c r="O161" s="7"/>
+      <c r="P161" s="5"/>
+    </row>
+    <row r="162" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A162" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B162" s="6">
+        <v>15.42</v>
+      </c>
+      <c r="C162" s="5">
+        <f t="shared" si="12"/>
+        <v>9.9699999999999989</v>
+      </c>
+      <c r="D162" s="5">
+        <f t="shared" si="13"/>
+        <v>20.87</v>
+      </c>
+      <c r="E162" s="5">
+        <v>15.42</v>
+      </c>
       <c r="F162">
         <v>11</v>
+      </c>
+      <c r="G162" s="8">
+        <v>15</v>
       </c>
       <c r="H162" s="8"/>
       <c r="I162" t="s">
@@ -8969,10 +9235,32 @@
       <c r="L162">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="163" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O162" s="7"/>
+      <c r="P162" s="5"/>
+    </row>
+    <row r="163" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A163" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B163" s="6">
+        <v>15.69</v>
+      </c>
+      <c r="C163" s="5">
+        <f t="shared" si="12"/>
+        <v>10.239999999999998</v>
+      </c>
+      <c r="D163" s="5">
+        <f t="shared" si="13"/>
+        <v>21.14</v>
+      </c>
+      <c r="E163" s="5">
+        <v>10.24</v>
+      </c>
       <c r="F163">
         <v>12</v>
+      </c>
+      <c r="G163" s="8">
+        <v>5</v>
       </c>
       <c r="H163" s="8"/>
       <c r="I163" t="s">
@@ -8987,10 +9275,32 @@
       <c r="L163">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="164" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O163" s="7"/>
+      <c r="P163" s="5"/>
+    </row>
+    <row r="164" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A164" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B164" s="6">
+        <v>15.78</v>
+      </c>
+      <c r="C164" s="5">
+        <f t="shared" si="12"/>
+        <v>10.329999999999998</v>
+      </c>
+      <c r="D164" s="5">
+        <f t="shared" si="13"/>
+        <v>21.23</v>
+      </c>
+      <c r="E164" s="5">
+        <v>15.78</v>
+      </c>
       <c r="F164">
         <v>13</v>
+      </c>
+      <c r="G164" s="8">
+        <v>16</v>
       </c>
       <c r="H164" s="8"/>
       <c r="I164" t="s">
@@ -9005,10 +9315,33 @@
       <c r="L164">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="165" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N164" s="6"/>
+      <c r="O164" s="7"/>
+      <c r="P164" s="5"/>
+    </row>
+    <row r="165" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A165" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B165" s="6">
+        <v>15.85</v>
+      </c>
+      <c r="C165" s="5">
+        <f t="shared" si="12"/>
+        <v>10.399999999999999</v>
+      </c>
+      <c r="D165" s="5">
+        <f t="shared" si="13"/>
+        <v>21.3</v>
+      </c>
+      <c r="E165" s="5">
+        <v>10.4</v>
+      </c>
       <c r="F165">
         <v>14</v>
+      </c>
+      <c r="G165" s="8">
+        <v>6</v>
       </c>
       <c r="H165" s="8"/>
       <c r="I165" t="s">
@@ -9023,10 +9356,32 @@
       <c r="L165">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="166" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O165" s="7"/>
+      <c r="P165" s="5"/>
+    </row>
+    <row r="166" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A166" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B166" s="6">
+        <v>16.27</v>
+      </c>
+      <c r="C166" s="5">
+        <f t="shared" si="12"/>
+        <v>10.82</v>
+      </c>
+      <c r="D166" s="5">
+        <f t="shared" si="13"/>
+        <v>21.72</v>
+      </c>
+      <c r="E166" s="5">
+        <v>10.82</v>
+      </c>
       <c r="F166">
         <v>15</v>
+      </c>
+      <c r="G166" s="8">
+        <v>9</v>
       </c>
       <c r="H166" s="8"/>
       <c r="I166" t="s">
@@ -9041,10 +9396,32 @@
       <c r="L166">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="167" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O166" s="7"/>
+      <c r="P166" s="5"/>
+    </row>
+    <row r="167" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A167" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B167" s="6">
+        <v>16.760000000000002</v>
+      </c>
+      <c r="C167" s="5">
+        <f t="shared" si="12"/>
+        <v>11.310000000000002</v>
+      </c>
+      <c r="D167" s="5">
+        <f t="shared" si="13"/>
+        <v>22.21</v>
+      </c>
+      <c r="E167" s="5">
+        <v>16.760000000000002</v>
+      </c>
       <c r="F167">
         <v>16</v>
+      </c>
+      <c r="G167" s="8">
+        <v>18</v>
       </c>
       <c r="H167" s="8"/>
       <c r="I167" t="s">
@@ -9059,10 +9436,33 @@
       <c r="L167">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="168" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N167" s="6"/>
+      <c r="O167" s="7"/>
+      <c r="P167" s="5"/>
+    </row>
+    <row r="168" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A168" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B168" s="6">
+        <v>17.23</v>
+      </c>
+      <c r="C168" s="5">
+        <f t="shared" si="12"/>
+        <v>11.780000000000001</v>
+      </c>
+      <c r="D168" s="5">
+        <f t="shared" si="13"/>
+        <v>22.68</v>
+      </c>
+      <c r="E168" s="5">
+        <v>17.23</v>
+      </c>
       <c r="F168">
         <v>17</v>
+      </c>
+      <c r="G168" s="8">
+        <v>19</v>
       </c>
       <c r="H168" s="8"/>
       <c r="I168" t="s">
@@ -9077,10 +9477,32 @@
       <c r="L168">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="169" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O168" s="7"/>
+      <c r="P168" s="5"/>
+    </row>
+    <row r="169" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A169" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B169" s="6">
+        <v>17.670000000000002</v>
+      </c>
+      <c r="C169" s="5">
+        <f t="shared" si="12"/>
+        <v>12.220000000000002</v>
+      </c>
+      <c r="D169" s="5">
+        <f t="shared" si="13"/>
+        <v>23.12</v>
+      </c>
+      <c r="E169" s="5">
+        <v>17.670000000000002</v>
+      </c>
       <c r="F169">
         <v>18</v>
+      </c>
+      <c r="G169" s="8">
+        <v>20</v>
       </c>
       <c r="H169" s="8"/>
       <c r="I169" t="s">
@@ -9095,10 +9517,32 @@
       <c r="L169">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="170" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O169" s="7"/>
+      <c r="P169" s="5"/>
+    </row>
+    <row r="170" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A170" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B170" s="6">
+        <v>17.7</v>
+      </c>
+      <c r="C170" s="5">
+        <f t="shared" si="12"/>
+        <v>12.25</v>
+      </c>
+      <c r="D170" s="5">
+        <f t="shared" si="13"/>
+        <v>23.15</v>
+      </c>
+      <c r="E170" s="5">
+        <v>17.7</v>
+      </c>
       <c r="F170">
         <v>19</v>
+      </c>
+      <c r="G170" s="8">
+        <v>21</v>
       </c>
       <c r="H170" s="8"/>
       <c r="I170" t="s">
@@ -9113,10 +9557,33 @@
       <c r="L170">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="171" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N170" s="6"/>
+      <c r="O170" s="7"/>
+      <c r="P170" s="5"/>
+    </row>
+    <row r="171" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A171" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B171" s="6">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="C171" s="5">
+        <f t="shared" si="12"/>
+        <v>12.45</v>
+      </c>
+      <c r="D171" s="5">
+        <f t="shared" si="13"/>
+        <v>23.349999999999998</v>
+      </c>
+      <c r="E171" s="5">
+        <v>12.45</v>
+      </c>
       <c r="F171">
         <v>20</v>
+      </c>
+      <c r="G171" s="8">
+        <v>10</v>
       </c>
       <c r="H171" s="8"/>
       <c r="I171" t="s">
@@ -9131,10 +9598,32 @@
       <c r="L171">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="172" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O171" s="7"/>
+      <c r="P171" s="5"/>
+    </row>
+    <row r="172" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A172" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B172" s="6">
+        <v>18.149999999999999</v>
+      </c>
+      <c r="C172" s="5">
+        <f t="shared" si="12"/>
+        <v>12.7</v>
+      </c>
+      <c r="D172" s="5">
+        <f t="shared" si="13"/>
+        <v>23.599999999999998</v>
+      </c>
+      <c r="E172" s="5">
+        <v>12.7</v>
+      </c>
       <c r="F172">
         <v>21</v>
+      </c>
+      <c r="G172" s="8">
+        <v>11</v>
       </c>
       <c r="H172" s="8"/>
       <c r="I172" t="s">
@@ -9149,10 +9638,32 @@
       <c r="L172">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="173" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O172" s="7"/>
+      <c r="P172" s="5"/>
+    </row>
+    <row r="173" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A173" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B173" s="6">
+        <v>18.39</v>
+      </c>
+      <c r="C173" s="5">
+        <f t="shared" si="12"/>
+        <v>12.940000000000001</v>
+      </c>
+      <c r="D173" s="5">
+        <f t="shared" si="13"/>
+        <v>23.84</v>
+      </c>
+      <c r="E173" s="5">
+        <v>23.84</v>
+      </c>
       <c r="F173">
         <v>22</v>
+      </c>
+      <c r="G173" s="8">
+        <v>25</v>
       </c>
       <c r="H173" s="8"/>
       <c r="I173" t="s">
@@ -9167,10 +9678,33 @@
       <c r="L173">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="174" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N173" s="6"/>
+      <c r="O173" s="7"/>
+      <c r="P173" s="5"/>
+    </row>
+    <row r="174" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A174" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B174" s="6">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="C174" s="5">
+        <f t="shared" si="12"/>
+        <v>13.95</v>
+      </c>
+      <c r="D174" s="5">
+        <f t="shared" si="13"/>
+        <v>24.849999999999998</v>
+      </c>
+      <c r="E174" s="5">
+        <v>24.85</v>
+      </c>
       <c r="F174">
         <v>23</v>
+      </c>
+      <c r="G174" s="8">
+        <v>26</v>
       </c>
       <c r="H174" s="8"/>
       <c r="I174" t="s">
@@ -9185,10 +9719,32 @@
       <c r="L174">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="175" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O174" s="7"/>
+      <c r="P174" s="5"/>
+    </row>
+    <row r="175" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A175" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B175" s="6">
+        <v>19.57</v>
+      </c>
+      <c r="C175" s="5">
+        <f t="shared" si="12"/>
+        <v>14.120000000000001</v>
+      </c>
+      <c r="D175" s="5">
+        <f t="shared" si="13"/>
+        <v>25.02</v>
+      </c>
+      <c r="E175" s="5">
+        <v>25.02</v>
+      </c>
       <c r="F175">
         <v>24</v>
+      </c>
+      <c r="G175" s="8">
+        <v>27</v>
       </c>
       <c r="H175" s="8"/>
       <c r="I175" t="s">
@@ -9203,10 +9759,32 @@
       <c r="L175">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="176" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="O175" s="7"/>
+      <c r="P175" s="5"/>
+    </row>
+    <row r="176" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A176" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B176" s="6">
+        <v>19.739999999999998</v>
+      </c>
+      <c r="C176" s="5">
+        <f t="shared" si="12"/>
+        <v>14.29</v>
+      </c>
+      <c r="D176" s="5">
+        <f t="shared" si="13"/>
+        <v>25.189999999999998</v>
+      </c>
+      <c r="E176" s="5">
+        <v>19.739999999999998</v>
+      </c>
       <c r="F176">
         <v>25</v>
+      </c>
+      <c r="G176" s="8">
+        <v>22</v>
       </c>
       <c r="H176" s="8"/>
       <c r="I176" t="s">
@@ -9221,53 +9799,354 @@
       <c r="L176">
         <v>5.45</v>
       </c>
-    </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="N176" s="6"/>
+      <c r="O176" s="7"/>
+      <c r="P176" s="5"/>
+    </row>
+    <row r="177" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A177" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B177" s="6">
+        <v>20.86</v>
+      </c>
+      <c r="C177" s="5">
+        <f t="shared" si="12"/>
+        <v>15.41</v>
+      </c>
+      <c r="D177" s="5">
+        <f t="shared" si="13"/>
+        <v>26.31</v>
+      </c>
+      <c r="E177" s="5">
+        <v>26.31</v>
+      </c>
+      <c r="F177">
+        <v>26</v>
+      </c>
+      <c r="G177" s="8">
+        <v>28</v>
+      </c>
       <c r="H177" s="8"/>
-    </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I177" t="s">
+        <v>90</v>
+      </c>
+      <c r="J177" t="s">
+        <v>85</v>
+      </c>
+      <c r="K177" t="s">
+        <v>77</v>
+      </c>
+      <c r="L177">
+        <v>5.45</v>
+      </c>
+      <c r="O177" s="7"/>
+      <c r="P177" s="5"/>
+    </row>
+    <row r="178" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A178" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B178" s="6">
+        <v>21.69</v>
+      </c>
+      <c r="C178" s="5">
+        <f t="shared" si="12"/>
+        <v>16.240000000000002</v>
+      </c>
+      <c r="D178" s="5">
+        <f t="shared" si="13"/>
+        <v>27.14</v>
+      </c>
+      <c r="E178" s="5">
+        <v>27.14</v>
+      </c>
+      <c r="F178">
+        <v>27</v>
+      </c>
+      <c r="G178" s="8">
+        <v>29</v>
+      </c>
       <c r="H178" s="8"/>
-    </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I178" t="s">
+        <v>90</v>
+      </c>
+      <c r="J178" t="s">
+        <v>85</v>
+      </c>
+      <c r="K178" t="s">
+        <v>77</v>
+      </c>
+      <c r="L178">
+        <v>5.45</v>
+      </c>
+      <c r="O178" s="7"/>
+      <c r="P178" s="5"/>
+    </row>
+    <row r="179" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A179" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B179" s="6">
+        <v>21.9</v>
+      </c>
+      <c r="C179" s="5">
+        <f t="shared" si="12"/>
+        <v>16.45</v>
+      </c>
+      <c r="D179" s="5">
+        <f t="shared" si="13"/>
+        <v>27.349999999999998</v>
+      </c>
+      <c r="E179" s="5">
+        <v>27.35</v>
+      </c>
+      <c r="F179">
+        <v>28</v>
+      </c>
+      <c r="G179" s="8">
+        <v>30</v>
+      </c>
       <c r="H179" s="8"/>
-    </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I179" t="s">
+        <v>90</v>
+      </c>
+      <c r="J179" t="s">
+        <v>85</v>
+      </c>
+      <c r="K179" t="s">
+        <v>77</v>
+      </c>
+      <c r="L179">
+        <v>5.45</v>
+      </c>
+      <c r="N179" s="6"/>
+      <c r="O179" s="7"/>
+      <c r="P179" s="5"/>
+    </row>
+    <row r="180" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A180" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B180" s="6">
+        <v>21.96</v>
+      </c>
+      <c r="C180" s="5">
+        <f t="shared" si="12"/>
+        <v>16.510000000000002</v>
+      </c>
+      <c r="D180" s="5">
+        <f t="shared" si="13"/>
+        <v>27.41</v>
+      </c>
+      <c r="E180" s="5">
+        <v>27.41</v>
+      </c>
+      <c r="F180">
+        <v>29</v>
+      </c>
+      <c r="G180" s="8">
+        <v>31</v>
+      </c>
       <c r="H180" s="8"/>
-    </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I180" t="s">
+        <v>90</v>
+      </c>
+      <c r="J180" t="s">
+        <v>85</v>
+      </c>
+      <c r="K180" t="s">
+        <v>77</v>
+      </c>
+      <c r="L180">
+        <v>5.45</v>
+      </c>
+      <c r="O180" s="7"/>
+      <c r="P180" s="5"/>
+    </row>
+    <row r="181" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A181" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B181" s="6">
+        <v>22.02</v>
+      </c>
+      <c r="C181" s="5">
+        <f t="shared" si="12"/>
+        <v>16.57</v>
+      </c>
+      <c r="D181" s="5">
+        <f t="shared" si="13"/>
+        <v>27.47</v>
+      </c>
+      <c r="E181" s="5">
+        <v>16.57</v>
+      </c>
+      <c r="F181">
+        <v>30</v>
+      </c>
+      <c r="G181" s="8">
+        <v>17</v>
+      </c>
       <c r="H181" s="8"/>
-    </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I181" t="s">
+        <v>90</v>
+      </c>
+      <c r="J181" t="s">
+        <v>85</v>
+      </c>
+      <c r="K181" t="s">
+        <v>77</v>
+      </c>
+      <c r="L181">
+        <v>5.45</v>
+      </c>
+      <c r="O181" s="7"/>
+      <c r="P181" s="5"/>
+    </row>
+    <row r="182" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A182" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B182" s="6">
+        <v>22.27</v>
+      </c>
+      <c r="C182" s="5">
+        <f t="shared" si="12"/>
+        <v>16.82</v>
+      </c>
+      <c r="D182" s="5">
+        <f t="shared" si="13"/>
+        <v>27.72</v>
+      </c>
+      <c r="E182" s="5">
+        <v>22.27</v>
+      </c>
+      <c r="F182">
+        <v>31</v>
+      </c>
+      <c r="G182" s="8">
+        <v>24</v>
+      </c>
       <c r="H182" s="8"/>
-    </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I182" t="s">
+        <v>90</v>
+      </c>
+      <c r="J182" t="s">
+        <v>85</v>
+      </c>
+      <c r="K182" t="s">
+        <v>77</v>
+      </c>
+      <c r="L182">
+        <v>5.45</v>
+      </c>
+      <c r="N182" s="6"/>
+      <c r="O182" s="7"/>
+      <c r="P182" s="5"/>
+    </row>
+    <row r="183" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A183" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B183" s="6">
+        <v>22.72</v>
+      </c>
+      <c r="C183" s="5">
+        <f t="shared" si="12"/>
+        <v>17.27</v>
+      </c>
+      <c r="D183" s="5">
+        <f t="shared" si="13"/>
+        <v>28.169999999999998</v>
+      </c>
+      <c r="E183" s="5">
+        <v>28.17</v>
+      </c>
+      <c r="F183">
+        <v>32</v>
+      </c>
+      <c r="G183" s="8">
+        <v>32</v>
+      </c>
       <c r="H183" s="8"/>
-    </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I183" t="s">
+        <v>90</v>
+      </c>
+      <c r="J183" t="s">
+        <v>85</v>
+      </c>
+      <c r="K183" t="s">
+        <v>77</v>
+      </c>
+      <c r="L183">
+        <v>5.45</v>
+      </c>
+      <c r="O183" s="7"/>
+      <c r="P183" s="5"/>
+    </row>
+    <row r="184" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+      <c r="A184" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B184" s="6">
+        <v>22.92</v>
+      </c>
+      <c r="C184" s="5">
+        <f t="shared" si="12"/>
+        <v>17.470000000000002</v>
+      </c>
+      <c r="D184" s="5">
+        <f t="shared" si="13"/>
+        <v>28.37</v>
+      </c>
+      <c r="E184" s="5">
+        <v>28.37</v>
+      </c>
+      <c r="F184">
+        <v>33</v>
+      </c>
+      <c r="G184" s="8">
+        <v>33</v>
+      </c>
       <c r="H184" s="8"/>
-    </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I184" t="s">
+        <v>90</v>
+      </c>
+      <c r="J184" t="s">
+        <v>85</v>
+      </c>
+      <c r="K184" t="s">
+        <v>77</v>
+      </c>
+      <c r="L184">
+        <v>5.45</v>
+      </c>
+      <c r="O184" s="7"/>
+      <c r="P184" s="5"/>
+    </row>
+    <row r="185" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H185" s="8"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H186" s="8"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H187" s="8"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H188" s="8"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H189" s="8"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H190" s="8"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H191" s="8"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="H192" s="8"/>
     </row>
     <row r="193" spans="8:8" x14ac:dyDescent="0.55000000000000004">
@@ -9766,8 +10645,8 @@
       <c r="H357" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N128:O152">
-    <sortCondition ref="O128:O152"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="O152:P184">
+    <sortCondition ref="P152:P184"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated dataset and results page for Indyar
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A5625F-8D04-4ADB-BFD0-F0DA21AC4B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0318EF4D-6065-44FF-9195-AC7A6C5D3CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1804" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2029" uniqueCount="109">
   <si>
     <t>Model</t>
   </si>
@@ -367,6 +367,9 @@
   <si>
     <t>Streets of Detroit</t>
   </si>
+  <si>
+    <t>World Wide Technology Raceway</t>
+  </si>
 </sst>
 </file>
 
@@ -468,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -501,7 +504,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2487,7 +2489,7 @@
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B12" s="1"/>
@@ -10709,7 +10711,9 @@
       <c r="G185" s="8">
         <v>1</v>
       </c>
-      <c r="H185" s="8"/>
+      <c r="H185" s="8">
+        <v>1</v>
+      </c>
       <c r="I185" t="s">
         <v>107</v>
       </c>
@@ -10749,7 +10753,9 @@
       <c r="G186" s="8">
         <v>7</v>
       </c>
-      <c r="H186" s="8"/>
+      <c r="H186" s="8">
+        <v>24</v>
+      </c>
       <c r="I186" t="s">
         <v>107</v>
       </c>
@@ -10789,7 +10795,9 @@
       <c r="G187" s="8">
         <v>2</v>
       </c>
-      <c r="H187" s="8"/>
+      <c r="H187" s="8">
+        <v>2</v>
+      </c>
       <c r="I187" t="s">
         <v>107</v>
       </c>
@@ -10829,7 +10837,9 @@
       <c r="G188" s="8">
         <v>8</v>
       </c>
-      <c r="H188" s="8"/>
+      <c r="H188" s="8">
+        <v>5</v>
+      </c>
       <c r="I188" t="s">
         <v>107</v>
       </c>
@@ -10869,7 +10879,9 @@
       <c r="G189" s="8">
         <v>3</v>
       </c>
-      <c r="H189" s="8"/>
+      <c r="H189" s="8">
+        <v>4</v>
+      </c>
       <c r="I189" t="s">
         <v>107</v>
       </c>
@@ -10909,7 +10921,9 @@
       <c r="G190" s="8">
         <v>4</v>
       </c>
-      <c r="H190" s="8"/>
+      <c r="H190" s="8">
+        <v>19</v>
+      </c>
       <c r="I190" t="s">
         <v>107</v>
       </c>
@@ -10949,7 +10963,9 @@
       <c r="G191" s="8">
         <v>9</v>
       </c>
-      <c r="H191" s="8"/>
+      <c r="H191" s="8">
+        <v>10</v>
+      </c>
       <c r="I191" t="s">
         <v>107</v>
       </c>
@@ -10989,7 +11005,9 @@
       <c r="G192" s="8">
         <v>5</v>
       </c>
-      <c r="H192" s="8"/>
+      <c r="H192" s="8">
+        <v>18</v>
+      </c>
       <c r="I192" t="s">
         <v>107</v>
       </c>
@@ -11029,7 +11047,9 @@
       <c r="G193" s="8">
         <v>10</v>
       </c>
-      <c r="H193" s="8"/>
+      <c r="H193" s="8">
+        <v>22</v>
+      </c>
       <c r="I193" t="s">
         <v>107</v>
       </c>
@@ -11069,7 +11089,9 @@
       <c r="G194" s="8">
         <v>17</v>
       </c>
-      <c r="H194" s="8"/>
+      <c r="H194" s="8">
+        <v>8</v>
+      </c>
       <c r="I194" t="s">
         <v>107</v>
       </c>
@@ -11109,7 +11131,9 @@
       <c r="G195" s="8">
         <v>11</v>
       </c>
-      <c r="H195" s="8"/>
+      <c r="H195" s="8">
+        <v>11</v>
+      </c>
       <c r="I195" t="s">
         <v>107</v>
       </c>
@@ -11149,7 +11173,9 @@
       <c r="G196" s="8">
         <v>18</v>
       </c>
-      <c r="H196" s="8"/>
+      <c r="H196" s="8">
+        <v>3</v>
+      </c>
       <c r="I196" t="s">
         <v>107</v>
       </c>
@@ -11189,7 +11215,9 @@
       <c r="G197" s="8">
         <v>12</v>
       </c>
-      <c r="H197" s="8"/>
+      <c r="H197" s="8">
+        <v>9</v>
+      </c>
       <c r="I197" t="s">
         <v>107</v>
       </c>
@@ -11229,7 +11257,9 @@
       <c r="G198" s="8">
         <v>6</v>
       </c>
-      <c r="H198" s="8"/>
+      <c r="H198" s="8">
+        <v>6</v>
+      </c>
       <c r="I198" t="s">
         <v>107</v>
       </c>
@@ -11269,7 +11299,9 @@
       <c r="G199" s="8">
         <v>13</v>
       </c>
-      <c r="H199" s="8"/>
+      <c r="H199" s="8">
+        <v>17</v>
+      </c>
       <c r="I199" t="s">
         <v>107</v>
       </c>
@@ -11309,7 +11341,9 @@
       <c r="G200" s="8">
         <v>19</v>
       </c>
-      <c r="H200" s="8"/>
+      <c r="H200" s="8">
+        <v>12</v>
+      </c>
       <c r="I200" t="s">
         <v>107</v>
       </c>
@@ -11349,7 +11383,9 @@
       <c r="G201" s="8">
         <v>14</v>
       </c>
-      <c r="H201" s="8"/>
+      <c r="H201" s="8">
+        <v>13</v>
+      </c>
       <c r="I201" t="s">
         <v>107</v>
       </c>
@@ -11389,7 +11425,9 @@
       <c r="G202" s="8">
         <v>20</v>
       </c>
-      <c r="H202" s="8"/>
+      <c r="H202" s="8">
+        <v>7</v>
+      </c>
       <c r="I202" t="s">
         <v>107</v>
       </c>
@@ -11429,7 +11467,9 @@
       <c r="G203" s="8">
         <v>21</v>
       </c>
-      <c r="H203" s="8"/>
+      <c r="H203" s="8">
+        <v>15</v>
+      </c>
       <c r="I203" t="s">
         <v>107</v>
       </c>
@@ -11469,7 +11509,9 @@
       <c r="G204" s="8">
         <v>15</v>
       </c>
-      <c r="H204" s="8"/>
+      <c r="H204" s="8">
+        <v>23</v>
+      </c>
       <c r="I204" t="s">
         <v>107</v>
       </c>
@@ -11509,7 +11551,9 @@
       <c r="G205" s="8">
         <v>22</v>
       </c>
-      <c r="H205" s="8"/>
+      <c r="H205" s="8">
+        <v>25</v>
+      </c>
       <c r="I205" t="s">
         <v>107</v>
       </c>
@@ -11549,7 +11593,9 @@
       <c r="G206" s="8">
         <v>16</v>
       </c>
-      <c r="H206" s="8"/>
+      <c r="H206" s="8">
+        <v>20</v>
+      </c>
       <c r="I206" t="s">
         <v>107</v>
       </c>
@@ -11589,7 +11635,9 @@
       <c r="G207" s="8">
         <v>23</v>
       </c>
-      <c r="H207" s="8"/>
+      <c r="H207" s="8">
+        <v>16</v>
+      </c>
       <c r="I207" t="s">
         <v>107</v>
       </c>
@@ -11629,7 +11677,9 @@
       <c r="G208" s="8">
         <v>24</v>
       </c>
-      <c r="H208" s="8"/>
+      <c r="H208" s="8">
+        <v>21</v>
+      </c>
       <c r="I208" t="s">
         <v>107</v>
       </c>
@@ -11645,7 +11695,7 @@
       <c r="N208" s="6"/>
       <c r="O208" s="5"/>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A209" s="6" t="s">
         <v>43</v>
       </c>
@@ -11669,7 +11719,9 @@
       <c r="G209" s="8">
         <v>25</v>
       </c>
-      <c r="H209" s="8"/>
+      <c r="H209" s="8">
+        <v>14</v>
+      </c>
       <c r="I209" t="s">
         <v>107</v>
       </c>
@@ -11682,128 +11734,1027 @@
       <c r="L209">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G210" s="8"/>
+      <c r="N209" s="6"/>
+      <c r="O209" s="5"/>
+    </row>
+    <row r="210" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A210" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B210" s="6">
+        <v>10.51</v>
+      </c>
+      <c r="C210" s="5">
+        <f>B210-L210</f>
+        <v>5.08</v>
+      </c>
+      <c r="D210" s="5">
+        <f>B210+L210</f>
+        <v>15.94</v>
+      </c>
+      <c r="E210" s="5">
+        <v>10.51</v>
+      </c>
+      <c r="F210">
+        <v>1</v>
+      </c>
+      <c r="G210" s="8">
+        <v>8</v>
+      </c>
       <c r="H210" s="8"/>
-    </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G211" s="8"/>
+      <c r="I210" t="s">
+        <v>108</v>
+      </c>
+      <c r="J210" t="s">
+        <v>85</v>
+      </c>
+      <c r="K210" t="s">
+        <v>77</v>
+      </c>
+      <c r="L210">
+        <v>5.43</v>
+      </c>
+      <c r="N210" s="6"/>
+      <c r="O210" s="5"/>
+    </row>
+    <row r="211" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A211" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B211" s="6">
+        <v>10.58</v>
+      </c>
+      <c r="C211" s="5">
+        <f t="shared" ref="C211:C234" si="16">B211-L211</f>
+        <v>5.15</v>
+      </c>
+      <c r="D211" s="5">
+        <f t="shared" ref="D211:D234" si="17">B211+L211</f>
+        <v>16.009999999999998</v>
+      </c>
+      <c r="E211" s="5">
+        <v>10.58</v>
+      </c>
+      <c r="F211">
+        <v>2</v>
+      </c>
+      <c r="G211" s="8">
+        <v>9</v>
+      </c>
       <c r="H211" s="8"/>
-    </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G212" s="8"/>
+      <c r="I211" t="s">
+        <v>108</v>
+      </c>
+      <c r="J211" t="s">
+        <v>85</v>
+      </c>
+      <c r="K211" t="s">
+        <v>77</v>
+      </c>
+      <c r="L211">
+        <v>5.43</v>
+      </c>
+      <c r="N211" s="6"/>
+      <c r="O211" s="5"/>
+    </row>
+    <row r="212" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A212" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B212" s="6">
+        <v>11.03</v>
+      </c>
+      <c r="C212" s="5">
+        <f t="shared" si="16"/>
+        <v>5.6</v>
+      </c>
+      <c r="D212" s="5">
+        <f t="shared" si="17"/>
+        <v>16.46</v>
+      </c>
+      <c r="E212" s="5">
+        <v>5.6</v>
+      </c>
+      <c r="F212">
+        <v>3</v>
+      </c>
+      <c r="G212" s="8">
+        <v>1</v>
+      </c>
       <c r="H212" s="8"/>
-    </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G213" s="8"/>
+      <c r="I212" t="s">
+        <v>108</v>
+      </c>
+      <c r="J212" t="s">
+        <v>85</v>
+      </c>
+      <c r="K212" t="s">
+        <v>77</v>
+      </c>
+      <c r="L212">
+        <v>5.43</v>
+      </c>
+      <c r="N212" s="6"/>
+    </row>
+    <row r="213" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A213" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B213" s="6">
+        <v>11.18</v>
+      </c>
+      <c r="C213" s="5">
+        <f t="shared" si="16"/>
+        <v>5.75</v>
+      </c>
+      <c r="D213" s="5">
+        <f t="shared" si="17"/>
+        <v>16.61</v>
+      </c>
+      <c r="E213" s="5">
+        <v>5.75</v>
+      </c>
+      <c r="F213">
+        <v>4</v>
+      </c>
+      <c r="G213" s="8">
+        <v>2</v>
+      </c>
       <c r="H213" s="8"/>
-    </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G214" s="8"/>
+      <c r="I213" t="s">
+        <v>108</v>
+      </c>
+      <c r="J213" t="s">
+        <v>85</v>
+      </c>
+      <c r="K213" t="s">
+        <v>77</v>
+      </c>
+      <c r="L213">
+        <v>5.43</v>
+      </c>
+      <c r="N213" s="6"/>
+      <c r="O213" s="5"/>
+    </row>
+    <row r="214" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A214" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B214" s="6">
+        <v>11.32</v>
+      </c>
+      <c r="C214" s="5">
+        <f t="shared" si="16"/>
+        <v>5.8900000000000006</v>
+      </c>
+      <c r="D214" s="5">
+        <f t="shared" si="17"/>
+        <v>16.75</v>
+      </c>
+      <c r="E214" s="5">
+        <v>5.89</v>
+      </c>
+      <c r="F214">
+        <v>5</v>
+      </c>
+      <c r="G214" s="8">
+        <v>3</v>
+      </c>
       <c r="H214" s="8"/>
-    </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G215" s="8"/>
+      <c r="I214" t="s">
+        <v>108</v>
+      </c>
+      <c r="J214" t="s">
+        <v>85</v>
+      </c>
+      <c r="K214" t="s">
+        <v>77</v>
+      </c>
+      <c r="L214">
+        <v>5.43</v>
+      </c>
+      <c r="N214" s="6"/>
+      <c r="O214" s="5"/>
+    </row>
+    <row r="215" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A215" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B215" s="6">
+        <v>11.46</v>
+      </c>
+      <c r="C215" s="5">
+        <f t="shared" si="16"/>
+        <v>6.0300000000000011</v>
+      </c>
+      <c r="D215" s="5">
+        <f t="shared" si="17"/>
+        <v>16.89</v>
+      </c>
+      <c r="E215">
+        <v>6.03</v>
+      </c>
+      <c r="F215">
+        <v>6</v>
+      </c>
+      <c r="G215" s="8">
+        <v>4</v>
+      </c>
       <c r="H215" s="8"/>
-    </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G216" s="8"/>
+      <c r="I215" t="s">
+        <v>108</v>
+      </c>
+      <c r="J215" t="s">
+        <v>85</v>
+      </c>
+      <c r="K215" t="s">
+        <v>77</v>
+      </c>
+      <c r="L215">
+        <v>5.43</v>
+      </c>
+      <c r="N215" s="6"/>
+      <c r="O215" s="5"/>
+    </row>
+    <row r="216" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A216" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B216" s="6">
+        <v>12.77</v>
+      </c>
+      <c r="C216" s="5">
+        <f t="shared" si="16"/>
+        <v>7.34</v>
+      </c>
+      <c r="D216" s="5">
+        <f t="shared" si="17"/>
+        <v>18.2</v>
+      </c>
+      <c r="E216" s="5">
+        <v>7.34</v>
+      </c>
+      <c r="F216">
+        <v>7</v>
+      </c>
+      <c r="G216" s="8">
+        <v>5</v>
+      </c>
       <c r="H216" s="8"/>
-    </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G217" s="8"/>
+      <c r="I216" t="s">
+        <v>108</v>
+      </c>
+      <c r="J216" t="s">
+        <v>85</v>
+      </c>
+      <c r="K216" t="s">
+        <v>77</v>
+      </c>
+      <c r="L216">
+        <v>5.43</v>
+      </c>
+      <c r="N216" s="6"/>
+      <c r="O216" s="5"/>
+    </row>
+    <row r="217" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A217" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B217" s="6">
+        <v>12.87</v>
+      </c>
+      <c r="C217" s="5">
+        <f t="shared" si="16"/>
+        <v>7.4399999999999995</v>
+      </c>
+      <c r="D217" s="5">
+        <f t="shared" si="17"/>
+        <v>18.299999999999997</v>
+      </c>
+      <c r="E217" s="5">
+        <v>18.3</v>
+      </c>
+      <c r="F217">
+        <v>8</v>
+      </c>
+      <c r="G217" s="8">
+        <v>21</v>
+      </c>
       <c r="H217" s="8"/>
-    </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G218" s="8"/>
+      <c r="I217" t="s">
+        <v>108</v>
+      </c>
+      <c r="J217" t="s">
+        <v>85</v>
+      </c>
+      <c r="K217" t="s">
+        <v>77</v>
+      </c>
+      <c r="L217">
+        <v>5.43</v>
+      </c>
+      <c r="N217" s="6"/>
+      <c r="O217" s="5"/>
+    </row>
+    <row r="218" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A218" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B218" s="6">
+        <v>12.9</v>
+      </c>
+      <c r="C218" s="5">
+        <f t="shared" si="16"/>
+        <v>7.4700000000000006</v>
+      </c>
+      <c r="D218" s="5">
+        <f t="shared" si="17"/>
+        <v>18.329999999999998</v>
+      </c>
+      <c r="E218" s="5">
+        <v>12.9</v>
+      </c>
+      <c r="F218">
+        <v>9</v>
+      </c>
+      <c r="G218" s="8">
+        <v>10</v>
+      </c>
       <c r="H218" s="8"/>
-    </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G219" s="8"/>
+      <c r="I218" t="s">
+        <v>108</v>
+      </c>
+      <c r="J218" t="s">
+        <v>85</v>
+      </c>
+      <c r="K218" t="s">
+        <v>77</v>
+      </c>
+      <c r="L218">
+        <v>5.43</v>
+      </c>
+      <c r="N218" s="6"/>
+      <c r="O218" s="5"/>
+    </row>
+    <row r="219" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A219" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B219" s="6">
+        <v>12.98</v>
+      </c>
+      <c r="C219" s="5">
+        <f t="shared" si="16"/>
+        <v>7.5500000000000007</v>
+      </c>
+      <c r="D219" s="5">
+        <f t="shared" si="17"/>
+        <v>18.41</v>
+      </c>
+      <c r="E219" s="5">
+        <v>12.98</v>
+      </c>
+      <c r="F219">
+        <v>10</v>
+      </c>
+      <c r="G219" s="8">
+        <v>11</v>
+      </c>
       <c r="H219" s="8"/>
-    </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G220" s="8"/>
+      <c r="I219" t="s">
+        <v>108</v>
+      </c>
+      <c r="J219" t="s">
+        <v>85</v>
+      </c>
+      <c r="K219" t="s">
+        <v>77</v>
+      </c>
+      <c r="L219">
+        <v>5.43</v>
+      </c>
+      <c r="N219" s="6"/>
+      <c r="O219" s="5"/>
+    </row>
+    <row r="220" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A220" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B220" s="6">
+        <v>13.11</v>
+      </c>
+      <c r="C220" s="5">
+        <f t="shared" si="16"/>
+        <v>7.68</v>
+      </c>
+      <c r="D220" s="5">
+        <f t="shared" si="17"/>
+        <v>18.54</v>
+      </c>
+      <c r="E220" s="5">
+        <v>7.68</v>
+      </c>
+      <c r="F220">
+        <v>11</v>
+      </c>
+      <c r="G220" s="8">
+        <v>6</v>
+      </c>
       <c r="H220" s="8"/>
-    </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G221" s="8"/>
+      <c r="I220" t="s">
+        <v>108</v>
+      </c>
+      <c r="J220" t="s">
+        <v>85</v>
+      </c>
+      <c r="K220" t="s">
+        <v>77</v>
+      </c>
+      <c r="L220">
+        <v>5.43</v>
+      </c>
+      <c r="N220" s="6"/>
+      <c r="O220" s="5"/>
+    </row>
+    <row r="221" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A221" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B221" s="6">
+        <v>13.2</v>
+      </c>
+      <c r="C221" s="5">
+        <f t="shared" si="16"/>
+        <v>7.77</v>
+      </c>
+      <c r="D221" s="5">
+        <f t="shared" si="17"/>
+        <v>18.63</v>
+      </c>
+      <c r="E221" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="F221">
+        <v>12</v>
+      </c>
+      <c r="G221" s="8">
+        <v>12</v>
+      </c>
       <c r="H221" s="8"/>
-    </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G222" s="8"/>
+      <c r="I221" t="s">
+        <v>108</v>
+      </c>
+      <c r="J221" t="s">
+        <v>85</v>
+      </c>
+      <c r="K221" t="s">
+        <v>77</v>
+      </c>
+      <c r="L221">
+        <v>5.43</v>
+      </c>
+      <c r="N221" s="6"/>
+      <c r="O221" s="5"/>
+    </row>
+    <row r="222" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A222" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B222" s="6">
+        <v>13.22</v>
+      </c>
+      <c r="C222" s="5">
+        <f t="shared" si="16"/>
+        <v>7.7900000000000009</v>
+      </c>
+      <c r="D222" s="5">
+        <f t="shared" si="17"/>
+        <v>18.649999999999999</v>
+      </c>
+      <c r="E222" s="5">
+        <v>7.79</v>
+      </c>
+      <c r="F222">
+        <v>13</v>
+      </c>
+      <c r="G222" s="8">
+        <v>7</v>
+      </c>
       <c r="H222" s="8"/>
-    </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G223" s="8"/>
+      <c r="I222" t="s">
+        <v>108</v>
+      </c>
+      <c r="J222" t="s">
+        <v>85</v>
+      </c>
+      <c r="K222" t="s">
+        <v>77</v>
+      </c>
+      <c r="L222">
+        <v>5.43</v>
+      </c>
+      <c r="N222" s="6"/>
+      <c r="O222" s="5"/>
+    </row>
+    <row r="223" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A223" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B223" s="6">
+        <v>13.24</v>
+      </c>
+      <c r="C223" s="5">
+        <f t="shared" si="16"/>
+        <v>7.8100000000000005</v>
+      </c>
+      <c r="D223" s="5">
+        <f t="shared" si="17"/>
+        <v>18.670000000000002</v>
+      </c>
+      <c r="E223" s="5">
+        <v>13.24</v>
+      </c>
+      <c r="F223">
+        <v>14</v>
+      </c>
+      <c r="G223" s="8">
+        <v>13</v>
+      </c>
       <c r="H223" s="8"/>
-    </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="G224" s="8"/>
+      <c r="I223" t="s">
+        <v>108</v>
+      </c>
+      <c r="J223" t="s">
+        <v>85</v>
+      </c>
+      <c r="K223" t="s">
+        <v>77</v>
+      </c>
+      <c r="L223">
+        <v>5.43</v>
+      </c>
+      <c r="N223" s="6"/>
+      <c r="O223" s="5"/>
+    </row>
+    <row r="224" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A224" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B224" s="6">
+        <v>13.46</v>
+      </c>
+      <c r="C224" s="5">
+        <f t="shared" si="16"/>
+        <v>8.0300000000000011</v>
+      </c>
+      <c r="D224" s="5">
+        <f t="shared" si="17"/>
+        <v>18.89</v>
+      </c>
+      <c r="E224" s="5">
+        <v>18.89</v>
+      </c>
+      <c r="F224">
+        <v>15</v>
+      </c>
+      <c r="G224" s="8">
+        <v>22</v>
+      </c>
       <c r="H224" s="8"/>
-    </row>
-    <row r="225" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G225" s="8"/>
+      <c r="I224" t="s">
+        <v>108</v>
+      </c>
+      <c r="J224" t="s">
+        <v>85</v>
+      </c>
+      <c r="K224" t="s">
+        <v>77</v>
+      </c>
+      <c r="L224">
+        <v>5.43</v>
+      </c>
+      <c r="N224" s="6"/>
+      <c r="O224" s="5"/>
+    </row>
+    <row r="225" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A225" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B225" s="6">
+        <v>13.52</v>
+      </c>
+      <c r="C225" s="5">
+        <f t="shared" si="16"/>
+        <v>8.09</v>
+      </c>
+      <c r="D225" s="5">
+        <f t="shared" si="17"/>
+        <v>18.95</v>
+      </c>
+      <c r="E225" s="5">
+        <v>13.52</v>
+      </c>
+      <c r="F225">
+        <v>16</v>
+      </c>
+      <c r="G225" s="8">
+        <v>14</v>
+      </c>
       <c r="H225" s="8"/>
-    </row>
-    <row r="226" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G226" s="8"/>
+      <c r="I225" t="s">
+        <v>108</v>
+      </c>
+      <c r="J225" t="s">
+        <v>85</v>
+      </c>
+      <c r="K225" t="s">
+        <v>77</v>
+      </c>
+      <c r="L225">
+        <v>5.43</v>
+      </c>
+      <c r="N225" s="6"/>
+      <c r="O225" s="5"/>
+    </row>
+    <row r="226" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A226" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B226" s="6">
+        <v>13.68</v>
+      </c>
+      <c r="C226" s="5">
+        <f t="shared" si="16"/>
+        <v>8.25</v>
+      </c>
+      <c r="D226" s="5">
+        <f t="shared" si="17"/>
+        <v>19.11</v>
+      </c>
+      <c r="E226" s="5">
+        <v>13.68</v>
+      </c>
+      <c r="F226">
+        <v>17</v>
+      </c>
+      <c r="G226" s="8">
+        <v>15</v>
+      </c>
       <c r="H226" s="8"/>
-    </row>
-    <row r="227" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G227" s="8"/>
+      <c r="I226" t="s">
+        <v>108</v>
+      </c>
+      <c r="J226" t="s">
+        <v>85</v>
+      </c>
+      <c r="K226" t="s">
+        <v>77</v>
+      </c>
+      <c r="L226">
+        <v>5.43</v>
+      </c>
+      <c r="N226" s="6"/>
+      <c r="O226" s="5"/>
+    </row>
+    <row r="227" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A227" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B227" s="6">
+        <v>14.59</v>
+      </c>
+      <c r="C227" s="5">
+        <f t="shared" si="16"/>
+        <v>9.16</v>
+      </c>
+      <c r="D227" s="5">
+        <f t="shared" si="17"/>
+        <v>20.02</v>
+      </c>
+      <c r="E227" s="5">
+        <v>14.59</v>
+      </c>
+      <c r="F227">
+        <v>18</v>
+      </c>
+      <c r="G227" s="8">
+        <v>16</v>
+      </c>
       <c r="H227" s="8"/>
-    </row>
-    <row r="228" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G228" s="8"/>
+      <c r="I227" t="s">
+        <v>108</v>
+      </c>
+      <c r="J227" t="s">
+        <v>85</v>
+      </c>
+      <c r="K227" t="s">
+        <v>77</v>
+      </c>
+      <c r="L227">
+        <v>5.43</v>
+      </c>
+      <c r="N227" s="6"/>
+      <c r="O227" s="5"/>
+    </row>
+    <row r="228" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A228" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B228" s="6">
+        <v>14.71</v>
+      </c>
+      <c r="C228" s="5">
+        <f t="shared" si="16"/>
+        <v>9.2800000000000011</v>
+      </c>
+      <c r="D228" s="5">
+        <f t="shared" si="17"/>
+        <v>20.14</v>
+      </c>
+      <c r="E228" s="5">
+        <v>14.71</v>
+      </c>
+      <c r="F228">
+        <v>19</v>
+      </c>
+      <c r="G228" s="8">
+        <v>17</v>
+      </c>
       <c r="H228" s="8"/>
-    </row>
-    <row r="229" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G229" s="8"/>
+      <c r="I228" t="s">
+        <v>108</v>
+      </c>
+      <c r="J228" t="s">
+        <v>85</v>
+      </c>
+      <c r="K228" t="s">
+        <v>77</v>
+      </c>
+      <c r="L228">
+        <v>5.43</v>
+      </c>
+      <c r="N228" s="6"/>
+      <c r="O228" s="5"/>
+    </row>
+    <row r="229" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A229" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B229" s="6">
+        <v>14.94</v>
+      </c>
+      <c r="C229" s="5">
+        <f t="shared" si="16"/>
+        <v>9.51</v>
+      </c>
+      <c r="D229" s="5">
+        <f t="shared" si="17"/>
+        <v>20.369999999999997</v>
+      </c>
+      <c r="E229" s="5">
+        <v>20.37</v>
+      </c>
+      <c r="F229">
+        <v>20</v>
+      </c>
+      <c r="G229" s="8">
+        <v>23</v>
+      </c>
       <c r="H229" s="8"/>
-    </row>
-    <row r="230" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G230" s="8"/>
+      <c r="I229" t="s">
+        <v>108</v>
+      </c>
+      <c r="J229" t="s">
+        <v>85</v>
+      </c>
+      <c r="K229" t="s">
+        <v>77</v>
+      </c>
+      <c r="L229">
+        <v>5.43</v>
+      </c>
+      <c r="N229" s="6"/>
+      <c r="O229" s="5"/>
+    </row>
+    <row r="230" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A230" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B230" s="6">
+        <v>15.08</v>
+      </c>
+      <c r="C230" s="5">
+        <f t="shared" si="16"/>
+        <v>9.65</v>
+      </c>
+      <c r="D230" s="5">
+        <f t="shared" si="17"/>
+        <v>20.509999999999998</v>
+      </c>
+      <c r="E230" s="5">
+        <v>20.51</v>
+      </c>
+      <c r="F230">
+        <v>21</v>
+      </c>
+      <c r="G230" s="8">
+        <v>24</v>
+      </c>
       <c r="H230" s="8"/>
-    </row>
-    <row r="231" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G231" s="8"/>
+      <c r="I230" t="s">
+        <v>108</v>
+      </c>
+      <c r="J230" t="s">
+        <v>85</v>
+      </c>
+      <c r="K230" t="s">
+        <v>77</v>
+      </c>
+      <c r="L230">
+        <v>5.43</v>
+      </c>
+      <c r="N230" s="6"/>
+      <c r="O230" s="5"/>
+    </row>
+    <row r="231" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A231" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B231" s="6">
+        <v>15.11</v>
+      </c>
+      <c r="C231" s="5">
+        <f t="shared" si="16"/>
+        <v>9.68</v>
+      </c>
+      <c r="D231" s="5">
+        <f t="shared" si="17"/>
+        <v>20.54</v>
+      </c>
+      <c r="E231" s="5">
+        <v>15.11</v>
+      </c>
+      <c r="F231">
+        <v>22</v>
+      </c>
+      <c r="G231" s="8">
+        <v>18</v>
+      </c>
       <c r="H231" s="8"/>
-    </row>
-    <row r="232" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G232" s="8"/>
+      <c r="I231" t="s">
+        <v>108</v>
+      </c>
+      <c r="J231" t="s">
+        <v>85</v>
+      </c>
+      <c r="K231" t="s">
+        <v>77</v>
+      </c>
+      <c r="L231">
+        <v>5.43</v>
+      </c>
+      <c r="N231" s="6"/>
+      <c r="O231" s="5"/>
+    </row>
+    <row r="232" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A232" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B232" s="6">
+        <v>15.26</v>
+      </c>
+      <c r="C232" s="5">
+        <f t="shared" si="16"/>
+        <v>9.83</v>
+      </c>
+      <c r="D232" s="5">
+        <f t="shared" si="17"/>
+        <v>20.689999999999998</v>
+      </c>
+      <c r="E232" s="5">
+        <v>15.26</v>
+      </c>
+      <c r="F232">
+        <v>23</v>
+      </c>
+      <c r="G232" s="8">
+        <v>19</v>
+      </c>
       <c r="H232" s="8"/>
-    </row>
-    <row r="233" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G233" s="8"/>
+      <c r="I232" t="s">
+        <v>108</v>
+      </c>
+      <c r="J232" t="s">
+        <v>85</v>
+      </c>
+      <c r="K232" t="s">
+        <v>77</v>
+      </c>
+      <c r="L232">
+        <v>5.43</v>
+      </c>
+      <c r="N232" s="6"/>
+      <c r="O232" s="5"/>
+    </row>
+    <row r="233" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A233" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B233" s="6">
+        <v>15.31</v>
+      </c>
+      <c r="C233" s="5">
+        <f t="shared" si="16"/>
+        <v>9.8800000000000008</v>
+      </c>
+      <c r="D233" s="5">
+        <f t="shared" si="17"/>
+        <v>20.740000000000002</v>
+      </c>
+      <c r="E233" s="5">
+        <v>20.74</v>
+      </c>
+      <c r="F233">
+        <v>24</v>
+      </c>
+      <c r="G233" s="8">
+        <v>25</v>
+      </c>
       <c r="H233" s="8"/>
-    </row>
-    <row r="234" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G234" s="8"/>
+      <c r="I233" t="s">
+        <v>108</v>
+      </c>
+      <c r="J233" t="s">
+        <v>85</v>
+      </c>
+      <c r="K233" t="s">
+        <v>77</v>
+      </c>
+      <c r="L233">
+        <v>5.43</v>
+      </c>
+      <c r="N233" s="6"/>
+      <c r="O233" s="5"/>
+    </row>
+    <row r="234" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A234" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B234" s="6">
+        <v>15.38</v>
+      </c>
+      <c r="C234" s="5">
+        <f>B234-L234</f>
+        <v>9.9500000000000011</v>
+      </c>
+      <c r="D234" s="5">
+        <f t="shared" si="17"/>
+        <v>20.810000000000002</v>
+      </c>
+      <c r="E234" s="5">
+        <v>15.38</v>
+      </c>
+      <c r="F234">
+        <v>25</v>
+      </c>
+      <c r="G234" s="8">
+        <v>20</v>
+      </c>
       <c r="H234" s="8"/>
-    </row>
-    <row r="235" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I234" t="s">
+        <v>108</v>
+      </c>
+      <c r="J234" t="s">
+        <v>85</v>
+      </c>
+      <c r="K234" t="s">
+        <v>77</v>
+      </c>
+      <c r="L234">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="235" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="G235" s="8"/>
       <c r="H235" s="8"/>
     </row>
-    <row r="236" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="236" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="G236" s="8"/>
       <c r="H236" s="8"/>
     </row>
-    <row r="237" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="237" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="G237" s="8"/>
       <c r="H237" s="8"/>
     </row>
-    <row r="238" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="238" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="G238" s="8"/>
       <c r="H238" s="8"/>
     </row>
-    <row r="239" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="239" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="G239" s="8"/>
       <c r="H239" s="8"/>
     </row>
-    <row r="240" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="240" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="G240" s="8"/>
       <c r="H240" s="8"/>
     </row>
@@ -12274,8 +13225,8 @@
       <c r="H357" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N185:O208">
-    <sortCondition ref="O184:O208"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N209:O233">
+    <sortCondition ref="O209:O233"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12288,7 +13239,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O209"/>
+  <dimension ref="A1:O234"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="18.3671875" bestFit="1" customWidth="1"/>
@@ -19951,9 +20902,32 @@
       <c r="O184" s="5"/>
     </row>
     <row r="185" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A185" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B185" s="6">
+        <v>6.13</v>
+      </c>
+      <c r="C185" s="5">
+        <f>B185-L185</f>
+        <v>1.04</v>
+      </c>
+      <c r="D185" s="5">
+        <f>B185+L185</f>
+        <v>11.219999999999999</v>
+      </c>
+      <c r="E185" s="5">
+        <v>1.04</v>
+      </c>
       <c r="F185">
         <v>1</v>
       </c>
+      <c r="G185" s="8">
+        <v>1</v>
+      </c>
+      <c r="H185" s="8">
+        <v>1</v>
+      </c>
       <c r="I185" t="s">
         <v>107</v>
       </c>
@@ -19966,11 +20940,36 @@
       <c r="L185" s="5">
         <v>5.09</v>
       </c>
+      <c r="N185" s="6"/>
+      <c r="O185" s="5"/>
     </row>
     <row r="186" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A186" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B186" s="6">
+        <v>7.16</v>
+      </c>
+      <c r="C186" s="5">
+        <f t="shared" ref="C186:C209" si="13">B186-L186</f>
+        <v>2.0700000000000003</v>
+      </c>
+      <c r="D186" s="5">
+        <f t="shared" ref="D186:D209" si="14">B186+L186</f>
+        <v>12.25</v>
+      </c>
+      <c r="E186" s="5">
+        <v>7.16</v>
+      </c>
       <c r="F186">
         <v>2</v>
       </c>
+      <c r="G186" s="8">
+        <v>5</v>
+      </c>
+      <c r="H186" s="8">
+        <v>24</v>
+      </c>
       <c r="I186" t="s">
         <v>107</v>
       </c>
@@ -19983,11 +20982,36 @@
       <c r="L186" s="5">
         <v>5.09</v>
       </c>
+      <c r="N186" s="6"/>
+      <c r="O186" s="5"/>
     </row>
     <row r="187" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A187" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B187" s="6">
+        <v>7.98</v>
+      </c>
+      <c r="C187" s="5">
+        <f t="shared" si="13"/>
+        <v>2.8900000000000006</v>
+      </c>
+      <c r="D187" s="5">
+        <f t="shared" si="14"/>
+        <v>13.07</v>
+      </c>
+      <c r="E187" s="5">
+        <v>2.89</v>
+      </c>
       <c r="F187">
         <v>3</v>
       </c>
+      <c r="G187" s="8">
+        <v>2</v>
+      </c>
+      <c r="H187" s="8">
+        <v>2</v>
+      </c>
       <c r="I187" t="s">
         <v>107</v>
       </c>
@@ -20000,11 +21024,36 @@
       <c r="L187" s="5">
         <v>5.09</v>
       </c>
+      <c r="N187" s="6"/>
+      <c r="O187" s="5"/>
     </row>
     <row r="188" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A188" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B188" s="6">
+        <v>8.35</v>
+      </c>
+      <c r="C188" s="5">
+        <f t="shared" si="13"/>
+        <v>3.26</v>
+      </c>
+      <c r="D188" s="5">
+        <f t="shared" si="14"/>
+        <v>13.44</v>
+      </c>
+      <c r="E188" s="5">
+        <v>8.35</v>
+      </c>
       <c r="F188">
         <v>4</v>
       </c>
+      <c r="G188" s="8">
+        <v>8</v>
+      </c>
+      <c r="H188" s="8">
+        <v>22</v>
+      </c>
       <c r="I188" t="s">
         <v>107</v>
       </c>
@@ -20017,11 +21066,36 @@
       <c r="L188" s="5">
         <v>5.09</v>
       </c>
+      <c r="N188" s="6"/>
+      <c r="O188" s="5"/>
     </row>
     <row r="189" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A189" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B189" s="6">
+        <v>8.4</v>
+      </c>
+      <c r="C189" s="5">
+        <f t="shared" si="13"/>
+        <v>3.3100000000000005</v>
+      </c>
+      <c r="D189" s="5">
+        <f t="shared" si="14"/>
+        <v>13.49</v>
+      </c>
+      <c r="E189" s="5">
+        <v>8.4</v>
+      </c>
       <c r="F189">
         <v>5</v>
       </c>
+      <c r="G189" s="8">
+        <v>9</v>
+      </c>
+      <c r="H189" s="8">
+        <v>5</v>
+      </c>
       <c r="I189" t="s">
         <v>107</v>
       </c>
@@ -20034,11 +21108,36 @@
       <c r="L189" s="5">
         <v>5.09</v>
       </c>
+      <c r="N189" s="6"/>
+      <c r="O189" s="5"/>
     </row>
     <row r="190" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A190" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B190" s="6">
+        <v>8.74</v>
+      </c>
+      <c r="C190" s="5">
+        <f t="shared" si="13"/>
+        <v>3.6500000000000004</v>
+      </c>
+      <c r="D190" s="5">
+        <f t="shared" si="14"/>
+        <v>13.83</v>
+      </c>
+      <c r="E190" s="5">
+        <v>8.74</v>
+      </c>
       <c r="F190">
         <v>6</v>
       </c>
+      <c r="G190" s="8">
+        <v>10</v>
+      </c>
+      <c r="H190" s="8">
+        <v>19</v>
+      </c>
       <c r="I190" t="s">
         <v>107</v>
       </c>
@@ -20051,11 +21150,36 @@
       <c r="L190" s="5">
         <v>5.09</v>
       </c>
+      <c r="N190" s="6"/>
+      <c r="O190" s="5"/>
     </row>
     <row r="191" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A191" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B191" s="6">
+        <v>9.7899999999999991</v>
+      </c>
+      <c r="C191" s="5">
+        <f t="shared" si="13"/>
+        <v>4.6999999999999993</v>
+      </c>
+      <c r="D191" s="5">
+        <f t="shared" si="14"/>
+        <v>14.879999999999999</v>
+      </c>
+      <c r="E191" s="5">
+        <v>4.7</v>
+      </c>
       <c r="F191">
         <v>7</v>
       </c>
+      <c r="G191" s="8">
+        <v>3</v>
+      </c>
+      <c r="H191" s="8">
+        <v>4</v>
+      </c>
       <c r="I191" t="s">
         <v>107</v>
       </c>
@@ -20068,11 +21192,36 @@
       <c r="L191" s="5">
         <v>5.09</v>
       </c>
+      <c r="N191" s="6"/>
+      <c r="O191" s="5"/>
     </row>
     <row r="192" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A192" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B192" s="6">
+        <v>10.220000000000001</v>
+      </c>
+      <c r="C192" s="5">
+        <f t="shared" si="13"/>
+        <v>5.1300000000000008</v>
+      </c>
+      <c r="D192" s="5">
+        <f t="shared" si="14"/>
+        <v>15.31</v>
+      </c>
+      <c r="E192" s="5">
+        <v>10.220000000000001</v>
+      </c>
       <c r="F192">
         <v>8</v>
       </c>
+      <c r="G192" s="8">
+        <v>11</v>
+      </c>
+      <c r="H192" s="8">
+        <v>11</v>
+      </c>
       <c r="I192" t="s">
         <v>107</v>
       </c>
@@ -20085,11 +21234,36 @@
       <c r="L192" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="193" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N192" s="6"/>
+      <c r="O192" s="5"/>
+    </row>
+    <row r="193" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A193" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B193" s="6">
+        <v>11.92</v>
+      </c>
+      <c r="C193" s="5">
+        <f t="shared" si="13"/>
+        <v>6.83</v>
+      </c>
+      <c r="D193" s="5">
+        <f t="shared" si="14"/>
+        <v>17.009999999999998</v>
+      </c>
+      <c r="E193" s="5">
+        <v>17.010000000000002</v>
+      </c>
       <c r="F193">
         <v>9</v>
       </c>
+      <c r="G193" s="8">
+        <v>17</v>
+      </c>
+      <c r="H193" s="8">
+        <v>8</v>
+      </c>
       <c r="I193" t="s">
         <v>107</v>
       </c>
@@ -20102,11 +21276,36 @@
       <c r="L193" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="194" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N193" s="6"/>
+      <c r="O193" s="5"/>
+    </row>
+    <row r="194" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A194" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B194" s="6">
+        <v>11.93</v>
+      </c>
+      <c r="C194" s="5">
+        <f t="shared" si="13"/>
+        <v>6.84</v>
+      </c>
+      <c r="D194" s="5">
+        <f t="shared" si="14"/>
+        <v>17.02</v>
+      </c>
+      <c r="E194" s="5">
+        <v>6.84</v>
+      </c>
       <c r="F194">
         <v>10</v>
       </c>
+      <c r="G194" s="8">
+        <v>4</v>
+      </c>
+      <c r="H194" s="8">
+        <v>9</v>
+      </c>
       <c r="I194" t="s">
         <v>107</v>
       </c>
@@ -20119,11 +21318,36 @@
       <c r="L194" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="195" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N194" s="6"/>
+      <c r="O194" s="5"/>
+    </row>
+    <row r="195" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A195" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B195" s="6">
+        <v>12.5</v>
+      </c>
+      <c r="C195" s="5">
+        <f t="shared" si="13"/>
+        <v>7.41</v>
+      </c>
+      <c r="D195" s="5">
+        <f t="shared" si="14"/>
+        <v>17.59</v>
+      </c>
+      <c r="E195" s="5">
+        <v>7.41</v>
+      </c>
       <c r="F195">
         <v>11</v>
       </c>
+      <c r="G195" s="8">
+        <v>6</v>
+      </c>
+      <c r="H195" s="8">
+        <v>6</v>
+      </c>
       <c r="I195" t="s">
         <v>107</v>
       </c>
@@ -20136,11 +21360,36 @@
       <c r="L195" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="196" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N195" s="6"/>
+      <c r="O195" s="5"/>
+    </row>
+    <row r="196" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A196" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B196" s="6">
+        <v>12.53</v>
+      </c>
+      <c r="C196" s="5">
+        <f t="shared" si="13"/>
+        <v>7.4399999999999995</v>
+      </c>
+      <c r="D196" s="5">
+        <f t="shared" si="14"/>
+        <v>17.619999999999997</v>
+      </c>
+      <c r="E196" s="5">
+        <v>12.53</v>
+      </c>
       <c r="F196">
         <v>12</v>
       </c>
+      <c r="G196" s="8">
+        <v>12</v>
+      </c>
+      <c r="H196" s="8">
+        <v>3</v>
+      </c>
       <c r="I196" t="s">
         <v>107</v>
       </c>
@@ -20153,11 +21402,36 @@
       <c r="L196" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="197" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N196" s="6"/>
+      <c r="O196" s="5"/>
+    </row>
+    <row r="197" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A197" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B197" s="6">
+        <v>12.98</v>
+      </c>
+      <c r="C197" s="5">
+        <f t="shared" si="13"/>
+        <v>7.8900000000000006</v>
+      </c>
+      <c r="D197" s="5">
+        <f t="shared" si="14"/>
+        <v>18.07</v>
+      </c>
+      <c r="E197" s="5">
+        <v>7.89</v>
+      </c>
       <c r="F197">
         <v>13</v>
       </c>
+      <c r="G197" s="8">
+        <v>7</v>
+      </c>
+      <c r="H197" s="8">
+        <v>18</v>
+      </c>
       <c r="I197" t="s">
         <v>107</v>
       </c>
@@ -20170,11 +21444,36 @@
       <c r="L197" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="198" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N197" s="6"/>
+      <c r="O197" s="5"/>
+    </row>
+    <row r="198" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A198" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B198" s="6">
+        <v>13.04</v>
+      </c>
+      <c r="C198" s="5">
+        <f t="shared" si="13"/>
+        <v>7.9499999999999993</v>
+      </c>
+      <c r="D198" s="5">
+        <f t="shared" si="14"/>
+        <v>18.13</v>
+      </c>
+      <c r="E198" s="5">
+        <v>18.13</v>
+      </c>
       <c r="F198">
         <v>14</v>
       </c>
+      <c r="G198" s="8">
+        <v>18</v>
+      </c>
+      <c r="H198" s="8">
+        <v>10</v>
+      </c>
       <c r="I198" t="s">
         <v>107</v>
       </c>
@@ -20187,11 +21486,36 @@
       <c r="L198" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="199" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N198" s="6"/>
+      <c r="O198" s="5"/>
+    </row>
+    <row r="199" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A199" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B199" s="6">
+        <v>13.17</v>
+      </c>
+      <c r="C199" s="5">
+        <f t="shared" si="13"/>
+        <v>8.08</v>
+      </c>
+      <c r="D199" s="5">
+        <f t="shared" si="14"/>
+        <v>18.259999999999998</v>
+      </c>
+      <c r="E199" s="5">
+        <v>13.17</v>
+      </c>
       <c r="F199">
         <v>15</v>
       </c>
+      <c r="G199" s="8">
+        <v>13</v>
+      </c>
+      <c r="H199" s="8">
+        <v>17</v>
+      </c>
       <c r="I199" t="s">
         <v>107</v>
       </c>
@@ -20204,11 +21528,36 @@
       <c r="L199" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="200" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N199" s="6"/>
+      <c r="O199" s="5"/>
+    </row>
+    <row r="200" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A200" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B200" s="6">
+        <v>13.94</v>
+      </c>
+      <c r="C200" s="5">
+        <f t="shared" si="13"/>
+        <v>8.85</v>
+      </c>
+      <c r="D200" s="5">
+        <f t="shared" si="14"/>
+        <v>19.03</v>
+      </c>
+      <c r="E200" s="5">
+        <v>19.03</v>
+      </c>
       <c r="F200">
         <v>16</v>
       </c>
+      <c r="G200" s="8">
+        <v>19</v>
+      </c>
+      <c r="H200" s="8">
+        <v>13</v>
+      </c>
       <c r="I200" t="s">
         <v>107</v>
       </c>
@@ -20221,11 +21570,36 @@
       <c r="L200" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="201" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N200" s="6"/>
+      <c r="O200" s="5"/>
+    </row>
+    <row r="201" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A201" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B201" s="6">
+        <v>14.17</v>
+      </c>
+      <c r="C201" s="5">
+        <f t="shared" si="13"/>
+        <v>9.08</v>
+      </c>
+      <c r="D201" s="5">
+        <f t="shared" si="14"/>
+        <v>19.259999999999998</v>
+      </c>
+      <c r="E201" s="5">
+        <v>19.260000000000002</v>
+      </c>
       <c r="F201">
         <v>17</v>
       </c>
+      <c r="G201" s="8">
+        <v>20</v>
+      </c>
+      <c r="H201" s="8">
+        <v>12</v>
+      </c>
       <c r="I201" t="s">
         <v>107</v>
       </c>
@@ -20238,11 +21612,36 @@
       <c r="L201" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="202" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N201" s="6"/>
+      <c r="O201" s="5"/>
+    </row>
+    <row r="202" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A202" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B202" s="6">
+        <v>14.44</v>
+      </c>
+      <c r="C202" s="5">
+        <f t="shared" si="13"/>
+        <v>9.35</v>
+      </c>
+      <c r="D202" s="5">
+        <f t="shared" si="14"/>
+        <v>19.53</v>
+      </c>
+      <c r="E202" s="5">
+        <v>19.53</v>
+      </c>
       <c r="F202">
         <v>18</v>
       </c>
+      <c r="G202" s="8">
+        <v>21</v>
+      </c>
+      <c r="H202" s="8">
+        <v>7</v>
+      </c>
       <c r="I202" t="s">
         <v>107</v>
       </c>
@@ -20255,11 +21654,36 @@
       <c r="L202" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="203" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N202" s="6"/>
+      <c r="O202" s="5"/>
+    </row>
+    <row r="203" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A203" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B203" s="6">
+        <v>14.96</v>
+      </c>
+      <c r="C203" s="5">
+        <f t="shared" si="13"/>
+        <v>9.870000000000001</v>
+      </c>
+      <c r="D203" s="5">
+        <f t="shared" si="14"/>
+        <v>20.05</v>
+      </c>
+      <c r="E203" s="5">
+        <v>20.05</v>
+      </c>
       <c r="F203">
         <v>19</v>
       </c>
+      <c r="G203" s="8">
+        <v>22</v>
+      </c>
+      <c r="H203" s="8">
+        <v>25</v>
+      </c>
       <c r="I203" t="s">
         <v>107</v>
       </c>
@@ -20272,11 +21696,36 @@
       <c r="L203" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="204" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N203" s="6"/>
+      <c r="O203" s="5"/>
+    </row>
+    <row r="204" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A204" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B204" s="6">
+        <v>15.33</v>
+      </c>
+      <c r="C204" s="5">
+        <f t="shared" si="13"/>
+        <v>10.24</v>
+      </c>
+      <c r="D204" s="5">
+        <f t="shared" si="14"/>
+        <v>20.420000000000002</v>
+      </c>
+      <c r="E204" s="5">
+        <v>15.33</v>
+      </c>
       <c r="F204">
         <v>20</v>
       </c>
+      <c r="G204" s="8">
+        <v>14</v>
+      </c>
+      <c r="H204" s="8">
+        <v>15</v>
+      </c>
       <c r="I204" t="s">
         <v>107</v>
       </c>
@@ -20289,11 +21738,36 @@
       <c r="L204" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="205" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N204" s="6"/>
+      <c r="O204" s="5"/>
+    </row>
+    <row r="205" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A205" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B205" s="6">
+        <v>16.46</v>
+      </c>
+      <c r="C205" s="5">
+        <f t="shared" si="13"/>
+        <v>11.370000000000001</v>
+      </c>
+      <c r="D205" s="5">
+        <f t="shared" si="14"/>
+        <v>21.55</v>
+      </c>
+      <c r="E205" s="5">
+        <v>16.46</v>
+      </c>
       <c r="F205">
         <v>21</v>
       </c>
+      <c r="G205" s="8">
+        <v>15</v>
+      </c>
+      <c r="H205" s="8">
+        <v>20</v>
+      </c>
       <c r="I205" t="s">
         <v>107</v>
       </c>
@@ -20306,11 +21780,36 @@
       <c r="L205" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="206" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N205" s="6"/>
+      <c r="O205" s="5"/>
+    </row>
+    <row r="206" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A206" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B206" s="6">
+        <v>16.46</v>
+      </c>
+      <c r="C206" s="5">
+        <f t="shared" si="13"/>
+        <v>11.370000000000001</v>
+      </c>
+      <c r="D206" s="5">
+        <f t="shared" si="14"/>
+        <v>21.55</v>
+      </c>
+      <c r="E206" s="5">
+        <v>21.55</v>
+      </c>
       <c r="F206">
         <v>22</v>
       </c>
+      <c r="G206" s="8">
+        <v>23</v>
+      </c>
+      <c r="H206" s="8">
+        <v>23</v>
+      </c>
       <c r="I206" t="s">
         <v>107</v>
       </c>
@@ -20323,11 +21822,36 @@
       <c r="L206" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="207" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N206" s="6"/>
+      <c r="O206" s="5"/>
+    </row>
+    <row r="207" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A207" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B207" s="6">
+        <v>17</v>
+      </c>
+      <c r="C207" s="5">
+        <f>B207-L207</f>
+        <v>11.91</v>
+      </c>
+      <c r="D207" s="5">
+        <f t="shared" si="14"/>
+        <v>22.09</v>
+      </c>
+      <c r="E207" s="5">
+        <v>17</v>
+      </c>
       <c r="F207">
         <v>23</v>
       </c>
+      <c r="G207" s="8">
+        <v>16</v>
+      </c>
+      <c r="H207" s="8">
+        <v>16</v>
+      </c>
       <c r="I207" t="s">
         <v>107</v>
       </c>
@@ -20340,11 +21864,36 @@
       <c r="L207" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="208" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N207" s="6"/>
+      <c r="O207" s="5"/>
+    </row>
+    <row r="208" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A208" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B208" s="6">
+        <v>18.05</v>
+      </c>
+      <c r="C208" s="5">
+        <f t="shared" si="13"/>
+        <v>12.96</v>
+      </c>
+      <c r="D208" s="5">
+        <f t="shared" si="14"/>
+        <v>23.14</v>
+      </c>
+      <c r="E208" s="5">
+        <v>23.14</v>
+      </c>
       <c r="F208">
         <v>24</v>
       </c>
+      <c r="G208" s="8">
+        <v>24</v>
+      </c>
+      <c r="H208" s="8">
+        <v>21</v>
+      </c>
       <c r="I208" t="s">
         <v>107</v>
       </c>
@@ -20357,11 +21906,36 @@
       <c r="L208" s="5">
         <v>5.09</v>
       </c>
-    </row>
-    <row r="209" spans="6:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N208" s="6"/>
+      <c r="O208" s="5"/>
+    </row>
+    <row r="209" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A209" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B209" s="6">
+        <v>18.079999999999998</v>
+      </c>
+      <c r="C209" s="5">
+        <f t="shared" si="13"/>
+        <v>12.989999999999998</v>
+      </c>
+      <c r="D209" s="5">
+        <f t="shared" si="14"/>
+        <v>23.169999999999998</v>
+      </c>
+      <c r="E209" s="5">
+        <v>23.17</v>
+      </c>
       <c r="F209">
         <v>25</v>
       </c>
+      <c r="G209" s="8">
+        <v>25</v>
+      </c>
+      <c r="H209" s="8">
+        <v>14</v>
+      </c>
       <c r="I209" t="s">
         <v>107</v>
       </c>
@@ -20374,10 +21948,987 @@
       <c r="L209" s="5">
         <v>5.09</v>
       </c>
+      <c r="N209" s="6"/>
+      <c r="O209" s="5"/>
+    </row>
+    <row r="210" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A210" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B210" s="6">
+        <v>8.33</v>
+      </c>
+      <c r="C210" s="5">
+        <f>B210-L210</f>
+        <v>3.24</v>
+      </c>
+      <c r="D210" s="5">
+        <f>B210+L210</f>
+        <v>13.42</v>
+      </c>
+      <c r="E210" s="5">
+        <v>3.24</v>
+      </c>
+      <c r="F210">
+        <v>1</v>
+      </c>
+      <c r="G210" s="8">
+        <v>1</v>
+      </c>
+      <c r="I210" t="s">
+        <v>108</v>
+      </c>
+      <c r="J210" t="s">
+        <v>85</v>
+      </c>
+      <c r="K210" t="s">
+        <v>86</v>
+      </c>
+      <c r="L210" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N210" s="6"/>
+      <c r="O210" s="5"/>
+    </row>
+    <row r="211" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A211" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B211" s="6">
+        <v>8.34</v>
+      </c>
+      <c r="C211" s="5">
+        <f t="shared" ref="C211:C234" si="15">B211-L211</f>
+        <v>3.25</v>
+      </c>
+      <c r="D211" s="5">
+        <f t="shared" ref="D211:D234" si="16">B211+L211</f>
+        <v>13.43</v>
+      </c>
+      <c r="E211" s="5">
+        <v>3.25</v>
+      </c>
+      <c r="F211">
+        <v>2</v>
+      </c>
+      <c r="G211" s="8">
+        <v>2</v>
+      </c>
+      <c r="I211" t="s">
+        <v>108</v>
+      </c>
+      <c r="J211" t="s">
+        <v>85</v>
+      </c>
+      <c r="K211" t="s">
+        <v>86</v>
+      </c>
+      <c r="L211" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N211" s="6"/>
+      <c r="O211" s="5"/>
+    </row>
+    <row r="212" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A212" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B212" s="6">
+        <v>9.3800000000000008</v>
+      </c>
+      <c r="C212" s="5">
+        <f t="shared" si="15"/>
+        <v>4.2900000000000009</v>
+      </c>
+      <c r="D212" s="5">
+        <f t="shared" si="16"/>
+        <v>14.47</v>
+      </c>
+      <c r="E212" s="5">
+        <v>9.3800000000000008</v>
+      </c>
+      <c r="F212">
+        <v>3</v>
+      </c>
+      <c r="G212" s="8">
+        <v>5</v>
+      </c>
+      <c r="I212" t="s">
+        <v>108</v>
+      </c>
+      <c r="J212" t="s">
+        <v>85</v>
+      </c>
+      <c r="K212" t="s">
+        <v>86</v>
+      </c>
+      <c r="L212" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N212" s="6"/>
+      <c r="O212" s="5"/>
+    </row>
+    <row r="213" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A213" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B213" s="6">
+        <v>9.51</v>
+      </c>
+      <c r="C213" s="5">
+        <f t="shared" si="15"/>
+        <v>4.42</v>
+      </c>
+      <c r="D213" s="5">
+        <f t="shared" si="16"/>
+        <v>14.6</v>
+      </c>
+      <c r="E213" s="5">
+        <v>9.51</v>
+      </c>
+      <c r="F213">
+        <v>4</v>
+      </c>
+      <c r="G213" s="8">
+        <v>7</v>
+      </c>
+      <c r="I213" t="s">
+        <v>108</v>
+      </c>
+      <c r="J213" t="s">
+        <v>85</v>
+      </c>
+      <c r="K213" t="s">
+        <v>86</v>
+      </c>
+      <c r="L213" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N213" s="6"/>
+      <c r="O213" s="5"/>
+    </row>
+    <row r="214" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A214" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B214" s="6">
+        <v>10.24</v>
+      </c>
+      <c r="C214" s="5">
+        <f t="shared" si="15"/>
+        <v>5.15</v>
+      </c>
+      <c r="D214" s="5">
+        <f t="shared" si="16"/>
+        <v>15.33</v>
+      </c>
+      <c r="E214" s="5">
+        <v>10.24</v>
+      </c>
+      <c r="F214">
+        <v>5</v>
+      </c>
+      <c r="G214" s="8">
+        <v>8</v>
+      </c>
+      <c r="I214" t="s">
+        <v>108</v>
+      </c>
+      <c r="J214" t="s">
+        <v>85</v>
+      </c>
+      <c r="K214" t="s">
+        <v>86</v>
+      </c>
+      <c r="L214" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N214" s="6"/>
+      <c r="O214" s="5"/>
+    </row>
+    <row r="215" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A215" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B215" s="6">
+        <v>10.34</v>
+      </c>
+      <c r="C215" s="5">
+        <f t="shared" si="15"/>
+        <v>5.25</v>
+      </c>
+      <c r="D215" s="5">
+        <f t="shared" si="16"/>
+        <v>15.43</v>
+      </c>
+      <c r="E215" s="5">
+        <v>10.34</v>
+      </c>
+      <c r="F215">
+        <v>6</v>
+      </c>
+      <c r="G215" s="8">
+        <v>9</v>
+      </c>
+      <c r="I215" t="s">
+        <v>108</v>
+      </c>
+      <c r="J215" t="s">
+        <v>85</v>
+      </c>
+      <c r="K215" t="s">
+        <v>86</v>
+      </c>
+      <c r="L215" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N215" s="6"/>
+      <c r="O215" s="5"/>
+    </row>
+    <row r="216" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A216" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B216" s="6">
+        <v>11.03</v>
+      </c>
+      <c r="C216" s="5">
+        <f t="shared" si="15"/>
+        <v>5.9399999999999995</v>
+      </c>
+      <c r="D216" s="5">
+        <f t="shared" si="16"/>
+        <v>16.119999999999997</v>
+      </c>
+      <c r="E216" s="5">
+        <v>11.03</v>
+      </c>
+      <c r="F216">
+        <v>7</v>
+      </c>
+      <c r="G216" s="8">
+        <v>10</v>
+      </c>
+      <c r="I216" t="s">
+        <v>108</v>
+      </c>
+      <c r="J216" t="s">
+        <v>85</v>
+      </c>
+      <c r="K216" t="s">
+        <v>86</v>
+      </c>
+      <c r="L216" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N216" s="6"/>
+      <c r="O216" s="5"/>
+    </row>
+    <row r="217" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A217" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B217" s="6">
+        <v>11.04</v>
+      </c>
+      <c r="C217" s="5">
+        <f t="shared" si="15"/>
+        <v>5.9499999999999993</v>
+      </c>
+      <c r="D217" s="5">
+        <f t="shared" si="16"/>
+        <v>16.13</v>
+      </c>
+      <c r="E217" s="5">
+        <v>5.95</v>
+      </c>
+      <c r="F217">
+        <v>8</v>
+      </c>
+      <c r="G217" s="8">
+        <v>3</v>
+      </c>
+      <c r="I217" t="s">
+        <v>108</v>
+      </c>
+      <c r="J217" t="s">
+        <v>85</v>
+      </c>
+      <c r="K217" t="s">
+        <v>86</v>
+      </c>
+      <c r="L217" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N217" s="6"/>
+      <c r="O217" s="5"/>
+    </row>
+    <row r="218" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A218" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B218" s="6">
+        <v>11.15</v>
+      </c>
+      <c r="C218" s="5">
+        <f t="shared" si="15"/>
+        <v>6.0600000000000005</v>
+      </c>
+      <c r="D218" s="5">
+        <f t="shared" si="16"/>
+        <v>16.240000000000002</v>
+      </c>
+      <c r="E218" s="5">
+        <v>6.06</v>
+      </c>
+      <c r="F218">
+        <v>9</v>
+      </c>
+      <c r="G218" s="8">
+        <v>4</v>
+      </c>
+      <c r="I218" t="s">
+        <v>108</v>
+      </c>
+      <c r="J218" t="s">
+        <v>85</v>
+      </c>
+      <c r="K218" t="s">
+        <v>86</v>
+      </c>
+      <c r="L218" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N218" s="6"/>
+      <c r="O218" s="5"/>
+    </row>
+    <row r="219" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A219" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B219" s="6">
+        <v>12.24</v>
+      </c>
+      <c r="C219" s="5">
+        <f t="shared" si="15"/>
+        <v>7.15</v>
+      </c>
+      <c r="D219" s="5">
+        <f t="shared" si="16"/>
+        <v>17.329999999999998</v>
+      </c>
+      <c r="E219" s="5">
+        <v>12.24</v>
+      </c>
+      <c r="F219">
+        <v>10</v>
+      </c>
+      <c r="G219" s="8">
+        <v>12</v>
+      </c>
+      <c r="I219" t="s">
+        <v>108</v>
+      </c>
+      <c r="J219" t="s">
+        <v>85</v>
+      </c>
+      <c r="K219" t="s">
+        <v>86</v>
+      </c>
+      <c r="L219" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N219" s="6"/>
+      <c r="O219" s="5"/>
+    </row>
+    <row r="220" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A220" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B220" s="6">
+        <v>12.83</v>
+      </c>
+      <c r="C220" s="5">
+        <f t="shared" si="15"/>
+        <v>7.74</v>
+      </c>
+      <c r="D220" s="5">
+        <f t="shared" si="16"/>
+        <v>17.920000000000002</v>
+      </c>
+      <c r="E220" s="5">
+        <v>12.83</v>
+      </c>
+      <c r="F220">
+        <v>11</v>
+      </c>
+      <c r="G220">
+        <v>13</v>
+      </c>
+      <c r="I220" t="s">
+        <v>108</v>
+      </c>
+      <c r="J220" t="s">
+        <v>85</v>
+      </c>
+      <c r="K220" t="s">
+        <v>86</v>
+      </c>
+      <c r="L220" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N220" s="6"/>
+      <c r="O220" s="5"/>
+    </row>
+    <row r="221" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A221" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B221" s="6">
+        <v>13.75</v>
+      </c>
+      <c r="C221" s="5">
+        <f t="shared" si="15"/>
+        <v>8.66</v>
+      </c>
+      <c r="D221" s="5">
+        <f t="shared" si="16"/>
+        <v>18.84</v>
+      </c>
+      <c r="E221" s="5">
+        <v>18.84</v>
+      </c>
+      <c r="F221">
+        <v>12</v>
+      </c>
+      <c r="G221" s="8">
+        <v>21</v>
+      </c>
+      <c r="I221" t="s">
+        <v>108</v>
+      </c>
+      <c r="J221" t="s">
+        <v>85</v>
+      </c>
+      <c r="K221" t="s">
+        <v>86</v>
+      </c>
+      <c r="L221" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N221" s="6"/>
+      <c r="O221" s="5"/>
+    </row>
+    <row r="222" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A222" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B222" s="6">
+        <v>13.87</v>
+      </c>
+      <c r="C222" s="5">
+        <f t="shared" si="15"/>
+        <v>8.7799999999999994</v>
+      </c>
+      <c r="D222" s="5">
+        <f t="shared" si="16"/>
+        <v>18.96</v>
+      </c>
+      <c r="E222" s="5">
+        <v>13.87</v>
+      </c>
+      <c r="F222">
+        <v>13</v>
+      </c>
+      <c r="G222" s="8">
+        <v>14</v>
+      </c>
+      <c r="I222" t="s">
+        <v>108</v>
+      </c>
+      <c r="J222" t="s">
+        <v>85</v>
+      </c>
+      <c r="K222" t="s">
+        <v>86</v>
+      </c>
+      <c r="L222" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N222" s="6"/>
+      <c r="O222" s="5"/>
+    </row>
+    <row r="223" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A223" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B223" s="6">
+        <v>14.05</v>
+      </c>
+      <c r="C223" s="5">
+        <f t="shared" si="15"/>
+        <v>8.9600000000000009</v>
+      </c>
+      <c r="D223" s="5">
+        <f t="shared" si="16"/>
+        <v>19.14</v>
+      </c>
+      <c r="E223" s="5">
+        <v>19.14</v>
+      </c>
+      <c r="F223">
+        <v>14</v>
+      </c>
+      <c r="G223" s="8">
+        <v>22</v>
+      </c>
+      <c r="I223" t="s">
+        <v>108</v>
+      </c>
+      <c r="J223" t="s">
+        <v>85</v>
+      </c>
+      <c r="K223" t="s">
+        <v>86</v>
+      </c>
+      <c r="L223" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N223" s="6"/>
+      <c r="O223" s="5"/>
+    </row>
+    <row r="224" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A224" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B224" s="6">
+        <v>14.33</v>
+      </c>
+      <c r="C224" s="5">
+        <f t="shared" si="15"/>
+        <v>9.24</v>
+      </c>
+      <c r="D224" s="5">
+        <f t="shared" si="16"/>
+        <v>19.420000000000002</v>
+      </c>
+      <c r="E224" s="5">
+        <v>14.33</v>
+      </c>
+      <c r="F224">
+        <v>15</v>
+      </c>
+      <c r="G224" s="8">
+        <v>15</v>
+      </c>
+      <c r="I224" t="s">
+        <v>108</v>
+      </c>
+      <c r="J224" t="s">
+        <v>85</v>
+      </c>
+      <c r="K224" t="s">
+        <v>86</v>
+      </c>
+      <c r="L224" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N224" s="6"/>
+      <c r="O224" s="5"/>
+    </row>
+    <row r="225" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A225" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B225" s="6">
+        <v>14.57</v>
+      </c>
+      <c r="C225" s="5">
+        <f t="shared" si="15"/>
+        <v>9.48</v>
+      </c>
+      <c r="D225" s="5">
+        <f t="shared" si="16"/>
+        <v>19.66</v>
+      </c>
+      <c r="E225" s="5">
+        <v>9.48</v>
+      </c>
+      <c r="F225">
+        <v>16</v>
+      </c>
+      <c r="G225" s="8">
+        <v>6</v>
+      </c>
+      <c r="I225" t="s">
+        <v>108</v>
+      </c>
+      <c r="J225" t="s">
+        <v>85</v>
+      </c>
+      <c r="K225" t="s">
+        <v>86</v>
+      </c>
+      <c r="L225" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N225" s="6"/>
+      <c r="O225" s="5"/>
+    </row>
+    <row r="226" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A226" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B226" s="6">
+        <v>14.59</v>
+      </c>
+      <c r="C226" s="5">
+        <f t="shared" si="15"/>
+        <v>9.5</v>
+      </c>
+      <c r="D226" s="5">
+        <f t="shared" si="16"/>
+        <v>19.68</v>
+      </c>
+      <c r="E226" s="5">
+        <v>14.59</v>
+      </c>
+      <c r="F226">
+        <v>17</v>
+      </c>
+      <c r="G226" s="8">
+        <v>16</v>
+      </c>
+      <c r="I226" t="s">
+        <v>108</v>
+      </c>
+      <c r="J226" t="s">
+        <v>85</v>
+      </c>
+      <c r="K226" t="s">
+        <v>86</v>
+      </c>
+      <c r="L226" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N226" s="6"/>
+      <c r="O226" s="5"/>
+    </row>
+    <row r="227" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A227" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B227" s="6">
+        <v>14.63</v>
+      </c>
+      <c r="C227" s="5">
+        <f t="shared" si="15"/>
+        <v>9.5400000000000009</v>
+      </c>
+      <c r="D227" s="5">
+        <f t="shared" si="16"/>
+        <v>19.72</v>
+      </c>
+      <c r="E227" s="5">
+        <v>14.63</v>
+      </c>
+      <c r="F227">
+        <v>18</v>
+      </c>
+      <c r="G227" s="8">
+        <v>17</v>
+      </c>
+      <c r="I227" t="s">
+        <v>108</v>
+      </c>
+      <c r="J227" t="s">
+        <v>85</v>
+      </c>
+      <c r="K227" t="s">
+        <v>86</v>
+      </c>
+      <c r="L227" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N227" s="6"/>
+      <c r="O227" s="5"/>
+    </row>
+    <row r="228" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A228" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B228" s="6">
+        <v>14.98</v>
+      </c>
+      <c r="C228" s="5">
+        <f t="shared" si="15"/>
+        <v>9.89</v>
+      </c>
+      <c r="D228" s="5">
+        <f t="shared" si="16"/>
+        <v>20.07</v>
+      </c>
+      <c r="E228" s="5">
+        <v>20.07</v>
+      </c>
+      <c r="F228">
+        <v>19</v>
+      </c>
+      <c r="G228" s="8">
+        <v>23</v>
+      </c>
+      <c r="I228" t="s">
+        <v>108</v>
+      </c>
+      <c r="J228" t="s">
+        <v>85</v>
+      </c>
+      <c r="K228" t="s">
+        <v>86</v>
+      </c>
+      <c r="L228" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N228" s="6"/>
+      <c r="O228" s="5"/>
+    </row>
+    <row r="229" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A229" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B229" s="6">
+        <v>14.98</v>
+      </c>
+      <c r="C229" s="5">
+        <f t="shared" si="15"/>
+        <v>9.89</v>
+      </c>
+      <c r="D229" s="5">
+        <f t="shared" si="16"/>
+        <v>20.07</v>
+      </c>
+      <c r="E229" s="5">
+        <v>14.98</v>
+      </c>
+      <c r="F229">
+        <v>20</v>
+      </c>
+      <c r="G229" s="8">
+        <v>18</v>
+      </c>
+      <c r="I229" t="s">
+        <v>108</v>
+      </c>
+      <c r="J229" t="s">
+        <v>85</v>
+      </c>
+      <c r="K229" t="s">
+        <v>86</v>
+      </c>
+      <c r="L229" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N229" s="6"/>
+      <c r="O229" s="5"/>
+    </row>
+    <row r="230" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A230" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B230" s="6">
+        <v>15.75</v>
+      </c>
+      <c r="C230" s="5">
+        <f t="shared" si="15"/>
+        <v>10.66</v>
+      </c>
+      <c r="D230" s="5">
+        <f t="shared" si="16"/>
+        <v>20.84</v>
+      </c>
+      <c r="E230" s="5">
+        <v>15.75</v>
+      </c>
+      <c r="F230">
+        <v>21</v>
+      </c>
+      <c r="G230" s="8">
+        <v>19</v>
+      </c>
+      <c r="I230" t="s">
+        <v>108</v>
+      </c>
+      <c r="J230" t="s">
+        <v>85</v>
+      </c>
+      <c r="K230" t="s">
+        <v>86</v>
+      </c>
+      <c r="L230" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N230" s="6"/>
+      <c r="O230" s="5"/>
+    </row>
+    <row r="231" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A231" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B231" s="6">
+        <v>16.239999999999998</v>
+      </c>
+      <c r="C231" s="5">
+        <f t="shared" si="15"/>
+        <v>11.149999999999999</v>
+      </c>
+      <c r="D231" s="5">
+        <f t="shared" si="16"/>
+        <v>21.33</v>
+      </c>
+      <c r="E231" s="5">
+        <v>11.15</v>
+      </c>
+      <c r="F231">
+        <v>22</v>
+      </c>
+      <c r="G231" s="8">
+        <v>11</v>
+      </c>
+      <c r="I231" t="s">
+        <v>108</v>
+      </c>
+      <c r="J231" t="s">
+        <v>85</v>
+      </c>
+      <c r="K231" t="s">
+        <v>86</v>
+      </c>
+      <c r="L231" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N231" s="6"/>
+      <c r="O231" s="5"/>
+    </row>
+    <row r="232" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A232" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B232" s="6">
+        <v>16.5</v>
+      </c>
+      <c r="C232" s="5">
+        <f t="shared" si="15"/>
+        <v>11.41</v>
+      </c>
+      <c r="D232" s="5">
+        <f t="shared" si="16"/>
+        <v>21.59</v>
+      </c>
+      <c r="E232" s="5">
+        <v>21.59</v>
+      </c>
+      <c r="F232">
+        <v>23</v>
+      </c>
+      <c r="G232" s="8">
+        <v>24</v>
+      </c>
+      <c r="I232" t="s">
+        <v>108</v>
+      </c>
+      <c r="J232" t="s">
+        <v>85</v>
+      </c>
+      <c r="K232" t="s">
+        <v>86</v>
+      </c>
+      <c r="L232" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N232" s="6"/>
+      <c r="O232" s="5"/>
+    </row>
+    <row r="233" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A233" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B233" s="6">
+        <v>16.55</v>
+      </c>
+      <c r="C233" s="5">
+        <f>B233-L233</f>
+        <v>11.46</v>
+      </c>
+      <c r="D233" s="5">
+        <f t="shared" si="16"/>
+        <v>21.64</v>
+      </c>
+      <c r="E233" s="5">
+        <v>16.55</v>
+      </c>
+      <c r="F233">
+        <v>24</v>
+      </c>
+      <c r="G233" s="8">
+        <v>20</v>
+      </c>
+      <c r="I233" t="s">
+        <v>108</v>
+      </c>
+      <c r="J233" t="s">
+        <v>85</v>
+      </c>
+      <c r="K233" t="s">
+        <v>86</v>
+      </c>
+      <c r="L233" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N233" s="6"/>
+      <c r="O233" s="5"/>
+    </row>
+    <row r="234" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A234" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B234" s="6">
+        <v>16.55</v>
+      </c>
+      <c r="C234" s="5">
+        <f t="shared" si="15"/>
+        <v>11.46</v>
+      </c>
+      <c r="D234" s="5">
+        <f t="shared" si="16"/>
+        <v>21.64</v>
+      </c>
+      <c r="E234" s="5">
+        <v>21.64</v>
+      </c>
+      <c r="F234">
+        <v>25</v>
+      </c>
+      <c r="G234" s="8">
+        <v>25</v>
+      </c>
+      <c r="I234" t="s">
+        <v>108</v>
+      </c>
+      <c r="J234" t="s">
+        <v>85</v>
+      </c>
+      <c r="K234" t="s">
+        <v>86</v>
+      </c>
+      <c r="L234" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N234" s="6"/>
+      <c r="O234" s="5"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N152:O184">
-    <sortCondition ref="O152:O184"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N210:O234">
+    <sortCondition ref="O210:O234"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated dataset and Fixed pages
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0318EF4D-6065-44FF-9195-AC7A6C5D3CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08571517-CCB6-4ABB-A404-FAE52C17D7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy_Model" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2029" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2329" uniqueCount="111">
   <si>
     <t>Model</t>
   </si>
@@ -370,13 +370,20 @@
   <si>
     <t>World Wide Technology Raceway</t>
   </si>
+  <si>
+    <t>Nashville Superpeedway</t>
+  </si>
+  <si>
+    <t>Milwaukee Mile</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -471,7 +478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -504,6 +511,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11785,7 +11793,7 @@
         <v>10.58</v>
       </c>
       <c r="C211" s="5">
-        <f t="shared" ref="C211:C234" si="16">B211-L211</f>
+        <f t="shared" ref="C211:C233" si="16">B211-L211</f>
         <v>5.15</v>
       </c>
       <c r="D211" s="5">
@@ -12735,218 +12743,1543 @@
       </c>
     </row>
     <row r="235" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A235" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B235" s="6">
+        <v>10.93</v>
+      </c>
       <c r="G235" s="8"/>
       <c r="H235" s="8"/>
+      <c r="I235" t="s">
+        <v>109</v>
+      </c>
+      <c r="J235" t="s">
+        <v>85</v>
+      </c>
+      <c r="K235" t="s">
+        <v>77</v>
+      </c>
+      <c r="L235">
+        <v>5.43</v>
+      </c>
     </row>
     <row r="236" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A236" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B236" s="6">
+        <v>10.96</v>
+      </c>
       <c r="G236" s="8"/>
       <c r="H236" s="8"/>
+      <c r="I236" t="s">
+        <v>109</v>
+      </c>
+      <c r="J236" t="s">
+        <v>85</v>
+      </c>
+      <c r="K236" t="s">
+        <v>77</v>
+      </c>
+      <c r="L236">
+        <v>5.43</v>
+      </c>
     </row>
     <row r="237" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A237" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B237" s="6">
+        <v>11.4</v>
+      </c>
       <c r="G237" s="8"/>
       <c r="H237" s="8"/>
+      <c r="I237" t="s">
+        <v>109</v>
+      </c>
+      <c r="J237" t="s">
+        <v>85</v>
+      </c>
+      <c r="K237" t="s">
+        <v>77</v>
+      </c>
+      <c r="L237">
+        <v>5.43</v>
+      </c>
     </row>
     <row r="238" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A238" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B238" s="6">
+        <v>11.91</v>
+      </c>
       <c r="G238" s="8"/>
       <c r="H238" s="8"/>
+      <c r="I238" t="s">
+        <v>109</v>
+      </c>
+      <c r="J238" t="s">
+        <v>85</v>
+      </c>
+      <c r="K238" t="s">
+        <v>77</v>
+      </c>
+      <c r="L238">
+        <v>5.43</v>
+      </c>
     </row>
     <row r="239" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A239" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B239" s="6">
+        <v>12.31</v>
+      </c>
       <c r="G239" s="8"/>
       <c r="H239" s="8"/>
+      <c r="I239" t="s">
+        <v>109</v>
+      </c>
+      <c r="J239" t="s">
+        <v>85</v>
+      </c>
+      <c r="K239" t="s">
+        <v>77</v>
+      </c>
+      <c r="L239">
+        <v>5.43</v>
+      </c>
     </row>
     <row r="240" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A240" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B240" s="6">
+        <v>12.61</v>
+      </c>
       <c r="G240" s="8"/>
       <c r="H240" s="8"/>
-    </row>
-    <row r="241" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I240" t="s">
+        <v>109</v>
+      </c>
+      <c r="J240" t="s">
+        <v>85</v>
+      </c>
+      <c r="K240" t="s">
+        <v>77</v>
+      </c>
+      <c r="L240">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="241" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A241" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B241" s="6">
+        <v>12.66</v>
+      </c>
       <c r="G241" s="8"/>
       <c r="H241" s="8"/>
-    </row>
-    <row r="242" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I241" t="s">
+        <v>109</v>
+      </c>
+      <c r="J241" t="s">
+        <v>85</v>
+      </c>
+      <c r="K241" t="s">
+        <v>77</v>
+      </c>
+      <c r="L241">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="242" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A242" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B242" s="6">
+        <v>12.76</v>
+      </c>
       <c r="G242" s="8"/>
       <c r="H242" s="8"/>
-    </row>
-    <row r="243" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I242" t="s">
+        <v>109</v>
+      </c>
+      <c r="J242" t="s">
+        <v>85</v>
+      </c>
+      <c r="K242" t="s">
+        <v>77</v>
+      </c>
+      <c r="L242">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="243" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A243" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B243" s="6">
+        <v>13.04</v>
+      </c>
       <c r="G243" s="8"/>
       <c r="H243" s="8"/>
-    </row>
-    <row r="244" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I243" t="s">
+        <v>109</v>
+      </c>
+      <c r="J243" t="s">
+        <v>85</v>
+      </c>
+      <c r="K243" t="s">
+        <v>77</v>
+      </c>
+      <c r="L243">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="244" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A244" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B244" s="6">
+        <v>13.07</v>
+      </c>
       <c r="G244" s="8"/>
       <c r="H244" s="8"/>
-    </row>
-    <row r="245" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I244" t="s">
+        <v>109</v>
+      </c>
+      <c r="J244" t="s">
+        <v>85</v>
+      </c>
+      <c r="K244" t="s">
+        <v>77</v>
+      </c>
+      <c r="L244">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="245" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A245" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B245" s="6">
+        <v>13.11</v>
+      </c>
       <c r="G245" s="8"/>
       <c r="H245" s="8"/>
-    </row>
-    <row r="246" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I245" t="s">
+        <v>109</v>
+      </c>
+      <c r="J245" t="s">
+        <v>85</v>
+      </c>
+      <c r="K245" t="s">
+        <v>77</v>
+      </c>
+      <c r="L245">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="246" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A246" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B246" s="6">
+        <v>13.11</v>
+      </c>
       <c r="G246" s="8"/>
       <c r="H246" s="8"/>
-    </row>
-    <row r="247" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I246" t="s">
+        <v>109</v>
+      </c>
+      <c r="J246" t="s">
+        <v>85</v>
+      </c>
+      <c r="K246" t="s">
+        <v>77</v>
+      </c>
+      <c r="L246">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="247" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A247" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B247" s="6">
+        <v>13.18</v>
+      </c>
       <c r="G247" s="8"/>
       <c r="H247" s="8"/>
-    </row>
-    <row r="248" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I247" t="s">
+        <v>109</v>
+      </c>
+      <c r="J247" t="s">
+        <v>85</v>
+      </c>
+      <c r="K247" t="s">
+        <v>77</v>
+      </c>
+      <c r="L247">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="248" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A248" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B248" s="6">
+        <v>13.34</v>
+      </c>
       <c r="G248" s="8"/>
       <c r="H248" s="8"/>
-    </row>
-    <row r="249" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I248" t="s">
+        <v>109</v>
+      </c>
+      <c r="J248" t="s">
+        <v>85</v>
+      </c>
+      <c r="K248" t="s">
+        <v>77</v>
+      </c>
+      <c r="L248">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="249" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A249" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B249" s="6">
+        <v>13.77</v>
+      </c>
       <c r="G249" s="8"/>
       <c r="H249" s="8"/>
-    </row>
-    <row r="250" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I249" t="s">
+        <v>109</v>
+      </c>
+      <c r="J249" t="s">
+        <v>85</v>
+      </c>
+      <c r="K249" t="s">
+        <v>77</v>
+      </c>
+      <c r="L249">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="250" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A250" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B250" s="6">
+        <v>14.11</v>
+      </c>
       <c r="G250" s="8"/>
       <c r="H250" s="8"/>
-    </row>
-    <row r="251" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I250" t="s">
+        <v>109</v>
+      </c>
+      <c r="J250" t="s">
+        <v>85</v>
+      </c>
+      <c r="K250" t="s">
+        <v>77</v>
+      </c>
+      <c r="L250">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="251" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A251" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B251" s="6">
+        <v>14.19</v>
+      </c>
       <c r="G251" s="8"/>
       <c r="H251" s="8"/>
-    </row>
-    <row r="252" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I251" t="s">
+        <v>109</v>
+      </c>
+      <c r="J251" t="s">
+        <v>85</v>
+      </c>
+      <c r="K251" t="s">
+        <v>77</v>
+      </c>
+      <c r="L251">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="252" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A252" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B252" s="6">
+        <v>14.9</v>
+      </c>
       <c r="G252" s="8"/>
       <c r="H252" s="8"/>
-    </row>
-    <row r="253" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I252" t="s">
+        <v>109</v>
+      </c>
+      <c r="J252" t="s">
+        <v>85</v>
+      </c>
+      <c r="K252" t="s">
+        <v>77</v>
+      </c>
+      <c r="L252">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="253" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A253" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B253" s="6">
+        <v>14.94</v>
+      </c>
       <c r="G253" s="8"/>
       <c r="H253" s="8"/>
-    </row>
-    <row r="254" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I253" t="s">
+        <v>109</v>
+      </c>
+      <c r="J253" t="s">
+        <v>85</v>
+      </c>
+      <c r="K253" t="s">
+        <v>77</v>
+      </c>
+      <c r="L253">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="254" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A254" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B254" s="6">
+        <v>15.13</v>
+      </c>
       <c r="G254" s="8"/>
       <c r="H254" s="8"/>
-    </row>
-    <row r="255" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I254" t="s">
+        <v>109</v>
+      </c>
+      <c r="J254" t="s">
+        <v>85</v>
+      </c>
+      <c r="K254" t="s">
+        <v>77</v>
+      </c>
+      <c r="L254">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="255" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A255" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B255" s="6">
+        <v>15.17</v>
+      </c>
       <c r="G255" s="8"/>
       <c r="H255" s="8"/>
-    </row>
-    <row r="256" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I255" t="s">
+        <v>109</v>
+      </c>
+      <c r="J255" t="s">
+        <v>85</v>
+      </c>
+      <c r="K255" t="s">
+        <v>77</v>
+      </c>
+      <c r="L255">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="256" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A256" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B256" s="6">
+        <v>15.25</v>
+      </c>
       <c r="G256" s="8"/>
       <c r="H256" s="8"/>
-    </row>
-    <row r="257" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I256" t="s">
+        <v>109</v>
+      </c>
+      <c r="J256" t="s">
+        <v>85</v>
+      </c>
+      <c r="K256" t="s">
+        <v>77</v>
+      </c>
+      <c r="L256">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="257" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A257" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B257" s="6">
+        <v>15.26</v>
+      </c>
       <c r="G257" s="8"/>
       <c r="H257" s="8"/>
-    </row>
-    <row r="258" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I257" t="s">
+        <v>109</v>
+      </c>
+      <c r="J257" t="s">
+        <v>85</v>
+      </c>
+      <c r="K257" t="s">
+        <v>77</v>
+      </c>
+      <c r="L257">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="258" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A258" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B258" s="6">
+        <v>15.3</v>
+      </c>
       <c r="G258" s="8"/>
       <c r="H258" s="8"/>
-    </row>
-    <row r="259" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I258" t="s">
+        <v>109</v>
+      </c>
+      <c r="J258" t="s">
+        <v>85</v>
+      </c>
+      <c r="K258" t="s">
+        <v>77</v>
+      </c>
+      <c r="L258">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="259" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A259" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B259" s="6">
+        <v>15.54</v>
+      </c>
       <c r="G259" s="8"/>
       <c r="H259" s="8"/>
-    </row>
-    <row r="260" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G260" s="8"/>
+      <c r="I259" t="s">
+        <v>109</v>
+      </c>
+      <c r="J259" t="s">
+        <v>85</v>
+      </c>
+      <c r="K259" t="s">
+        <v>77</v>
+      </c>
+      <c r="L259">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="260" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A260" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B260" s="6">
+        <v>7.71</v>
+      </c>
+      <c r="C260">
+        <f>B260-L260</f>
+        <v>2.2800000000000002</v>
+      </c>
+      <c r="D260">
+        <f>B260+L260</f>
+        <v>13.14</v>
+      </c>
+      <c r="E260">
+        <v>7.71</v>
+      </c>
+      <c r="F260">
+        <v>1</v>
+      </c>
+      <c r="G260" s="8">
+        <v>5</v>
+      </c>
       <c r="H260" s="8"/>
-    </row>
-    <row r="261" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G261" s="8"/>
+      <c r="I260" t="s">
+        <v>110</v>
+      </c>
+      <c r="J260" t="s">
+        <v>85</v>
+      </c>
+      <c r="K260" t="s">
+        <v>77</v>
+      </c>
+      <c r="L260">
+        <v>5.43</v>
+      </c>
+      <c r="N260" s="6"/>
+    </row>
+    <row r="261" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A261" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B261" s="6">
+        <v>8.11</v>
+      </c>
+      <c r="C261">
+        <f>B261-L261</f>
+        <v>2.6799999999999997</v>
+      </c>
+      <c r="D261">
+        <f t="shared" ref="D261:D284" si="18">B261+L261</f>
+        <v>13.54</v>
+      </c>
+      <c r="E261">
+        <v>2.68</v>
+      </c>
+      <c r="F261">
+        <v>2</v>
+      </c>
+      <c r="G261" s="8">
+        <v>1</v>
+      </c>
       <c r="H261" s="8"/>
-    </row>
-    <row r="262" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G262" s="8"/>
+      <c r="I261" t="s">
+        <v>110</v>
+      </c>
+      <c r="J261" t="s">
+        <v>85</v>
+      </c>
+      <c r="K261" t="s">
+        <v>77</v>
+      </c>
+      <c r="L261">
+        <v>5.43</v>
+      </c>
+      <c r="N261" s="6"/>
+    </row>
+    <row r="262" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A262" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B262" s="6">
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="C262">
+        <f t="shared" ref="C261:C284" si="19">B262-L262</f>
+        <v>2.8499999999999996</v>
+      </c>
+      <c r="D262">
+        <f t="shared" si="18"/>
+        <v>13.709999999999999</v>
+      </c>
+      <c r="E262">
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="F262">
+        <v>3</v>
+      </c>
+      <c r="G262" s="8">
+        <v>7</v>
+      </c>
       <c r="H262" s="8"/>
-    </row>
-    <row r="263" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G263" s="8"/>
+      <c r="I262" t="s">
+        <v>110</v>
+      </c>
+      <c r="J262" t="s">
+        <v>85</v>
+      </c>
+      <c r="K262" t="s">
+        <v>77</v>
+      </c>
+      <c r="L262">
+        <v>5.43</v>
+      </c>
+      <c r="N262" s="6"/>
+    </row>
+    <row r="263" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A263" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B263" s="6">
+        <v>8.51</v>
+      </c>
+      <c r="C263">
+        <f t="shared" si="19"/>
+        <v>3.08</v>
+      </c>
+      <c r="D263">
+        <f t="shared" si="18"/>
+        <v>13.94</v>
+      </c>
+      <c r="E263">
+        <v>3.08</v>
+      </c>
+      <c r="F263">
+        <v>4</v>
+      </c>
+      <c r="G263" s="8">
+        <v>2</v>
+      </c>
       <c r="H263" s="8"/>
-    </row>
-    <row r="264" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G264" s="8"/>
+      <c r="I263" t="s">
+        <v>110</v>
+      </c>
+      <c r="J263" t="s">
+        <v>85</v>
+      </c>
+      <c r="K263" t="s">
+        <v>77</v>
+      </c>
+      <c r="L263">
+        <v>5.43</v>
+      </c>
+      <c r="N263" s="6"/>
+    </row>
+    <row r="264" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A264" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B264" s="6">
+        <v>9.23</v>
+      </c>
+      <c r="C264" s="16">
+        <f t="shared" si="19"/>
+        <v>3.8000000000000007</v>
+      </c>
+      <c r="D264">
+        <f t="shared" si="18"/>
+        <v>14.66</v>
+      </c>
+      <c r="E264">
+        <v>3.8</v>
+      </c>
+      <c r="F264">
+        <v>5</v>
+      </c>
+      <c r="G264" s="8">
+        <v>3</v>
+      </c>
       <c r="H264" s="8"/>
-    </row>
-    <row r="265" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G265" s="8"/>
+      <c r="I264" t="s">
+        <v>110</v>
+      </c>
+      <c r="J264" t="s">
+        <v>85</v>
+      </c>
+      <c r="K264" t="s">
+        <v>77</v>
+      </c>
+      <c r="L264">
+        <v>5.43</v>
+      </c>
+      <c r="N264" s="6"/>
+    </row>
+    <row r="265" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A265" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B265" s="6">
+        <v>9.23</v>
+      </c>
+      <c r="C265" s="16">
+        <f t="shared" si="19"/>
+        <v>3.8000000000000007</v>
+      </c>
+      <c r="D265">
+        <f t="shared" si="18"/>
+        <v>14.66</v>
+      </c>
+      <c r="E265">
+        <v>14.66</v>
+      </c>
+      <c r="F265">
+        <v>6</v>
+      </c>
+      <c r="G265" s="8">
+        <v>18</v>
+      </c>
       <c r="H265" s="8"/>
-    </row>
-    <row r="266" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G266" s="8"/>
+      <c r="I265" t="s">
+        <v>110</v>
+      </c>
+      <c r="J265" t="s">
+        <v>85</v>
+      </c>
+      <c r="K265" t="s">
+        <v>77</v>
+      </c>
+      <c r="L265">
+        <v>5.43</v>
+      </c>
+      <c r="N265" s="6"/>
+    </row>
+    <row r="266" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A266" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B266" s="6">
+        <v>9.26</v>
+      </c>
+      <c r="C266">
+        <f t="shared" si="19"/>
+        <v>3.83</v>
+      </c>
+      <c r="D266">
+        <f t="shared" si="18"/>
+        <v>14.69</v>
+      </c>
+      <c r="E266">
+        <v>9.26</v>
+      </c>
+      <c r="F266">
+        <v>7</v>
+      </c>
+      <c r="G266" s="8">
+        <v>10</v>
+      </c>
       <c r="H266" s="8"/>
-    </row>
-    <row r="267" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G267" s="8"/>
+      <c r="I266" t="s">
+        <v>110</v>
+      </c>
+      <c r="J266" t="s">
+        <v>85</v>
+      </c>
+      <c r="K266" t="s">
+        <v>77</v>
+      </c>
+      <c r="L266">
+        <v>5.43</v>
+      </c>
+      <c r="N266" s="6"/>
+    </row>
+    <row r="267" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A267" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B267" s="6">
+        <v>10.77</v>
+      </c>
+      <c r="C267">
+        <f t="shared" si="19"/>
+        <v>5.34</v>
+      </c>
+      <c r="D267">
+        <f t="shared" si="18"/>
+        <v>16.2</v>
+      </c>
+      <c r="E267">
+        <v>10.77</v>
+      </c>
+      <c r="F267">
+        <v>8</v>
+      </c>
+      <c r="G267" s="8">
+        <v>11</v>
+      </c>
       <c r="H267" s="8"/>
-    </row>
-    <row r="268" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G268" s="8"/>
+      <c r="I267" t="s">
+        <v>110</v>
+      </c>
+      <c r="J267" t="s">
+        <v>85</v>
+      </c>
+      <c r="K267" t="s">
+        <v>77</v>
+      </c>
+      <c r="L267">
+        <v>5.43</v>
+      </c>
+      <c r="N267" s="6"/>
+    </row>
+    <row r="268" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A268" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B268" s="6">
+        <v>10.94</v>
+      </c>
+      <c r="C268">
+        <f t="shared" si="19"/>
+        <v>5.51</v>
+      </c>
+      <c r="D268">
+        <f t="shared" si="18"/>
+        <v>16.369999999999997</v>
+      </c>
+      <c r="E268">
+        <v>10.94</v>
+      </c>
+      <c r="F268">
+        <v>9</v>
+      </c>
+      <c r="G268" s="8">
+        <v>12</v>
+      </c>
       <c r="H268" s="8"/>
-    </row>
-    <row r="269" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G269" s="8"/>
+      <c r="I268" t="s">
+        <v>110</v>
+      </c>
+      <c r="J268" t="s">
+        <v>85</v>
+      </c>
+      <c r="K268" t="s">
+        <v>77</v>
+      </c>
+      <c r="L268">
+        <v>5.43</v>
+      </c>
+      <c r="N268" s="6"/>
+    </row>
+    <row r="269" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A269" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B269" s="6">
+        <v>10.97</v>
+      </c>
+      <c r="C269">
+        <f t="shared" si="19"/>
+        <v>5.5400000000000009</v>
+      </c>
+      <c r="D269">
+        <f t="shared" si="18"/>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="E269">
+        <v>10.97</v>
+      </c>
+      <c r="F269">
+        <v>10</v>
+      </c>
+      <c r="G269" s="8">
+        <v>13</v>
+      </c>
       <c r="H269" s="8"/>
-    </row>
-    <row r="270" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G270" s="8"/>
+      <c r="I269" t="s">
+        <v>110</v>
+      </c>
+      <c r="J269" t="s">
+        <v>85</v>
+      </c>
+      <c r="K269" t="s">
+        <v>77</v>
+      </c>
+      <c r="L269">
+        <v>5.43</v>
+      </c>
+      <c r="N269" s="6"/>
+    </row>
+    <row r="270" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A270" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B270" s="6">
+        <v>11.25</v>
+      </c>
+      <c r="C270">
+        <f t="shared" si="19"/>
+        <v>5.82</v>
+      </c>
+      <c r="D270">
+        <f t="shared" si="18"/>
+        <v>16.68</v>
+      </c>
+      <c r="E270">
+        <v>5.82</v>
+      </c>
+      <c r="F270">
+        <v>11</v>
+      </c>
+      <c r="G270" s="8">
+        <v>4</v>
+      </c>
       <c r="H270" s="8"/>
-    </row>
-    <row r="271" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G271" s="8"/>
+      <c r="I270" t="s">
+        <v>110</v>
+      </c>
+      <c r="J270" t="s">
+        <v>85</v>
+      </c>
+      <c r="K270" t="s">
+        <v>77</v>
+      </c>
+      <c r="L270">
+        <v>5.43</v>
+      </c>
+      <c r="N270" s="6"/>
+    </row>
+    <row r="271" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A271" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B271" s="6">
+        <v>11.52</v>
+      </c>
+      <c r="C271">
+        <f t="shared" si="19"/>
+        <v>6.09</v>
+      </c>
+      <c r="D271">
+        <f t="shared" si="18"/>
+        <v>16.95</v>
+      </c>
+      <c r="E271">
+        <v>11.53</v>
+      </c>
+      <c r="F271">
+        <v>12</v>
+      </c>
+      <c r="G271" s="8">
+        <v>14</v>
+      </c>
       <c r="H271" s="8"/>
-    </row>
-    <row r="272" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G272" s="8"/>
+      <c r="I271" t="s">
+        <v>110</v>
+      </c>
+      <c r="J271" t="s">
+        <v>85</v>
+      </c>
+      <c r="K271" t="s">
+        <v>77</v>
+      </c>
+      <c r="L271">
+        <v>5.43</v>
+      </c>
+      <c r="N271" s="6"/>
+    </row>
+    <row r="272" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A272" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B272" s="6">
+        <v>12.71</v>
+      </c>
+      <c r="C272">
+        <f t="shared" si="19"/>
+        <v>7.2800000000000011</v>
+      </c>
+      <c r="D272">
+        <f t="shared" si="18"/>
+        <v>18.14</v>
+      </c>
+      <c r="E272">
+        <v>12.71</v>
+      </c>
+      <c r="F272">
+        <v>13</v>
+      </c>
+      <c r="G272" s="8">
+        <v>16</v>
+      </c>
       <c r="H272" s="8"/>
-    </row>
-    <row r="273" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G273" s="8"/>
+      <c r="I272" t="s">
+        <v>110</v>
+      </c>
+      <c r="J272" t="s">
+        <v>85</v>
+      </c>
+      <c r="K272" t="s">
+        <v>77</v>
+      </c>
+      <c r="L272">
+        <v>5.43</v>
+      </c>
+      <c r="N272" s="6"/>
+    </row>
+    <row r="273" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A273" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B273" s="6">
+        <v>13.03</v>
+      </c>
+      <c r="C273">
+        <f t="shared" si="19"/>
+        <v>7.6</v>
+      </c>
+      <c r="D273">
+        <f t="shared" si="18"/>
+        <v>18.46</v>
+      </c>
+      <c r="E273">
+        <v>18.46</v>
+      </c>
+      <c r="F273">
+        <v>14</v>
+      </c>
+      <c r="G273" s="8">
+        <v>23</v>
+      </c>
       <c r="H273" s="8"/>
-    </row>
-    <row r="274" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G274" s="8"/>
+      <c r="I273" t="s">
+        <v>110</v>
+      </c>
+      <c r="J273" t="s">
+        <v>85</v>
+      </c>
+      <c r="K273" t="s">
+        <v>77</v>
+      </c>
+      <c r="L273">
+        <v>5.43</v>
+      </c>
+      <c r="N273" s="6"/>
+    </row>
+    <row r="274" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A274" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B274" s="6">
+        <v>13.18</v>
+      </c>
+      <c r="C274">
+        <f t="shared" si="19"/>
+        <v>7.75</v>
+      </c>
+      <c r="D274">
+        <f t="shared" si="18"/>
+        <v>18.61</v>
+      </c>
+      <c r="E274">
+        <v>7.75</v>
+      </c>
+      <c r="F274">
+        <v>15</v>
+      </c>
+      <c r="G274" s="8">
+        <v>6</v>
+      </c>
       <c r="H274" s="8"/>
-    </row>
-    <row r="275" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G275" s="8"/>
+      <c r="I274" t="s">
+        <v>110</v>
+      </c>
+      <c r="J274" t="s">
+        <v>85</v>
+      </c>
+      <c r="K274" t="s">
+        <v>77</v>
+      </c>
+      <c r="L274">
+        <v>5.43</v>
+      </c>
+      <c r="N274" s="6"/>
+    </row>
+    <row r="275" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A275" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B275" s="6">
+        <v>14.17</v>
+      </c>
+      <c r="C275">
+        <f t="shared" si="19"/>
+        <v>8.74</v>
+      </c>
+      <c r="D275">
+        <f t="shared" si="18"/>
+        <v>19.600000000000001</v>
+      </c>
+      <c r="E275">
+        <v>8.74</v>
+      </c>
+      <c r="F275">
+        <v>16</v>
+      </c>
+      <c r="G275" s="8">
+        <v>8</v>
+      </c>
       <c r="H275" s="8"/>
-    </row>
-    <row r="276" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G276" s="8"/>
+      <c r="I275" t="s">
+        <v>110</v>
+      </c>
+      <c r="J275" t="s">
+        <v>85</v>
+      </c>
+      <c r="K275" t="s">
+        <v>77</v>
+      </c>
+      <c r="L275">
+        <v>5.43</v>
+      </c>
+      <c r="N275" s="6"/>
+    </row>
+    <row r="276" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A276" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B276" s="6">
+        <v>14.29</v>
+      </c>
+      <c r="C276">
+        <f t="shared" si="19"/>
+        <v>8.86</v>
+      </c>
+      <c r="D276">
+        <f t="shared" si="18"/>
+        <v>19.72</v>
+      </c>
+      <c r="E276">
+        <v>8.86</v>
+      </c>
+      <c r="F276">
+        <v>17</v>
+      </c>
+      <c r="G276" s="8">
+        <v>9</v>
+      </c>
       <c r="H276" s="8"/>
-    </row>
-    <row r="277" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G277" s="8"/>
+      <c r="I276" t="s">
+        <v>110</v>
+      </c>
+      <c r="J276" t="s">
+        <v>85</v>
+      </c>
+      <c r="K276" t="s">
+        <v>77</v>
+      </c>
+      <c r="L276">
+        <v>5.43</v>
+      </c>
+      <c r="N276" s="6"/>
+    </row>
+    <row r="277" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A277" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B277" s="6">
+        <v>14.53</v>
+      </c>
+      <c r="C277">
+        <f t="shared" si="19"/>
+        <v>9.1</v>
+      </c>
+      <c r="D277">
+        <f t="shared" si="18"/>
+        <v>19.96</v>
+      </c>
+      <c r="E277">
+        <v>14.53</v>
+      </c>
+      <c r="F277">
+        <v>18</v>
+      </c>
+      <c r="G277" s="8">
+        <v>17</v>
+      </c>
       <c r="H277" s="8"/>
-    </row>
-    <row r="278" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G278" s="8"/>
+      <c r="I277" t="s">
+        <v>110</v>
+      </c>
+      <c r="J277" t="s">
+        <v>85</v>
+      </c>
+      <c r="K277" t="s">
+        <v>77</v>
+      </c>
+      <c r="L277">
+        <v>5.43</v>
+      </c>
+      <c r="N277" s="6"/>
+    </row>
+    <row r="278" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A278" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B278" s="6">
+        <v>14.84</v>
+      </c>
+      <c r="C278">
+        <f t="shared" si="19"/>
+        <v>9.41</v>
+      </c>
+      <c r="D278">
+        <f t="shared" si="18"/>
+        <v>20.27</v>
+      </c>
+      <c r="E278">
+        <v>14.84</v>
+      </c>
+      <c r="F278">
+        <v>19</v>
+      </c>
+      <c r="G278" s="8">
+        <v>19</v>
+      </c>
       <c r="H278" s="8"/>
-    </row>
-    <row r="279" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G279" s="8"/>
+      <c r="I278" t="s">
+        <v>110</v>
+      </c>
+      <c r="J278" t="s">
+        <v>85</v>
+      </c>
+      <c r="K278" t="s">
+        <v>77</v>
+      </c>
+      <c r="L278">
+        <v>5.43</v>
+      </c>
+      <c r="N278" s="6"/>
+    </row>
+    <row r="279" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A279" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B279" s="6">
+        <v>15.58</v>
+      </c>
+      <c r="C279">
+        <f t="shared" si="19"/>
+        <v>10.15</v>
+      </c>
+      <c r="D279">
+        <f t="shared" si="18"/>
+        <v>21.009999999999998</v>
+      </c>
+      <c r="E279">
+        <v>15.58</v>
+      </c>
+      <c r="F279">
+        <v>20</v>
+      </c>
+      <c r="G279" s="8">
+        <v>20</v>
+      </c>
       <c r="H279" s="8"/>
-    </row>
-    <row r="280" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G280" s="8"/>
+      <c r="I279" t="s">
+        <v>110</v>
+      </c>
+      <c r="J279" t="s">
+        <v>85</v>
+      </c>
+      <c r="K279" t="s">
+        <v>77</v>
+      </c>
+      <c r="L279">
+        <v>5.43</v>
+      </c>
+      <c r="N279" s="6"/>
+    </row>
+    <row r="280" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A280" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B280" s="6">
+        <v>15.82</v>
+      </c>
+      <c r="C280">
+        <f t="shared" si="19"/>
+        <v>10.39</v>
+      </c>
+      <c r="D280">
+        <f t="shared" si="18"/>
+        <v>21.25</v>
+      </c>
+      <c r="E280">
+        <v>15.82</v>
+      </c>
+      <c r="F280">
+        <v>21</v>
+      </c>
+      <c r="G280" s="8">
+        <v>21</v>
+      </c>
       <c r="H280" s="8"/>
-    </row>
-    <row r="281" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G281" s="8"/>
+      <c r="I280" t="s">
+        <v>110</v>
+      </c>
+      <c r="J280" t="s">
+        <v>85</v>
+      </c>
+      <c r="K280" t="s">
+        <v>77</v>
+      </c>
+      <c r="L280">
+        <v>5.43</v>
+      </c>
+      <c r="N280" s="6"/>
+    </row>
+    <row r="281" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A281" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B281" s="6">
+        <v>16.52</v>
+      </c>
+      <c r="C281">
+        <f t="shared" si="19"/>
+        <v>11.09</v>
+      </c>
+      <c r="D281">
+        <f t="shared" si="18"/>
+        <v>21.95</v>
+      </c>
+      <c r="E281">
+        <v>21.95</v>
+      </c>
+      <c r="F281">
+        <v>22</v>
+      </c>
+      <c r="G281" s="8">
+        <v>24</v>
+      </c>
       <c r="H281" s="8"/>
-    </row>
-    <row r="282" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G282" s="8"/>
+      <c r="I281" t="s">
+        <v>110</v>
+      </c>
+      <c r="J281" t="s">
+        <v>85</v>
+      </c>
+      <c r="K281" t="s">
+        <v>77</v>
+      </c>
+      <c r="L281">
+        <v>5.43</v>
+      </c>
+      <c r="N281" s="6"/>
+    </row>
+    <row r="282" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A282" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B282" s="6">
+        <v>16.690000000000001</v>
+      </c>
+      <c r="C282">
+        <f t="shared" si="19"/>
+        <v>11.260000000000002</v>
+      </c>
+      <c r="D282">
+        <f t="shared" si="18"/>
+        <v>22.12</v>
+      </c>
+      <c r="E282">
+        <v>16.690000000000001</v>
+      </c>
+      <c r="F282">
+        <v>23</v>
+      </c>
+      <c r="G282" s="8">
+        <v>22</v>
+      </c>
       <c r="H282" s="8"/>
-    </row>
-    <row r="283" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G283" s="8"/>
+      <c r="I282" t="s">
+        <v>110</v>
+      </c>
+      <c r="J282" t="s">
+        <v>85</v>
+      </c>
+      <c r="K282" t="s">
+        <v>77</v>
+      </c>
+      <c r="L282">
+        <v>5.43</v>
+      </c>
+      <c r="N282" s="6"/>
+    </row>
+    <row r="283" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A283" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B283" s="6">
+        <v>16.97</v>
+      </c>
+      <c r="C283">
+        <f t="shared" si="19"/>
+        <v>11.54</v>
+      </c>
+      <c r="D283">
+        <f t="shared" si="18"/>
+        <v>22.4</v>
+      </c>
+      <c r="E283">
+        <v>11.54</v>
+      </c>
+      <c r="F283">
+        <v>24</v>
+      </c>
+      <c r="G283" s="8">
+        <v>15</v>
+      </c>
       <c r="H283" s="8"/>
-    </row>
-    <row r="284" spans="7:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="G284" s="8"/>
+      <c r="I283" t="s">
+        <v>110</v>
+      </c>
+      <c r="J283" t="s">
+        <v>85</v>
+      </c>
+      <c r="K283" t="s">
+        <v>77</v>
+      </c>
+      <c r="L283">
+        <v>5.43</v>
+      </c>
+      <c r="N283" s="6"/>
+    </row>
+    <row r="284" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A284" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B284" s="6">
+        <v>17.149999999999999</v>
+      </c>
+      <c r="C284">
+        <f t="shared" si="19"/>
+        <v>11.719999999999999</v>
+      </c>
+      <c r="D284">
+        <f t="shared" si="18"/>
+        <v>22.58</v>
+      </c>
+      <c r="E284">
+        <v>22.58</v>
+      </c>
+      <c r="F284">
+        <v>25</v>
+      </c>
+      <c r="G284" s="8">
+        <v>25</v>
+      </c>
       <c r="H284" s="8"/>
-    </row>
-    <row r="285" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="I284" t="s">
+        <v>110</v>
+      </c>
+      <c r="J284" t="s">
+        <v>85</v>
+      </c>
+      <c r="K284" t="s">
+        <v>77</v>
+      </c>
+      <c r="L284">
+        <v>5.43</v>
+      </c>
+      <c r="N284" s="6"/>
+    </row>
+    <row r="285" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="G285" s="8"/>
       <c r="H285" s="8"/>
     </row>
-    <row r="286" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="286" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="G286" s="8"/>
       <c r="H286" s="8"/>
     </row>
-    <row r="287" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="287" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="G287" s="8"/>
       <c r="H287" s="8"/>
     </row>
-    <row r="288" spans="7:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="288" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="G288" s="8"/>
       <c r="H288" s="8"/>
     </row>
@@ -13225,8 +14558,8 @@
       <c r="H357" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N209:O233">
-    <sortCondition ref="O209:O233"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N260:O284">
+    <sortCondition ref="O260:O284"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13239,13 +14572,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O234"/>
+  <dimension ref="A1:O259"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="18.3671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.47265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.05078125" customWidth="1"/>
-    <col min="5" max="5" width="10.68359375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.47265625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="8.05078125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="0" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="10.68359375" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="9.47265625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.89453125" customWidth="1"/>
     <col min="8" max="8" width="10.3125" bestFit="1" customWidth="1"/>
@@ -22926,9 +24260,984 @@
       <c r="N234" s="6"/>
       <c r="O234" s="5"/>
     </row>
+    <row r="235" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A235" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B235" s="6">
+        <v>8.65</v>
+      </c>
+      <c r="C235" s="5">
+        <f>B235-L235</f>
+        <v>3.5600000000000005</v>
+      </c>
+      <c r="D235" s="5">
+        <f>B235+L235</f>
+        <v>13.74</v>
+      </c>
+      <c r="E235" s="5">
+        <v>8.65</v>
+      </c>
+      <c r="F235">
+        <v>1</v>
+      </c>
+      <c r="G235" s="8">
+        <v>6</v>
+      </c>
+      <c r="I235" t="s">
+        <v>109</v>
+      </c>
+      <c r="J235" t="s">
+        <v>85</v>
+      </c>
+      <c r="K235" t="s">
+        <v>86</v>
+      </c>
+      <c r="L235" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N235" s="6"/>
+      <c r="O235" s="5"/>
+    </row>
+    <row r="236" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A236" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B236" s="6">
+        <v>8.69</v>
+      </c>
+      <c r="C236" s="5">
+        <f t="shared" ref="C236:C259" si="17">B236-L236</f>
+        <v>3.5999999999999996</v>
+      </c>
+      <c r="D236" s="5">
+        <f t="shared" ref="D236:D259" si="18">B236+L236</f>
+        <v>13.78</v>
+      </c>
+      <c r="E236" s="5">
+        <v>3.6</v>
+      </c>
+      <c r="F236">
+        <v>2</v>
+      </c>
+      <c r="G236" s="8">
+        <v>1</v>
+      </c>
+      <c r="I236" t="s">
+        <v>109</v>
+      </c>
+      <c r="J236" t="s">
+        <v>85</v>
+      </c>
+      <c r="K236" t="s">
+        <v>86</v>
+      </c>
+      <c r="L236" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N236" s="6"/>
+      <c r="O236" s="5"/>
+    </row>
+    <row r="237" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A237" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B237" s="6">
+        <v>8.85</v>
+      </c>
+      <c r="C237" s="5">
+        <f t="shared" si="17"/>
+        <v>3.76</v>
+      </c>
+      <c r="D237" s="5">
+        <f t="shared" si="18"/>
+        <v>13.94</v>
+      </c>
+      <c r="E237" s="5">
+        <v>3.76</v>
+      </c>
+      <c r="F237">
+        <v>3</v>
+      </c>
+      <c r="G237" s="8">
+        <v>2</v>
+      </c>
+      <c r="I237" t="s">
+        <v>109</v>
+      </c>
+      <c r="J237" t="s">
+        <v>85</v>
+      </c>
+      <c r="K237" t="s">
+        <v>86</v>
+      </c>
+      <c r="L237" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N237" s="6"/>
+      <c r="O237" s="5"/>
+    </row>
+    <row r="238" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A238" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B238" s="6">
+        <v>9.5</v>
+      </c>
+      <c r="C238" s="5">
+        <f t="shared" si="17"/>
+        <v>4.41</v>
+      </c>
+      <c r="D238" s="5">
+        <f t="shared" si="18"/>
+        <v>14.59</v>
+      </c>
+      <c r="E238" s="5">
+        <v>9.5</v>
+      </c>
+      <c r="F238">
+        <v>4</v>
+      </c>
+      <c r="G238" s="8">
+        <v>7</v>
+      </c>
+      <c r="I238" t="s">
+        <v>109</v>
+      </c>
+      <c r="J238" t="s">
+        <v>85</v>
+      </c>
+      <c r="K238" t="s">
+        <v>86</v>
+      </c>
+      <c r="L238" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N238" s="6"/>
+      <c r="O238" s="5"/>
+    </row>
+    <row r="239" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A239" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B239" s="6">
+        <v>11.32</v>
+      </c>
+      <c r="C239" s="5">
+        <f t="shared" si="17"/>
+        <v>6.23</v>
+      </c>
+      <c r="D239" s="5">
+        <f t="shared" si="18"/>
+        <v>16.41</v>
+      </c>
+      <c r="E239" s="5">
+        <v>11.32</v>
+      </c>
+      <c r="F239">
+        <v>5</v>
+      </c>
+      <c r="G239" s="8">
+        <v>10</v>
+      </c>
+      <c r="I239" t="s">
+        <v>109</v>
+      </c>
+      <c r="J239" t="s">
+        <v>85</v>
+      </c>
+      <c r="K239" t="s">
+        <v>86</v>
+      </c>
+      <c r="L239" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N239" s="6"/>
+      <c r="O239" s="5"/>
+    </row>
+    <row r="240" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A240" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B240" s="6">
+        <v>11.42</v>
+      </c>
+      <c r="C240" s="5">
+        <f t="shared" si="17"/>
+        <v>6.33</v>
+      </c>
+      <c r="D240" s="5">
+        <f t="shared" si="18"/>
+        <v>16.509999999999998</v>
+      </c>
+      <c r="E240" s="5">
+        <v>6.33</v>
+      </c>
+      <c r="F240">
+        <v>6</v>
+      </c>
+      <c r="G240" s="8">
+        <v>3</v>
+      </c>
+      <c r="I240" t="s">
+        <v>109</v>
+      </c>
+      <c r="J240" t="s">
+        <v>85</v>
+      </c>
+      <c r="K240" t="s">
+        <v>86</v>
+      </c>
+      <c r="L240" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N240" s="6"/>
+      <c r="O240" s="5"/>
+    </row>
+    <row r="241" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A241" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B241" s="6">
+        <v>11.42</v>
+      </c>
+      <c r="C241" s="5">
+        <f t="shared" si="17"/>
+        <v>6.33</v>
+      </c>
+      <c r="D241" s="5">
+        <f t="shared" si="18"/>
+        <v>16.509999999999998</v>
+      </c>
+      <c r="E241" s="5">
+        <v>11.42</v>
+      </c>
+      <c r="F241">
+        <v>7</v>
+      </c>
+      <c r="G241" s="8">
+        <v>11</v>
+      </c>
+      <c r="I241" t="s">
+        <v>109</v>
+      </c>
+      <c r="J241" t="s">
+        <v>85</v>
+      </c>
+      <c r="K241" t="s">
+        <v>86</v>
+      </c>
+      <c r="L241" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N241" s="6"/>
+      <c r="O241" s="5"/>
+    </row>
+    <row r="242" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A242" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B242" s="6">
+        <v>11.69</v>
+      </c>
+      <c r="C242" s="5">
+        <f t="shared" si="17"/>
+        <v>6.6</v>
+      </c>
+      <c r="D242" s="5">
+        <f t="shared" si="18"/>
+        <v>16.78</v>
+      </c>
+      <c r="E242" s="5">
+        <v>11.69</v>
+      </c>
+      <c r="F242">
+        <v>8</v>
+      </c>
+      <c r="G242" s="8">
+        <v>12</v>
+      </c>
+      <c r="I242" t="s">
+        <v>109</v>
+      </c>
+      <c r="J242" t="s">
+        <v>85</v>
+      </c>
+      <c r="K242" t="s">
+        <v>86</v>
+      </c>
+      <c r="L242" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N242" s="6"/>
+      <c r="O242" s="5"/>
+    </row>
+    <row r="243" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A243" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B243" s="6">
+        <v>11.79</v>
+      </c>
+      <c r="C243" s="5">
+        <f t="shared" si="17"/>
+        <v>6.6999999999999993</v>
+      </c>
+      <c r="D243" s="5">
+        <f t="shared" si="18"/>
+        <v>16.88</v>
+      </c>
+      <c r="E243" s="5">
+        <v>6.7</v>
+      </c>
+      <c r="F243">
+        <v>9</v>
+      </c>
+      <c r="G243" s="8">
+        <v>4</v>
+      </c>
+      <c r="I243" t="s">
+        <v>109</v>
+      </c>
+      <c r="J243" t="s">
+        <v>85</v>
+      </c>
+      <c r="K243" t="s">
+        <v>86</v>
+      </c>
+      <c r="L243" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N243" s="6"/>
+      <c r="O243" s="5"/>
+    </row>
+    <row r="244" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A244" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B244" s="6">
+        <v>12.28</v>
+      </c>
+      <c r="C244" s="5">
+        <f t="shared" si="17"/>
+        <v>7.1899999999999995</v>
+      </c>
+      <c r="D244" s="5">
+        <f t="shared" si="18"/>
+        <v>17.369999999999997</v>
+      </c>
+      <c r="E244" s="5">
+        <v>12.28</v>
+      </c>
+      <c r="F244">
+        <v>10</v>
+      </c>
+      <c r="G244" s="8">
+        <v>13</v>
+      </c>
+      <c r="I244" t="s">
+        <v>109</v>
+      </c>
+      <c r="J244" t="s">
+        <v>85</v>
+      </c>
+      <c r="K244" t="s">
+        <v>86</v>
+      </c>
+      <c r="L244" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N244" s="6"/>
+      <c r="O244" s="5"/>
+    </row>
+    <row r="245" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A245" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B245" s="6">
+        <v>12.53</v>
+      </c>
+      <c r="C245" s="5">
+        <f t="shared" si="17"/>
+        <v>7.4399999999999995</v>
+      </c>
+      <c r="D245" s="5">
+        <f t="shared" si="18"/>
+        <v>17.619999999999997</v>
+      </c>
+      <c r="E245" s="5">
+        <v>12.53</v>
+      </c>
+      <c r="F245">
+        <v>11</v>
+      </c>
+      <c r="G245" s="8">
+        <v>14</v>
+      </c>
+      <c r="I245" t="s">
+        <v>109</v>
+      </c>
+      <c r="J245" t="s">
+        <v>85</v>
+      </c>
+      <c r="K245" t="s">
+        <v>86</v>
+      </c>
+      <c r="L245" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N245" s="6"/>
+      <c r="O245" s="5"/>
+    </row>
+    <row r="246" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A246" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B246" s="6">
+        <v>13.39</v>
+      </c>
+      <c r="C246" s="5">
+        <f t="shared" si="17"/>
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="D246" s="5">
+        <f t="shared" si="18"/>
+        <v>18.48</v>
+      </c>
+      <c r="E246" s="5">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="F246">
+        <v>12</v>
+      </c>
+      <c r="G246" s="8">
+        <v>5</v>
+      </c>
+      <c r="I246" t="s">
+        <v>109</v>
+      </c>
+      <c r="J246" t="s">
+        <v>85</v>
+      </c>
+      <c r="K246" t="s">
+        <v>86</v>
+      </c>
+      <c r="L246" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N246" s="6"/>
+      <c r="O246" s="5"/>
+    </row>
+    <row r="247" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A247" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B247" s="6">
+        <v>13.5</v>
+      </c>
+      <c r="C247" s="5">
+        <f t="shared" si="17"/>
+        <v>8.41</v>
+      </c>
+      <c r="D247" s="5">
+        <f t="shared" si="18"/>
+        <v>18.59</v>
+      </c>
+      <c r="E247" s="5">
+        <v>13.5</v>
+      </c>
+      <c r="F247">
+        <v>13</v>
+      </c>
+      <c r="G247" s="8">
+        <v>15</v>
+      </c>
+      <c r="I247" t="s">
+        <v>109</v>
+      </c>
+      <c r="J247" t="s">
+        <v>85</v>
+      </c>
+      <c r="K247" t="s">
+        <v>86</v>
+      </c>
+      <c r="L247" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N247" s="6"/>
+      <c r="O247" s="5"/>
+    </row>
+    <row r="248" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A248" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B248" s="6">
+        <v>13.8</v>
+      </c>
+      <c r="C248" s="5">
+        <f t="shared" si="17"/>
+        <v>8.7100000000000009</v>
+      </c>
+      <c r="D248" s="5">
+        <f t="shared" si="18"/>
+        <v>18.89</v>
+      </c>
+      <c r="E248" s="5">
+        <v>13.8</v>
+      </c>
+      <c r="F248">
+        <v>14</v>
+      </c>
+      <c r="G248" s="8">
+        <v>16</v>
+      </c>
+      <c r="I248" t="s">
+        <v>109</v>
+      </c>
+      <c r="J248" t="s">
+        <v>85</v>
+      </c>
+      <c r="K248" t="s">
+        <v>86</v>
+      </c>
+      <c r="L248" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N248" s="6"/>
+      <c r="O248" s="5"/>
+    </row>
+    <row r="249" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A249" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B249" s="6">
+        <v>14.3</v>
+      </c>
+      <c r="C249" s="5">
+        <f t="shared" si="17"/>
+        <v>9.2100000000000009</v>
+      </c>
+      <c r="D249" s="5">
+        <f t="shared" si="18"/>
+        <v>19.39</v>
+      </c>
+      <c r="E249" s="5">
+        <v>19.39</v>
+      </c>
+      <c r="F249">
+        <v>15</v>
+      </c>
+      <c r="G249" s="8">
+        <v>20</v>
+      </c>
+      <c r="I249" t="s">
+        <v>109</v>
+      </c>
+      <c r="J249" t="s">
+        <v>85</v>
+      </c>
+      <c r="K249" t="s">
+        <v>86</v>
+      </c>
+      <c r="L249" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N249" s="6"/>
+      <c r="O249" s="5"/>
+    </row>
+    <row r="250" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A250" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B250" s="6">
+        <v>14.41</v>
+      </c>
+      <c r="C250" s="5">
+        <f t="shared" si="17"/>
+        <v>9.32</v>
+      </c>
+      <c r="D250" s="5">
+        <f t="shared" si="18"/>
+        <v>19.5</v>
+      </c>
+      <c r="E250" s="5">
+        <v>19.5</v>
+      </c>
+      <c r="F250">
+        <v>16</v>
+      </c>
+      <c r="G250" s="8">
+        <v>21</v>
+      </c>
+      <c r="I250" t="s">
+        <v>109</v>
+      </c>
+      <c r="J250" t="s">
+        <v>85</v>
+      </c>
+      <c r="K250" t="s">
+        <v>86</v>
+      </c>
+      <c r="L250" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N250" s="6"/>
+      <c r="O250" s="5"/>
+    </row>
+    <row r="251" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A251" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B251" s="6">
+        <v>14.42</v>
+      </c>
+      <c r="C251" s="5">
+        <f t="shared" si="17"/>
+        <v>9.33</v>
+      </c>
+      <c r="D251" s="5">
+        <f t="shared" si="18"/>
+        <v>19.509999999999998</v>
+      </c>
+      <c r="E251" s="5">
+        <v>19.510000000000002</v>
+      </c>
+      <c r="F251">
+        <v>17</v>
+      </c>
+      <c r="G251" s="8">
+        <v>22</v>
+      </c>
+      <c r="I251" t="s">
+        <v>109</v>
+      </c>
+      <c r="J251" t="s">
+        <v>85</v>
+      </c>
+      <c r="K251" t="s">
+        <v>86</v>
+      </c>
+      <c r="L251" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N251" s="6"/>
+      <c r="O251" s="5"/>
+    </row>
+    <row r="252" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A252" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B252" s="6">
+        <v>14.75</v>
+      </c>
+      <c r="C252" s="5">
+        <f t="shared" si="17"/>
+        <v>9.66</v>
+      </c>
+      <c r="D252" s="5">
+        <f t="shared" si="18"/>
+        <v>19.84</v>
+      </c>
+      <c r="E252" s="5">
+        <v>9.66</v>
+      </c>
+      <c r="F252">
+        <v>18</v>
+      </c>
+      <c r="G252" s="8">
+        <v>8</v>
+      </c>
+      <c r="I252" t="s">
+        <v>109</v>
+      </c>
+      <c r="J252" t="s">
+        <v>85</v>
+      </c>
+      <c r="K252" t="s">
+        <v>86</v>
+      </c>
+      <c r="L252" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N252" s="6"/>
+      <c r="O252" s="5"/>
+    </row>
+    <row r="253" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A253" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B253" s="6">
+        <v>15.08</v>
+      </c>
+      <c r="C253" s="5">
+        <f t="shared" si="17"/>
+        <v>9.99</v>
+      </c>
+      <c r="D253" s="5">
+        <f t="shared" si="18"/>
+        <v>20.170000000000002</v>
+      </c>
+      <c r="E253" s="5">
+        <v>9.99</v>
+      </c>
+      <c r="F253">
+        <v>19</v>
+      </c>
+      <c r="G253" s="8">
+        <v>9</v>
+      </c>
+      <c r="I253" t="s">
+        <v>109</v>
+      </c>
+      <c r="J253" t="s">
+        <v>85</v>
+      </c>
+      <c r="K253" t="s">
+        <v>86</v>
+      </c>
+      <c r="L253" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N253" s="6"/>
+      <c r="O253" s="5"/>
+    </row>
+    <row r="254" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A254" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B254" s="6">
+        <v>15.15</v>
+      </c>
+      <c r="C254" s="5">
+        <f t="shared" si="17"/>
+        <v>10.06</v>
+      </c>
+      <c r="D254" s="5">
+        <f t="shared" si="18"/>
+        <v>20.240000000000002</v>
+      </c>
+      <c r="E254" s="5">
+        <v>15.15</v>
+      </c>
+      <c r="F254">
+        <v>20</v>
+      </c>
+      <c r="G254" s="8">
+        <v>17</v>
+      </c>
+      <c r="I254" t="s">
+        <v>109</v>
+      </c>
+      <c r="J254" t="s">
+        <v>85</v>
+      </c>
+      <c r="K254" t="s">
+        <v>86</v>
+      </c>
+      <c r="L254" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N254" s="6"/>
+      <c r="O254" s="5"/>
+    </row>
+    <row r="255" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A255" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B255" s="6">
+        <v>15.31</v>
+      </c>
+      <c r="C255" s="5">
+        <f t="shared" si="17"/>
+        <v>10.220000000000001</v>
+      </c>
+      <c r="D255" s="5">
+        <f t="shared" si="18"/>
+        <v>20.399999999999999</v>
+      </c>
+      <c r="E255" s="5">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="F255">
+        <v>21</v>
+      </c>
+      <c r="G255" s="8">
+        <v>23</v>
+      </c>
+      <c r="I255" t="s">
+        <v>109</v>
+      </c>
+      <c r="J255" t="s">
+        <v>85</v>
+      </c>
+      <c r="K255" t="s">
+        <v>86</v>
+      </c>
+      <c r="L255" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N255" s="6"/>
+      <c r="O255" s="5"/>
+    </row>
+    <row r="256" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A256" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B256" s="6">
+        <v>15.66</v>
+      </c>
+      <c r="C256" s="5">
+        <f t="shared" si="17"/>
+        <v>10.57</v>
+      </c>
+      <c r="D256" s="5">
+        <f t="shared" si="18"/>
+        <v>20.75</v>
+      </c>
+      <c r="E256" s="5">
+        <v>15.66</v>
+      </c>
+      <c r="F256">
+        <v>22</v>
+      </c>
+      <c r="G256" s="8">
+        <v>18</v>
+      </c>
+      <c r="I256" t="s">
+        <v>109</v>
+      </c>
+      <c r="J256" t="s">
+        <v>85</v>
+      </c>
+      <c r="K256" t="s">
+        <v>86</v>
+      </c>
+      <c r="L256" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N256" s="6"/>
+      <c r="O256" s="5"/>
+    </row>
+    <row r="257" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A257" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B257" s="6">
+        <v>16</v>
+      </c>
+      <c r="C257" s="5">
+        <f t="shared" si="17"/>
+        <v>10.91</v>
+      </c>
+      <c r="D257" s="5">
+        <f t="shared" si="18"/>
+        <v>21.09</v>
+      </c>
+      <c r="E257" s="5">
+        <v>21.09</v>
+      </c>
+      <c r="F257">
+        <v>23</v>
+      </c>
+      <c r="G257" s="8">
+        <v>24</v>
+      </c>
+      <c r="I257" t="s">
+        <v>109</v>
+      </c>
+      <c r="J257" t="s">
+        <v>85</v>
+      </c>
+      <c r="K257" t="s">
+        <v>86</v>
+      </c>
+      <c r="L257" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N257" s="6"/>
+      <c r="O257" s="5"/>
+    </row>
+    <row r="258" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A258" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B258" s="6">
+        <v>16.14</v>
+      </c>
+      <c r="C258" s="5">
+        <f t="shared" si="17"/>
+        <v>11.05</v>
+      </c>
+      <c r="D258" s="5">
+        <f t="shared" si="18"/>
+        <v>21.23</v>
+      </c>
+      <c r="E258" s="5">
+        <v>16.14</v>
+      </c>
+      <c r="F258">
+        <v>24</v>
+      </c>
+      <c r="G258" s="8">
+        <v>19</v>
+      </c>
+      <c r="I258" t="s">
+        <v>109</v>
+      </c>
+      <c r="J258" t="s">
+        <v>85</v>
+      </c>
+      <c r="K258" t="s">
+        <v>86</v>
+      </c>
+      <c r="L258" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N258" s="6"/>
+      <c r="O258" s="5"/>
+    </row>
+    <row r="259" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A259" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B259" s="6">
+        <v>16.14</v>
+      </c>
+      <c r="C259" s="5">
+        <f t="shared" si="17"/>
+        <v>11.05</v>
+      </c>
+      <c r="D259" s="5">
+        <f t="shared" si="18"/>
+        <v>21.23</v>
+      </c>
+      <c r="E259" s="5">
+        <v>21.23</v>
+      </c>
+      <c r="F259">
+        <v>25</v>
+      </c>
+      <c r="G259" s="8">
+        <v>25</v>
+      </c>
+      <c r="I259" t="s">
+        <v>109</v>
+      </c>
+      <c r="J259" t="s">
+        <v>85</v>
+      </c>
+      <c r="K259" t="s">
+        <v>86</v>
+      </c>
+      <c r="L259" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N259" s="6"/>
+      <c r="O259" s="5"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N210:O234">
-    <sortCondition ref="O210:O234"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N235:O259">
+    <sortCondition ref="O235:O259"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated Prediction Results for the IndyCar page
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08571517-CCB6-4ABB-A404-FAE52C17D7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8355DD-90BB-46F4-89E9-7603B9782255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy_Model" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2329" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2529" uniqueCount="113">
   <si>
     <t>Model</t>
   </si>
@@ -376,6 +376,12 @@
   <si>
     <t>Milwaukee Mile</t>
   </si>
+  <si>
+    <t>Milwuakee Mile (Race 1)</t>
+  </si>
+  <si>
+    <t>Milwuakee Mile (Race 2)</t>
+  </si>
 </sst>
 </file>
 
@@ -383,7 +389,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -478,7 +484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -499,6 +505,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -511,7 +521,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1089,22 +1098,22 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="12" t="s">
+      <c r="C1" s="17"/>
+      <c r="D1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="13" t="s">
+      <c r="E1" s="14"/>
+      <c r="F1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13" t="s">
+      <c r="G1" s="15"/>
+      <c r="H1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="13"/>
+      <c r="I1" s="15"/>
       <c r="J1" t="s">
         <v>51</v>
       </c>
@@ -1372,22 +1381,22 @@
       <c r="A12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="12" t="s">
+      <c r="C12" s="17"/>
+      <c r="D12" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13" t="s">
+      <c r="E12" s="14"/>
+      <c r="F12" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13" t="s">
+      <c r="G12" s="15"/>
+      <c r="H12" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I12" s="13"/>
+      <c r="I12" s="15"/>
       <c r="J12" t="s">
         <v>50</v>
       </c>
@@ -1943,41 +1952,41 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="12" t="s">
+      <c r="C1" s="17"/>
+      <c r="D1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="13" t="s">
+      <c r="E1" s="14"/>
+      <c r="F1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13" t="s">
+      <c r="G1" s="15"/>
+      <c r="H1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="13"/>
+      <c r="I1" s="15"/>
       <c r="L1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="M1" s="14" t="s">
+      <c r="M1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="15"/>
-      <c r="O1" s="12" t="s">
+      <c r="N1" s="17"/>
+      <c r="O1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="13" t="s">
+      <c r="P1" s="14"/>
+      <c r="Q1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13" t="s">
+      <c r="R1" s="15"/>
+      <c r="S1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="13"/>
+      <c r="T1" s="15"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1"/>
@@ -13378,7 +13387,7 @@
         <v>8.2799999999999994</v>
       </c>
       <c r="C262">
-        <f t="shared" ref="C261:C284" si="19">B262-L262</f>
+        <f t="shared" ref="C262:C284" si="19">B262-L262</f>
         <v>2.8499999999999996</v>
       </c>
       <c r="D262">
@@ -13455,7 +13464,7 @@
       <c r="B264" s="6">
         <v>9.23</v>
       </c>
-      <c r="C264" s="16">
+      <c r="C264" s="12">
         <f t="shared" si="19"/>
         <v>3.8000000000000007</v>
       </c>
@@ -13494,7 +13503,7 @@
       <c r="B265" s="6">
         <v>9.23</v>
       </c>
-      <c r="C265" s="16">
+      <c r="C265" s="12">
         <f t="shared" si="19"/>
         <v>3.8000000000000007</v>
       </c>
@@ -14572,14 +14581,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O259"/>
+  <dimension ref="A1:O309"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="18.3671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.47265625" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="8.05078125" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="0" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.68359375" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="8.47265625" customWidth="1"/>
+    <col min="3" max="3" width="8.05078125" customWidth="1"/>
+    <col min="4" max="4" width="8.83984375" customWidth="1"/>
+    <col min="5" max="5" width="10.68359375" customWidth="1"/>
     <col min="6" max="6" width="9.47265625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.89453125" customWidth="1"/>
     <col min="8" max="8" width="10.3125" bestFit="1" customWidth="1"/>
@@ -23309,6 +23318,9 @@
       <c r="G210" s="8">
         <v>1</v>
       </c>
+      <c r="H210" s="8">
+        <v>7</v>
+      </c>
       <c r="I210" t="s">
         <v>108</v>
       </c>
@@ -23348,6 +23360,9 @@
       <c r="G211" s="8">
         <v>2</v>
       </c>
+      <c r="H211" s="8">
+        <v>17</v>
+      </c>
       <c r="I211" t="s">
         <v>108</v>
       </c>
@@ -23387,6 +23402,9 @@
       <c r="G212" s="8">
         <v>5</v>
       </c>
+      <c r="H212" s="8">
+        <v>12</v>
+      </c>
       <c r="I212" t="s">
         <v>108</v>
       </c>
@@ -23426,6 +23444,9 @@
       <c r="G213" s="8">
         <v>7</v>
       </c>
+      <c r="H213" s="8">
+        <v>5</v>
+      </c>
       <c r="I213" t="s">
         <v>108</v>
       </c>
@@ -23465,6 +23486,9 @@
       <c r="G214" s="8">
         <v>8</v>
       </c>
+      <c r="H214" s="8">
+        <v>1</v>
+      </c>
       <c r="I214" t="s">
         <v>108</v>
       </c>
@@ -23504,6 +23528,9 @@
       <c r="G215" s="8">
         <v>9</v>
       </c>
+      <c r="H215" s="8">
+        <v>14</v>
+      </c>
       <c r="I215" t="s">
         <v>108</v>
       </c>
@@ -23543,6 +23570,9 @@
       <c r="G216" s="8">
         <v>10</v>
       </c>
+      <c r="H216" s="8">
+        <v>6</v>
+      </c>
       <c r="I216" t="s">
         <v>108</v>
       </c>
@@ -23582,6 +23612,9 @@
       <c r="G217" s="8">
         <v>3</v>
       </c>
+      <c r="H217" s="8">
+        <v>11</v>
+      </c>
       <c r="I217" t="s">
         <v>108</v>
       </c>
@@ -23621,6 +23654,9 @@
       <c r="G218" s="8">
         <v>4</v>
       </c>
+      <c r="H218" s="8">
+        <v>9</v>
+      </c>
       <c r="I218" t="s">
         <v>108</v>
       </c>
@@ -23660,6 +23696,9 @@
       <c r="G219" s="8">
         <v>12</v>
       </c>
+      <c r="H219" s="8">
+        <v>13</v>
+      </c>
       <c r="I219" t="s">
         <v>108</v>
       </c>
@@ -23699,6 +23738,9 @@
       <c r="G220">
         <v>13</v>
       </c>
+      <c r="H220" s="8">
+        <v>18</v>
+      </c>
       <c r="I220" t="s">
         <v>108</v>
       </c>
@@ -23738,6 +23780,9 @@
       <c r="G221" s="8">
         <v>21</v>
       </c>
+      <c r="H221" s="8">
+        <v>10</v>
+      </c>
       <c r="I221" t="s">
         <v>108</v>
       </c>
@@ -23777,6 +23822,9 @@
       <c r="G222" s="8">
         <v>14</v>
       </c>
+      <c r="H222" s="8">
+        <v>4</v>
+      </c>
       <c r="I222" t="s">
         <v>108</v>
       </c>
@@ -23816,6 +23864,9 @@
       <c r="G223" s="8">
         <v>22</v>
       </c>
+      <c r="H223" s="8">
+        <v>21</v>
+      </c>
       <c r="I223" t="s">
         <v>108</v>
       </c>
@@ -23855,6 +23906,9 @@
       <c r="G224" s="8">
         <v>15</v>
       </c>
+      <c r="H224" s="8">
+        <v>23</v>
+      </c>
       <c r="I224" t="s">
         <v>108</v>
       </c>
@@ -23894,6 +23948,9 @@
       <c r="G225" s="8">
         <v>6</v>
       </c>
+      <c r="H225" s="8">
+        <v>3</v>
+      </c>
       <c r="I225" t="s">
         <v>108</v>
       </c>
@@ -23933,6 +23990,9 @@
       <c r="G226" s="8">
         <v>16</v>
       </c>
+      <c r="H226" s="8">
+        <v>8</v>
+      </c>
       <c r="I226" t="s">
         <v>108</v>
       </c>
@@ -23972,6 +24032,9 @@
       <c r="G227" s="8">
         <v>17</v>
       </c>
+      <c r="H227" s="8">
+        <v>2</v>
+      </c>
       <c r="I227" t="s">
         <v>108</v>
       </c>
@@ -24011,6 +24074,9 @@
       <c r="G228" s="8">
         <v>23</v>
       </c>
+      <c r="H228" s="8">
+        <v>20</v>
+      </c>
       <c r="I228" t="s">
         <v>108</v>
       </c>
@@ -24050,6 +24116,9 @@
       <c r="G229" s="8">
         <v>18</v>
       </c>
+      <c r="H229" s="8">
+        <v>16</v>
+      </c>
       <c r="I229" t="s">
         <v>108</v>
       </c>
@@ -24089,6 +24158,9 @@
       <c r="G230" s="8">
         <v>19</v>
       </c>
+      <c r="H230" s="8">
+        <v>24</v>
+      </c>
       <c r="I230" t="s">
         <v>108</v>
       </c>
@@ -24128,6 +24200,9 @@
       <c r="G231" s="8">
         <v>11</v>
       </c>
+      <c r="H231" s="8">
+        <v>22</v>
+      </c>
       <c r="I231" t="s">
         <v>108</v>
       </c>
@@ -24167,6 +24242,9 @@
       <c r="G232" s="8">
         <v>24</v>
       </c>
+      <c r="H232" s="8">
+        <v>19</v>
+      </c>
       <c r="I232" t="s">
         <v>108</v>
       </c>
@@ -24206,6 +24284,9 @@
       <c r="G233" s="8">
         <v>20</v>
       </c>
+      <c r="H233" s="8">
+        <v>15</v>
+      </c>
       <c r="I233" t="s">
         <v>108</v>
       </c>
@@ -24245,6 +24326,9 @@
       <c r="G234" s="8">
         <v>25</v>
       </c>
+      <c r="H234" s="8">
+        <v>25</v>
+      </c>
       <c r="I234" t="s">
         <v>108</v>
       </c>
@@ -24284,6 +24368,9 @@
       <c r="G235" s="8">
         <v>6</v>
       </c>
+      <c r="H235" s="8">
+        <v>4</v>
+      </c>
       <c r="I235" t="s">
         <v>109</v>
       </c>
@@ -24323,6 +24410,9 @@
       <c r="G236" s="8">
         <v>1</v>
       </c>
+      <c r="H236" s="8">
+        <v>2</v>
+      </c>
       <c r="I236" t="s">
         <v>109</v>
       </c>
@@ -24362,6 +24452,9 @@
       <c r="G237" s="8">
         <v>2</v>
       </c>
+      <c r="H237" s="8">
+        <v>10</v>
+      </c>
       <c r="I237" t="s">
         <v>109</v>
       </c>
@@ -24401,6 +24494,9 @@
       <c r="G238" s="8">
         <v>7</v>
       </c>
+      <c r="H238" s="8">
+        <v>1</v>
+      </c>
       <c r="I238" t="s">
         <v>109</v>
       </c>
@@ -24440,6 +24536,9 @@
       <c r="G239" s="8">
         <v>10</v>
       </c>
+      <c r="H239" s="8">
+        <v>18</v>
+      </c>
       <c r="I239" t="s">
         <v>109</v>
       </c>
@@ -24479,6 +24578,9 @@
       <c r="G240" s="8">
         <v>3</v>
       </c>
+      <c r="H240" s="8">
+        <v>22</v>
+      </c>
       <c r="I240" t="s">
         <v>109</v>
       </c>
@@ -24518,6 +24620,9 @@
       <c r="G241" s="8">
         <v>11</v>
       </c>
+      <c r="H241" s="8">
+        <v>23</v>
+      </c>
       <c r="I241" t="s">
         <v>109</v>
       </c>
@@ -24557,6 +24662,9 @@
       <c r="G242" s="8">
         <v>12</v>
       </c>
+      <c r="H242" s="8">
+        <v>13</v>
+      </c>
       <c r="I242" t="s">
         <v>109</v>
       </c>
@@ -24596,6 +24704,9 @@
       <c r="G243" s="8">
         <v>4</v>
       </c>
+      <c r="H243" s="8">
+        <v>7</v>
+      </c>
       <c r="I243" t="s">
         <v>109</v>
       </c>
@@ -24635,6 +24746,9 @@
       <c r="G244" s="8">
         <v>13</v>
       </c>
+      <c r="H244" s="8">
+        <v>24</v>
+      </c>
       <c r="I244" t="s">
         <v>109</v>
       </c>
@@ -24674,6 +24788,9 @@
       <c r="G245" s="8">
         <v>14</v>
       </c>
+      <c r="H245" s="8">
+        <v>12</v>
+      </c>
       <c r="I245" t="s">
         <v>109</v>
       </c>
@@ -24713,6 +24830,9 @@
       <c r="G246" s="8">
         <v>5</v>
       </c>
+      <c r="H246" s="8">
+        <v>20</v>
+      </c>
       <c r="I246" t="s">
         <v>109</v>
       </c>
@@ -24752,6 +24872,9 @@
       <c r="G247" s="8">
         <v>15</v>
       </c>
+      <c r="H247" s="8">
+        <v>5</v>
+      </c>
       <c r="I247" t="s">
         <v>109</v>
       </c>
@@ -24791,6 +24914,9 @@
       <c r="G248" s="8">
         <v>16</v>
       </c>
+      <c r="H248" s="8">
+        <v>6</v>
+      </c>
       <c r="I248" t="s">
         <v>109</v>
       </c>
@@ -24830,6 +24956,9 @@
       <c r="G249" s="8">
         <v>20</v>
       </c>
+      <c r="H249" s="8">
+        <v>9</v>
+      </c>
       <c r="I249" t="s">
         <v>109</v>
       </c>
@@ -24869,6 +24998,7 @@
       <c r="G250" s="8">
         <v>21</v>
       </c>
+      <c r="H250" s="8"/>
       <c r="I250" t="s">
         <v>109</v>
       </c>
@@ -24908,6 +25038,9 @@
       <c r="G251" s="8">
         <v>22</v>
       </c>
+      <c r="H251" s="8">
+        <v>16</v>
+      </c>
       <c r="I251" t="s">
         <v>109</v>
       </c>
@@ -24947,6 +25080,9 @@
       <c r="G252" s="8">
         <v>8</v>
       </c>
+      <c r="H252" s="8">
+        <v>3</v>
+      </c>
       <c r="I252" t="s">
         <v>109</v>
       </c>
@@ -24986,6 +25122,9 @@
       <c r="G253" s="8">
         <v>9</v>
       </c>
+      <c r="H253" s="8">
+        <v>25</v>
+      </c>
       <c r="I253" t="s">
         <v>109</v>
       </c>
@@ -25025,6 +25164,9 @@
       <c r="G254" s="8">
         <v>17</v>
       </c>
+      <c r="H254" s="8">
+        <v>11</v>
+      </c>
       <c r="I254" t="s">
         <v>109</v>
       </c>
@@ -25064,6 +25206,9 @@
       <c r="G255" s="8">
         <v>23</v>
       </c>
+      <c r="H255" s="8">
+        <v>19</v>
+      </c>
       <c r="I255" t="s">
         <v>109</v>
       </c>
@@ -25103,6 +25248,9 @@
       <c r="G256" s="8">
         <v>18</v>
       </c>
+      <c r="H256" s="8">
+        <v>17</v>
+      </c>
       <c r="I256" t="s">
         <v>109</v>
       </c>
@@ -25142,6 +25290,9 @@
       <c r="G257" s="8">
         <v>24</v>
       </c>
+      <c r="H257" s="8">
+        <v>15</v>
+      </c>
       <c r="I257" t="s">
         <v>109</v>
       </c>
@@ -25181,6 +25332,9 @@
       <c r="G258" s="8">
         <v>19</v>
       </c>
+      <c r="H258" s="8">
+        <v>14</v>
+      </c>
       <c r="I258" t="s">
         <v>109</v>
       </c>
@@ -25220,6 +25374,9 @@
       <c r="G259" s="8">
         <v>25</v>
       </c>
+      <c r="H259" s="8">
+        <v>21</v>
+      </c>
       <c r="I259" t="s">
         <v>109</v>
       </c>
@@ -25235,9 +25392,2007 @@
       <c r="N259" s="6"/>
       <c r="O259" s="5"/>
     </row>
+    <row r="260" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A260" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B260" s="6">
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="C260" s="13">
+        <f>B260-L260</f>
+        <v>3.1899999999999995</v>
+      </c>
+      <c r="D260" s="5">
+        <f>B260+L260</f>
+        <v>13.37</v>
+      </c>
+      <c r="E260" s="5">
+        <v>3.19</v>
+      </c>
+      <c r="F260">
+        <v>1</v>
+      </c>
+      <c r="G260" s="8">
+        <v>1</v>
+      </c>
+      <c r="H260" s="8"/>
+      <c r="I260" t="s">
+        <v>111</v>
+      </c>
+      <c r="J260" t="s">
+        <v>85</v>
+      </c>
+      <c r="K260" t="s">
+        <v>86</v>
+      </c>
+      <c r="L260" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N260" s="6"/>
+      <c r="O260" s="5"/>
+    </row>
+    <row r="261" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A261" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B261" s="6">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="C261" s="13">
+        <f t="shared" ref="C261:C284" si="19">B261-L261</f>
+        <v>3.2100000000000009</v>
+      </c>
+      <c r="D261" s="5">
+        <f t="shared" ref="D261:D284" si="20">B261+L261</f>
+        <v>13.39</v>
+      </c>
+      <c r="E261" s="5">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="F261">
+        <v>2</v>
+      </c>
+      <c r="G261" s="8">
+        <v>7</v>
+      </c>
+      <c r="H261" s="8"/>
+      <c r="I261" t="s">
+        <v>111</v>
+      </c>
+      <c r="J261" t="s">
+        <v>85</v>
+      </c>
+      <c r="K261" t="s">
+        <v>86</v>
+      </c>
+      <c r="L261" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N261" s="6"/>
+      <c r="O261" s="5"/>
+    </row>
+    <row r="262" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A262" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B262" s="6">
+        <v>8.31</v>
+      </c>
+      <c r="C262" s="13">
+        <f t="shared" si="19"/>
+        <v>3.2200000000000006</v>
+      </c>
+      <c r="D262" s="5">
+        <f t="shared" si="20"/>
+        <v>13.4</v>
+      </c>
+      <c r="E262" s="5">
+        <v>3.22</v>
+      </c>
+      <c r="F262">
+        <v>3</v>
+      </c>
+      <c r="G262" s="8">
+        <v>2</v>
+      </c>
+      <c r="H262" s="8"/>
+      <c r="I262" t="s">
+        <v>111</v>
+      </c>
+      <c r="J262" t="s">
+        <v>85</v>
+      </c>
+      <c r="K262" t="s">
+        <v>86</v>
+      </c>
+      <c r="L262" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N262" s="6"/>
+      <c r="O262" s="5"/>
+    </row>
+    <row r="263" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A263" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B263" s="6">
+        <v>8.57</v>
+      </c>
+      <c r="C263" s="13">
+        <f t="shared" si="19"/>
+        <v>3.4800000000000004</v>
+      </c>
+      <c r="D263" s="5">
+        <f t="shared" si="20"/>
+        <v>13.66</v>
+      </c>
+      <c r="E263" s="5">
+        <v>3.48</v>
+      </c>
+      <c r="F263">
+        <v>4</v>
+      </c>
+      <c r="G263" s="8">
+        <v>3</v>
+      </c>
+      <c r="H263" s="8"/>
+      <c r="I263" t="s">
+        <v>111</v>
+      </c>
+      <c r="J263" t="s">
+        <v>85</v>
+      </c>
+      <c r="K263" t="s">
+        <v>86</v>
+      </c>
+      <c r="L263" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N263" s="6"/>
+      <c r="O263" s="5"/>
+    </row>
+    <row r="264" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A264" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B264" s="6">
+        <v>9.68</v>
+      </c>
+      <c r="C264" s="13">
+        <f t="shared" si="19"/>
+        <v>4.59</v>
+      </c>
+      <c r="D264" s="5">
+        <f t="shared" si="20"/>
+        <v>14.77</v>
+      </c>
+      <c r="E264" s="5">
+        <v>4.59</v>
+      </c>
+      <c r="F264">
+        <v>5</v>
+      </c>
+      <c r="G264" s="8">
+        <v>4</v>
+      </c>
+      <c r="H264" s="8"/>
+      <c r="I264" t="s">
+        <v>111</v>
+      </c>
+      <c r="J264" t="s">
+        <v>85</v>
+      </c>
+      <c r="K264" t="s">
+        <v>86</v>
+      </c>
+      <c r="L264" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N264" s="6"/>
+      <c r="O264" s="5"/>
+    </row>
+    <row r="265" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A265" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B265" s="6">
+        <v>10.119999999999999</v>
+      </c>
+      <c r="C265" s="13">
+        <f t="shared" si="19"/>
+        <v>5.0299999999999994</v>
+      </c>
+      <c r="D265" s="5">
+        <f t="shared" si="20"/>
+        <v>15.209999999999999</v>
+      </c>
+      <c r="E265" s="5">
+        <v>5.03</v>
+      </c>
+      <c r="F265">
+        <v>6</v>
+      </c>
+      <c r="G265" s="8">
+        <v>5</v>
+      </c>
+      <c r="H265" s="8"/>
+      <c r="I265" t="s">
+        <v>111</v>
+      </c>
+      <c r="J265" t="s">
+        <v>85</v>
+      </c>
+      <c r="K265" t="s">
+        <v>86</v>
+      </c>
+      <c r="L265" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N265" s="6"/>
+      <c r="O265" s="5"/>
+    </row>
+    <row r="266" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A266" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B266" s="6">
+        <v>10.23</v>
+      </c>
+      <c r="C266" s="13">
+        <f t="shared" si="19"/>
+        <v>5.1400000000000006</v>
+      </c>
+      <c r="D266" s="5">
+        <f t="shared" si="20"/>
+        <v>15.32</v>
+      </c>
+      <c r="E266" s="5">
+        <v>15.32</v>
+      </c>
+      <c r="F266">
+        <v>7</v>
+      </c>
+      <c r="G266" s="8">
+        <v>18</v>
+      </c>
+      <c r="H266" s="8"/>
+      <c r="I266" t="s">
+        <v>111</v>
+      </c>
+      <c r="J266" t="s">
+        <v>85</v>
+      </c>
+      <c r="K266" t="s">
+        <v>86</v>
+      </c>
+      <c r="L266" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N266" s="6"/>
+      <c r="O266" s="5"/>
+    </row>
+    <row r="267" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A267" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B267" s="6">
+        <v>10.78</v>
+      </c>
+      <c r="C267" s="13">
+        <f t="shared" si="19"/>
+        <v>5.6899999999999995</v>
+      </c>
+      <c r="D267" s="5">
+        <f t="shared" si="20"/>
+        <v>15.87</v>
+      </c>
+      <c r="E267" s="5">
+        <v>10.78</v>
+      </c>
+      <c r="F267">
+        <v>8</v>
+      </c>
+      <c r="G267" s="8">
+        <v>9</v>
+      </c>
+      <c r="H267" s="8"/>
+      <c r="I267" t="s">
+        <v>111</v>
+      </c>
+      <c r="J267" t="s">
+        <v>85</v>
+      </c>
+      <c r="K267" t="s">
+        <v>86</v>
+      </c>
+      <c r="L267" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N267" s="6"/>
+      <c r="O267" s="5"/>
+    </row>
+    <row r="268" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A268" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B268" s="6">
+        <v>11.28</v>
+      </c>
+      <c r="C268" s="13">
+        <f t="shared" si="19"/>
+        <v>6.1899999999999995</v>
+      </c>
+      <c r="D268" s="5">
+        <f t="shared" si="20"/>
+        <v>16.369999999999997</v>
+      </c>
+      <c r="E268" s="5">
+        <v>6.19</v>
+      </c>
+      <c r="F268">
+        <v>9</v>
+      </c>
+      <c r="G268" s="8">
+        <v>6</v>
+      </c>
+      <c r="H268" s="8"/>
+      <c r="I268" t="s">
+        <v>111</v>
+      </c>
+      <c r="J268" t="s">
+        <v>85</v>
+      </c>
+      <c r="K268" t="s">
+        <v>86</v>
+      </c>
+      <c r="L268" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N268" s="6"/>
+      <c r="O268" s="5"/>
+    </row>
+    <row r="269" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A269" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B269" s="6">
+        <v>11.92</v>
+      </c>
+      <c r="C269" s="13">
+        <f t="shared" si="19"/>
+        <v>6.83</v>
+      </c>
+      <c r="D269" s="5">
+        <f t="shared" si="20"/>
+        <v>17.009999999999998</v>
+      </c>
+      <c r="E269" s="5">
+        <v>11.92</v>
+      </c>
+      <c r="F269">
+        <v>10</v>
+      </c>
+      <c r="G269" s="8">
+        <v>11</v>
+      </c>
+      <c r="H269" s="8"/>
+      <c r="I269" t="s">
+        <v>111</v>
+      </c>
+      <c r="J269" t="s">
+        <v>85</v>
+      </c>
+      <c r="K269" t="s">
+        <v>86</v>
+      </c>
+      <c r="L269" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N269" s="6"/>
+      <c r="O269" s="5"/>
+    </row>
+    <row r="270" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A270" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B270" s="6">
+        <v>12.16</v>
+      </c>
+      <c r="C270" s="13">
+        <f t="shared" si="19"/>
+        <v>7.07</v>
+      </c>
+      <c r="D270" s="5">
+        <f t="shared" si="20"/>
+        <v>17.25</v>
+      </c>
+      <c r="E270" s="5">
+        <v>12.16</v>
+      </c>
+      <c r="F270">
+        <v>11</v>
+      </c>
+      <c r="G270" s="8">
+        <v>13</v>
+      </c>
+      <c r="H270" s="8"/>
+      <c r="I270" t="s">
+        <v>111</v>
+      </c>
+      <c r="J270" t="s">
+        <v>85</v>
+      </c>
+      <c r="K270" t="s">
+        <v>86</v>
+      </c>
+      <c r="L270" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N270" s="6"/>
+      <c r="O270" s="5"/>
+    </row>
+    <row r="271" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A271" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B271" s="6">
+        <v>12.87</v>
+      </c>
+      <c r="C271" s="13">
+        <f t="shared" si="19"/>
+        <v>7.7799999999999994</v>
+      </c>
+      <c r="D271" s="5">
+        <f t="shared" si="20"/>
+        <v>17.96</v>
+      </c>
+      <c r="E271" s="5">
+        <v>17.96</v>
+      </c>
+      <c r="F271">
+        <v>12</v>
+      </c>
+      <c r="G271" s="8">
+        <v>21</v>
+      </c>
+      <c r="H271" s="8"/>
+      <c r="I271" t="s">
+        <v>111</v>
+      </c>
+      <c r="J271" t="s">
+        <v>85</v>
+      </c>
+      <c r="K271" t="s">
+        <v>86</v>
+      </c>
+      <c r="L271" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N271" s="6"/>
+      <c r="O271" s="5"/>
+    </row>
+    <row r="272" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A272" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B272" s="6">
+        <v>13.09</v>
+      </c>
+      <c r="C272" s="13">
+        <f t="shared" si="19"/>
+        <v>8</v>
+      </c>
+      <c r="D272" s="5">
+        <f t="shared" si="20"/>
+        <v>18.18</v>
+      </c>
+      <c r="E272" s="5">
+        <v>18.18</v>
+      </c>
+      <c r="F272">
+        <v>13</v>
+      </c>
+      <c r="G272" s="8">
+        <v>22</v>
+      </c>
+      <c r="H272" s="8"/>
+      <c r="I272" t="s">
+        <v>111</v>
+      </c>
+      <c r="J272" t="s">
+        <v>85</v>
+      </c>
+      <c r="K272" t="s">
+        <v>86</v>
+      </c>
+      <c r="L272" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N272" s="6"/>
+      <c r="O272" s="5"/>
+    </row>
+    <row r="273" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A273" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B273" s="6">
+        <v>13.67</v>
+      </c>
+      <c r="C273" s="13">
+        <f t="shared" si="19"/>
+        <v>8.58</v>
+      </c>
+      <c r="D273" s="5">
+        <f t="shared" si="20"/>
+        <v>18.759999999999998</v>
+      </c>
+      <c r="E273" s="5">
+        <v>13.67</v>
+      </c>
+      <c r="F273">
+        <v>14</v>
+      </c>
+      <c r="G273" s="8">
+        <v>14</v>
+      </c>
+      <c r="H273" s="8"/>
+      <c r="I273" t="s">
+        <v>111</v>
+      </c>
+      <c r="J273" t="s">
+        <v>85</v>
+      </c>
+      <c r="K273" t="s">
+        <v>86</v>
+      </c>
+      <c r="L273" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N273" s="6"/>
+      <c r="O273" s="5"/>
+    </row>
+    <row r="274" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A274" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B274" s="6">
+        <v>13.89</v>
+      </c>
+      <c r="C274" s="13">
+        <f t="shared" si="19"/>
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="D274" s="5">
+        <f t="shared" si="20"/>
+        <v>18.98</v>
+      </c>
+      <c r="E274" s="5">
+        <v>13.89</v>
+      </c>
+      <c r="F274">
+        <v>15</v>
+      </c>
+      <c r="G274" s="8">
+        <v>15</v>
+      </c>
+      <c r="H274" s="8"/>
+      <c r="I274" t="s">
+        <v>111</v>
+      </c>
+      <c r="J274" t="s">
+        <v>85</v>
+      </c>
+      <c r="K274" t="s">
+        <v>86</v>
+      </c>
+      <c r="L274" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N274" s="6"/>
+      <c r="O274" s="5"/>
+    </row>
+    <row r="275" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A275" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B275" s="6">
+        <v>13.92</v>
+      </c>
+      <c r="C275" s="13">
+        <f t="shared" si="19"/>
+        <v>8.83</v>
+      </c>
+      <c r="D275" s="5">
+        <f t="shared" si="20"/>
+        <v>19.009999999999998</v>
+      </c>
+      <c r="E275" s="5">
+        <v>8.83</v>
+      </c>
+      <c r="F275">
+        <v>16</v>
+      </c>
+      <c r="G275" s="8">
+        <v>8</v>
+      </c>
+      <c r="H275" s="8"/>
+      <c r="I275" t="s">
+        <v>111</v>
+      </c>
+      <c r="J275" t="s">
+        <v>85</v>
+      </c>
+      <c r="K275" t="s">
+        <v>86</v>
+      </c>
+      <c r="L275" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N275" s="6"/>
+      <c r="O275" s="5"/>
+    </row>
+    <row r="276" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A276" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B276" s="6">
+        <v>13.92</v>
+      </c>
+      <c r="C276" s="13">
+        <f t="shared" si="19"/>
+        <v>8.83</v>
+      </c>
+      <c r="D276" s="5">
+        <f t="shared" si="20"/>
+        <v>19.009999999999998</v>
+      </c>
+      <c r="E276" s="5">
+        <v>13.92</v>
+      </c>
+      <c r="F276">
+        <v>17</v>
+      </c>
+      <c r="G276" s="8">
+        <v>16</v>
+      </c>
+      <c r="H276" s="8"/>
+      <c r="I276" t="s">
+        <v>111</v>
+      </c>
+      <c r="J276" t="s">
+        <v>85</v>
+      </c>
+      <c r="K276" t="s">
+        <v>86</v>
+      </c>
+      <c r="L276" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N276" s="6"/>
+      <c r="O276" s="5"/>
+    </row>
+    <row r="277" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A277" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B277" s="6">
+        <v>14.08</v>
+      </c>
+      <c r="C277" s="13">
+        <f t="shared" si="19"/>
+        <v>8.99</v>
+      </c>
+      <c r="D277" s="5">
+        <f t="shared" si="20"/>
+        <v>19.170000000000002</v>
+      </c>
+      <c r="E277" s="5">
+        <v>19.170000000000002</v>
+      </c>
+      <c r="F277">
+        <v>18</v>
+      </c>
+      <c r="G277" s="8">
+        <v>23</v>
+      </c>
+      <c r="H277" s="8"/>
+      <c r="I277" t="s">
+        <v>111</v>
+      </c>
+      <c r="J277" t="s">
+        <v>85</v>
+      </c>
+      <c r="K277" t="s">
+        <v>86</v>
+      </c>
+      <c r="L277" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N277" s="6"/>
+      <c r="O277" s="5"/>
+    </row>
+    <row r="278" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A278" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B278" s="6">
+        <v>14.92</v>
+      </c>
+      <c r="C278" s="13">
+        <f t="shared" si="19"/>
+        <v>9.83</v>
+      </c>
+      <c r="D278" s="5">
+        <f t="shared" si="20"/>
+        <v>20.009999999999998</v>
+      </c>
+      <c r="E278" s="5">
+        <v>14.92</v>
+      </c>
+      <c r="F278">
+        <v>19</v>
+      </c>
+      <c r="G278" s="8">
+        <v>17</v>
+      </c>
+      <c r="H278" s="8"/>
+      <c r="I278" t="s">
+        <v>111</v>
+      </c>
+      <c r="J278" t="s">
+        <v>85</v>
+      </c>
+      <c r="K278" t="s">
+        <v>86</v>
+      </c>
+      <c r="L278" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N278" s="6"/>
+      <c r="O278" s="5"/>
+    </row>
+    <row r="279" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A279" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B279" s="6">
+        <v>15.33</v>
+      </c>
+      <c r="C279" s="13">
+        <f t="shared" si="19"/>
+        <v>10.24</v>
+      </c>
+      <c r="D279" s="5">
+        <f t="shared" si="20"/>
+        <v>20.420000000000002</v>
+      </c>
+      <c r="E279" s="5">
+        <v>15.33</v>
+      </c>
+      <c r="F279">
+        <v>20</v>
+      </c>
+      <c r="G279" s="8">
+        <v>19</v>
+      </c>
+      <c r="H279" s="8"/>
+      <c r="I279" t="s">
+        <v>111</v>
+      </c>
+      <c r="J279" t="s">
+        <v>85</v>
+      </c>
+      <c r="K279" t="s">
+        <v>86</v>
+      </c>
+      <c r="L279" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N279" s="6"/>
+      <c r="O279" s="5"/>
+    </row>
+    <row r="280" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A280" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B280" s="6">
+        <v>15.71</v>
+      </c>
+      <c r="C280" s="13">
+        <f t="shared" si="19"/>
+        <v>10.620000000000001</v>
+      </c>
+      <c r="D280" s="5">
+        <f t="shared" si="20"/>
+        <v>20.8</v>
+      </c>
+      <c r="E280" s="5">
+        <v>20.8</v>
+      </c>
+      <c r="F280">
+        <v>21</v>
+      </c>
+      <c r="G280" s="8">
+        <v>24</v>
+      </c>
+      <c r="H280" s="8"/>
+      <c r="I280" t="s">
+        <v>111</v>
+      </c>
+      <c r="J280" t="s">
+        <v>85</v>
+      </c>
+      <c r="K280" t="s">
+        <v>86</v>
+      </c>
+      <c r="L280" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N280" s="6"/>
+      <c r="O280" s="5"/>
+    </row>
+    <row r="281" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A281" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B281" s="6">
+        <v>15.89</v>
+      </c>
+      <c r="C281" s="13">
+        <f t="shared" si="19"/>
+        <v>10.8</v>
+      </c>
+      <c r="D281" s="5">
+        <f t="shared" si="20"/>
+        <v>20.98</v>
+      </c>
+      <c r="E281" s="5">
+        <v>10.8</v>
+      </c>
+      <c r="F281">
+        <v>22</v>
+      </c>
+      <c r="G281" s="8">
+        <v>10</v>
+      </c>
+      <c r="H281" s="8"/>
+      <c r="I281" t="s">
+        <v>111</v>
+      </c>
+      <c r="J281" t="s">
+        <v>85</v>
+      </c>
+      <c r="K281" t="s">
+        <v>86</v>
+      </c>
+      <c r="L281" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N281" s="6"/>
+      <c r="O281" s="5"/>
+    </row>
+    <row r="282" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A282" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B282" s="6">
+        <v>16.510000000000002</v>
+      </c>
+      <c r="C282" s="13">
+        <f t="shared" si="19"/>
+        <v>11.420000000000002</v>
+      </c>
+      <c r="D282" s="5">
+        <f t="shared" si="20"/>
+        <v>21.6</v>
+      </c>
+      <c r="E282" s="5">
+        <v>16.510000000000002</v>
+      </c>
+      <c r="F282">
+        <v>23</v>
+      </c>
+      <c r="G282" s="8">
+        <v>20</v>
+      </c>
+      <c r="H282" s="8"/>
+      <c r="I282" t="s">
+        <v>111</v>
+      </c>
+      <c r="J282" t="s">
+        <v>85</v>
+      </c>
+      <c r="K282" t="s">
+        <v>86</v>
+      </c>
+      <c r="L282" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N282" s="6"/>
+      <c r="O282" s="5"/>
+    </row>
+    <row r="283" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A283" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B283" s="6">
+        <v>17.23</v>
+      </c>
+      <c r="C283" s="13">
+        <f t="shared" si="19"/>
+        <v>12.14</v>
+      </c>
+      <c r="D283" s="5">
+        <f t="shared" si="20"/>
+        <v>22.32</v>
+      </c>
+      <c r="E283" s="5">
+        <v>12.14</v>
+      </c>
+      <c r="F283">
+        <v>24</v>
+      </c>
+      <c r="G283" s="8">
+        <v>12</v>
+      </c>
+      <c r="H283" s="8"/>
+      <c r="I283" t="s">
+        <v>111</v>
+      </c>
+      <c r="J283" t="s">
+        <v>85</v>
+      </c>
+      <c r="K283" t="s">
+        <v>86</v>
+      </c>
+      <c r="L283" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N283" s="6"/>
+      <c r="O283" s="5"/>
+    </row>
+    <row r="284" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A284" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B284" s="6">
+        <v>17.579999999999998</v>
+      </c>
+      <c r="C284" s="13">
+        <f t="shared" si="19"/>
+        <v>12.489999999999998</v>
+      </c>
+      <c r="D284" s="5">
+        <f t="shared" si="20"/>
+        <v>22.669999999999998</v>
+      </c>
+      <c r="E284" s="5">
+        <v>22.67</v>
+      </c>
+      <c r="F284">
+        <v>25</v>
+      </c>
+      <c r="G284" s="8">
+        <v>25</v>
+      </c>
+      <c r="H284" s="8"/>
+      <c r="I284" t="s">
+        <v>111</v>
+      </c>
+      <c r="J284" t="s">
+        <v>85</v>
+      </c>
+      <c r="K284" t="s">
+        <v>86</v>
+      </c>
+      <c r="L284" s="5">
+        <v>5.09</v>
+      </c>
+    </row>
+    <row r="285" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A285" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B285" s="6">
+        <v>6.76</v>
+      </c>
+      <c r="C285" s="5">
+        <f>B285-L285</f>
+        <v>1.67</v>
+      </c>
+      <c r="D285" s="5">
+        <f>B285+L285</f>
+        <v>11.85</v>
+      </c>
+      <c r="E285" s="5">
+        <v>6.76</v>
+      </c>
+      <c r="F285">
+        <v>1</v>
+      </c>
+      <c r="G285" s="8">
+        <v>7</v>
+      </c>
+      <c r="H285" s="8"/>
+      <c r="I285" t="s">
+        <v>112</v>
+      </c>
+      <c r="J285" t="s">
+        <v>85</v>
+      </c>
+      <c r="K285" t="s">
+        <v>86</v>
+      </c>
+      <c r="L285" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N285" s="6"/>
+      <c r="O285" s="5"/>
+    </row>
+    <row r="286" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A286" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B286" s="6">
+        <v>7.7</v>
+      </c>
+      <c r="C286" s="5">
+        <f t="shared" ref="C286:C309" si="21">B286-L286</f>
+        <v>2.6100000000000003</v>
+      </c>
+      <c r="D286" s="5">
+        <f t="shared" ref="D286:D309" si="22">B286+L286</f>
+        <v>12.79</v>
+      </c>
+      <c r="E286" s="5">
+        <v>2.61</v>
+      </c>
+      <c r="F286">
+        <v>2</v>
+      </c>
+      <c r="G286" s="8">
+        <v>1</v>
+      </c>
+      <c r="H286" s="8"/>
+      <c r="I286" t="s">
+        <v>112</v>
+      </c>
+      <c r="J286" t="s">
+        <v>85</v>
+      </c>
+      <c r="K286" t="s">
+        <v>86</v>
+      </c>
+      <c r="L286" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N286" s="6"/>
+      <c r="O286" s="5"/>
+    </row>
+    <row r="287" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A287" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B287" s="6">
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="C287" s="5">
+        <f t="shared" si="21"/>
+        <v>3.1899999999999995</v>
+      </c>
+      <c r="D287" s="5">
+        <f t="shared" si="22"/>
+        <v>13.37</v>
+      </c>
+      <c r="E287" s="5">
+        <v>3.19</v>
+      </c>
+      <c r="F287">
+        <v>3</v>
+      </c>
+      <c r="G287" s="8">
+        <v>2</v>
+      </c>
+      <c r="H287" s="8"/>
+      <c r="I287" t="s">
+        <v>112</v>
+      </c>
+      <c r="J287" t="s">
+        <v>85</v>
+      </c>
+      <c r="K287" t="s">
+        <v>86</v>
+      </c>
+      <c r="L287" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N287" s="6"/>
+      <c r="O287" s="5"/>
+    </row>
+    <row r="288" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A288" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B288" s="6">
+        <v>8.49</v>
+      </c>
+      <c r="C288" s="5">
+        <f t="shared" si="21"/>
+        <v>3.4000000000000004</v>
+      </c>
+      <c r="D288" s="5">
+        <f t="shared" si="22"/>
+        <v>13.58</v>
+      </c>
+      <c r="E288" s="5">
+        <v>3.4</v>
+      </c>
+      <c r="F288">
+        <v>4</v>
+      </c>
+      <c r="G288" s="8">
+        <v>3</v>
+      </c>
+      <c r="H288" s="8"/>
+      <c r="I288" t="s">
+        <v>112</v>
+      </c>
+      <c r="J288" t="s">
+        <v>85</v>
+      </c>
+      <c r="K288" t="s">
+        <v>86</v>
+      </c>
+      <c r="L288" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N288" s="6"/>
+      <c r="O288" s="5"/>
+    </row>
+    <row r="289" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A289" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B289" s="6">
+        <v>9.94</v>
+      </c>
+      <c r="C289" s="5">
+        <f t="shared" si="21"/>
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="D289" s="5">
+        <f t="shared" si="22"/>
+        <v>15.03</v>
+      </c>
+      <c r="E289" s="5">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="F289">
+        <v>5</v>
+      </c>
+      <c r="G289" s="8">
+        <v>4</v>
+      </c>
+      <c r="H289" s="8"/>
+      <c r="I289" t="s">
+        <v>112</v>
+      </c>
+      <c r="J289" t="s">
+        <v>85</v>
+      </c>
+      <c r="K289" t="s">
+        <v>86</v>
+      </c>
+      <c r="L289" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N289" s="6"/>
+      <c r="O289" s="5"/>
+    </row>
+    <row r="290" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A290" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B290" s="6">
+        <v>10.42</v>
+      </c>
+      <c r="C290" s="5">
+        <f t="shared" si="21"/>
+        <v>5.33</v>
+      </c>
+      <c r="D290" s="5">
+        <f t="shared" si="22"/>
+        <v>15.51</v>
+      </c>
+      <c r="E290" s="5">
+        <v>5.33</v>
+      </c>
+      <c r="F290">
+        <v>6</v>
+      </c>
+      <c r="G290" s="8">
+        <v>5</v>
+      </c>
+      <c r="H290" s="8"/>
+      <c r="I290" t="s">
+        <v>112</v>
+      </c>
+      <c r="J290" t="s">
+        <v>85</v>
+      </c>
+      <c r="K290" t="s">
+        <v>86</v>
+      </c>
+      <c r="L290" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N290" s="6"/>
+      <c r="O290" s="5"/>
+    </row>
+    <row r="291" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A291" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B291" s="6">
+        <v>10.59</v>
+      </c>
+      <c r="C291" s="5">
+        <f t="shared" si="21"/>
+        <v>5.5</v>
+      </c>
+      <c r="D291" s="5">
+        <f t="shared" si="22"/>
+        <v>15.68</v>
+      </c>
+      <c r="E291" s="5">
+        <v>10.59</v>
+      </c>
+      <c r="F291">
+        <v>7</v>
+      </c>
+      <c r="G291" s="8">
+        <v>11</v>
+      </c>
+      <c r="H291" s="8"/>
+      <c r="I291" t="s">
+        <v>112</v>
+      </c>
+      <c r="J291" t="s">
+        <v>85</v>
+      </c>
+      <c r="K291" t="s">
+        <v>86</v>
+      </c>
+      <c r="L291" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N291" s="6"/>
+      <c r="O291" s="5"/>
+    </row>
+    <row r="292" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A292" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B292" s="6">
+        <v>11.28</v>
+      </c>
+      <c r="C292" s="5">
+        <f t="shared" si="21"/>
+        <v>6.1899999999999995</v>
+      </c>
+      <c r="D292" s="5">
+        <f t="shared" si="22"/>
+        <v>16.369999999999997</v>
+      </c>
+      <c r="E292" s="5">
+        <v>6.19</v>
+      </c>
+      <c r="F292">
+        <v>8</v>
+      </c>
+      <c r="G292" s="8">
+        <v>6</v>
+      </c>
+      <c r="H292" s="8"/>
+      <c r="I292" t="s">
+        <v>112</v>
+      </c>
+      <c r="J292" t="s">
+        <v>85</v>
+      </c>
+      <c r="K292" t="s">
+        <v>86</v>
+      </c>
+      <c r="L292" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N292" s="6"/>
+      <c r="O292" s="5"/>
+    </row>
+    <row r="293" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A293" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B293" s="6">
+        <v>11.47</v>
+      </c>
+      <c r="C293" s="5">
+        <f t="shared" si="21"/>
+        <v>6.3800000000000008</v>
+      </c>
+      <c r="D293" s="5">
+        <f t="shared" si="22"/>
+        <v>16.560000000000002</v>
+      </c>
+      <c r="E293" s="5">
+        <v>11.47</v>
+      </c>
+      <c r="F293">
+        <v>9</v>
+      </c>
+      <c r="G293" s="8">
+        <v>12</v>
+      </c>
+      <c r="H293" s="8"/>
+      <c r="I293" t="s">
+        <v>112</v>
+      </c>
+      <c r="J293" t="s">
+        <v>85</v>
+      </c>
+      <c r="K293" t="s">
+        <v>86</v>
+      </c>
+      <c r="L293" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N293" s="6"/>
+      <c r="O293" s="5"/>
+    </row>
+    <row r="294" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A294" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B294" s="6">
+        <v>11.9</v>
+      </c>
+      <c r="C294" s="5">
+        <f t="shared" si="21"/>
+        <v>6.8100000000000005</v>
+      </c>
+      <c r="D294" s="5">
+        <f t="shared" si="22"/>
+        <v>16.990000000000002</v>
+      </c>
+      <c r="E294" s="5">
+        <v>6.81</v>
+      </c>
+      <c r="F294">
+        <v>10</v>
+      </c>
+      <c r="G294" s="8">
+        <v>8</v>
+      </c>
+      <c r="H294" s="8"/>
+      <c r="I294" t="s">
+        <v>112</v>
+      </c>
+      <c r="J294" t="s">
+        <v>85</v>
+      </c>
+      <c r="K294" t="s">
+        <v>86</v>
+      </c>
+      <c r="L294" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N294" s="6"/>
+      <c r="O294" s="5"/>
+    </row>
+    <row r="295" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A295" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B295" s="6">
+        <v>12.18</v>
+      </c>
+      <c r="C295" s="5">
+        <f t="shared" si="21"/>
+        <v>7.09</v>
+      </c>
+      <c r="D295" s="5">
+        <f t="shared" si="22"/>
+        <v>17.27</v>
+      </c>
+      <c r="E295" s="5">
+        <v>12.18</v>
+      </c>
+      <c r="F295">
+        <v>11</v>
+      </c>
+      <c r="G295" s="8">
+        <v>13</v>
+      </c>
+      <c r="H295" s="8"/>
+      <c r="I295" t="s">
+        <v>112</v>
+      </c>
+      <c r="J295" t="s">
+        <v>85</v>
+      </c>
+      <c r="K295" t="s">
+        <v>86</v>
+      </c>
+      <c r="L295" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N295" s="6"/>
+      <c r="O295" s="5"/>
+    </row>
+    <row r="296" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A296" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B296" s="6">
+        <v>12.33</v>
+      </c>
+      <c r="C296" s="5">
+        <f t="shared" si="21"/>
+        <v>7.24</v>
+      </c>
+      <c r="D296" s="5">
+        <f t="shared" si="22"/>
+        <v>17.420000000000002</v>
+      </c>
+      <c r="E296" s="5">
+        <v>12.33</v>
+      </c>
+      <c r="F296">
+        <v>12</v>
+      </c>
+      <c r="G296" s="8">
+        <v>14</v>
+      </c>
+      <c r="H296" s="8"/>
+      <c r="I296" t="s">
+        <v>112</v>
+      </c>
+      <c r="J296" t="s">
+        <v>85</v>
+      </c>
+      <c r="K296" t="s">
+        <v>86</v>
+      </c>
+      <c r="L296" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N296" s="6"/>
+      <c r="O296" s="5"/>
+    </row>
+    <row r="297" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A297" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B297" s="6">
+        <v>13.35</v>
+      </c>
+      <c r="C297" s="5">
+        <f t="shared" si="21"/>
+        <v>8.26</v>
+      </c>
+      <c r="D297" s="5">
+        <f t="shared" si="22"/>
+        <v>18.439999999999998</v>
+      </c>
+      <c r="E297" s="5">
+        <v>18.440000000000001</v>
+      </c>
+      <c r="F297">
+        <v>13</v>
+      </c>
+      <c r="G297" s="8">
+        <v>21</v>
+      </c>
+      <c r="H297" s="8"/>
+      <c r="I297" t="s">
+        <v>112</v>
+      </c>
+      <c r="J297" t="s">
+        <v>85</v>
+      </c>
+      <c r="K297" t="s">
+        <v>86</v>
+      </c>
+      <c r="L297" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N297" s="6"/>
+      <c r="O297" s="5"/>
+    </row>
+    <row r="298" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A298" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B298" s="6">
+        <v>13.42</v>
+      </c>
+      <c r="C298" s="5">
+        <f t="shared" si="21"/>
+        <v>8.33</v>
+      </c>
+      <c r="D298" s="5">
+        <f t="shared" si="22"/>
+        <v>18.509999999999998</v>
+      </c>
+      <c r="E298" s="5">
+        <v>13.42</v>
+      </c>
+      <c r="F298">
+        <v>14</v>
+      </c>
+      <c r="G298" s="8">
+        <v>15</v>
+      </c>
+      <c r="H298" s="8"/>
+      <c r="I298" t="s">
+        <v>112</v>
+      </c>
+      <c r="J298" t="s">
+        <v>85</v>
+      </c>
+      <c r="K298" t="s">
+        <v>86</v>
+      </c>
+      <c r="L298" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N298" s="6"/>
+      <c r="O298" s="5"/>
+    </row>
+    <row r="299" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A299" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B299" s="6">
+        <v>13.67</v>
+      </c>
+      <c r="C299" s="5">
+        <f t="shared" si="21"/>
+        <v>8.58</v>
+      </c>
+      <c r="D299" s="5">
+        <f t="shared" si="22"/>
+        <v>18.759999999999998</v>
+      </c>
+      <c r="E299" s="5">
+        <v>13.67</v>
+      </c>
+      <c r="F299">
+        <v>15</v>
+      </c>
+      <c r="G299" s="8">
+        <v>16</v>
+      </c>
+      <c r="H299" s="8"/>
+      <c r="I299" t="s">
+        <v>112</v>
+      </c>
+      <c r="J299" t="s">
+        <v>85</v>
+      </c>
+      <c r="K299" t="s">
+        <v>86</v>
+      </c>
+      <c r="L299" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N299" s="6"/>
+      <c r="O299" s="5"/>
+    </row>
+    <row r="300" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A300" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B300" s="6">
+        <v>13.89</v>
+      </c>
+      <c r="C300" s="5">
+        <f t="shared" si="21"/>
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="D300" s="5">
+        <f t="shared" si="22"/>
+        <v>18.98</v>
+      </c>
+      <c r="E300" s="5">
+        <v>18.98</v>
+      </c>
+      <c r="F300">
+        <v>16</v>
+      </c>
+      <c r="G300" s="8">
+        <v>22</v>
+      </c>
+      <c r="H300" s="8"/>
+      <c r="I300" t="s">
+        <v>112</v>
+      </c>
+      <c r="J300" t="s">
+        <v>85</v>
+      </c>
+      <c r="K300" t="s">
+        <v>86</v>
+      </c>
+      <c r="L300" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N300" s="6"/>
+      <c r="O300" s="5"/>
+    </row>
+    <row r="301" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A301" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B301" s="6">
+        <v>14.08</v>
+      </c>
+      <c r="C301" s="5">
+        <f t="shared" si="21"/>
+        <v>8.99</v>
+      </c>
+      <c r="D301" s="5">
+        <f t="shared" si="22"/>
+        <v>19.170000000000002</v>
+      </c>
+      <c r="E301" s="5">
+        <v>14.08</v>
+      </c>
+      <c r="F301">
+        <v>17</v>
+      </c>
+      <c r="G301" s="8">
+        <v>17</v>
+      </c>
+      <c r="H301" s="8"/>
+      <c r="I301" t="s">
+        <v>112</v>
+      </c>
+      <c r="J301" t="s">
+        <v>85</v>
+      </c>
+      <c r="K301" t="s">
+        <v>86</v>
+      </c>
+      <c r="L301" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N301" s="6"/>
+      <c r="O301" s="5"/>
+    </row>
+    <row r="302" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A302" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B302" s="6">
+        <v>14.12</v>
+      </c>
+      <c r="C302" s="5">
+        <f t="shared" si="21"/>
+        <v>9.0299999999999994</v>
+      </c>
+      <c r="D302" s="5">
+        <f t="shared" si="22"/>
+        <v>19.21</v>
+      </c>
+      <c r="E302" s="5">
+        <v>9.0299999999999994</v>
+      </c>
+      <c r="F302">
+        <v>18</v>
+      </c>
+      <c r="G302" s="8">
+        <v>9</v>
+      </c>
+      <c r="H302" s="8"/>
+      <c r="I302" t="s">
+        <v>112</v>
+      </c>
+      <c r="J302" t="s">
+        <v>85</v>
+      </c>
+      <c r="K302" t="s">
+        <v>86</v>
+      </c>
+      <c r="L302" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N302" s="6"/>
+      <c r="O302" s="5"/>
+    </row>
+    <row r="303" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A303" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B303" s="6">
+        <v>14.92</v>
+      </c>
+      <c r="C303" s="5">
+        <f t="shared" si="21"/>
+        <v>9.83</v>
+      </c>
+      <c r="D303" s="5">
+        <f t="shared" si="22"/>
+        <v>20.009999999999998</v>
+      </c>
+      <c r="E303" s="5">
+        <v>20.010000000000002</v>
+      </c>
+      <c r="F303">
+        <v>19</v>
+      </c>
+      <c r="G303" s="8">
+        <v>23</v>
+      </c>
+      <c r="H303" s="8"/>
+      <c r="I303" t="s">
+        <v>112</v>
+      </c>
+      <c r="J303" t="s">
+        <v>85</v>
+      </c>
+      <c r="K303" t="s">
+        <v>86</v>
+      </c>
+      <c r="L303" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N303" s="6"/>
+      <c r="O303" s="5"/>
+    </row>
+    <row r="304" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A304" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B304" s="6">
+        <v>15.62</v>
+      </c>
+      <c r="C304" s="5">
+        <f t="shared" si="21"/>
+        <v>10.53</v>
+      </c>
+      <c r="D304" s="5">
+        <f t="shared" si="22"/>
+        <v>20.71</v>
+      </c>
+      <c r="E304" s="5">
+        <v>10.53</v>
+      </c>
+      <c r="F304">
+        <v>20</v>
+      </c>
+      <c r="G304" s="8">
+        <v>10</v>
+      </c>
+      <c r="H304" s="8"/>
+      <c r="I304" t="s">
+        <v>112</v>
+      </c>
+      <c r="J304" t="s">
+        <v>85</v>
+      </c>
+      <c r="K304" t="s">
+        <v>86</v>
+      </c>
+      <c r="L304" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N304" s="6"/>
+      <c r="O304" s="5"/>
+    </row>
+    <row r="305" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A305" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B305" s="6">
+        <v>16.350000000000001</v>
+      </c>
+      <c r="C305" s="5">
+        <f t="shared" si="21"/>
+        <v>11.260000000000002</v>
+      </c>
+      <c r="D305" s="5">
+        <f t="shared" si="22"/>
+        <v>21.44</v>
+      </c>
+      <c r="E305" s="5">
+        <v>16.350000000000001</v>
+      </c>
+      <c r="F305">
+        <v>21</v>
+      </c>
+      <c r="G305" s="8">
+        <v>18</v>
+      </c>
+      <c r="H305" s="8"/>
+      <c r="I305" t="s">
+        <v>112</v>
+      </c>
+      <c r="J305" t="s">
+        <v>85</v>
+      </c>
+      <c r="K305" t="s">
+        <v>86</v>
+      </c>
+      <c r="L305" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N305" s="6"/>
+      <c r="O305" s="5"/>
+    </row>
+    <row r="306" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A306" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B306" s="6">
+        <v>16.510000000000002</v>
+      </c>
+      <c r="C306" s="5">
+        <f t="shared" si="21"/>
+        <v>11.420000000000002</v>
+      </c>
+      <c r="D306" s="5">
+        <f t="shared" si="22"/>
+        <v>21.6</v>
+      </c>
+      <c r="E306" s="5">
+        <v>16.510000000000002</v>
+      </c>
+      <c r="F306">
+        <v>22</v>
+      </c>
+      <c r="G306" s="8">
+        <v>19</v>
+      </c>
+      <c r="H306" s="8"/>
+      <c r="I306" t="s">
+        <v>112</v>
+      </c>
+      <c r="J306" t="s">
+        <v>85</v>
+      </c>
+      <c r="K306" t="s">
+        <v>86</v>
+      </c>
+      <c r="L306" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N306" s="6"/>
+      <c r="O306" s="5"/>
+    </row>
+    <row r="307" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A307" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B307" s="6">
+        <v>16.8</v>
+      </c>
+      <c r="C307" s="5">
+        <f t="shared" si="21"/>
+        <v>11.71</v>
+      </c>
+      <c r="D307" s="5">
+        <f t="shared" si="22"/>
+        <v>21.89</v>
+      </c>
+      <c r="E307" s="5">
+        <v>21.89</v>
+      </c>
+      <c r="F307">
+        <v>23</v>
+      </c>
+      <c r="G307" s="8">
+        <v>24</v>
+      </c>
+      <c r="H307" s="8"/>
+      <c r="I307" t="s">
+        <v>112</v>
+      </c>
+      <c r="J307" t="s">
+        <v>85</v>
+      </c>
+      <c r="K307" t="s">
+        <v>86</v>
+      </c>
+      <c r="L307" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N307" s="6"/>
+      <c r="O307" s="5"/>
+    </row>
+    <row r="308" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A308" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B308" s="6">
+        <v>17.350000000000001</v>
+      </c>
+      <c r="C308" s="5">
+        <f t="shared" si="21"/>
+        <v>12.260000000000002</v>
+      </c>
+      <c r="D308" s="5">
+        <f t="shared" si="22"/>
+        <v>22.44</v>
+      </c>
+      <c r="E308" s="5">
+        <v>22.44</v>
+      </c>
+      <c r="F308">
+        <v>24</v>
+      </c>
+      <c r="G308" s="8">
+        <v>25</v>
+      </c>
+      <c r="H308" s="8"/>
+      <c r="I308" t="s">
+        <v>112</v>
+      </c>
+      <c r="J308" t="s">
+        <v>85</v>
+      </c>
+      <c r="K308" t="s">
+        <v>86</v>
+      </c>
+      <c r="L308" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N308" s="6"/>
+      <c r="O308" s="5"/>
+    </row>
+    <row r="309" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A309" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B309" s="6">
+        <v>17.510000000000002</v>
+      </c>
+      <c r="C309" s="5">
+        <f t="shared" si="21"/>
+        <v>12.420000000000002</v>
+      </c>
+      <c r="D309" s="5">
+        <f t="shared" si="22"/>
+        <v>22.6</v>
+      </c>
+      <c r="E309" s="5">
+        <v>17.510000000000002</v>
+      </c>
+      <c r="F309">
+        <v>25</v>
+      </c>
+      <c r="G309" s="8">
+        <v>20</v>
+      </c>
+      <c r="H309" s="8"/>
+      <c r="I309" t="s">
+        <v>112</v>
+      </c>
+      <c r="J309" t="s">
+        <v>85</v>
+      </c>
+      <c r="K309" t="s">
+        <v>86</v>
+      </c>
+      <c r="L309" s="5">
+        <v>5.09</v>
+      </c>
+      <c r="N309" s="6"/>
+      <c r="O309" s="5"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N235:O259">
-    <sortCondition ref="O235:O259"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N285:O309">
+    <sortCondition ref="O285:O309"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated IndyCar dataset to latest results & Results page
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8355DD-90BB-46F4-89E9-7603B9782255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5278E5-2037-4ADB-9A48-BAEDE6D7BB51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy_Model" sheetId="1" r:id="rId1"/>
@@ -374,13 +374,13 @@
     <t>Nashville Superpeedway</t>
   </si>
   <si>
-    <t>Milwaukee Mile</t>
-  </si>
-  <si>
     <t>Milwuakee Mile (Race 1)</t>
   </si>
   <si>
     <t>Milwuakee Mile (Race 2)</t>
+  </si>
+  <si>
+    <t>Milwaukee Mile (Avg of both races)</t>
   </si>
 </sst>
 </file>
@@ -11778,7 +11778,9 @@
       <c r="G210" s="8">
         <v>8</v>
       </c>
-      <c r="H210" s="8"/>
+      <c r="H210" s="8">
+        <v>1</v>
+      </c>
       <c r="I210" t="s">
         <v>108</v>
       </c>
@@ -11792,7 +11794,7 @@
         <v>5.43</v>
       </c>
       <c r="N210" s="6"/>
-      <c r="O210" s="5"/>
+      <c r="O210" s="8"/>
     </row>
     <row r="211" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A211" s="6" t="s">
@@ -11818,7 +11820,9 @@
       <c r="G211" s="8">
         <v>9</v>
       </c>
-      <c r="H211" s="8"/>
+      <c r="H211" s="8">
+        <v>5</v>
+      </c>
       <c r="I211" t="s">
         <v>108</v>
       </c>
@@ -11832,7 +11836,7 @@
         <v>5.43</v>
       </c>
       <c r="N211" s="6"/>
-      <c r="O211" s="5"/>
+      <c r="O211" s="8"/>
     </row>
     <row r="212" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A212" s="6" t="s">
@@ -11858,7 +11862,9 @@
       <c r="G212" s="8">
         <v>1</v>
       </c>
-      <c r="H212" s="8"/>
+      <c r="H212" s="8">
+        <v>11</v>
+      </c>
       <c r="I212" t="s">
         <v>108</v>
       </c>
@@ -11872,6 +11878,7 @@
         <v>5.43</v>
       </c>
       <c r="N212" s="6"/>
+      <c r="O212" s="8"/>
     </row>
     <row r="213" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A213" s="6" t="s">
@@ -11897,7 +11904,9 @@
       <c r="G213" s="8">
         <v>2</v>
       </c>
-      <c r="H213" s="8"/>
+      <c r="H213" s="8">
+        <v>7</v>
+      </c>
       <c r="I213" t="s">
         <v>108</v>
       </c>
@@ -11911,7 +11920,7 @@
         <v>5.43</v>
       </c>
       <c r="N213" s="6"/>
-      <c r="O213" s="5"/>
+      <c r="O213" s="8"/>
     </row>
     <row r="214" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A214" s="6" t="s">
@@ -11937,7 +11946,9 @@
       <c r="G214" s="8">
         <v>3</v>
       </c>
-      <c r="H214" s="8"/>
+      <c r="H214" s="8">
+        <v>12</v>
+      </c>
       <c r="I214" t="s">
         <v>108</v>
       </c>
@@ -11951,7 +11962,7 @@
         <v>5.43</v>
       </c>
       <c r="N214" s="6"/>
-      <c r="O214" s="5"/>
+      <c r="O214" s="8"/>
     </row>
     <row r="215" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A215" s="6" t="s">
@@ -11977,7 +11988,9 @@
       <c r="G215" s="8">
         <v>4</v>
       </c>
-      <c r="H215" s="8"/>
+      <c r="H215" s="8">
+        <v>17</v>
+      </c>
       <c r="I215" t="s">
         <v>108</v>
       </c>
@@ -11991,7 +12004,7 @@
         <v>5.43</v>
       </c>
       <c r="N215" s="6"/>
-      <c r="O215" s="5"/>
+      <c r="O215" s="8"/>
     </row>
     <row r="216" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A216" s="6" t="s">
@@ -12017,7 +12030,9 @@
       <c r="G216" s="8">
         <v>5</v>
       </c>
-      <c r="H216" s="8"/>
+      <c r="H216" s="8">
+        <v>13</v>
+      </c>
       <c r="I216" t="s">
         <v>108</v>
       </c>
@@ -12031,7 +12046,7 @@
         <v>5.43</v>
       </c>
       <c r="N216" s="6"/>
-      <c r="O216" s="5"/>
+      <c r="O216" s="8"/>
     </row>
     <row r="217" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A217" s="6" t="s">
@@ -12057,7 +12072,9 @@
       <c r="G217" s="8">
         <v>21</v>
       </c>
-      <c r="H217" s="8"/>
+      <c r="H217" s="8">
+        <v>21</v>
+      </c>
       <c r="I217" t="s">
         <v>108</v>
       </c>
@@ -12071,7 +12088,7 @@
         <v>5.43</v>
       </c>
       <c r="N217" s="6"/>
-      <c r="O217" s="5"/>
+      <c r="O217" s="8"/>
     </row>
     <row r="218" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A218" s="6" t="s">
@@ -12097,7 +12114,9 @@
       <c r="G218" s="8">
         <v>10</v>
       </c>
-      <c r="H218" s="8"/>
+      <c r="H218" s="8">
+        <v>18</v>
+      </c>
       <c r="I218" t="s">
         <v>108</v>
       </c>
@@ -12111,7 +12130,7 @@
         <v>5.43</v>
       </c>
       <c r="N218" s="6"/>
-      <c r="O218" s="5"/>
+      <c r="O218" s="8"/>
     </row>
     <row r="219" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A219" s="6" t="s">
@@ -12137,7 +12156,9 @@
       <c r="G219" s="8">
         <v>11</v>
       </c>
-      <c r="H219" s="8"/>
+      <c r="H219" s="8">
+        <v>14</v>
+      </c>
       <c r="I219" t="s">
         <v>108</v>
       </c>
@@ -12151,7 +12172,7 @@
         <v>5.43</v>
       </c>
       <c r="N219" s="6"/>
-      <c r="O219" s="5"/>
+      <c r="O219" s="8"/>
     </row>
     <row r="220" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A220" s="6" t="s">
@@ -12177,7 +12198,9 @@
       <c r="G220" s="8">
         <v>6</v>
       </c>
-      <c r="H220" s="8"/>
+      <c r="H220" s="8">
+        <v>3</v>
+      </c>
       <c r="I220" t="s">
         <v>108</v>
       </c>
@@ -12191,7 +12214,7 @@
         <v>5.43</v>
       </c>
       <c r="N220" s="6"/>
-      <c r="O220" s="5"/>
+      <c r="O220" s="8"/>
     </row>
     <row r="221" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A221" s="6" t="s">
@@ -12217,7 +12240,9 @@
       <c r="G221" s="8">
         <v>12</v>
       </c>
-      <c r="H221" s="8"/>
+      <c r="H221" s="8">
+        <v>4</v>
+      </c>
       <c r="I221" t="s">
         <v>108</v>
       </c>
@@ -12231,7 +12256,7 @@
         <v>5.43</v>
       </c>
       <c r="N221" s="6"/>
-      <c r="O221" s="5"/>
+      <c r="O221" s="8"/>
     </row>
     <row r="222" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A222" s="6" t="s">
@@ -12257,7 +12282,9 @@
       <c r="G222" s="8">
         <v>7</v>
       </c>
-      <c r="H222" s="8"/>
+      <c r="H222" s="8">
+        <v>9</v>
+      </c>
       <c r="I222" t="s">
         <v>108</v>
       </c>
@@ -12271,7 +12298,7 @@
         <v>5.43</v>
       </c>
       <c r="N222" s="6"/>
-      <c r="O222" s="5"/>
+      <c r="O222" s="8"/>
     </row>
     <row r="223" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A223" s="6" t="s">
@@ -12297,7 +12324,9 @@
       <c r="G223" s="8">
         <v>13</v>
       </c>
-      <c r="H223" s="8"/>
+      <c r="H223" s="8">
+        <v>8</v>
+      </c>
       <c r="I223" t="s">
         <v>108</v>
       </c>
@@ -12311,7 +12340,7 @@
         <v>5.43</v>
       </c>
       <c r="N223" s="6"/>
-      <c r="O223" s="5"/>
+      <c r="O223" s="8"/>
     </row>
     <row r="224" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A224" s="6" t="s">
@@ -12337,7 +12366,9 @@
       <c r="G224" s="8">
         <v>22</v>
       </c>
-      <c r="H224" s="8"/>
+      <c r="H224" s="8">
+        <v>10</v>
+      </c>
       <c r="I224" t="s">
         <v>108</v>
       </c>
@@ -12351,7 +12382,7 @@
         <v>5.43</v>
       </c>
       <c r="N224" s="6"/>
-      <c r="O224" s="5"/>
+      <c r="O224" s="8"/>
     </row>
     <row r="225" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A225" s="6" t="s">
@@ -12377,7 +12408,9 @@
       <c r="G225" s="8">
         <v>14</v>
       </c>
-      <c r="H225" s="8"/>
+      <c r="H225" s="8">
+        <v>6</v>
+      </c>
       <c r="I225" t="s">
         <v>108</v>
       </c>
@@ -12391,7 +12424,7 @@
         <v>5.43</v>
       </c>
       <c r="N225" s="6"/>
-      <c r="O225" s="5"/>
+      <c r="O225" s="8"/>
     </row>
     <row r="226" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A226" s="6" t="s">
@@ -12417,7 +12450,9 @@
       <c r="G226" s="8">
         <v>15</v>
       </c>
-      <c r="H226" s="8"/>
+      <c r="H226" s="8">
+        <v>24</v>
+      </c>
       <c r="I226" t="s">
         <v>108</v>
       </c>
@@ -12431,7 +12466,7 @@
         <v>5.43</v>
       </c>
       <c r="N226" s="6"/>
-      <c r="O226" s="5"/>
+      <c r="O226" s="8"/>
     </row>
     <row r="227" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A227" s="6" t="s">
@@ -12457,7 +12492,9 @@
       <c r="G227" s="8">
         <v>16</v>
       </c>
-      <c r="H227" s="8"/>
+      <c r="H227" s="8">
+        <v>23</v>
+      </c>
       <c r="I227" t="s">
         <v>108</v>
       </c>
@@ -12471,7 +12508,7 @@
         <v>5.43</v>
       </c>
       <c r="N227" s="6"/>
-      <c r="O227" s="5"/>
+      <c r="O227" s="8"/>
     </row>
     <row r="228" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A228" s="6" t="s">
@@ -12497,7 +12534,9 @@
       <c r="G228" s="8">
         <v>17</v>
       </c>
-      <c r="H228" s="8"/>
+      <c r="H228" s="8">
+        <v>2</v>
+      </c>
       <c r="I228" t="s">
         <v>108</v>
       </c>
@@ -12511,7 +12550,7 @@
         <v>5.43</v>
       </c>
       <c r="N228" s="6"/>
-      <c r="O228" s="5"/>
+      <c r="O228" s="8"/>
     </row>
     <row r="229" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A229" s="6" t="s">
@@ -12537,7 +12576,9 @@
       <c r="G229" s="8">
         <v>23</v>
       </c>
-      <c r="H229" s="8"/>
+      <c r="H229" s="8">
+        <v>25</v>
+      </c>
       <c r="I229" t="s">
         <v>108</v>
       </c>
@@ -12551,7 +12592,7 @@
         <v>5.43</v>
       </c>
       <c r="N229" s="6"/>
-      <c r="O229" s="5"/>
+      <c r="O229" s="8"/>
     </row>
     <row r="230" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A230" s="6" t="s">
@@ -12577,7 +12618,9 @@
       <c r="G230" s="8">
         <v>24</v>
       </c>
-      <c r="H230" s="8"/>
+      <c r="H230" s="8">
+        <v>20</v>
+      </c>
       <c r="I230" t="s">
         <v>108</v>
       </c>
@@ -12591,7 +12634,7 @@
         <v>5.43</v>
       </c>
       <c r="N230" s="6"/>
-      <c r="O230" s="5"/>
+      <c r="O230" s="8"/>
     </row>
     <row r="231" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A231" s="6" t="s">
@@ -12617,7 +12660,9 @@
       <c r="G231" s="8">
         <v>18</v>
       </c>
-      <c r="H231" s="8"/>
+      <c r="H231" s="8">
+        <v>15</v>
+      </c>
       <c r="I231" t="s">
         <v>108</v>
       </c>
@@ -12631,7 +12676,7 @@
         <v>5.43</v>
       </c>
       <c r="N231" s="6"/>
-      <c r="O231" s="5"/>
+      <c r="O231" s="8"/>
     </row>
     <row r="232" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A232" s="6" t="s">
@@ -12657,7 +12702,9 @@
       <c r="G232" s="8">
         <v>19</v>
       </c>
-      <c r="H232" s="8"/>
+      <c r="H232" s="8">
+        <v>22</v>
+      </c>
       <c r="I232" t="s">
         <v>108</v>
       </c>
@@ -12671,7 +12718,7 @@
         <v>5.43</v>
       </c>
       <c r="N232" s="6"/>
-      <c r="O232" s="5"/>
+      <c r="O232" s="8"/>
     </row>
     <row r="233" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A233" s="6" t="s">
@@ -12697,7 +12744,9 @@
       <c r="G233" s="8">
         <v>25</v>
       </c>
-      <c r="H233" s="8"/>
+      <c r="H233" s="8">
+        <v>19</v>
+      </c>
       <c r="I233" t="s">
         <v>108</v>
       </c>
@@ -12711,7 +12760,7 @@
         <v>5.43</v>
       </c>
       <c r="N233" s="6"/>
-      <c r="O233" s="5"/>
+      <c r="O233" s="8"/>
     </row>
     <row r="234" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A234" s="6" t="s">
@@ -12737,7 +12786,9 @@
       <c r="G234" s="8">
         <v>20</v>
       </c>
-      <c r="H234" s="8"/>
+      <c r="H234" s="8">
+        <v>16</v>
+      </c>
       <c r="I234" t="s">
         <v>108</v>
       </c>
@@ -12750,6 +12801,8 @@
       <c r="L234">
         <v>5.43</v>
       </c>
+      <c r="N234" s="6"/>
+      <c r="O234" s="8"/>
     </row>
     <row r="235" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A235" s="6" t="s">
@@ -12758,8 +12811,26 @@
       <c r="B235" s="6">
         <v>10.93</v>
       </c>
-      <c r="G235" s="8"/>
-      <c r="H235" s="8"/>
+      <c r="C235" s="5">
+        <f>B235-L235</f>
+        <v>5.5</v>
+      </c>
+      <c r="D235" s="5">
+        <f>B235+L235</f>
+        <v>16.36</v>
+      </c>
+      <c r="E235" s="5">
+        <v>10.93</v>
+      </c>
+      <c r="F235">
+        <v>1</v>
+      </c>
+      <c r="G235" s="8">
+        <v>8</v>
+      </c>
+      <c r="H235" s="8">
+        <v>4</v>
+      </c>
       <c r="I235" t="s">
         <v>109</v>
       </c>
@@ -12780,8 +12851,26 @@
       <c r="B236" s="6">
         <v>10.96</v>
       </c>
-      <c r="G236" s="8"/>
-      <c r="H236" s="8"/>
+      <c r="C236" s="5">
+        <f t="shared" ref="C236:C259" si="18">B236-L236</f>
+        <v>5.5300000000000011</v>
+      </c>
+      <c r="D236" s="5">
+        <f t="shared" ref="D236:D259" si="19">B236+L236</f>
+        <v>16.39</v>
+      </c>
+      <c r="E236" s="5">
+        <v>5.53</v>
+      </c>
+      <c r="F236">
+        <v>2</v>
+      </c>
+      <c r="G236" s="8">
+        <v>1</v>
+      </c>
+      <c r="H236" s="8">
+        <v>2</v>
+      </c>
       <c r="I236" t="s">
         <v>109</v>
       </c>
@@ -12794,6 +12883,8 @@
       <c r="L236">
         <v>5.43</v>
       </c>
+      <c r="N236" s="6"/>
+      <c r="O236" s="8"/>
     </row>
     <row r="237" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A237" s="6" t="s">
@@ -12802,8 +12893,26 @@
       <c r="B237" s="6">
         <v>11.4</v>
       </c>
-      <c r="G237" s="8"/>
-      <c r="H237" s="8"/>
+      <c r="C237" s="5">
+        <f t="shared" si="18"/>
+        <v>5.9700000000000006</v>
+      </c>
+      <c r="D237" s="5">
+        <f t="shared" si="19"/>
+        <v>16.829999999999998</v>
+      </c>
+      <c r="E237" s="5">
+        <v>5.97</v>
+      </c>
+      <c r="F237">
+        <v>3</v>
+      </c>
+      <c r="G237" s="8">
+        <v>2</v>
+      </c>
+      <c r="H237" s="8">
+        <v>7</v>
+      </c>
       <c r="I237" t="s">
         <v>109</v>
       </c>
@@ -12816,6 +12925,8 @@
       <c r="L237">
         <v>5.43</v>
       </c>
+      <c r="N237" s="6"/>
+      <c r="O237" s="8"/>
     </row>
     <row r="238" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A238" s="6" t="s">
@@ -12824,8 +12935,26 @@
       <c r="B238" s="6">
         <v>11.91</v>
       </c>
-      <c r="G238" s="8"/>
-      <c r="H238" s="8"/>
+      <c r="C238" s="5">
+        <f t="shared" si="18"/>
+        <v>6.48</v>
+      </c>
+      <c r="D238" s="5">
+        <f t="shared" si="19"/>
+        <v>17.34</v>
+      </c>
+      <c r="E238" s="5">
+        <v>6.48</v>
+      </c>
+      <c r="F238">
+        <v>4</v>
+      </c>
+      <c r="G238" s="8">
+        <v>3</v>
+      </c>
+      <c r="H238" s="8">
+        <v>3</v>
+      </c>
       <c r="I238" t="s">
         <v>109</v>
       </c>
@@ -12838,6 +12967,8 @@
       <c r="L238">
         <v>5.43</v>
       </c>
+      <c r="N238" s="6"/>
+      <c r="O238" s="8"/>
     </row>
     <row r="239" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A239" s="6" t="s">
@@ -12846,8 +12977,26 @@
       <c r="B239" s="6">
         <v>12.31</v>
       </c>
-      <c r="G239" s="8"/>
-      <c r="H239" s="8"/>
+      <c r="C239" s="5">
+        <f t="shared" si="18"/>
+        <v>6.8800000000000008</v>
+      </c>
+      <c r="D239" s="5">
+        <f t="shared" si="19"/>
+        <v>17.740000000000002</v>
+      </c>
+      <c r="E239" s="5">
+        <v>12.31</v>
+      </c>
+      <c r="F239">
+        <v>5</v>
+      </c>
+      <c r="G239" s="8">
+        <v>9</v>
+      </c>
+      <c r="H239" s="8">
+        <v>10</v>
+      </c>
       <c r="I239" t="s">
         <v>109</v>
       </c>
@@ -12860,6 +13009,8 @@
       <c r="L239">
         <v>5.43</v>
       </c>
+      <c r="N239" s="6"/>
+      <c r="O239" s="8"/>
     </row>
     <row r="240" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A240" s="6" t="s">
@@ -12868,8 +13019,26 @@
       <c r="B240" s="6">
         <v>12.61</v>
       </c>
-      <c r="G240" s="8"/>
-      <c r="H240" s="8"/>
+      <c r="C240" s="5">
+        <f t="shared" si="18"/>
+        <v>7.18</v>
+      </c>
+      <c r="D240" s="5">
+        <f t="shared" si="19"/>
+        <v>18.04</v>
+      </c>
+      <c r="E240" s="5">
+        <v>12.61</v>
+      </c>
+      <c r="F240">
+        <v>6</v>
+      </c>
+      <c r="G240" s="8">
+        <v>10</v>
+      </c>
+      <c r="H240" s="8">
+        <v>1</v>
+      </c>
       <c r="I240" t="s">
         <v>109</v>
       </c>
@@ -12882,16 +13051,36 @@
       <c r="L240">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N240" s="6"/>
+      <c r="O240" s="8"/>
+    </row>
+    <row r="241" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A241" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B241" s="6">
         <v>12.66</v>
       </c>
-      <c r="G241" s="8"/>
-      <c r="H241" s="8"/>
+      <c r="C241" s="5">
+        <f t="shared" si="18"/>
+        <v>7.23</v>
+      </c>
+      <c r="D241" s="5">
+        <f t="shared" si="19"/>
+        <v>18.09</v>
+      </c>
+      <c r="E241" s="5">
+        <v>12.66</v>
+      </c>
+      <c r="F241">
+        <v>7</v>
+      </c>
+      <c r="G241" s="8">
+        <v>11</v>
+      </c>
+      <c r="H241" s="8">
+        <v>18</v>
+      </c>
       <c r="I241" t="s">
         <v>109</v>
       </c>
@@ -12904,16 +13093,36 @@
       <c r="L241">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N241" s="6"/>
+      <c r="O241" s="8"/>
+    </row>
+    <row r="242" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A242" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B242" s="6">
         <v>12.76</v>
       </c>
-      <c r="G242" s="8"/>
-      <c r="H242" s="8"/>
+      <c r="C242" s="5">
+        <f t="shared" si="18"/>
+        <v>7.33</v>
+      </c>
+      <c r="D242" s="5">
+        <f t="shared" si="19"/>
+        <v>18.189999999999998</v>
+      </c>
+      <c r="E242" s="5">
+        <v>7.33</v>
+      </c>
+      <c r="F242">
+        <v>8</v>
+      </c>
+      <c r="G242" s="8">
+        <v>4</v>
+      </c>
+      <c r="H242" s="8">
+        <v>13</v>
+      </c>
       <c r="I242" t="s">
         <v>109</v>
       </c>
@@ -12926,16 +13135,36 @@
       <c r="L242">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N242" s="6"/>
+      <c r="O242" s="8"/>
+    </row>
+    <row r="243" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A243" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B243" s="6">
         <v>13.04</v>
       </c>
-      <c r="G243" s="8"/>
-      <c r="H243" s="8"/>
+      <c r="C243" s="5">
+        <f t="shared" si="18"/>
+        <v>7.6099999999999994</v>
+      </c>
+      <c r="D243" s="5">
+        <f t="shared" si="19"/>
+        <v>18.47</v>
+      </c>
+      <c r="E243" s="5">
+        <v>13.04</v>
+      </c>
+      <c r="F243">
+        <v>9</v>
+      </c>
+      <c r="G243" s="8">
+        <v>12</v>
+      </c>
+      <c r="H243" s="8">
+        <v>23</v>
+      </c>
       <c r="I243" t="s">
         <v>109</v>
       </c>
@@ -12948,16 +13177,36 @@
       <c r="L243">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N243" s="6"/>
+      <c r="O243" s="8"/>
+    </row>
+    <row r="244" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A244" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B244" s="6">
         <v>13.07</v>
       </c>
-      <c r="G244" s="8"/>
-      <c r="H244" s="8"/>
+      <c r="C244" s="5">
+        <f t="shared" si="18"/>
+        <v>7.6400000000000006</v>
+      </c>
+      <c r="D244" s="5">
+        <f t="shared" si="19"/>
+        <v>18.5</v>
+      </c>
+      <c r="E244" s="5">
+        <v>13.07</v>
+      </c>
+      <c r="F244">
+        <v>10</v>
+      </c>
+      <c r="G244" s="8">
+        <v>13</v>
+      </c>
+      <c r="H244" s="8">
+        <v>12</v>
+      </c>
       <c r="I244" t="s">
         <v>109</v>
       </c>
@@ -12970,16 +13219,36 @@
       <c r="L244">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N244" s="6"/>
+      <c r="O244" s="8"/>
+    </row>
+    <row r="245" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A245" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B245" s="6">
         <v>13.11</v>
       </c>
-      <c r="G245" s="8"/>
-      <c r="H245" s="8"/>
+      <c r="C245" s="5">
+        <f t="shared" si="18"/>
+        <v>7.68</v>
+      </c>
+      <c r="D245" s="5">
+        <f t="shared" si="19"/>
+        <v>18.54</v>
+      </c>
+      <c r="E245" s="5">
+        <v>7.68</v>
+      </c>
+      <c r="F245">
+        <v>11</v>
+      </c>
+      <c r="G245" s="8">
+        <v>5</v>
+      </c>
+      <c r="H245" s="8">
+        <v>22</v>
+      </c>
       <c r="I245" t="s">
         <v>109</v>
       </c>
@@ -12992,16 +13261,36 @@
       <c r="L245">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N245" s="6"/>
+      <c r="O245" s="8"/>
+    </row>
+    <row r="246" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A246" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B246" s="6">
         <v>13.11</v>
       </c>
-      <c r="G246" s="8"/>
-      <c r="H246" s="8"/>
+      <c r="C246" s="5">
+        <f t="shared" si="18"/>
+        <v>7.68</v>
+      </c>
+      <c r="D246" s="5">
+        <f t="shared" si="19"/>
+        <v>18.54</v>
+      </c>
+      <c r="E246" s="5">
+        <v>13.11</v>
+      </c>
+      <c r="F246">
+        <v>12</v>
+      </c>
+      <c r="G246" s="8">
+        <v>14</v>
+      </c>
+      <c r="H246" s="8">
+        <v>24</v>
+      </c>
       <c r="I246" t="s">
         <v>109</v>
       </c>
@@ -13014,16 +13303,36 @@
       <c r="L246">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N246" s="6"/>
+      <c r="O246" s="8"/>
+    </row>
+    <row r="247" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A247" s="6" t="s">
         <v>44</v>
       </c>
       <c r="B247" s="6">
         <v>13.18</v>
       </c>
-      <c r="G247" s="8"/>
-      <c r="H247" s="8"/>
+      <c r="C247" s="5">
+        <f t="shared" si="18"/>
+        <v>7.75</v>
+      </c>
+      <c r="D247" s="5">
+        <f t="shared" si="19"/>
+        <v>18.61</v>
+      </c>
+      <c r="E247" s="5">
+        <v>13.18</v>
+      </c>
+      <c r="F247">
+        <v>13</v>
+      </c>
+      <c r="G247" s="8">
+        <v>15</v>
+      </c>
+      <c r="H247" s="8">
+        <v>5</v>
+      </c>
       <c r="I247" t="s">
         <v>109</v>
       </c>
@@ -13036,16 +13345,36 @@
       <c r="L247">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N247" s="6"/>
+      <c r="O247" s="8"/>
+    </row>
+    <row r="248" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A248" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B248" s="6">
         <v>13.34</v>
       </c>
-      <c r="G248" s="8"/>
-      <c r="H248" s="8"/>
+      <c r="C248" s="5">
+        <f t="shared" si="18"/>
+        <v>7.91</v>
+      </c>
+      <c r="D248" s="5">
+        <f t="shared" si="19"/>
+        <v>18.77</v>
+      </c>
+      <c r="E248" s="5">
+        <v>7.91</v>
+      </c>
+      <c r="F248">
+        <v>14</v>
+      </c>
+      <c r="G248" s="8">
+        <v>6</v>
+      </c>
+      <c r="H248" s="8">
+        <v>20</v>
+      </c>
       <c r="I248" t="s">
         <v>109</v>
       </c>
@@ -13058,16 +13387,36 @@
       <c r="L248">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N248" s="6"/>
+      <c r="O248" s="8"/>
+    </row>
+    <row r="249" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A249" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B249" s="6">
         <v>13.77</v>
       </c>
-      <c r="G249" s="8"/>
-      <c r="H249" s="8"/>
+      <c r="C249" s="5">
+        <f t="shared" si="18"/>
+        <v>8.34</v>
+      </c>
+      <c r="D249" s="5">
+        <f t="shared" si="19"/>
+        <v>19.2</v>
+      </c>
+      <c r="E249" s="5">
+        <v>19.2</v>
+      </c>
+      <c r="F249">
+        <v>15</v>
+      </c>
+      <c r="G249" s="8">
+        <v>21</v>
+      </c>
+      <c r="H249" s="8">
+        <v>16</v>
+      </c>
       <c r="I249" t="s">
         <v>109</v>
       </c>
@@ -13080,16 +13429,36 @@
       <c r="L249">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N249" s="6"/>
+      <c r="O249" s="8"/>
+    </row>
+    <row r="250" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A250" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B250" s="6">
         <v>14.11</v>
       </c>
-      <c r="G250" s="8"/>
-      <c r="H250" s="8"/>
+      <c r="C250" s="5">
+        <f t="shared" si="18"/>
+        <v>8.68</v>
+      </c>
+      <c r="D250" s="5">
+        <f t="shared" si="19"/>
+        <v>19.54</v>
+      </c>
+      <c r="E250" s="5">
+        <v>19.54</v>
+      </c>
+      <c r="F250">
+        <v>16</v>
+      </c>
+      <c r="G250" s="8">
+        <v>22</v>
+      </c>
+      <c r="H250" s="8">
+        <v>9</v>
+      </c>
       <c r="I250" t="s">
         <v>109</v>
       </c>
@@ -13102,16 +13471,36 @@
       <c r="L250">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N250" s="6"/>
+      <c r="O250" s="8"/>
+    </row>
+    <row r="251" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A251" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B251" s="6">
         <v>14.19</v>
       </c>
-      <c r="G251" s="8"/>
-      <c r="H251" s="8"/>
+      <c r="C251" s="5">
+        <f t="shared" si="18"/>
+        <v>8.76</v>
+      </c>
+      <c r="D251" s="5">
+        <f t="shared" si="19"/>
+        <v>19.619999999999997</v>
+      </c>
+      <c r="E251" s="5">
+        <v>14.19</v>
+      </c>
+      <c r="F251">
+        <v>17</v>
+      </c>
+      <c r="G251" s="8">
+        <v>16</v>
+      </c>
+      <c r="H251" s="8">
+        <v>6</v>
+      </c>
       <c r="I251" t="s">
         <v>109</v>
       </c>
@@ -13124,16 +13513,36 @@
       <c r="L251">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N251" s="6"/>
+      <c r="O251" s="8"/>
+    </row>
+    <row r="252" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A252" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B252" s="6">
         <v>14.9</v>
       </c>
-      <c r="G252" s="8"/>
-      <c r="H252" s="8"/>
+      <c r="C252" s="5">
+        <f t="shared" si="18"/>
+        <v>9.4700000000000006</v>
+      </c>
+      <c r="D252" s="5">
+        <f t="shared" si="19"/>
+        <v>20.329999999999998</v>
+      </c>
+      <c r="E252" s="5">
+        <v>20.329999999999998</v>
+      </c>
+      <c r="F252">
+        <v>18</v>
+      </c>
+      <c r="G252" s="8">
+        <v>23</v>
+      </c>
+      <c r="H252" s="8">
+        <v>19</v>
+      </c>
       <c r="I252" t="s">
         <v>109</v>
       </c>
@@ -13146,16 +13555,36 @@
       <c r="L252">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N252" s="6"/>
+      <c r="O252" s="8"/>
+    </row>
+    <row r="253" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A253" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B253" s="6">
         <v>14.94</v>
       </c>
-      <c r="G253" s="8"/>
-      <c r="H253" s="8"/>
+      <c r="C253" s="5">
+        <f t="shared" si="18"/>
+        <v>9.51</v>
+      </c>
+      <c r="D253" s="5">
+        <f t="shared" si="19"/>
+        <v>20.369999999999997</v>
+      </c>
+      <c r="E253" s="5">
+        <v>14.94</v>
+      </c>
+      <c r="F253">
+        <v>19</v>
+      </c>
+      <c r="G253" s="8">
+        <v>17</v>
+      </c>
+      <c r="H253" s="8">
+        <v>11</v>
+      </c>
       <c r="I253" t="s">
         <v>109</v>
       </c>
@@ -13168,16 +13597,36 @@
       <c r="L253">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N253" s="6"/>
+      <c r="O253" s="8"/>
+    </row>
+    <row r="254" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A254" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B254" s="6">
         <v>15.13</v>
       </c>
-      <c r="G254" s="8"/>
-      <c r="H254" s="8"/>
+      <c r="C254" s="5">
+        <f t="shared" si="18"/>
+        <v>9.7000000000000011</v>
+      </c>
+      <c r="D254" s="5">
+        <f t="shared" si="19"/>
+        <v>20.560000000000002</v>
+      </c>
+      <c r="E254" s="5">
+        <v>20.56</v>
+      </c>
+      <c r="F254">
+        <v>20</v>
+      </c>
+      <c r="G254" s="8">
+        <v>24</v>
+      </c>
+      <c r="H254" s="8">
+        <v>21</v>
+      </c>
       <c r="I254" t="s">
         <v>109</v>
       </c>
@@ -13190,16 +13639,36 @@
       <c r="L254">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N254" s="6"/>
+      <c r="O254" s="8"/>
+    </row>
+    <row r="255" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A255" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B255" s="6">
         <v>15.17</v>
       </c>
-      <c r="G255" s="8"/>
-      <c r="H255" s="8"/>
+      <c r="C255" s="5">
+        <f t="shared" si="18"/>
+        <v>9.74</v>
+      </c>
+      <c r="D255" s="5">
+        <f t="shared" si="19"/>
+        <v>20.6</v>
+      </c>
+      <c r="E255" s="5">
+        <v>20.6</v>
+      </c>
+      <c r="F255">
+        <v>21</v>
+      </c>
+      <c r="G255" s="8">
+        <v>25</v>
+      </c>
+      <c r="H255" s="8">
+        <v>15</v>
+      </c>
       <c r="I255" t="s">
         <v>109</v>
       </c>
@@ -13212,16 +13681,36 @@
       <c r="L255">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="N255" s="6"/>
+      <c r="O255" s="8"/>
+    </row>
+    <row r="256" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A256" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B256" s="6">
         <v>15.25</v>
       </c>
-      <c r="G256" s="8"/>
-      <c r="H256" s="8"/>
+      <c r="C256" s="5">
+        <f t="shared" si="18"/>
+        <v>9.82</v>
+      </c>
+      <c r="D256" s="5">
+        <f t="shared" si="19"/>
+        <v>20.68</v>
+      </c>
+      <c r="E256" s="5">
+        <v>15.25</v>
+      </c>
+      <c r="F256">
+        <v>22</v>
+      </c>
+      <c r="G256" s="8">
+        <v>18</v>
+      </c>
+      <c r="H256" s="8">
+        <v>17</v>
+      </c>
       <c r="I256" t="s">
         <v>109</v>
       </c>
@@ -13234,16 +13723,36 @@
       <c r="L256">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="257" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="N256" s="6"/>
+      <c r="O256" s="8"/>
+    </row>
+    <row r="257" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A257" s="6" t="s">
         <v>26</v>
       </c>
       <c r="B257" s="6">
         <v>15.26</v>
       </c>
-      <c r="G257" s="8"/>
-      <c r="H257" s="8"/>
+      <c r="C257" s="5">
+        <f t="shared" si="18"/>
+        <v>9.83</v>
+      </c>
+      <c r="D257" s="5">
+        <f t="shared" si="19"/>
+        <v>20.689999999999998</v>
+      </c>
+      <c r="E257" s="5">
+        <v>9.83</v>
+      </c>
+      <c r="F257">
+        <v>23</v>
+      </c>
+      <c r="G257" s="8">
+        <v>7</v>
+      </c>
+      <c r="H257" s="8">
+        <v>25</v>
+      </c>
       <c r="I257" t="s">
         <v>109</v>
       </c>
@@ -13256,16 +13765,36 @@
       <c r="L257">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="258" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="N257" s="6"/>
+      <c r="O257" s="8"/>
+    </row>
+    <row r="258" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A258" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B258" s="6">
         <v>15.3</v>
       </c>
-      <c r="G258" s="8"/>
-      <c r="H258" s="8"/>
+      <c r="C258" s="5">
+        <f t="shared" si="18"/>
+        <v>9.870000000000001</v>
+      </c>
+      <c r="D258" s="5">
+        <f t="shared" si="19"/>
+        <v>20.73</v>
+      </c>
+      <c r="E258" s="5">
+        <v>15.3</v>
+      </c>
+      <c r="F258">
+        <v>24</v>
+      </c>
+      <c r="G258" s="8">
+        <v>19</v>
+      </c>
+      <c r="H258" s="8">
+        <v>14</v>
+      </c>
       <c r="I258" t="s">
         <v>109</v>
       </c>
@@ -13278,16 +13807,36 @@
       <c r="L258">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="259" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="N258" s="6"/>
+      <c r="O258" s="8"/>
+    </row>
+    <row r="259" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A259" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B259" s="6">
         <v>15.54</v>
       </c>
-      <c r="G259" s="8"/>
-      <c r="H259" s="8"/>
+      <c r="C259" s="5">
+        <f t="shared" si="18"/>
+        <v>10.11</v>
+      </c>
+      <c r="D259" s="5">
+        <f t="shared" si="19"/>
+        <v>20.97</v>
+      </c>
+      <c r="E259" s="5">
+        <v>15.54</v>
+      </c>
+      <c r="F259">
+        <v>25</v>
+      </c>
+      <c r="G259" s="8">
+        <v>20</v>
+      </c>
+      <c r="H259" s="8">
+        <v>8</v>
+      </c>
       <c r="I259" t="s">
         <v>109</v>
       </c>
@@ -13300,8 +13849,10 @@
       <c r="L259">
         <v>5.43</v>
       </c>
-    </row>
-    <row r="260" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="N259" s="6"/>
+      <c r="O259" s="8"/>
+    </row>
+    <row r="260" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A260" s="6" t="s">
         <v>36</v>
       </c>
@@ -13325,9 +13876,11 @@
       <c r="G260" s="8">
         <v>5</v>
       </c>
-      <c r="H260" s="8"/>
+      <c r="H260" s="8">
+        <v>3</v>
+      </c>
       <c r="I260" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J260" t="s">
         <v>85</v>
@@ -13339,8 +13892,9 @@
         <v>5.43</v>
       </c>
       <c r="N260" s="6"/>
-    </row>
-    <row r="261" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="O260" s="8"/>
+    </row>
+    <row r="261" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A261" s="6" t="s">
         <v>35</v>
       </c>
@@ -13352,7 +13906,7 @@
         <v>2.6799999999999997</v>
       </c>
       <c r="D261">
-        <f t="shared" ref="D261:D284" si="18">B261+L261</f>
+        <f t="shared" ref="D261:D284" si="20">B261+L261</f>
         <v>13.54</v>
       </c>
       <c r="E261">
@@ -13364,9 +13918,11 @@
       <c r="G261" s="8">
         <v>1</v>
       </c>
-      <c r="H261" s="8"/>
+      <c r="H261" s="8">
+        <v>4</v>
+      </c>
       <c r="I261" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J261" t="s">
         <v>85</v>
@@ -13379,7 +13935,7 @@
       </c>
       <c r="N261" s="6"/>
     </row>
-    <row r="262" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A262" s="6" t="s">
         <v>39</v>
       </c>
@@ -13387,11 +13943,11 @@
         <v>8.2799999999999994</v>
       </c>
       <c r="C262">
-        <f t="shared" ref="C262:C284" si="19">B262-L262</f>
+        <f t="shared" ref="C262:C284" si="21">B262-L262</f>
         <v>2.8499999999999996</v>
       </c>
       <c r="D262">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>13.709999999999999</v>
       </c>
       <c r="E262">
@@ -13403,9 +13959,11 @@
       <c r="G262" s="8">
         <v>7</v>
       </c>
-      <c r="H262" s="8"/>
+      <c r="H262" s="8">
+        <v>8</v>
+      </c>
       <c r="I262" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J262" t="s">
         <v>85</v>
@@ -13418,7 +13976,7 @@
       </c>
       <c r="N262" s="6"/>
     </row>
-    <row r="263" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A263" s="6" t="s">
         <v>38</v>
       </c>
@@ -13426,11 +13984,11 @@
         <v>8.51</v>
       </c>
       <c r="C263">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>3.08</v>
       </c>
       <c r="D263">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>13.94</v>
       </c>
       <c r="E263">
@@ -13442,9 +14000,11 @@
       <c r="G263" s="8">
         <v>2</v>
       </c>
-      <c r="H263" s="8"/>
+      <c r="H263" s="8">
+        <v>1</v>
+      </c>
       <c r="I263" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J263" t="s">
         <v>85</v>
@@ -13457,7 +14017,7 @@
       </c>
       <c r="N263" s="6"/>
     </row>
-    <row r="264" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A264" s="6" t="s">
         <v>37</v>
       </c>
@@ -13465,11 +14025,11 @@
         <v>9.23</v>
       </c>
       <c r="C264" s="12">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>3.8000000000000007</v>
       </c>
       <c r="D264">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>14.66</v>
       </c>
       <c r="E264">
@@ -13481,9 +14041,11 @@
       <c r="G264" s="8">
         <v>3</v>
       </c>
-      <c r="H264" s="8"/>
+      <c r="H264" s="8">
+        <v>16</v>
+      </c>
       <c r="I264" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J264" t="s">
         <v>85</v>
@@ -13496,7 +14058,7 @@
       </c>
       <c r="N264" s="6"/>
     </row>
-    <row r="265" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A265" s="6" t="s">
         <v>34</v>
       </c>
@@ -13504,11 +14066,11 @@
         <v>9.23</v>
       </c>
       <c r="C265" s="12">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>3.8000000000000007</v>
       </c>
       <c r="D265">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>14.66</v>
       </c>
       <c r="E265">
@@ -13520,9 +14082,11 @@
       <c r="G265" s="8">
         <v>18</v>
       </c>
-      <c r="H265" s="8"/>
+      <c r="H265" s="8">
+        <v>5</v>
+      </c>
       <c r="I265" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J265" t="s">
         <v>85</v>
@@ -13535,7 +14099,7 @@
       </c>
       <c r="N265" s="6"/>
     </row>
-    <row r="266" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="266" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A266" s="6" t="s">
         <v>33</v>
       </c>
@@ -13543,11 +14107,11 @@
         <v>9.26</v>
       </c>
       <c r="C266">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>3.83</v>
       </c>
       <c r="D266">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>14.69</v>
       </c>
       <c r="E266">
@@ -13559,9 +14123,11 @@
       <c r="G266" s="8">
         <v>10</v>
       </c>
-      <c r="H266" s="8"/>
+      <c r="H266" s="8">
+        <v>11</v>
+      </c>
       <c r="I266" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J266" t="s">
         <v>85</v>
@@ -13574,7 +14140,7 @@
       </c>
       <c r="N266" s="6"/>
     </row>
-    <row r="267" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="267" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A267" s="6" t="s">
         <v>49</v>
       </c>
@@ -13582,11 +14148,11 @@
         <v>10.77</v>
       </c>
       <c r="C267">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>5.34</v>
       </c>
       <c r="D267">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>16.2</v>
       </c>
       <c r="E267">
@@ -13598,9 +14164,11 @@
       <c r="G267" s="8">
         <v>11</v>
       </c>
-      <c r="H267" s="8"/>
+      <c r="H267" s="8">
+        <v>5</v>
+      </c>
       <c r="I267" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J267" t="s">
         <v>85</v>
@@ -13613,7 +14181,7 @@
       </c>
       <c r="N267" s="6"/>
     </row>
-    <row r="268" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="268" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A268" s="6" t="s">
         <v>27</v>
       </c>
@@ -13621,11 +14189,11 @@
         <v>10.94</v>
       </c>
       <c r="C268">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>5.51</v>
       </c>
       <c r="D268">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>16.369999999999997</v>
       </c>
       <c r="E268">
@@ -13637,9 +14205,11 @@
       <c r="G268" s="8">
         <v>12</v>
       </c>
-      <c r="H268" s="8"/>
+      <c r="H268" s="8">
+        <v>17</v>
+      </c>
       <c r="I268" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J268" t="s">
         <v>85</v>
@@ -13652,7 +14222,7 @@
       </c>
       <c r="N268" s="6"/>
     </row>
-    <row r="269" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="269" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A269" s="6" t="s">
         <v>28</v>
       </c>
@@ -13660,11 +14230,11 @@
         <v>10.97</v>
       </c>
       <c r="C269">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>5.5400000000000009</v>
       </c>
       <c r="D269">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>16.399999999999999</v>
       </c>
       <c r="E269">
@@ -13676,9 +14246,11 @@
       <c r="G269" s="8">
         <v>13</v>
       </c>
-      <c r="H269" s="8"/>
+      <c r="H269" s="8">
+        <v>9</v>
+      </c>
       <c r="I269" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J269" t="s">
         <v>85</v>
@@ -13691,7 +14263,7 @@
       </c>
       <c r="N269" s="6"/>
     </row>
-    <row r="270" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="270" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A270" s="6" t="s">
         <v>40</v>
       </c>
@@ -13699,11 +14271,11 @@
         <v>11.25</v>
       </c>
       <c r="C270">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>5.82</v>
       </c>
       <c r="D270">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>16.68</v>
       </c>
       <c r="E270">
@@ -13715,9 +14287,11 @@
       <c r="G270" s="8">
         <v>4</v>
       </c>
-      <c r="H270" s="8"/>
+      <c r="H270" s="8">
+        <v>20</v>
+      </c>
       <c r="I270" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J270" t="s">
         <v>85</v>
@@ -13730,7 +14304,7 @@
       </c>
       <c r="N270" s="6"/>
     </row>
-    <row r="271" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="271" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A271" s="6" t="s">
         <v>44</v>
       </c>
@@ -13738,11 +14312,11 @@
         <v>11.52</v>
       </c>
       <c r="C271">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>6.09</v>
       </c>
       <c r="D271">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>16.95</v>
       </c>
       <c r="E271">
@@ -13754,9 +14328,11 @@
       <c r="G271" s="8">
         <v>14</v>
       </c>
-      <c r="H271" s="8"/>
+      <c r="H271" s="8">
+        <v>19</v>
+      </c>
       <c r="I271" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J271" t="s">
         <v>85</v>
@@ -13769,7 +14345,7 @@
       </c>
       <c r="N271" s="6"/>
     </row>
-    <row r="272" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="272" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A272" s="6" t="s">
         <v>45</v>
       </c>
@@ -13777,11 +14353,11 @@
         <v>12.71</v>
       </c>
       <c r="C272">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>7.2800000000000011</v>
       </c>
       <c r="D272">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>18.14</v>
       </c>
       <c r="E272">
@@ -13793,9 +14369,11 @@
       <c r="G272" s="8">
         <v>16</v>
       </c>
-      <c r="H272" s="8"/>
+      <c r="H272" s="8">
+        <v>14</v>
+      </c>
       <c r="I272" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J272" t="s">
         <v>85</v>
@@ -13816,11 +14394,11 @@
         <v>13.03</v>
       </c>
       <c r="C273">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>7.6</v>
       </c>
       <c r="D273">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>18.46</v>
       </c>
       <c r="E273">
@@ -13832,9 +14410,11 @@
       <c r="G273" s="8">
         <v>23</v>
       </c>
-      <c r="H273" s="8"/>
+      <c r="H273" s="8">
+        <v>18</v>
+      </c>
       <c r="I273" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J273" t="s">
         <v>85</v>
@@ -13855,11 +14435,11 @@
         <v>13.18</v>
       </c>
       <c r="C274">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>7.75</v>
       </c>
       <c r="D274">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>18.61</v>
       </c>
       <c r="E274">
@@ -13871,9 +14451,11 @@
       <c r="G274" s="8">
         <v>6</v>
       </c>
-      <c r="H274" s="8"/>
+      <c r="H274" s="8">
+        <v>16</v>
+      </c>
       <c r="I274" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J274" t="s">
         <v>85</v>
@@ -13894,11 +14476,11 @@
         <v>14.17</v>
       </c>
       <c r="C275">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>8.74</v>
       </c>
       <c r="D275">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>19.600000000000001</v>
       </c>
       <c r="E275">
@@ -13910,9 +14492,11 @@
       <c r="G275" s="8">
         <v>8</v>
       </c>
-      <c r="H275" s="8"/>
+      <c r="H275" s="8">
+        <v>15</v>
+      </c>
       <c r="I275" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J275" t="s">
         <v>85</v>
@@ -13933,11 +14517,11 @@
         <v>14.29</v>
       </c>
       <c r="C276">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>8.86</v>
       </c>
       <c r="D276">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>19.72</v>
       </c>
       <c r="E276">
@@ -13949,9 +14533,11 @@
       <c r="G276" s="8">
         <v>9</v>
       </c>
-      <c r="H276" s="8"/>
+      <c r="H276" s="8">
+        <v>7</v>
+      </c>
       <c r="I276" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J276" t="s">
         <v>85</v>
@@ -13972,11 +14558,11 @@
         <v>14.53</v>
       </c>
       <c r="C277">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>9.1</v>
       </c>
       <c r="D277">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>19.96</v>
       </c>
       <c r="E277">
@@ -13988,9 +14574,11 @@
       <c r="G277" s="8">
         <v>17</v>
       </c>
-      <c r="H277" s="8"/>
+      <c r="H277" s="8">
+        <v>23</v>
+      </c>
       <c r="I277" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J277" t="s">
         <v>85</v>
@@ -14011,11 +14599,11 @@
         <v>14.84</v>
       </c>
       <c r="C278">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>9.41</v>
       </c>
       <c r="D278">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>20.27</v>
       </c>
       <c r="E278">
@@ -14027,9 +14615,11 @@
       <c r="G278" s="8">
         <v>19</v>
       </c>
-      <c r="H278" s="8"/>
+      <c r="H278" s="8">
+        <v>15</v>
+      </c>
       <c r="I278" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J278" t="s">
         <v>85</v>
@@ -14050,11 +14640,11 @@
         <v>15.58</v>
       </c>
       <c r="C279">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>10.15</v>
       </c>
       <c r="D279">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>21.009999999999998</v>
       </c>
       <c r="E279">
@@ -14066,9 +14656,11 @@
       <c r="G279" s="8">
         <v>20</v>
       </c>
-      <c r="H279" s="8"/>
+      <c r="H279" s="8">
+        <v>22</v>
+      </c>
       <c r="I279" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J279" t="s">
         <v>85</v>
@@ -14089,11 +14681,11 @@
         <v>15.82</v>
       </c>
       <c r="C280">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>10.39</v>
       </c>
       <c r="D280">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>21.25</v>
       </c>
       <c r="E280">
@@ -14105,9 +14697,11 @@
       <c r="G280" s="8">
         <v>21</v>
       </c>
-      <c r="H280" s="8"/>
+      <c r="H280" s="8">
+        <v>13</v>
+      </c>
       <c r="I280" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J280" t="s">
         <v>85</v>
@@ -14128,11 +14722,11 @@
         <v>16.52</v>
       </c>
       <c r="C281">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>11.09</v>
       </c>
       <c r="D281">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>21.95</v>
       </c>
       <c r="E281">
@@ -14144,9 +14738,11 @@
       <c r="G281" s="8">
         <v>24</v>
       </c>
-      <c r="H281" s="8"/>
+      <c r="H281" s="8">
+        <v>21</v>
+      </c>
       <c r="I281" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J281" t="s">
         <v>85</v>
@@ -14167,11 +14763,11 @@
         <v>16.690000000000001</v>
       </c>
       <c r="C282">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>11.260000000000002</v>
       </c>
       <c r="D282">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>22.12</v>
       </c>
       <c r="E282">
@@ -14183,9 +14779,11 @@
       <c r="G282" s="8">
         <v>22</v>
       </c>
-      <c r="H282" s="8"/>
+      <c r="H282" s="8">
+        <v>12</v>
+      </c>
       <c r="I282" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J282" t="s">
         <v>85</v>
@@ -14206,11 +14804,11 @@
         <v>16.97</v>
       </c>
       <c r="C283">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>11.54</v>
       </c>
       <c r="D283">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>22.4</v>
       </c>
       <c r="E283">
@@ -14222,9 +14820,11 @@
       <c r="G283" s="8">
         <v>15</v>
       </c>
-      <c r="H283" s="8"/>
+      <c r="H283" s="8">
+        <v>25</v>
+      </c>
       <c r="I283" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J283" t="s">
         <v>85</v>
@@ -14245,11 +14845,11 @@
         <v>17.149999999999999</v>
       </c>
       <c r="C284">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>11.719999999999999</v>
       </c>
       <c r="D284">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>22.58</v>
       </c>
       <c r="E284">
@@ -14261,9 +14861,11 @@
       <c r="G284" s="8">
         <v>25</v>
       </c>
-      <c r="H284" s="8"/>
+      <c r="H284" s="8">
+        <v>24</v>
+      </c>
       <c r="I284" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J284" t="s">
         <v>85</v>
@@ -14567,8 +15169,8 @@
       <c r="H357" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N260:O284">
-    <sortCondition ref="O260:O284"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N210:O234">
+    <sortCondition ref="O210:O234"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24998,7 +25600,9 @@
       <c r="G250" s="8">
         <v>21</v>
       </c>
-      <c r="H250" s="8"/>
+      <c r="H250" s="8">
+        <v>8</v>
+      </c>
       <c r="I250" t="s">
         <v>109</v>
       </c>
@@ -25416,9 +26020,11 @@
       <c r="G260" s="8">
         <v>1</v>
       </c>
-      <c r="H260" s="8"/>
+      <c r="H260" s="8">
+        <v>1</v>
+      </c>
       <c r="I260" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J260" t="s">
         <v>85</v>
@@ -25456,9 +26062,11 @@
       <c r="G261" s="8">
         <v>7</v>
       </c>
-      <c r="H261" s="8"/>
+      <c r="H261" s="8">
+        <v>10</v>
+      </c>
       <c r="I261" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J261" t="s">
         <v>85</v>
@@ -25496,9 +26104,11 @@
       <c r="G262" s="8">
         <v>2</v>
       </c>
-      <c r="H262" s="8"/>
+      <c r="H262" s="8">
+        <v>7</v>
+      </c>
       <c r="I262" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J262" t="s">
         <v>85</v>
@@ -25536,9 +26146,11 @@
       <c r="G263" s="8">
         <v>3</v>
       </c>
-      <c r="H263" s="8"/>
+      <c r="H263" s="8">
+        <v>4</v>
+      </c>
       <c r="I263" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J263" t="s">
         <v>85</v>
@@ -25576,9 +26188,11 @@
       <c r="G264" s="8">
         <v>4</v>
       </c>
-      <c r="H264" s="8"/>
+      <c r="H264" s="8">
+        <v>25</v>
+      </c>
       <c r="I264" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J264" t="s">
         <v>85</v>
@@ -25616,9 +26230,11 @@
       <c r="G265" s="8">
         <v>5</v>
       </c>
-      <c r="H265" s="8"/>
+      <c r="H265" s="8">
+        <v>2</v>
+      </c>
       <c r="I265" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J265" t="s">
         <v>85</v>
@@ -25656,9 +26272,11 @@
       <c r="G266" s="8">
         <v>18</v>
       </c>
-      <c r="H266" s="8"/>
+      <c r="H266" s="8">
+        <v>6</v>
+      </c>
       <c r="I266" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J266" t="s">
         <v>85</v>
@@ -25696,9 +26314,11 @@
       <c r="G267" s="8">
         <v>9</v>
       </c>
-      <c r="H267" s="8"/>
+      <c r="H267" s="8">
+        <v>18</v>
+      </c>
       <c r="I267" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J267" t="s">
         <v>85</v>
@@ -25736,9 +26356,11 @@
       <c r="G268" s="8">
         <v>6</v>
       </c>
-      <c r="H268" s="8"/>
+      <c r="H268" s="8">
+        <v>17</v>
+      </c>
       <c r="I268" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J268" t="s">
         <v>85</v>
@@ -25776,9 +26398,11 @@
       <c r="G269" s="8">
         <v>11</v>
       </c>
-      <c r="H269" s="8"/>
+      <c r="H269" s="8">
+        <v>14</v>
+      </c>
       <c r="I269" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J269" t="s">
         <v>85</v>
@@ -25816,9 +26440,11 @@
       <c r="G270" s="8">
         <v>13</v>
       </c>
-      <c r="H270" s="8"/>
+      <c r="H270" s="8">
+        <v>8</v>
+      </c>
       <c r="I270" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J270" t="s">
         <v>85</v>
@@ -25856,9 +26482,11 @@
       <c r="G271" s="8">
         <v>21</v>
       </c>
-      <c r="H271" s="8"/>
+      <c r="H271" s="8">
+        <v>21</v>
+      </c>
       <c r="I271" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J271" t="s">
         <v>85</v>
@@ -25896,9 +26524,11 @@
       <c r="G272" s="8">
         <v>22</v>
       </c>
-      <c r="H272" s="8"/>
+      <c r="H272" s="8">
+        <v>16</v>
+      </c>
       <c r="I272" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J272" t="s">
         <v>85</v>
@@ -25936,9 +26566,11 @@
       <c r="G273" s="8">
         <v>14</v>
       </c>
-      <c r="H273" s="8"/>
+      <c r="H273" s="8">
+        <v>15</v>
+      </c>
       <c r="I273" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J273" t="s">
         <v>85</v>
@@ -25976,9 +26608,11 @@
       <c r="G274" s="8">
         <v>15</v>
       </c>
-      <c r="H274" s="8"/>
+      <c r="H274" s="8">
+        <v>20</v>
+      </c>
       <c r="I274" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J274" t="s">
         <v>85</v>
@@ -26016,9 +26650,11 @@
       <c r="G275" s="8">
         <v>8</v>
       </c>
-      <c r="H275" s="8"/>
+      <c r="H275" s="8">
+        <v>9</v>
+      </c>
       <c r="I275" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J275" t="s">
         <v>85</v>
@@ -26056,9 +26692,11 @@
       <c r="G276" s="8">
         <v>16</v>
       </c>
-      <c r="H276" s="8"/>
+      <c r="H276" s="8">
+        <v>3</v>
+      </c>
       <c r="I276" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J276" t="s">
         <v>85</v>
@@ -26096,9 +26734,11 @@
       <c r="G277" s="8">
         <v>23</v>
       </c>
-      <c r="H277" s="8"/>
+      <c r="H277" s="8">
+        <v>11</v>
+      </c>
       <c r="I277" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J277" t="s">
         <v>85</v>
@@ -26136,9 +26776,11 @@
       <c r="G278" s="8">
         <v>17</v>
       </c>
-      <c r="H278" s="8"/>
+      <c r="H278" s="8">
+        <v>23</v>
+      </c>
       <c r="I278" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J278" t="s">
         <v>85</v>
@@ -26176,9 +26818,11 @@
       <c r="G279" s="8">
         <v>19</v>
       </c>
-      <c r="H279" s="8"/>
+      <c r="H279" s="8">
+        <v>19</v>
+      </c>
       <c r="I279" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J279" t="s">
         <v>85</v>
@@ -26216,9 +26860,11 @@
       <c r="G280" s="8">
         <v>24</v>
       </c>
-      <c r="H280" s="8"/>
+      <c r="H280" s="8">
+        <v>12</v>
+      </c>
       <c r="I280" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J280" t="s">
         <v>85</v>
@@ -26256,9 +26902,11 @@
       <c r="G281" s="8">
         <v>10</v>
       </c>
-      <c r="H281" s="8"/>
+      <c r="H281" s="8">
+        <v>5</v>
+      </c>
       <c r="I281" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J281" t="s">
         <v>85</v>
@@ -26296,9 +26944,11 @@
       <c r="G282" s="8">
         <v>20</v>
       </c>
-      <c r="H282" s="8"/>
+      <c r="H282" s="8">
+        <v>13</v>
+      </c>
       <c r="I282" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J282" t="s">
         <v>85</v>
@@ -26336,9 +26986,11 @@
       <c r="G283" s="8">
         <v>12</v>
       </c>
-      <c r="H283" s="8"/>
+      <c r="H283" s="8">
+        <v>24</v>
+      </c>
       <c r="I283" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J283" t="s">
         <v>85</v>
@@ -26376,9 +27028,11 @@
       <c r="G284" s="8">
         <v>25</v>
       </c>
-      <c r="H284" s="8"/>
+      <c r="H284" s="8">
+        <v>22</v>
+      </c>
       <c r="I284" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J284" t="s">
         <v>85</v>
@@ -26414,9 +27068,11 @@
       <c r="G285" s="8">
         <v>7</v>
       </c>
-      <c r="H285" s="8"/>
+      <c r="H285" s="8">
+        <v>5</v>
+      </c>
       <c r="I285" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J285" t="s">
         <v>85</v>
@@ -26454,9 +27110,11 @@
       <c r="G286" s="8">
         <v>1</v>
       </c>
-      <c r="H286" s="8"/>
+      <c r="H286" s="8">
+        <v>2</v>
+      </c>
       <c r="I286" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J286" t="s">
         <v>85</v>
@@ -26494,9 +27152,11 @@
       <c r="G287" s="8">
         <v>2</v>
       </c>
-      <c r="H287" s="8"/>
+      <c r="H287" s="8">
+        <v>1</v>
+      </c>
       <c r="I287" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J287" t="s">
         <v>85</v>
@@ -26534,9 +27194,11 @@
       <c r="G288" s="8">
         <v>3</v>
       </c>
-      <c r="H288" s="8"/>
+      <c r="H288" s="8">
+        <v>25</v>
+      </c>
       <c r="I288" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J288" t="s">
         <v>85</v>
@@ -26574,9 +27236,11 @@
       <c r="G289" s="8">
         <v>4</v>
       </c>
-      <c r="H289" s="8"/>
+      <c r="H289" s="8">
+        <v>4</v>
+      </c>
       <c r="I289" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J289" t="s">
         <v>85</v>
@@ -26614,9 +27278,11 @@
       <c r="G290" s="8">
         <v>5</v>
       </c>
-      <c r="H290" s="8"/>
+      <c r="H290" s="8">
+        <v>14</v>
+      </c>
       <c r="I290" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J290" t="s">
         <v>85</v>
@@ -26654,9 +27320,11 @@
       <c r="G291" s="8">
         <v>11</v>
       </c>
-      <c r="H291" s="8"/>
+      <c r="H291" s="8">
+        <v>15</v>
+      </c>
       <c r="I291" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J291" t="s">
         <v>85</v>
@@ -26694,9 +27362,11 @@
       <c r="G292" s="8">
         <v>6</v>
       </c>
-      <c r="H292" s="8"/>
+      <c r="H292" s="8">
+        <v>20</v>
+      </c>
       <c r="I292" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J292" t="s">
         <v>85</v>
@@ -26734,9 +27404,11 @@
       <c r="G293" s="8">
         <v>12</v>
       </c>
-      <c r="H293" s="8"/>
+      <c r="H293" s="8">
+        <v>3</v>
+      </c>
       <c r="I293" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J293" t="s">
         <v>85</v>
@@ -26774,9 +27446,11 @@
       <c r="G294" s="8">
         <v>8</v>
       </c>
-      <c r="H294" s="8"/>
+      <c r="H294" s="8">
+        <v>7</v>
+      </c>
       <c r="I294" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J294" t="s">
         <v>85</v>
@@ -26814,9 +27488,11 @@
       <c r="G295" s="8">
         <v>13</v>
       </c>
-      <c r="H295" s="8"/>
+      <c r="H295" s="8">
+        <v>9</v>
+      </c>
       <c r="I295" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J295" t="s">
         <v>85</v>
@@ -26854,9 +27530,11 @@
       <c r="G296" s="8">
         <v>14</v>
       </c>
-      <c r="H296" s="8"/>
+      <c r="H296" s="8">
+        <v>13</v>
+      </c>
       <c r="I296" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J296" t="s">
         <v>85</v>
@@ -26894,9 +27572,11 @@
       <c r="G297" s="8">
         <v>21</v>
       </c>
-      <c r="H297" s="8"/>
+      <c r="H297" s="8">
+        <v>19</v>
+      </c>
       <c r="I297" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J297" t="s">
         <v>85</v>
@@ -26934,9 +27614,11 @@
       <c r="G298" s="8">
         <v>15</v>
       </c>
-      <c r="H298" s="8"/>
+      <c r="H298" s="8">
+        <v>16</v>
+      </c>
       <c r="I298" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J298" t="s">
         <v>85</v>
@@ -26974,9 +27656,11 @@
       <c r="G299" s="8">
         <v>16</v>
       </c>
-      <c r="H299" s="8"/>
+      <c r="H299" s="8">
+        <v>6</v>
+      </c>
       <c r="I299" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J299" t="s">
         <v>85</v>
@@ -27014,9 +27698,11 @@
       <c r="G300" s="8">
         <v>22</v>
       </c>
-      <c r="H300" s="8"/>
+      <c r="H300" s="8">
+        <v>12</v>
+      </c>
       <c r="I300" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J300" t="s">
         <v>85</v>
@@ -27054,9 +27740,11 @@
       <c r="G301" s="8">
         <v>17</v>
       </c>
-      <c r="H301" s="8"/>
+      <c r="H301" s="8">
+        <v>10</v>
+      </c>
       <c r="I301" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J301" t="s">
         <v>85</v>
@@ -27094,9 +27782,11 @@
       <c r="G302" s="8">
         <v>9</v>
       </c>
-      <c r="H302" s="8"/>
+      <c r="H302" s="8">
+        <v>11</v>
+      </c>
       <c r="I302" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J302" t="s">
         <v>85</v>
@@ -27134,9 +27824,11 @@
       <c r="G303" s="8">
         <v>23</v>
       </c>
-      <c r="H303" s="8"/>
+      <c r="H303" s="8">
+        <v>22</v>
+      </c>
       <c r="I303" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J303" t="s">
         <v>85</v>
@@ -27174,9 +27866,11 @@
       <c r="G304" s="8">
         <v>10</v>
       </c>
-      <c r="H304" s="8"/>
+      <c r="H304" s="8">
+        <v>8</v>
+      </c>
       <c r="I304" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J304" t="s">
         <v>85</v>
@@ -27214,9 +27908,11 @@
       <c r="G305" s="8">
         <v>18</v>
       </c>
-      <c r="H305" s="8"/>
+      <c r="H305" s="8">
+        <v>24</v>
+      </c>
       <c r="I305" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J305" t="s">
         <v>85</v>
@@ -27254,9 +27950,11 @@
       <c r="G306" s="8">
         <v>19</v>
       </c>
-      <c r="H306" s="8"/>
+      <c r="H306" s="8">
+        <v>17</v>
+      </c>
       <c r="I306" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J306" t="s">
         <v>85</v>
@@ -27294,9 +27992,11 @@
       <c r="G307" s="8">
         <v>24</v>
       </c>
-      <c r="H307" s="8"/>
+      <c r="H307" s="8">
+        <v>21</v>
+      </c>
       <c r="I307" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J307" t="s">
         <v>85</v>
@@ -27334,9 +28034,11 @@
       <c r="G308" s="8">
         <v>25</v>
       </c>
-      <c r="H308" s="8"/>
+      <c r="H308" s="8">
+        <v>18</v>
+      </c>
       <c r="I308" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J308" t="s">
         <v>85</v>
@@ -27374,9 +28076,11 @@
       <c r="G309" s="8">
         <v>20</v>
       </c>
-      <c r="H309" s="8"/>
+      <c r="H309" s="8">
+        <v>23</v>
+      </c>
       <c r="I309" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J309" t="s">
         <v>85</v>

</xml_diff>